<commit_message>
fix(workbook): gráficos sem texto sobreposto no Excel
- Título e legenda com overlay desligado: o Excel desenhava os dois por cima
  da área do gráfico e dos rótulos do eixo.
- Barras negativas (pago) sem inversão de cor: saíam brancas.
- Rankings (categorias, clientes, estados) com o valor na ponta da barra e
  sem eixo de valores, que ia para o topo e encostava no título.
- Rótulos das categorias como texto (strRef).
- O cache dos gráficos agora é gravado também no XML sem prefixo "c:"
  (openpyxl): o arquivo abre com os gráficos preenchidos sem recálculo.
- Nomes longos de fornecedor reduzem a fonte em vez de cortar; nota da aba
  Despesas em duas linhas para não passar por baixo do gráfico.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NefkA2otxn5XifgkSQBnwE
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v2.xlsx
+++ b/public/workbook_fechamento_v2.xlsx
@@ -209,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -307,6 +307,9 @@
     </xf>
     <xf numFmtId="166" fontId="13" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" shrinkToFit="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -481,6 +484,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -503,10 +507,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resultado'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -531,10 +536,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resultado'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -580,6 +586,11 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <strRef>
+              <f>'Resultado'!$C$4:$N$4</f>
+            </strRef>
+          </cat>
           <val>
             <numRef>
               <f>'Resultado'!$C$90:$N$90</f>
@@ -686,6 +697,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -744,6 +756,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -780,9 +793,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Redes'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -823,9 +836,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Redes'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -933,6 +946,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -991,6 +1005,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1013,10 +1028,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1041,10 +1057,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1151,6 +1168,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1209,6 +1227,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -1245,9 +1264,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1288,9 +1307,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1331,9 +1350,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1440,6 +1459,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1498,6 +1518,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1520,10 +1541,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Caixa'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1548,10 +1570,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Caixa'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1597,6 +1620,11 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <strRef>
+              <f>'Caixa'!$C$4:$N$4</f>
+            </strRef>
+          </cat>
           <val>
             <numRef>
               <f>'Caixa'!$C$13:$N$13</f>
@@ -1702,6 +1730,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1760,6 +1789,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1782,10 +1812,42 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="800" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="1B1411"/>
+                    </a:solidFill>
+                    <a:latin typeface="Montserrat"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="1B1411"/>
+                  </a:solidFill>
+                  <a:latin typeface="Montserrat"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Despesas'!$B$5:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1844,18 +1906,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="E4DCD2"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -1925,6 +1977,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1947,10 +2000,42 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="800" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="1B1411"/>
+                    </a:solidFill>
+                    <a:latin typeface="Montserrat"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="1B1411"/>
+                  </a:solidFill>
+                  <a:latin typeface="Montserrat"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Clientes'!$B$5:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2009,18 +2094,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="E4DCD2"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -2090,6 +2165,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2112,10 +2188,42 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="800" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="1B1411"/>
+                    </a:solidFill>
+                    <a:latin typeface="Montserrat"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="1B1411"/>
+                  </a:solidFill>
+                  <a:latin typeface="Montserrat"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Estados'!$B$5:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2174,18 +2282,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="E4DCD2"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -2255,6 +2353,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2277,10 +2376,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Capital de giro'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2305,10 +2405,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Capital de giro'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2415,6 +2516,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -2473,6 +2575,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2495,10 +2598,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Estoque'!$B$5:$B$28</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2523,10 +2627,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Estoque'!$B$5:$B$28</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2634,6 +2739,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -5257,51 +5363,51 @@
           <t>ganho no mês</t>
         </is>
       </c>
-      <c r="C6" s="43">
+      <c r="C6" s="44">
         <f>IF(AND(ISNUMBER(C5),ISNUMBER(Dados!$W$29)),C5-Dados!$W$29,"")</f>
         <v/>
       </c>
-      <c r="D6" s="43">
+      <c r="D6" s="44">
         <f>IF(AND(ISNUMBER(D5),ISNUMBER(C5)),D5-C5,"")</f>
         <v/>
       </c>
-      <c r="E6" s="43">
+      <c r="E6" s="44">
         <f>IF(AND(ISNUMBER(E5),ISNUMBER(D5)),E5-D5,"")</f>
         <v/>
       </c>
-      <c r="F6" s="43">
+      <c r="F6" s="44">
         <f>IF(AND(ISNUMBER(F5),ISNUMBER(E5)),F5-E5,"")</f>
         <v/>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="44">
         <f>IF(AND(ISNUMBER(G5),ISNUMBER(F5)),G5-F5,"")</f>
         <v/>
       </c>
-      <c r="H6" s="43">
+      <c r="H6" s="44">
         <f>IF(AND(ISNUMBER(H5),ISNUMBER(G5)),H5-G5,"")</f>
         <v/>
       </c>
-      <c r="I6" s="43">
+      <c r="I6" s="44">
         <f>IF(AND(ISNUMBER(I5),ISNUMBER(H5)),I5-H5,"")</f>
         <v/>
       </c>
-      <c r="J6" s="43">
+      <c r="J6" s="44">
         <f>IF(AND(ISNUMBER(J5),ISNUMBER(I5)),J5-I5,"")</f>
         <v/>
       </c>
-      <c r="K6" s="43">
+      <c r="K6" s="44">
         <f>IF(AND(ISNUMBER(K5),ISNUMBER(J5)),K5-J5,"")</f>
         <v/>
       </c>
-      <c r="L6" s="43">
+      <c r="L6" s="44">
         <f>IF(AND(ISNUMBER(L5),ISNUMBER(K5)),L5-K5,"")</f>
         <v/>
       </c>
-      <c r="M6" s="43">
+      <c r="M6" s="44">
         <f>IF(AND(ISNUMBER(M5),ISNUMBER(L5)),M5-L5,"")</f>
         <v/>
       </c>
-      <c r="N6" s="43">
+      <c r="N6" s="44">
         <f>IF(AND(ISNUMBER(N5),ISNUMBER(M5)),N5-M5,"")</f>
         <v/>
       </c>
@@ -5372,51 +5478,51 @@
           <t>ganho no mês</t>
         </is>
       </c>
-      <c r="C8" s="43">
+      <c r="C8" s="44">
         <f>IF(AND(ISNUMBER(C7),ISNUMBER(Dados!$X$29)),C7-Dados!$X$29,"")</f>
         <v/>
       </c>
-      <c r="D8" s="43">
+      <c r="D8" s="44">
         <f>IF(AND(ISNUMBER(D7),ISNUMBER(C7)),D7-C7,"")</f>
         <v/>
       </c>
-      <c r="E8" s="43">
+      <c r="E8" s="44">
         <f>IF(AND(ISNUMBER(E7),ISNUMBER(D7)),E7-D7,"")</f>
         <v/>
       </c>
-      <c r="F8" s="43">
+      <c r="F8" s="44">
         <f>IF(AND(ISNUMBER(F7),ISNUMBER(E7)),F7-E7,"")</f>
         <v/>
       </c>
-      <c r="G8" s="43">
+      <c r="G8" s="44">
         <f>IF(AND(ISNUMBER(G7),ISNUMBER(F7)),G7-F7,"")</f>
         <v/>
       </c>
-      <c r="H8" s="43">
+      <c r="H8" s="44">
         <f>IF(AND(ISNUMBER(H7),ISNUMBER(G7)),H7-G7,"")</f>
         <v/>
       </c>
-      <c r="I8" s="43">
+      <c r="I8" s="44">
         <f>IF(AND(ISNUMBER(I7),ISNUMBER(H7)),I7-H7,"")</f>
         <v/>
       </c>
-      <c r="J8" s="43">
+      <c r="J8" s="44">
         <f>IF(AND(ISNUMBER(J7),ISNUMBER(I7)),J7-I7,"")</f>
         <v/>
       </c>
-      <c r="K8" s="43">
+      <c r="K8" s="44">
         <f>IF(AND(ISNUMBER(K7),ISNUMBER(J7)),K7-J7,"")</f>
         <v/>
       </c>
-      <c r="L8" s="43">
+      <c r="L8" s="44">
         <f>IF(AND(ISNUMBER(L7),ISNUMBER(K7)),L7-K7,"")</f>
         <v/>
       </c>
-      <c r="M8" s="43">
+      <c r="M8" s="44">
         <f>IF(AND(ISNUMBER(M7),ISNUMBER(L7)),M7-L7,"")</f>
         <v/>
       </c>
-      <c r="N8" s="43">
+      <c r="N8" s="44">
         <f>IF(AND(ISNUMBER(N7),ISNUMBER(M7)),N7-M7,"")</f>
         <v/>
       </c>
@@ -5753,1854 +5859,1854 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>Rótulo</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="45" t="inlineStr">
         <is>
           <t>Fechado</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
+      <c r="D4" s="45" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="E4" s="44" t="inlineStr">
+      <c r="E4" s="45" t="inlineStr">
         <is>
           <t>Pago</t>
         </is>
       </c>
-      <c r="F4" s="44" t="inlineStr">
+      <c r="F4" s="45" t="inlineStr">
         <is>
           <t>Faturamento</t>
         </is>
       </c>
-      <c r="G4" s="44" t="inlineStr">
+      <c r="G4" s="45" t="inlineStr">
         <is>
           <t>Caixa final</t>
         </is>
       </c>
-      <c r="H4" s="44" t="inlineStr">
+      <c r="H4" s="45" t="inlineStr">
         <is>
           <t>Caixa calculado (ERP)</t>
         </is>
       </c>
-      <c r="I4" s="44" t="inlineStr">
+      <c r="I4" s="45" t="inlineStr">
         <is>
           <t>Ajuste ao extrato</t>
         </is>
       </c>
-      <c r="J4" s="44" t="inlineStr">
+      <c r="J4" s="45" t="inlineStr">
         <is>
           <t>Bloqueado</t>
         </is>
       </c>
-      <c r="K4" s="44" t="inlineStr">
+      <c r="K4" s="45" t="inlineStr">
         <is>
           <t>Estoque produtos</t>
         </is>
       </c>
-      <c r="L4" s="44" t="inlineStr">
+      <c r="L4" s="45" t="inlineStr">
         <is>
           <t>Estoque materiais</t>
         </is>
       </c>
-      <c r="M4" s="44" t="inlineStr">
+      <c r="M4" s="45" t="inlineStr">
         <is>
           <t>Receber a vencer 0-30</t>
         </is>
       </c>
-      <c r="N4" s="44" t="inlineStr">
+      <c r="N4" s="45" t="inlineStr">
         <is>
           <t>Receber a vencer 31-90</t>
         </is>
       </c>
-      <c r="O4" s="44" t="inlineStr">
+      <c r="O4" s="45" t="inlineStr">
         <is>
           <t>Receber a vencer &gt;90</t>
         </is>
       </c>
-      <c r="P4" s="44" t="inlineStr">
+      <c r="P4" s="45" t="inlineStr">
         <is>
           <t>Receber vencido 0-30</t>
         </is>
       </c>
-      <c r="Q4" s="44" t="inlineStr">
+      <c r="Q4" s="45" t="inlineStr">
         <is>
           <t>Receber vencido &gt;30</t>
         </is>
       </c>
-      <c r="R4" s="44" t="inlineStr">
+      <c r="R4" s="45" t="inlineStr">
         <is>
           <t>Pagar a vencer 0-30</t>
         </is>
       </c>
-      <c r="S4" s="44" t="inlineStr">
+      <c r="S4" s="45" t="inlineStr">
         <is>
           <t>Pagar a vencer 31-90</t>
         </is>
       </c>
-      <c r="T4" s="44" t="inlineStr">
+      <c r="T4" s="45" t="inlineStr">
         <is>
           <t>Pagar a vencer &gt;90</t>
         </is>
       </c>
-      <c r="U4" s="44" t="inlineStr">
+      <c r="U4" s="45" t="inlineStr">
         <is>
           <t>Pagar vencido 0-30</t>
         </is>
       </c>
-      <c r="V4" s="44" t="inlineStr">
+      <c r="V4" s="45" t="inlineStr">
         <is>
           <t>Pagar vencido &gt;30</t>
         </is>
       </c>
-      <c r="W4" s="44" t="inlineStr">
+      <c r="W4" s="45" t="inlineStr">
         <is>
           <t>Seguidores LinkedIn</t>
         </is>
       </c>
-      <c r="X4" s="44" t="inlineStr">
+      <c r="X4" s="45" t="inlineStr">
         <is>
           <t>Seguidores Instagram</t>
         </is>
       </c>
-      <c r="Y4" s="44" t="inlineStr">
+      <c r="Y4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 1</t>
         </is>
       </c>
-      <c r="Z4" s="44" t="inlineStr">
+      <c r="Z4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 2</t>
         </is>
       </c>
-      <c r="AA4" s="44" t="inlineStr">
+      <c r="AA4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 3</t>
         </is>
       </c>
-      <c r="AB4" s="44" t="inlineStr">
+      <c r="AB4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 4</t>
         </is>
       </c>
-      <c r="AC4" s="44" t="inlineStr">
+      <c r="AC4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 1</t>
         </is>
       </c>
-      <c r="AD4" s="44" t="inlineStr">
+      <c r="AD4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 2</t>
         </is>
       </c>
-      <c r="AE4" s="44" t="inlineStr">
+      <c r="AE4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 3</t>
         </is>
       </c>
-      <c r="AF4" s="44" t="inlineStr">
+      <c r="AF4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 4</t>
         </is>
       </c>
-      <c r="AH4" s="44" t="inlineStr">
+      <c r="AH4" s="45" t="inlineStr">
         <is>
           <t>Parâmetro</t>
         </is>
       </c>
-      <c r="AI4" s="44" t="inlineStr">
+      <c r="AI4" s="45" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="AK4" s="44" t="inlineStr">
+      <c r="AK4" s="45" t="inlineStr">
         <is>
           <t>Cliente (grupo)</t>
         </is>
       </c>
-      <c r="AL4" s="44" t="inlineStr">
+      <c r="AL4" s="45" t="inlineStr">
         <is>
           <t>1ª compra</t>
         </is>
       </c>
-      <c r="AN4" s="44" t="inlineStr">
+      <c r="AN4" s="45" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="AO4" s="44" t="inlineStr">
+      <c r="AO4" s="45" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="AQ4" s="44" t="inlineStr">
+      <c r="AQ4" s="45" t="inlineStr">
         <is>
           <t>Categoria de despesa</t>
         </is>
       </c>
-      <c r="AS4" s="44" t="inlineStr">
+      <c r="AS4" s="45" t="inlineStr">
         <is>
           <t>Fornecedor do mês</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="45" t="n"/>
-      <c r="B5" s="46" t="n"/>
-      <c r="C5" s="47" t="n"/>
-      <c r="D5" s="48" t="n"/>
-      <c r="E5" s="48" t="n"/>
-      <c r="F5" s="48" t="n"/>
-      <c r="G5" s="48" t="n"/>
-      <c r="H5" s="48" t="n"/>
-      <c r="I5" s="48" t="n"/>
-      <c r="J5" s="48" t="n"/>
-      <c r="K5" s="48" t="n"/>
-      <c r="L5" s="48" t="n"/>
-      <c r="M5" s="48" t="n"/>
-      <c r="N5" s="48" t="n"/>
-      <c r="O5" s="48" t="n"/>
-      <c r="P5" s="48" t="n"/>
-      <c r="Q5" s="48" t="n"/>
-      <c r="R5" s="48" t="n"/>
-      <c r="S5" s="48" t="n"/>
-      <c r="T5" s="48" t="n"/>
-      <c r="U5" s="48" t="n"/>
-      <c r="V5" s="48" t="n"/>
-      <c r="W5" s="49" t="n"/>
-      <c r="X5" s="49" t="n"/>
-      <c r="Y5" s="48" t="n"/>
-      <c r="Z5" s="48" t="n"/>
-      <c r="AA5" s="48" t="n"/>
-      <c r="AB5" s="48" t="n"/>
-      <c r="AC5" s="48" t="n"/>
-      <c r="AD5" s="48" t="n"/>
-      <c r="AE5" s="48" t="n"/>
-      <c r="AF5" s="48" t="n"/>
-      <c r="AH5" s="46" t="inlineStr">
+      <c r="A5" s="46" t="n"/>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="48" t="n"/>
+      <c r="D5" s="49" t="n"/>
+      <c r="E5" s="49" t="n"/>
+      <c r="F5" s="49" t="n"/>
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="49" t="n"/>
+      <c r="I5" s="49" t="n"/>
+      <c r="J5" s="49" t="n"/>
+      <c r="K5" s="49" t="n"/>
+      <c r="L5" s="49" t="n"/>
+      <c r="M5" s="49" t="n"/>
+      <c r="N5" s="49" t="n"/>
+      <c r="O5" s="49" t="n"/>
+      <c r="P5" s="49" t="n"/>
+      <c r="Q5" s="49" t="n"/>
+      <c r="R5" s="49" t="n"/>
+      <c r="S5" s="49" t="n"/>
+      <c r="T5" s="49" t="n"/>
+      <c r="U5" s="49" t="n"/>
+      <c r="V5" s="49" t="n"/>
+      <c r="W5" s="50" t="n"/>
+      <c r="X5" s="50" t="n"/>
+      <c r="Y5" s="49" t="n"/>
+      <c r="Z5" s="49" t="n"/>
+      <c r="AA5" s="49" t="n"/>
+      <c r="AB5" s="49" t="n"/>
+      <c r="AC5" s="49" t="n"/>
+      <c r="AD5" s="49" t="n"/>
+      <c r="AE5" s="49" t="n"/>
+      <c r="AF5" s="49" t="n"/>
+      <c r="AH5" s="47" t="inlineStr">
         <is>
           <t>Competência</t>
         </is>
       </c>
-      <c r="AI5" s="45" t="n"/>
-      <c r="AK5" s="46" t="n"/>
-      <c r="AL5" s="46" t="n"/>
-      <c r="AN5" s="46" t="n"/>
-      <c r="AO5" s="46" t="n"/>
-      <c r="AQ5" s="46" t="n"/>
-      <c r="AS5" s="46" t="n"/>
+      <c r="AI5" s="46" t="n"/>
+      <c r="AK5" s="47" t="n"/>
+      <c r="AL5" s="47" t="n"/>
+      <c r="AN5" s="47" t="n"/>
+      <c r="AO5" s="47" t="n"/>
+      <c r="AQ5" s="47" t="n"/>
+      <c r="AS5" s="47" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="45" t="n"/>
-      <c r="B6" s="46" t="n"/>
-      <c r="C6" s="47" t="n"/>
-      <c r="D6" s="48" t="n"/>
-      <c r="E6" s="48" t="n"/>
-      <c r="F6" s="48" t="n"/>
-      <c r="G6" s="48" t="n"/>
-      <c r="H6" s="48" t="n"/>
-      <c r="I6" s="48" t="n"/>
-      <c r="J6" s="48" t="n"/>
-      <c r="K6" s="48" t="n"/>
-      <c r="L6" s="48" t="n"/>
-      <c r="M6" s="48" t="n"/>
-      <c r="N6" s="48" t="n"/>
-      <c r="O6" s="48" t="n"/>
-      <c r="P6" s="48" t="n"/>
-      <c r="Q6" s="48" t="n"/>
-      <c r="R6" s="48" t="n"/>
-      <c r="S6" s="48" t="n"/>
-      <c r="T6" s="48" t="n"/>
-      <c r="U6" s="48" t="n"/>
-      <c r="V6" s="48" t="n"/>
-      <c r="W6" s="49" t="n"/>
-      <c r="X6" s="49" t="n"/>
-      <c r="Y6" s="48" t="n"/>
-      <c r="Z6" s="48" t="n"/>
-      <c r="AA6" s="48" t="n"/>
-      <c r="AB6" s="48" t="n"/>
-      <c r="AC6" s="48" t="n"/>
-      <c r="AD6" s="48" t="n"/>
-      <c r="AE6" s="48" t="n"/>
-      <c r="AF6" s="48" t="n"/>
-      <c r="AH6" s="46" t="inlineStr">
+      <c r="A6" s="46" t="n"/>
+      <c r="B6" s="47" t="n"/>
+      <c r="C6" s="48" t="n"/>
+      <c r="D6" s="49" t="n"/>
+      <c r="E6" s="49" t="n"/>
+      <c r="F6" s="49" t="n"/>
+      <c r="G6" s="49" t="n"/>
+      <c r="H6" s="49" t="n"/>
+      <c r="I6" s="49" t="n"/>
+      <c r="J6" s="49" t="n"/>
+      <c r="K6" s="49" t="n"/>
+      <c r="L6" s="49" t="n"/>
+      <c r="M6" s="49" t="n"/>
+      <c r="N6" s="49" t="n"/>
+      <c r="O6" s="49" t="n"/>
+      <c r="P6" s="49" t="n"/>
+      <c r="Q6" s="49" t="n"/>
+      <c r="R6" s="49" t="n"/>
+      <c r="S6" s="49" t="n"/>
+      <c r="T6" s="49" t="n"/>
+      <c r="U6" s="49" t="n"/>
+      <c r="V6" s="49" t="n"/>
+      <c r="W6" s="50" t="n"/>
+      <c r="X6" s="50" t="n"/>
+      <c r="Y6" s="49" t="n"/>
+      <c r="Z6" s="49" t="n"/>
+      <c r="AA6" s="49" t="n"/>
+      <c r="AB6" s="49" t="n"/>
+      <c r="AC6" s="49" t="n"/>
+      <c r="AD6" s="49" t="n"/>
+      <c r="AE6" s="49" t="n"/>
+      <c r="AF6" s="49" t="n"/>
+      <c r="AH6" s="47" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="AI6" s="47" t="n"/>
-      <c r="AK6" s="46" t="n"/>
-      <c r="AL6" s="46" t="n"/>
-      <c r="AN6" s="46" t="n"/>
-      <c r="AO6" s="46" t="n"/>
-      <c r="AQ6" s="46" t="n"/>
-      <c r="AS6" s="46" t="n"/>
+      <c r="AI6" s="48" t="n"/>
+      <c r="AK6" s="47" t="n"/>
+      <c r="AL6" s="47" t="n"/>
+      <c r="AN6" s="47" t="n"/>
+      <c r="AO6" s="47" t="n"/>
+      <c r="AQ6" s="47" t="n"/>
+      <c r="AS6" s="47" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="45" t="n"/>
-      <c r="B7" s="46" t="n"/>
-      <c r="C7" s="47" t="n"/>
-      <c r="D7" s="48" t="n"/>
-      <c r="E7" s="48" t="n"/>
-      <c r="F7" s="48" t="n"/>
-      <c r="G7" s="48" t="n"/>
-      <c r="H7" s="48" t="n"/>
-      <c r="I7" s="48" t="n"/>
-      <c r="J7" s="48" t="n"/>
-      <c r="K7" s="48" t="n"/>
-      <c r="L7" s="48" t="n"/>
-      <c r="M7" s="48" t="n"/>
-      <c r="N7" s="48" t="n"/>
-      <c r="O7" s="48" t="n"/>
-      <c r="P7" s="48" t="n"/>
-      <c r="Q7" s="48" t="n"/>
-      <c r="R7" s="48" t="n"/>
-      <c r="S7" s="48" t="n"/>
-      <c r="T7" s="48" t="n"/>
-      <c r="U7" s="48" t="n"/>
-      <c r="V7" s="48" t="n"/>
-      <c r="W7" s="49" t="n"/>
-      <c r="X7" s="49" t="n"/>
-      <c r="Y7" s="48" t="n"/>
-      <c r="Z7" s="48" t="n"/>
-      <c r="AA7" s="48" t="n"/>
-      <c r="AB7" s="48" t="n"/>
-      <c r="AC7" s="48" t="n"/>
-      <c r="AD7" s="48" t="n"/>
-      <c r="AE7" s="48" t="n"/>
-      <c r="AF7" s="48" t="n"/>
-      <c r="AH7" s="46" t="inlineStr">
+      <c r="A7" s="46" t="n"/>
+      <c r="B7" s="47" t="n"/>
+      <c r="C7" s="48" t="n"/>
+      <c r="D7" s="49" t="n"/>
+      <c r="E7" s="49" t="n"/>
+      <c r="F7" s="49" t="n"/>
+      <c r="G7" s="49" t="n"/>
+      <c r="H7" s="49" t="n"/>
+      <c r="I7" s="49" t="n"/>
+      <c r="J7" s="49" t="n"/>
+      <c r="K7" s="49" t="n"/>
+      <c r="L7" s="49" t="n"/>
+      <c r="M7" s="49" t="n"/>
+      <c r="N7" s="49" t="n"/>
+      <c r="O7" s="49" t="n"/>
+      <c r="P7" s="49" t="n"/>
+      <c r="Q7" s="49" t="n"/>
+      <c r="R7" s="49" t="n"/>
+      <c r="S7" s="49" t="n"/>
+      <c r="T7" s="49" t="n"/>
+      <c r="U7" s="49" t="n"/>
+      <c r="V7" s="49" t="n"/>
+      <c r="W7" s="50" t="n"/>
+      <c r="X7" s="50" t="n"/>
+      <c r="Y7" s="49" t="n"/>
+      <c r="Z7" s="49" t="n"/>
+      <c r="AA7" s="49" t="n"/>
+      <c r="AB7" s="49" t="n"/>
+      <c r="AC7" s="49" t="n"/>
+      <c r="AD7" s="49" t="n"/>
+      <c r="AE7" s="49" t="n"/>
+      <c r="AF7" s="49" t="n"/>
+      <c r="AH7" s="47" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="AI7" s="47" t="n"/>
-      <c r="AK7" s="46" t="n"/>
-      <c r="AL7" s="46" t="n"/>
-      <c r="AN7" s="46" t="n"/>
-      <c r="AO7" s="46" t="n"/>
-      <c r="AQ7" s="46" t="n"/>
-      <c r="AS7" s="46" t="n"/>
+      <c r="AI7" s="48" t="n"/>
+      <c r="AK7" s="47" t="n"/>
+      <c r="AL7" s="47" t="n"/>
+      <c r="AN7" s="47" t="n"/>
+      <c r="AO7" s="47" t="n"/>
+      <c r="AQ7" s="47" t="n"/>
+      <c r="AS7" s="47" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="45" t="n"/>
-      <c r="B8" s="46" t="n"/>
-      <c r="C8" s="47" t="n"/>
-      <c r="D8" s="48" t="n"/>
-      <c r="E8" s="48" t="n"/>
-      <c r="F8" s="48" t="n"/>
-      <c r="G8" s="48" t="n"/>
-      <c r="H8" s="48" t="n"/>
-      <c r="I8" s="48" t="n"/>
-      <c r="J8" s="48" t="n"/>
-      <c r="K8" s="48" t="n"/>
-      <c r="L8" s="48" t="n"/>
-      <c r="M8" s="48" t="n"/>
-      <c r="N8" s="48" t="n"/>
-      <c r="O8" s="48" t="n"/>
-      <c r="P8" s="48" t="n"/>
-      <c r="Q8" s="48" t="n"/>
-      <c r="R8" s="48" t="n"/>
-      <c r="S8" s="48" t="n"/>
-      <c r="T8" s="48" t="n"/>
-      <c r="U8" s="48" t="n"/>
-      <c r="V8" s="48" t="n"/>
-      <c r="W8" s="49" t="n"/>
-      <c r="X8" s="49" t="n"/>
-      <c r="Y8" s="48" t="n"/>
-      <c r="Z8" s="48" t="n"/>
-      <c r="AA8" s="48" t="n"/>
-      <c r="AB8" s="48" t="n"/>
-      <c r="AC8" s="48" t="n"/>
-      <c r="AD8" s="48" t="n"/>
-      <c r="AE8" s="48" t="n"/>
-      <c r="AF8" s="48" t="n"/>
-      <c r="AH8" s="46" t="inlineStr">
+      <c r="A8" s="46" t="n"/>
+      <c r="B8" s="47" t="n"/>
+      <c r="C8" s="48" t="n"/>
+      <c r="D8" s="49" t="n"/>
+      <c r="E8" s="49" t="n"/>
+      <c r="F8" s="49" t="n"/>
+      <c r="G8" s="49" t="n"/>
+      <c r="H8" s="49" t="n"/>
+      <c r="I8" s="49" t="n"/>
+      <c r="J8" s="49" t="n"/>
+      <c r="K8" s="49" t="n"/>
+      <c r="L8" s="49" t="n"/>
+      <c r="M8" s="49" t="n"/>
+      <c r="N8" s="49" t="n"/>
+      <c r="O8" s="49" t="n"/>
+      <c r="P8" s="49" t="n"/>
+      <c r="Q8" s="49" t="n"/>
+      <c r="R8" s="49" t="n"/>
+      <c r="S8" s="49" t="n"/>
+      <c r="T8" s="49" t="n"/>
+      <c r="U8" s="49" t="n"/>
+      <c r="V8" s="49" t="n"/>
+      <c r="W8" s="50" t="n"/>
+      <c r="X8" s="50" t="n"/>
+      <c r="Y8" s="49" t="n"/>
+      <c r="Z8" s="49" t="n"/>
+      <c r="AA8" s="49" t="n"/>
+      <c r="AB8" s="49" t="n"/>
+      <c r="AC8" s="49" t="n"/>
+      <c r="AD8" s="49" t="n"/>
+      <c r="AE8" s="49" t="n"/>
+      <c r="AF8" s="49" t="n"/>
+      <c r="AH8" s="47" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="AI8" s="46" t="n"/>
-      <c r="AK8" s="46" t="n"/>
-      <c r="AL8" s="46" t="n"/>
-      <c r="AN8" s="46" t="n"/>
-      <c r="AO8" s="46" t="n"/>
-      <c r="AQ8" s="46" t="n"/>
-      <c r="AS8" s="46" t="n"/>
+      <c r="AI8" s="47" t="n"/>
+      <c r="AK8" s="47" t="n"/>
+      <c r="AL8" s="47" t="n"/>
+      <c r="AN8" s="47" t="n"/>
+      <c r="AO8" s="47" t="n"/>
+      <c r="AQ8" s="47" t="n"/>
+      <c r="AS8" s="47" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="45" t="n"/>
-      <c r="B9" s="46" t="n"/>
-      <c r="C9" s="47" t="n"/>
-      <c r="D9" s="48" t="n"/>
-      <c r="E9" s="48" t="n"/>
-      <c r="F9" s="48" t="n"/>
-      <c r="G9" s="48" t="n"/>
-      <c r="H9" s="48" t="n"/>
-      <c r="I9" s="48" t="n"/>
-      <c r="J9" s="48" t="n"/>
-      <c r="K9" s="48" t="n"/>
-      <c r="L9" s="48" t="n"/>
-      <c r="M9" s="48" t="n"/>
-      <c r="N9" s="48" t="n"/>
-      <c r="O9" s="48" t="n"/>
-      <c r="P9" s="48" t="n"/>
-      <c r="Q9" s="48" t="n"/>
-      <c r="R9" s="48" t="n"/>
-      <c r="S9" s="48" t="n"/>
-      <c r="T9" s="48" t="n"/>
-      <c r="U9" s="48" t="n"/>
-      <c r="V9" s="48" t="n"/>
-      <c r="W9" s="49" t="n"/>
-      <c r="X9" s="49" t="n"/>
-      <c r="Y9" s="48" t="n"/>
-      <c r="Z9" s="48" t="n"/>
-      <c r="AA9" s="48" t="n"/>
-      <c r="AB9" s="48" t="n"/>
-      <c r="AC9" s="48" t="n"/>
-      <c r="AD9" s="48" t="n"/>
-      <c r="AE9" s="48" t="n"/>
-      <c r="AF9" s="48" t="n"/>
-      <c r="AH9" s="46" t="inlineStr">
+      <c r="A9" s="46" t="n"/>
+      <c r="B9" s="47" t="n"/>
+      <c r="C9" s="48" t="n"/>
+      <c r="D9" s="49" t="n"/>
+      <c r="E9" s="49" t="n"/>
+      <c r="F9" s="49" t="n"/>
+      <c r="G9" s="49" t="n"/>
+      <c r="H9" s="49" t="n"/>
+      <c r="I9" s="49" t="n"/>
+      <c r="J9" s="49" t="n"/>
+      <c r="K9" s="49" t="n"/>
+      <c r="L9" s="49" t="n"/>
+      <c r="M9" s="49" t="n"/>
+      <c r="N9" s="49" t="n"/>
+      <c r="O9" s="49" t="n"/>
+      <c r="P9" s="49" t="n"/>
+      <c r="Q9" s="49" t="n"/>
+      <c r="R9" s="49" t="n"/>
+      <c r="S9" s="49" t="n"/>
+      <c r="T9" s="49" t="n"/>
+      <c r="U9" s="49" t="n"/>
+      <c r="V9" s="49" t="n"/>
+      <c r="W9" s="50" t="n"/>
+      <c r="X9" s="50" t="n"/>
+      <c r="Y9" s="49" t="n"/>
+      <c r="Z9" s="49" t="n"/>
+      <c r="AA9" s="49" t="n"/>
+      <c r="AB9" s="49" t="n"/>
+      <c r="AC9" s="49" t="n"/>
+      <c r="AD9" s="49" t="n"/>
+      <c r="AE9" s="49" t="n"/>
+      <c r="AF9" s="49" t="n"/>
+      <c r="AH9" s="47" t="inlineStr">
         <is>
           <t>Data-base</t>
         </is>
       </c>
-      <c r="AI9" s="50" t="n"/>
-      <c r="AK9" s="46" t="n"/>
-      <c r="AL9" s="46" t="n"/>
-      <c r="AN9" s="46" t="n"/>
-      <c r="AO9" s="46" t="n"/>
-      <c r="AQ9" s="46" t="n"/>
-      <c r="AS9" s="46" t="n"/>
+      <c r="AI9" s="51" t="n"/>
+      <c r="AK9" s="47" t="n"/>
+      <c r="AL9" s="47" t="n"/>
+      <c r="AN9" s="47" t="n"/>
+      <c r="AO9" s="47" t="n"/>
+      <c r="AQ9" s="47" t="n"/>
+      <c r="AS9" s="47" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="45" t="n"/>
-      <c r="B10" s="46" t="n"/>
-      <c r="C10" s="47" t="n"/>
-      <c r="D10" s="48" t="n"/>
-      <c r="E10" s="48" t="n"/>
-      <c r="F10" s="48" t="n"/>
-      <c r="G10" s="48" t="n"/>
-      <c r="H10" s="48" t="n"/>
-      <c r="I10" s="48" t="n"/>
-      <c r="J10" s="48" t="n"/>
-      <c r="K10" s="48" t="n"/>
-      <c r="L10" s="48" t="n"/>
-      <c r="M10" s="48" t="n"/>
-      <c r="N10" s="48" t="n"/>
-      <c r="O10" s="48" t="n"/>
-      <c r="P10" s="48" t="n"/>
-      <c r="Q10" s="48" t="n"/>
-      <c r="R10" s="48" t="n"/>
-      <c r="S10" s="48" t="n"/>
-      <c r="T10" s="48" t="n"/>
-      <c r="U10" s="48" t="n"/>
-      <c r="V10" s="48" t="n"/>
-      <c r="W10" s="49" t="n"/>
-      <c r="X10" s="49" t="n"/>
-      <c r="Y10" s="48" t="n"/>
-      <c r="Z10" s="48" t="n"/>
-      <c r="AA10" s="48" t="n"/>
-      <c r="AB10" s="48" t="n"/>
-      <c r="AC10" s="48" t="n"/>
-      <c r="AD10" s="48" t="n"/>
-      <c r="AE10" s="48" t="n"/>
-      <c r="AF10" s="48" t="n"/>
-      <c r="AH10" s="46" t="inlineStr">
+      <c r="A10" s="46" t="n"/>
+      <c r="B10" s="47" t="n"/>
+      <c r="C10" s="48" t="n"/>
+      <c r="D10" s="49" t="n"/>
+      <c r="E10" s="49" t="n"/>
+      <c r="F10" s="49" t="n"/>
+      <c r="G10" s="49" t="n"/>
+      <c r="H10" s="49" t="n"/>
+      <c r="I10" s="49" t="n"/>
+      <c r="J10" s="49" t="n"/>
+      <c r="K10" s="49" t="n"/>
+      <c r="L10" s="49" t="n"/>
+      <c r="M10" s="49" t="n"/>
+      <c r="N10" s="49" t="n"/>
+      <c r="O10" s="49" t="n"/>
+      <c r="P10" s="49" t="n"/>
+      <c r="Q10" s="49" t="n"/>
+      <c r="R10" s="49" t="n"/>
+      <c r="S10" s="49" t="n"/>
+      <c r="T10" s="49" t="n"/>
+      <c r="U10" s="49" t="n"/>
+      <c r="V10" s="49" t="n"/>
+      <c r="W10" s="50" t="n"/>
+      <c r="X10" s="50" t="n"/>
+      <c r="Y10" s="49" t="n"/>
+      <c r="Z10" s="49" t="n"/>
+      <c r="AA10" s="49" t="n"/>
+      <c r="AB10" s="49" t="n"/>
+      <c r="AC10" s="49" t="n"/>
+      <c r="AD10" s="49" t="n"/>
+      <c r="AE10" s="49" t="n"/>
+      <c r="AF10" s="49" t="n"/>
+      <c r="AH10" s="47" t="inlineStr">
         <is>
           <t>Gerado em</t>
         </is>
       </c>
-      <c r="AI10" s="50" t="n"/>
-      <c r="AK10" s="46" t="n"/>
-      <c r="AL10" s="46" t="n"/>
-      <c r="AN10" s="46" t="n"/>
-      <c r="AO10" s="46" t="n"/>
-      <c r="AQ10" s="46" t="n"/>
-      <c r="AS10" s="46" t="n"/>
+      <c r="AI10" s="51" t="n"/>
+      <c r="AK10" s="47" t="n"/>
+      <c r="AL10" s="47" t="n"/>
+      <c r="AN10" s="47" t="n"/>
+      <c r="AO10" s="47" t="n"/>
+      <c r="AQ10" s="47" t="n"/>
+      <c r="AS10" s="47" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="45" t="n"/>
-      <c r="B11" s="46" t="n"/>
-      <c r="C11" s="47" t="n"/>
-      <c r="D11" s="48" t="n"/>
-      <c r="E11" s="48" t="n"/>
-      <c r="F11" s="48" t="n"/>
-      <c r="G11" s="48" t="n"/>
-      <c r="H11" s="48" t="n"/>
-      <c r="I11" s="48" t="n"/>
-      <c r="J11" s="48" t="n"/>
-      <c r="K11" s="48" t="n"/>
-      <c r="L11" s="48" t="n"/>
-      <c r="M11" s="48" t="n"/>
-      <c r="N11" s="48" t="n"/>
-      <c r="O11" s="48" t="n"/>
-      <c r="P11" s="48" t="n"/>
-      <c r="Q11" s="48" t="n"/>
-      <c r="R11" s="48" t="n"/>
-      <c r="S11" s="48" t="n"/>
-      <c r="T11" s="48" t="n"/>
-      <c r="U11" s="48" t="n"/>
-      <c r="V11" s="48" t="n"/>
-      <c r="W11" s="49" t="n"/>
-      <c r="X11" s="49" t="n"/>
-      <c r="Y11" s="48" t="n"/>
-      <c r="Z11" s="48" t="n"/>
-      <c r="AA11" s="48" t="n"/>
-      <c r="AB11" s="48" t="n"/>
-      <c r="AC11" s="48" t="n"/>
-      <c r="AD11" s="48" t="n"/>
-      <c r="AE11" s="48" t="n"/>
-      <c r="AF11" s="48" t="n"/>
-      <c r="AH11" s="46" t="inlineStr">
+      <c r="A11" s="46" t="n"/>
+      <c r="B11" s="47" t="n"/>
+      <c r="C11" s="48" t="n"/>
+      <c r="D11" s="49" t="n"/>
+      <c r="E11" s="49" t="n"/>
+      <c r="F11" s="49" t="n"/>
+      <c r="G11" s="49" t="n"/>
+      <c r="H11" s="49" t="n"/>
+      <c r="I11" s="49" t="n"/>
+      <c r="J11" s="49" t="n"/>
+      <c r="K11" s="49" t="n"/>
+      <c r="L11" s="49" t="n"/>
+      <c r="M11" s="49" t="n"/>
+      <c r="N11" s="49" t="n"/>
+      <c r="O11" s="49" t="n"/>
+      <c r="P11" s="49" t="n"/>
+      <c r="Q11" s="49" t="n"/>
+      <c r="R11" s="49" t="n"/>
+      <c r="S11" s="49" t="n"/>
+      <c r="T11" s="49" t="n"/>
+      <c r="U11" s="49" t="n"/>
+      <c r="V11" s="49" t="n"/>
+      <c r="W11" s="50" t="n"/>
+      <c r="X11" s="50" t="n"/>
+      <c r="Y11" s="49" t="n"/>
+      <c r="Z11" s="49" t="n"/>
+      <c r="AA11" s="49" t="n"/>
+      <c r="AB11" s="49" t="n"/>
+      <c r="AC11" s="49" t="n"/>
+      <c r="AD11" s="49" t="n"/>
+      <c r="AE11" s="49" t="n"/>
+      <c r="AF11" s="49" t="n"/>
+      <c r="AH11" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano</t>
         </is>
       </c>
-      <c r="AI11" s="51" t="n"/>
-      <c r="AK11" s="46" t="n"/>
-      <c r="AL11" s="46" t="n"/>
-      <c r="AN11" s="46" t="n"/>
-      <c r="AO11" s="46" t="n"/>
-      <c r="AQ11" s="46" t="n"/>
-      <c r="AS11" s="46" t="n"/>
+      <c r="AI11" s="52" t="n"/>
+      <c r="AK11" s="47" t="n"/>
+      <c r="AL11" s="47" t="n"/>
+      <c r="AN11" s="47" t="n"/>
+      <c r="AO11" s="47" t="n"/>
+      <c r="AQ11" s="47" t="n"/>
+      <c r="AS11" s="47" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="45" t="n"/>
-      <c r="B12" s="46" t="n"/>
-      <c r="C12" s="47" t="n"/>
-      <c r="D12" s="48" t="n"/>
-      <c r="E12" s="48" t="n"/>
-      <c r="F12" s="48" t="n"/>
-      <c r="G12" s="48" t="n"/>
-      <c r="H12" s="48" t="n"/>
-      <c r="I12" s="48" t="n"/>
-      <c r="J12" s="48" t="n"/>
-      <c r="K12" s="48" t="n"/>
-      <c r="L12" s="48" t="n"/>
-      <c r="M12" s="48" t="n"/>
-      <c r="N12" s="48" t="n"/>
-      <c r="O12" s="48" t="n"/>
-      <c r="P12" s="48" t="n"/>
-      <c r="Q12" s="48" t="n"/>
-      <c r="R12" s="48" t="n"/>
-      <c r="S12" s="48" t="n"/>
-      <c r="T12" s="48" t="n"/>
-      <c r="U12" s="48" t="n"/>
-      <c r="V12" s="48" t="n"/>
-      <c r="W12" s="49" t="n"/>
-      <c r="X12" s="49" t="n"/>
-      <c r="Y12" s="48" t="n"/>
-      <c r="Z12" s="48" t="n"/>
-      <c r="AA12" s="48" t="n"/>
-      <c r="AB12" s="48" t="n"/>
-      <c r="AC12" s="48" t="n"/>
-      <c r="AD12" s="48" t="n"/>
-      <c r="AE12" s="48" t="n"/>
-      <c r="AF12" s="48" t="n"/>
-      <c r="AH12" s="46" t="inlineStr">
+      <c r="A12" s="46" t="n"/>
+      <c r="B12" s="47" t="n"/>
+      <c r="C12" s="48" t="n"/>
+      <c r="D12" s="49" t="n"/>
+      <c r="E12" s="49" t="n"/>
+      <c r="F12" s="49" t="n"/>
+      <c r="G12" s="49" t="n"/>
+      <c r="H12" s="49" t="n"/>
+      <c r="I12" s="49" t="n"/>
+      <c r="J12" s="49" t="n"/>
+      <c r="K12" s="49" t="n"/>
+      <c r="L12" s="49" t="n"/>
+      <c r="M12" s="49" t="n"/>
+      <c r="N12" s="49" t="n"/>
+      <c r="O12" s="49" t="n"/>
+      <c r="P12" s="49" t="n"/>
+      <c r="Q12" s="49" t="n"/>
+      <c r="R12" s="49" t="n"/>
+      <c r="S12" s="49" t="n"/>
+      <c r="T12" s="49" t="n"/>
+      <c r="U12" s="49" t="n"/>
+      <c r="V12" s="49" t="n"/>
+      <c r="W12" s="50" t="n"/>
+      <c r="X12" s="50" t="n"/>
+      <c r="Y12" s="49" t="n"/>
+      <c r="Z12" s="49" t="n"/>
+      <c r="AA12" s="49" t="n"/>
+      <c r="AB12" s="49" t="n"/>
+      <c r="AC12" s="49" t="n"/>
+      <c r="AD12" s="49" t="n"/>
+      <c r="AE12" s="49" t="n"/>
+      <c r="AF12" s="49" t="n"/>
+      <c r="AH12" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano anterior</t>
         </is>
       </c>
-      <c r="AI12" s="51" t="n"/>
-      <c r="AK12" s="46" t="n"/>
-      <c r="AL12" s="46" t="n"/>
-      <c r="AN12" s="46" t="n"/>
-      <c r="AO12" s="46" t="n"/>
-      <c r="AQ12" s="46" t="n"/>
-      <c r="AS12" s="46" t="n"/>
+      <c r="AI12" s="52" t="n"/>
+      <c r="AK12" s="47" t="n"/>
+      <c r="AL12" s="47" t="n"/>
+      <c r="AN12" s="47" t="n"/>
+      <c r="AO12" s="47" t="n"/>
+      <c r="AQ12" s="47" t="n"/>
+      <c r="AS12" s="47" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="45" t="n"/>
-      <c r="B13" s="46" t="n"/>
-      <c r="C13" s="47" t="n"/>
-      <c r="D13" s="48" t="n"/>
-      <c r="E13" s="48" t="n"/>
-      <c r="F13" s="48" t="n"/>
-      <c r="G13" s="48" t="n"/>
-      <c r="H13" s="48" t="n"/>
-      <c r="I13" s="48" t="n"/>
-      <c r="J13" s="48" t="n"/>
-      <c r="K13" s="48" t="n"/>
-      <c r="L13" s="48" t="n"/>
-      <c r="M13" s="48" t="n"/>
-      <c r="N13" s="48" t="n"/>
-      <c r="O13" s="48" t="n"/>
-      <c r="P13" s="48" t="n"/>
-      <c r="Q13" s="48" t="n"/>
-      <c r="R13" s="48" t="n"/>
-      <c r="S13" s="48" t="n"/>
-      <c r="T13" s="48" t="n"/>
-      <c r="U13" s="48" t="n"/>
-      <c r="V13" s="48" t="n"/>
-      <c r="W13" s="49" t="n"/>
-      <c r="X13" s="49" t="n"/>
-      <c r="Y13" s="48" t="n"/>
-      <c r="Z13" s="48" t="n"/>
-      <c r="AA13" s="48" t="n"/>
-      <c r="AB13" s="48" t="n"/>
-      <c r="AC13" s="48" t="n"/>
-      <c r="AD13" s="48" t="n"/>
-      <c r="AE13" s="48" t="n"/>
-      <c r="AF13" s="48" t="n"/>
-      <c r="AH13" s="46" t="inlineStr">
+      <c r="A13" s="46" t="n"/>
+      <c r="B13" s="47" t="n"/>
+      <c r="C13" s="48" t="n"/>
+      <c r="D13" s="49" t="n"/>
+      <c r="E13" s="49" t="n"/>
+      <c r="F13" s="49" t="n"/>
+      <c r="G13" s="49" t="n"/>
+      <c r="H13" s="49" t="n"/>
+      <c r="I13" s="49" t="n"/>
+      <c r="J13" s="49" t="n"/>
+      <c r="K13" s="49" t="n"/>
+      <c r="L13" s="49" t="n"/>
+      <c r="M13" s="49" t="n"/>
+      <c r="N13" s="49" t="n"/>
+      <c r="O13" s="49" t="n"/>
+      <c r="P13" s="49" t="n"/>
+      <c r="Q13" s="49" t="n"/>
+      <c r="R13" s="49" t="n"/>
+      <c r="S13" s="49" t="n"/>
+      <c r="T13" s="49" t="n"/>
+      <c r="U13" s="49" t="n"/>
+      <c r="V13" s="49" t="n"/>
+      <c r="W13" s="50" t="n"/>
+      <c r="X13" s="50" t="n"/>
+      <c r="Y13" s="49" t="n"/>
+      <c r="Z13" s="49" t="n"/>
+      <c r="AA13" s="49" t="n"/>
+      <c r="AB13" s="49" t="n"/>
+      <c r="AC13" s="49" t="n"/>
+      <c r="AD13" s="49" t="n"/>
+      <c r="AE13" s="49" t="n"/>
+      <c r="AF13" s="49" t="n"/>
+      <c r="AH13" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-2)</t>
         </is>
       </c>
-      <c r="AI13" s="48" t="n"/>
-      <c r="AK13" s="46" t="n"/>
-      <c r="AL13" s="46" t="n"/>
-      <c r="AN13" s="46" t="n"/>
-      <c r="AO13" s="46" t="n"/>
-      <c r="AQ13" s="46" t="n"/>
-      <c r="AS13" s="46" t="n"/>
+      <c r="AI13" s="49" t="n"/>
+      <c r="AK13" s="47" t="n"/>
+      <c r="AL13" s="47" t="n"/>
+      <c r="AN13" s="47" t="n"/>
+      <c r="AO13" s="47" t="n"/>
+      <c r="AQ13" s="47" t="n"/>
+      <c r="AS13" s="47" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="45" t="n"/>
-      <c r="B14" s="46" t="n"/>
-      <c r="C14" s="47" t="n"/>
-      <c r="D14" s="48" t="n"/>
-      <c r="E14" s="48" t="n"/>
-      <c r="F14" s="48" t="n"/>
-      <c r="G14" s="48" t="n"/>
-      <c r="H14" s="48" t="n"/>
-      <c r="I14" s="48" t="n"/>
-      <c r="J14" s="48" t="n"/>
-      <c r="K14" s="48" t="n"/>
-      <c r="L14" s="48" t="n"/>
-      <c r="M14" s="48" t="n"/>
-      <c r="N14" s="48" t="n"/>
-      <c r="O14" s="48" t="n"/>
-      <c r="P14" s="48" t="n"/>
-      <c r="Q14" s="48" t="n"/>
-      <c r="R14" s="48" t="n"/>
-      <c r="S14" s="48" t="n"/>
-      <c r="T14" s="48" t="n"/>
-      <c r="U14" s="48" t="n"/>
-      <c r="V14" s="48" t="n"/>
-      <c r="W14" s="49" t="n"/>
-      <c r="X14" s="49" t="n"/>
-      <c r="Y14" s="48" t="n"/>
-      <c r="Z14" s="48" t="n"/>
-      <c r="AA14" s="48" t="n"/>
-      <c r="AB14" s="48" t="n"/>
-      <c r="AC14" s="48" t="n"/>
-      <c r="AD14" s="48" t="n"/>
-      <c r="AE14" s="48" t="n"/>
-      <c r="AF14" s="48" t="n"/>
-      <c r="AH14" s="46" t="inlineStr">
+      <c r="A14" s="46" t="n"/>
+      <c r="B14" s="47" t="n"/>
+      <c r="C14" s="48" t="n"/>
+      <c r="D14" s="49" t="n"/>
+      <c r="E14" s="49" t="n"/>
+      <c r="F14" s="49" t="n"/>
+      <c r="G14" s="49" t="n"/>
+      <c r="H14" s="49" t="n"/>
+      <c r="I14" s="49" t="n"/>
+      <c r="J14" s="49" t="n"/>
+      <c r="K14" s="49" t="n"/>
+      <c r="L14" s="49" t="n"/>
+      <c r="M14" s="49" t="n"/>
+      <c r="N14" s="49" t="n"/>
+      <c r="O14" s="49" t="n"/>
+      <c r="P14" s="49" t="n"/>
+      <c r="Q14" s="49" t="n"/>
+      <c r="R14" s="49" t="n"/>
+      <c r="S14" s="49" t="n"/>
+      <c r="T14" s="49" t="n"/>
+      <c r="U14" s="49" t="n"/>
+      <c r="V14" s="49" t="n"/>
+      <c r="W14" s="50" t="n"/>
+      <c r="X14" s="50" t="n"/>
+      <c r="Y14" s="49" t="n"/>
+      <c r="Z14" s="49" t="n"/>
+      <c r="AA14" s="49" t="n"/>
+      <c r="AB14" s="49" t="n"/>
+      <c r="AC14" s="49" t="n"/>
+      <c r="AD14" s="49" t="n"/>
+      <c r="AE14" s="49" t="n"/>
+      <c r="AF14" s="49" t="n"/>
+      <c r="AH14" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-1)</t>
         </is>
       </c>
-      <c r="AI14" s="48" t="n"/>
-      <c r="AK14" s="46" t="n"/>
-      <c r="AL14" s="46" t="n"/>
-      <c r="AN14" s="46" t="n"/>
-      <c r="AO14" s="46" t="n"/>
-      <c r="AQ14" s="46" t="n"/>
-      <c r="AS14" s="46" t="n"/>
+      <c r="AI14" s="49" t="n"/>
+      <c r="AK14" s="47" t="n"/>
+      <c r="AL14" s="47" t="n"/>
+      <c r="AN14" s="47" t="n"/>
+      <c r="AO14" s="47" t="n"/>
+      <c r="AQ14" s="47" t="n"/>
+      <c r="AS14" s="47" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="46" t="n"/>
-      <c r="C15" s="47" t="n"/>
-      <c r="D15" s="48" t="n"/>
-      <c r="E15" s="48" t="n"/>
-      <c r="F15" s="48" t="n"/>
-      <c r="G15" s="48" t="n"/>
-      <c r="H15" s="48" t="n"/>
-      <c r="I15" s="48" t="n"/>
-      <c r="J15" s="48" t="n"/>
-      <c r="K15" s="48" t="n"/>
-      <c r="L15" s="48" t="n"/>
-      <c r="M15" s="48" t="n"/>
-      <c r="N15" s="48" t="n"/>
-      <c r="O15" s="48" t="n"/>
-      <c r="P15" s="48" t="n"/>
-      <c r="Q15" s="48" t="n"/>
-      <c r="R15" s="48" t="n"/>
-      <c r="S15" s="48" t="n"/>
-      <c r="T15" s="48" t="n"/>
-      <c r="U15" s="48" t="n"/>
-      <c r="V15" s="48" t="n"/>
-      <c r="W15" s="49" t="n"/>
-      <c r="X15" s="49" t="n"/>
-      <c r="Y15" s="48" t="n"/>
-      <c r="Z15" s="48" t="n"/>
-      <c r="AA15" s="48" t="n"/>
-      <c r="AB15" s="48" t="n"/>
-      <c r="AC15" s="48" t="n"/>
-      <c r="AD15" s="48" t="n"/>
-      <c r="AE15" s="48" t="n"/>
-      <c r="AF15" s="48" t="n"/>
-      <c r="AH15" s="46" t="inlineStr">
+      <c r="A15" s="46" t="n"/>
+      <c r="B15" s="47" t="n"/>
+      <c r="C15" s="48" t="n"/>
+      <c r="D15" s="49" t="n"/>
+      <c r="E15" s="49" t="n"/>
+      <c r="F15" s="49" t="n"/>
+      <c r="G15" s="49" t="n"/>
+      <c r="H15" s="49" t="n"/>
+      <c r="I15" s="49" t="n"/>
+      <c r="J15" s="49" t="n"/>
+      <c r="K15" s="49" t="n"/>
+      <c r="L15" s="49" t="n"/>
+      <c r="M15" s="49" t="n"/>
+      <c r="N15" s="49" t="n"/>
+      <c r="O15" s="49" t="n"/>
+      <c r="P15" s="49" t="n"/>
+      <c r="Q15" s="49" t="n"/>
+      <c r="R15" s="49" t="n"/>
+      <c r="S15" s="49" t="n"/>
+      <c r="T15" s="49" t="n"/>
+      <c r="U15" s="49" t="n"/>
+      <c r="V15" s="49" t="n"/>
+      <c r="W15" s="50" t="n"/>
+      <c r="X15" s="50" t="n"/>
+      <c r="Y15" s="49" t="n"/>
+      <c r="Z15" s="49" t="n"/>
+      <c r="AA15" s="49" t="n"/>
+      <c r="AB15" s="49" t="n"/>
+      <c r="AC15" s="49" t="n"/>
+      <c r="AD15" s="49" t="n"/>
+      <c r="AE15" s="49" t="n"/>
+      <c r="AF15" s="49" t="n"/>
+      <c r="AH15" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano)</t>
         </is>
       </c>
-      <c r="AI15" s="48" t="n"/>
-      <c r="AK15" s="46" t="n"/>
-      <c r="AL15" s="46" t="n"/>
-      <c r="AN15" s="46" t="n"/>
-      <c r="AO15" s="46" t="n"/>
-      <c r="AQ15" s="46" t="n"/>
-      <c r="AS15" s="46" t="n"/>
+      <c r="AI15" s="49" t="n"/>
+      <c r="AK15" s="47" t="n"/>
+      <c r="AL15" s="47" t="n"/>
+      <c r="AN15" s="47" t="n"/>
+      <c r="AO15" s="47" t="n"/>
+      <c r="AQ15" s="47" t="n"/>
+      <c r="AS15" s="47" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="46" t="n"/>
-      <c r="C16" s="47" t="n"/>
-      <c r="D16" s="48" t="n"/>
-      <c r="E16" s="48" t="n"/>
-      <c r="F16" s="48" t="n"/>
-      <c r="G16" s="48" t="n"/>
-      <c r="H16" s="48" t="n"/>
-      <c r="I16" s="48" t="n"/>
-      <c r="J16" s="48" t="n"/>
-      <c r="K16" s="48" t="n"/>
-      <c r="L16" s="48" t="n"/>
-      <c r="M16" s="48" t="n"/>
-      <c r="N16" s="48" t="n"/>
-      <c r="O16" s="48" t="n"/>
-      <c r="P16" s="48" t="n"/>
-      <c r="Q16" s="48" t="n"/>
-      <c r="R16" s="48" t="n"/>
-      <c r="S16" s="48" t="n"/>
-      <c r="T16" s="48" t="n"/>
-      <c r="U16" s="48" t="n"/>
-      <c r="V16" s="48" t="n"/>
-      <c r="W16" s="49" t="n"/>
-      <c r="X16" s="49" t="n"/>
-      <c r="Y16" s="48" t="n"/>
-      <c r="Z16" s="48" t="n"/>
-      <c r="AA16" s="48" t="n"/>
-      <c r="AB16" s="48" t="n"/>
-      <c r="AC16" s="48" t="n"/>
-      <c r="AD16" s="48" t="n"/>
-      <c r="AE16" s="48" t="n"/>
-      <c r="AF16" s="48" t="n"/>
-      <c r="AH16" s="46" t="inlineStr">
+      <c r="A16" s="46" t="n"/>
+      <c r="B16" s="47" t="n"/>
+      <c r="C16" s="48" t="n"/>
+      <c r="D16" s="49" t="n"/>
+      <c r="E16" s="49" t="n"/>
+      <c r="F16" s="49" t="n"/>
+      <c r="G16" s="49" t="n"/>
+      <c r="H16" s="49" t="n"/>
+      <c r="I16" s="49" t="n"/>
+      <c r="J16" s="49" t="n"/>
+      <c r="K16" s="49" t="n"/>
+      <c r="L16" s="49" t="n"/>
+      <c r="M16" s="49" t="n"/>
+      <c r="N16" s="49" t="n"/>
+      <c r="O16" s="49" t="n"/>
+      <c r="P16" s="49" t="n"/>
+      <c r="Q16" s="49" t="n"/>
+      <c r="R16" s="49" t="n"/>
+      <c r="S16" s="49" t="n"/>
+      <c r="T16" s="49" t="n"/>
+      <c r="U16" s="49" t="n"/>
+      <c r="V16" s="49" t="n"/>
+      <c r="W16" s="50" t="n"/>
+      <c r="X16" s="50" t="n"/>
+      <c r="Y16" s="49" t="n"/>
+      <c r="Z16" s="49" t="n"/>
+      <c r="AA16" s="49" t="n"/>
+      <c r="AB16" s="49" t="n"/>
+      <c r="AC16" s="49" t="n"/>
+      <c r="AD16" s="49" t="n"/>
+      <c r="AE16" s="49" t="n"/>
+      <c r="AF16" s="49" t="n"/>
+      <c r="AH16" s="47" t="inlineStr">
         <is>
           <t>Linhas do extrato pendentes</t>
         </is>
       </c>
-      <c r="AI16" s="47" t="n"/>
-      <c r="AK16" s="46" t="n"/>
-      <c r="AL16" s="46" t="n"/>
-      <c r="AN16" s="46" t="n"/>
-      <c r="AO16" s="46" t="n"/>
-      <c r="AQ16" s="46" t="n"/>
-      <c r="AS16" s="46" t="n"/>
+      <c r="AI16" s="48" t="n"/>
+      <c r="AK16" s="47" t="n"/>
+      <c r="AL16" s="47" t="n"/>
+      <c r="AN16" s="47" t="n"/>
+      <c r="AO16" s="47" t="n"/>
+      <c r="AQ16" s="47" t="n"/>
+      <c r="AS16" s="47" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="46" t="n"/>
-      <c r="C17" s="47" t="n"/>
-      <c r="D17" s="48" t="n"/>
-      <c r="E17" s="48" t="n"/>
-      <c r="F17" s="48" t="n"/>
-      <c r="G17" s="48" t="n"/>
-      <c r="H17" s="48" t="n"/>
-      <c r="I17" s="48" t="n"/>
-      <c r="J17" s="48" t="n"/>
-      <c r="K17" s="48" t="n"/>
-      <c r="L17" s="48" t="n"/>
-      <c r="M17" s="48" t="n"/>
-      <c r="N17" s="48" t="n"/>
-      <c r="O17" s="48" t="n"/>
-      <c r="P17" s="48" t="n"/>
-      <c r="Q17" s="48" t="n"/>
-      <c r="R17" s="48" t="n"/>
-      <c r="S17" s="48" t="n"/>
-      <c r="T17" s="48" t="n"/>
-      <c r="U17" s="48" t="n"/>
-      <c r="V17" s="48" t="n"/>
-      <c r="W17" s="49" t="n"/>
-      <c r="X17" s="49" t="n"/>
-      <c r="Y17" s="48" t="n"/>
-      <c r="Z17" s="48" t="n"/>
-      <c r="AA17" s="48" t="n"/>
-      <c r="AB17" s="48" t="n"/>
-      <c r="AC17" s="48" t="n"/>
-      <c r="AD17" s="48" t="n"/>
-      <c r="AE17" s="48" t="n"/>
-      <c r="AF17" s="48" t="n"/>
-      <c r="AH17" s="46" t="inlineStr">
+      <c r="A17" s="46" t="n"/>
+      <c r="B17" s="47" t="n"/>
+      <c r="C17" s="48" t="n"/>
+      <c r="D17" s="49" t="n"/>
+      <c r="E17" s="49" t="n"/>
+      <c r="F17" s="49" t="n"/>
+      <c r="G17" s="49" t="n"/>
+      <c r="H17" s="49" t="n"/>
+      <c r="I17" s="49" t="n"/>
+      <c r="J17" s="49" t="n"/>
+      <c r="K17" s="49" t="n"/>
+      <c r="L17" s="49" t="n"/>
+      <c r="M17" s="49" t="n"/>
+      <c r="N17" s="49" t="n"/>
+      <c r="O17" s="49" t="n"/>
+      <c r="P17" s="49" t="n"/>
+      <c r="Q17" s="49" t="n"/>
+      <c r="R17" s="49" t="n"/>
+      <c r="S17" s="49" t="n"/>
+      <c r="T17" s="49" t="n"/>
+      <c r="U17" s="49" t="n"/>
+      <c r="V17" s="49" t="n"/>
+      <c r="W17" s="50" t="n"/>
+      <c r="X17" s="50" t="n"/>
+      <c r="Y17" s="49" t="n"/>
+      <c r="Z17" s="49" t="n"/>
+      <c r="AA17" s="49" t="n"/>
+      <c r="AB17" s="49" t="n"/>
+      <c r="AC17" s="49" t="n"/>
+      <c r="AD17" s="49" t="n"/>
+      <c r="AE17" s="49" t="n"/>
+      <c r="AF17" s="49" t="n"/>
+      <c r="AH17" s="47" t="inlineStr">
         <is>
           <t>Último extrato importado</t>
         </is>
       </c>
-      <c r="AI17" s="50" t="n"/>
-      <c r="AK17" s="46" t="n"/>
-      <c r="AL17" s="46" t="n"/>
-      <c r="AN17" s="46" t="n"/>
-      <c r="AO17" s="46" t="n"/>
-      <c r="AQ17" s="46" t="n"/>
-      <c r="AS17" s="46" t="n"/>
+      <c r="AI17" s="51" t="n"/>
+      <c r="AK17" s="47" t="n"/>
+      <c r="AL17" s="47" t="n"/>
+      <c r="AN17" s="47" t="n"/>
+      <c r="AO17" s="47" t="n"/>
+      <c r="AQ17" s="47" t="n"/>
+      <c r="AS17" s="47" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="46" t="n"/>
-      <c r="C18" s="47" t="n"/>
-      <c r="D18" s="48" t="n"/>
-      <c r="E18" s="48" t="n"/>
-      <c r="F18" s="48" t="n"/>
-      <c r="G18" s="48" t="n"/>
-      <c r="H18" s="48" t="n"/>
-      <c r="I18" s="48" t="n"/>
-      <c r="J18" s="48" t="n"/>
-      <c r="K18" s="48" t="n"/>
-      <c r="L18" s="48" t="n"/>
-      <c r="M18" s="48" t="n"/>
-      <c r="N18" s="48" t="n"/>
-      <c r="O18" s="48" t="n"/>
-      <c r="P18" s="48" t="n"/>
-      <c r="Q18" s="48" t="n"/>
-      <c r="R18" s="48" t="n"/>
-      <c r="S18" s="48" t="n"/>
-      <c r="T18" s="48" t="n"/>
-      <c r="U18" s="48" t="n"/>
-      <c r="V18" s="48" t="n"/>
-      <c r="W18" s="49" t="n"/>
-      <c r="X18" s="49" t="n"/>
-      <c r="Y18" s="48" t="n"/>
-      <c r="Z18" s="48" t="n"/>
-      <c r="AA18" s="48" t="n"/>
-      <c r="AB18" s="48" t="n"/>
-      <c r="AC18" s="48" t="n"/>
-      <c r="AD18" s="48" t="n"/>
-      <c r="AE18" s="48" t="n"/>
-      <c r="AF18" s="48" t="n"/>
-      <c r="AH18" s="46" t="inlineStr">
+      <c r="A18" s="46" t="n"/>
+      <c r="B18" s="47" t="n"/>
+      <c r="C18" s="48" t="n"/>
+      <c r="D18" s="49" t="n"/>
+      <c r="E18" s="49" t="n"/>
+      <c r="F18" s="49" t="n"/>
+      <c r="G18" s="49" t="n"/>
+      <c r="H18" s="49" t="n"/>
+      <c r="I18" s="49" t="n"/>
+      <c r="J18" s="49" t="n"/>
+      <c r="K18" s="49" t="n"/>
+      <c r="L18" s="49" t="n"/>
+      <c r="M18" s="49" t="n"/>
+      <c r="N18" s="49" t="n"/>
+      <c r="O18" s="49" t="n"/>
+      <c r="P18" s="49" t="n"/>
+      <c r="Q18" s="49" t="n"/>
+      <c r="R18" s="49" t="n"/>
+      <c r="S18" s="49" t="n"/>
+      <c r="T18" s="49" t="n"/>
+      <c r="U18" s="49" t="n"/>
+      <c r="V18" s="49" t="n"/>
+      <c r="W18" s="50" t="n"/>
+      <c r="X18" s="50" t="n"/>
+      <c r="Y18" s="49" t="n"/>
+      <c r="Z18" s="49" t="n"/>
+      <c r="AA18" s="49" t="n"/>
+      <c r="AB18" s="49" t="n"/>
+      <c r="AC18" s="49" t="n"/>
+      <c r="AD18" s="49" t="n"/>
+      <c r="AE18" s="49" t="n"/>
+      <c r="AF18" s="49" t="n"/>
+      <c r="AH18" s="47" t="inlineStr">
         <is>
           <t>Notas de saída no mês</t>
         </is>
       </c>
-      <c r="AI18" s="47" t="n"/>
-      <c r="AK18" s="46" t="n"/>
-      <c r="AL18" s="46" t="n"/>
-      <c r="AN18" s="46" t="n"/>
-      <c r="AO18" s="46" t="n"/>
-      <c r="AQ18" s="46" t="n"/>
-      <c r="AS18" s="46" t="n"/>
+      <c r="AI18" s="48" t="n"/>
+      <c r="AK18" s="47" t="n"/>
+      <c r="AL18" s="47" t="n"/>
+      <c r="AN18" s="47" t="n"/>
+      <c r="AO18" s="47" t="n"/>
+      <c r="AQ18" s="47" t="n"/>
+      <c r="AS18" s="47" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="45" t="n"/>
-      <c r="B19" s="46" t="n"/>
-      <c r="C19" s="47" t="n"/>
-      <c r="D19" s="48" t="n"/>
-      <c r="E19" s="48" t="n"/>
-      <c r="F19" s="48" t="n"/>
-      <c r="G19" s="48" t="n"/>
-      <c r="H19" s="48" t="n"/>
-      <c r="I19" s="48" t="n"/>
-      <c r="J19" s="48" t="n"/>
-      <c r="K19" s="48" t="n"/>
-      <c r="L19" s="48" t="n"/>
-      <c r="M19" s="48" t="n"/>
-      <c r="N19" s="48" t="n"/>
-      <c r="O19" s="48" t="n"/>
-      <c r="P19" s="48" t="n"/>
-      <c r="Q19" s="48" t="n"/>
-      <c r="R19" s="48" t="n"/>
-      <c r="S19" s="48" t="n"/>
-      <c r="T19" s="48" t="n"/>
-      <c r="U19" s="48" t="n"/>
-      <c r="V19" s="48" t="n"/>
-      <c r="W19" s="49" t="n"/>
-      <c r="X19" s="49" t="n"/>
-      <c r="Y19" s="48" t="n"/>
-      <c r="Z19" s="48" t="n"/>
-      <c r="AA19" s="48" t="n"/>
-      <c r="AB19" s="48" t="n"/>
-      <c r="AC19" s="48" t="n"/>
-      <c r="AD19" s="48" t="n"/>
-      <c r="AE19" s="48" t="n"/>
-      <c r="AF19" s="48" t="n"/>
-      <c r="AH19" s="46" t="inlineStr">
+      <c r="A19" s="46" t="n"/>
+      <c r="B19" s="47" t="n"/>
+      <c r="C19" s="48" t="n"/>
+      <c r="D19" s="49" t="n"/>
+      <c r="E19" s="49" t="n"/>
+      <c r="F19" s="49" t="n"/>
+      <c r="G19" s="49" t="n"/>
+      <c r="H19" s="49" t="n"/>
+      <c r="I19" s="49" t="n"/>
+      <c r="J19" s="49" t="n"/>
+      <c r="K19" s="49" t="n"/>
+      <c r="L19" s="49" t="n"/>
+      <c r="M19" s="49" t="n"/>
+      <c r="N19" s="49" t="n"/>
+      <c r="O19" s="49" t="n"/>
+      <c r="P19" s="49" t="n"/>
+      <c r="Q19" s="49" t="n"/>
+      <c r="R19" s="49" t="n"/>
+      <c r="S19" s="49" t="n"/>
+      <c r="T19" s="49" t="n"/>
+      <c r="U19" s="49" t="n"/>
+      <c r="V19" s="49" t="n"/>
+      <c r="W19" s="50" t="n"/>
+      <c r="X19" s="50" t="n"/>
+      <c r="Y19" s="49" t="n"/>
+      <c r="Z19" s="49" t="n"/>
+      <c r="AA19" s="49" t="n"/>
+      <c r="AB19" s="49" t="n"/>
+      <c r="AC19" s="49" t="n"/>
+      <c r="AD19" s="49" t="n"/>
+      <c r="AE19" s="49" t="n"/>
+      <c r="AF19" s="49" t="n"/>
+      <c r="AH19" s="47" t="inlineStr">
         <is>
           <t>Sócio 1</t>
         </is>
       </c>
-      <c r="AI19" s="46" t="n"/>
-      <c r="AK19" s="46" t="n"/>
-      <c r="AL19" s="46" t="n"/>
-      <c r="AN19" s="46" t="n"/>
-      <c r="AO19" s="46" t="n"/>
-      <c r="AQ19" s="46" t="n"/>
-      <c r="AS19" s="46" t="n"/>
+      <c r="AI19" s="47" t="n"/>
+      <c r="AK19" s="47" t="n"/>
+      <c r="AL19" s="47" t="n"/>
+      <c r="AN19" s="47" t="n"/>
+      <c r="AO19" s="47" t="n"/>
+      <c r="AQ19" s="47" t="n"/>
+      <c r="AS19" s="47" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="46" t="n"/>
-      <c r="C20" s="47" t="n"/>
-      <c r="D20" s="48" t="n"/>
-      <c r="E20" s="48" t="n"/>
-      <c r="F20" s="48" t="n"/>
-      <c r="G20" s="48" t="n"/>
-      <c r="H20" s="48" t="n"/>
-      <c r="I20" s="48" t="n"/>
-      <c r="J20" s="48" t="n"/>
-      <c r="K20" s="48" t="n"/>
-      <c r="L20" s="48" t="n"/>
-      <c r="M20" s="48" t="n"/>
-      <c r="N20" s="48" t="n"/>
-      <c r="O20" s="48" t="n"/>
-      <c r="P20" s="48" t="n"/>
-      <c r="Q20" s="48" t="n"/>
-      <c r="R20" s="48" t="n"/>
-      <c r="S20" s="48" t="n"/>
-      <c r="T20" s="48" t="n"/>
-      <c r="U20" s="48" t="n"/>
-      <c r="V20" s="48" t="n"/>
-      <c r="W20" s="49" t="n"/>
-      <c r="X20" s="49" t="n"/>
-      <c r="Y20" s="48" t="n"/>
-      <c r="Z20" s="48" t="n"/>
-      <c r="AA20" s="48" t="n"/>
-      <c r="AB20" s="48" t="n"/>
-      <c r="AC20" s="48" t="n"/>
-      <c r="AD20" s="48" t="n"/>
-      <c r="AE20" s="48" t="n"/>
-      <c r="AF20" s="48" t="n"/>
-      <c r="AH20" s="46" t="inlineStr">
+      <c r="A20" s="46" t="n"/>
+      <c r="B20" s="47" t="n"/>
+      <c r="C20" s="48" t="n"/>
+      <c r="D20" s="49" t="n"/>
+      <c r="E20" s="49" t="n"/>
+      <c r="F20" s="49" t="n"/>
+      <c r="G20" s="49" t="n"/>
+      <c r="H20" s="49" t="n"/>
+      <c r="I20" s="49" t="n"/>
+      <c r="J20" s="49" t="n"/>
+      <c r="K20" s="49" t="n"/>
+      <c r="L20" s="49" t="n"/>
+      <c r="M20" s="49" t="n"/>
+      <c r="N20" s="49" t="n"/>
+      <c r="O20" s="49" t="n"/>
+      <c r="P20" s="49" t="n"/>
+      <c r="Q20" s="49" t="n"/>
+      <c r="R20" s="49" t="n"/>
+      <c r="S20" s="49" t="n"/>
+      <c r="T20" s="49" t="n"/>
+      <c r="U20" s="49" t="n"/>
+      <c r="V20" s="49" t="n"/>
+      <c r="W20" s="50" t="n"/>
+      <c r="X20" s="50" t="n"/>
+      <c r="Y20" s="49" t="n"/>
+      <c r="Z20" s="49" t="n"/>
+      <c r="AA20" s="49" t="n"/>
+      <c r="AB20" s="49" t="n"/>
+      <c r="AC20" s="49" t="n"/>
+      <c r="AD20" s="49" t="n"/>
+      <c r="AE20" s="49" t="n"/>
+      <c r="AF20" s="49" t="n"/>
+      <c r="AH20" s="47" t="inlineStr">
         <is>
           <t>Sócio 2</t>
         </is>
       </c>
-      <c r="AI20" s="46" t="n"/>
-      <c r="AK20" s="46" t="n"/>
-      <c r="AL20" s="46" t="n"/>
-      <c r="AN20" s="46" t="n"/>
-      <c r="AO20" s="46" t="n"/>
-      <c r="AQ20" s="46" t="n"/>
-      <c r="AS20" s="46" t="n"/>
+      <c r="AI20" s="47" t="n"/>
+      <c r="AK20" s="47" t="n"/>
+      <c r="AL20" s="47" t="n"/>
+      <c r="AN20" s="47" t="n"/>
+      <c r="AO20" s="47" t="n"/>
+      <c r="AQ20" s="47" t="n"/>
+      <c r="AS20" s="47" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="46" t="n"/>
-      <c r="C21" s="47" t="n"/>
-      <c r="D21" s="48" t="n"/>
-      <c r="E21" s="48" t="n"/>
-      <c r="F21" s="48" t="n"/>
-      <c r="G21" s="48" t="n"/>
-      <c r="H21" s="48" t="n"/>
-      <c r="I21" s="48" t="n"/>
-      <c r="J21" s="48" t="n"/>
-      <c r="K21" s="48" t="n"/>
-      <c r="L21" s="48" t="n"/>
-      <c r="M21" s="48" t="n"/>
-      <c r="N21" s="48" t="n"/>
-      <c r="O21" s="48" t="n"/>
-      <c r="P21" s="48" t="n"/>
-      <c r="Q21" s="48" t="n"/>
-      <c r="R21" s="48" t="n"/>
-      <c r="S21" s="48" t="n"/>
-      <c r="T21" s="48" t="n"/>
-      <c r="U21" s="48" t="n"/>
-      <c r="V21" s="48" t="n"/>
-      <c r="W21" s="49" t="n"/>
-      <c r="X21" s="49" t="n"/>
-      <c r="Y21" s="48" t="n"/>
-      <c r="Z21" s="48" t="n"/>
-      <c r="AA21" s="48" t="n"/>
-      <c r="AB21" s="48" t="n"/>
-      <c r="AC21" s="48" t="n"/>
-      <c r="AD21" s="48" t="n"/>
-      <c r="AE21" s="48" t="n"/>
-      <c r="AF21" s="48" t="n"/>
-      <c r="AH21" s="46" t="inlineStr">
+      <c r="A21" s="46" t="n"/>
+      <c r="B21" s="47" t="n"/>
+      <c r="C21" s="48" t="n"/>
+      <c r="D21" s="49" t="n"/>
+      <c r="E21" s="49" t="n"/>
+      <c r="F21" s="49" t="n"/>
+      <c r="G21" s="49" t="n"/>
+      <c r="H21" s="49" t="n"/>
+      <c r="I21" s="49" t="n"/>
+      <c r="J21" s="49" t="n"/>
+      <c r="K21" s="49" t="n"/>
+      <c r="L21" s="49" t="n"/>
+      <c r="M21" s="49" t="n"/>
+      <c r="N21" s="49" t="n"/>
+      <c r="O21" s="49" t="n"/>
+      <c r="P21" s="49" t="n"/>
+      <c r="Q21" s="49" t="n"/>
+      <c r="R21" s="49" t="n"/>
+      <c r="S21" s="49" t="n"/>
+      <c r="T21" s="49" t="n"/>
+      <c r="U21" s="49" t="n"/>
+      <c r="V21" s="49" t="n"/>
+      <c r="W21" s="50" t="n"/>
+      <c r="X21" s="50" t="n"/>
+      <c r="Y21" s="49" t="n"/>
+      <c r="Z21" s="49" t="n"/>
+      <c r="AA21" s="49" t="n"/>
+      <c r="AB21" s="49" t="n"/>
+      <c r="AC21" s="49" t="n"/>
+      <c r="AD21" s="49" t="n"/>
+      <c r="AE21" s="49" t="n"/>
+      <c r="AF21" s="49" t="n"/>
+      <c r="AH21" s="47" t="inlineStr">
         <is>
           <t>Sócio 3</t>
         </is>
       </c>
-      <c r="AI21" s="46" t="n"/>
-      <c r="AK21" s="46" t="n"/>
-      <c r="AL21" s="46" t="n"/>
-      <c r="AN21" s="46" t="n"/>
-      <c r="AO21" s="46" t="n"/>
-      <c r="AQ21" s="46" t="n"/>
-      <c r="AS21" s="46" t="n"/>
+      <c r="AI21" s="47" t="n"/>
+      <c r="AK21" s="47" t="n"/>
+      <c r="AL21" s="47" t="n"/>
+      <c r="AN21" s="47" t="n"/>
+      <c r="AO21" s="47" t="n"/>
+      <c r="AQ21" s="47" t="n"/>
+      <c r="AS21" s="47" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="n"/>
-      <c r="C22" s="47" t="n"/>
-      <c r="D22" s="48" t="n"/>
-      <c r="E22" s="48" t="n"/>
-      <c r="F22" s="48" t="n"/>
-      <c r="G22" s="48" t="n"/>
-      <c r="H22" s="48" t="n"/>
-      <c r="I22" s="48" t="n"/>
-      <c r="J22" s="48" t="n"/>
-      <c r="K22" s="48" t="n"/>
-      <c r="L22" s="48" t="n"/>
-      <c r="M22" s="48" t="n"/>
-      <c r="N22" s="48" t="n"/>
-      <c r="O22" s="48" t="n"/>
-      <c r="P22" s="48" t="n"/>
-      <c r="Q22" s="48" t="n"/>
-      <c r="R22" s="48" t="n"/>
-      <c r="S22" s="48" t="n"/>
-      <c r="T22" s="48" t="n"/>
-      <c r="U22" s="48" t="n"/>
-      <c r="V22" s="48" t="n"/>
-      <c r="W22" s="49" t="n"/>
-      <c r="X22" s="49" t="n"/>
-      <c r="Y22" s="48" t="n"/>
-      <c r="Z22" s="48" t="n"/>
-      <c r="AA22" s="48" t="n"/>
-      <c r="AB22" s="48" t="n"/>
-      <c r="AC22" s="48" t="n"/>
-      <c r="AD22" s="48" t="n"/>
-      <c r="AE22" s="48" t="n"/>
-      <c r="AF22" s="48" t="n"/>
-      <c r="AH22" s="46" t="inlineStr">
+      <c r="A22" s="46" t="n"/>
+      <c r="B22" s="47" t="n"/>
+      <c r="C22" s="48" t="n"/>
+      <c r="D22" s="49" t="n"/>
+      <c r="E22" s="49" t="n"/>
+      <c r="F22" s="49" t="n"/>
+      <c r="G22" s="49" t="n"/>
+      <c r="H22" s="49" t="n"/>
+      <c r="I22" s="49" t="n"/>
+      <c r="J22" s="49" t="n"/>
+      <c r="K22" s="49" t="n"/>
+      <c r="L22" s="49" t="n"/>
+      <c r="M22" s="49" t="n"/>
+      <c r="N22" s="49" t="n"/>
+      <c r="O22" s="49" t="n"/>
+      <c r="P22" s="49" t="n"/>
+      <c r="Q22" s="49" t="n"/>
+      <c r="R22" s="49" t="n"/>
+      <c r="S22" s="49" t="n"/>
+      <c r="T22" s="49" t="n"/>
+      <c r="U22" s="49" t="n"/>
+      <c r="V22" s="49" t="n"/>
+      <c r="W22" s="50" t="n"/>
+      <c r="X22" s="50" t="n"/>
+      <c r="Y22" s="49" t="n"/>
+      <c r="Z22" s="49" t="n"/>
+      <c r="AA22" s="49" t="n"/>
+      <c r="AB22" s="49" t="n"/>
+      <c r="AC22" s="49" t="n"/>
+      <c r="AD22" s="49" t="n"/>
+      <c r="AE22" s="49" t="n"/>
+      <c r="AF22" s="49" t="n"/>
+      <c r="AH22" s="47" t="inlineStr">
         <is>
           <t>Sócio 4</t>
         </is>
       </c>
-      <c r="AI22" s="46" t="n"/>
-      <c r="AK22" s="46" t="n"/>
-      <c r="AL22" s="46" t="n"/>
-      <c r="AN22" s="46" t="n"/>
-      <c r="AO22" s="46" t="n"/>
-      <c r="AQ22" s="46" t="n"/>
-      <c r="AS22" s="46" t="n"/>
+      <c r="AI22" s="47" t="n"/>
+      <c r="AK22" s="47" t="n"/>
+      <c r="AL22" s="47" t="n"/>
+      <c r="AN22" s="47" t="n"/>
+      <c r="AO22" s="47" t="n"/>
+      <c r="AQ22" s="47" t="n"/>
+      <c r="AS22" s="47" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="n"/>
-      <c r="C23" s="47" t="n"/>
-      <c r="D23" s="48" t="n"/>
-      <c r="E23" s="48" t="n"/>
-      <c r="F23" s="48" t="n"/>
-      <c r="G23" s="48" t="n"/>
-      <c r="H23" s="48" t="n"/>
-      <c r="I23" s="48" t="n"/>
-      <c r="J23" s="48" t="n"/>
-      <c r="K23" s="48" t="n"/>
-      <c r="L23" s="48" t="n"/>
-      <c r="M23" s="48" t="n"/>
-      <c r="N23" s="48" t="n"/>
-      <c r="O23" s="48" t="n"/>
-      <c r="P23" s="48" t="n"/>
-      <c r="Q23" s="48" t="n"/>
-      <c r="R23" s="48" t="n"/>
-      <c r="S23" s="48" t="n"/>
-      <c r="T23" s="48" t="n"/>
-      <c r="U23" s="48" t="n"/>
-      <c r="V23" s="48" t="n"/>
-      <c r="W23" s="49" t="n"/>
-      <c r="X23" s="49" t="n"/>
-      <c r="Y23" s="48" t="n"/>
-      <c r="Z23" s="48" t="n"/>
-      <c r="AA23" s="48" t="n"/>
-      <c r="AB23" s="48" t="n"/>
-      <c r="AC23" s="48" t="n"/>
-      <c r="AD23" s="48" t="n"/>
-      <c r="AE23" s="48" t="n"/>
-      <c r="AF23" s="48" t="n"/>
-      <c r="AH23" s="46" t="inlineStr">
+      <c r="A23" s="46" t="n"/>
+      <c r="B23" s="47" t="n"/>
+      <c r="C23" s="48" t="n"/>
+      <c r="D23" s="49" t="n"/>
+      <c r="E23" s="49" t="n"/>
+      <c r="F23" s="49" t="n"/>
+      <c r="G23" s="49" t="n"/>
+      <c r="H23" s="49" t="n"/>
+      <c r="I23" s="49" t="n"/>
+      <c r="J23" s="49" t="n"/>
+      <c r="K23" s="49" t="n"/>
+      <c r="L23" s="49" t="n"/>
+      <c r="M23" s="49" t="n"/>
+      <c r="N23" s="49" t="n"/>
+      <c r="O23" s="49" t="n"/>
+      <c r="P23" s="49" t="n"/>
+      <c r="Q23" s="49" t="n"/>
+      <c r="R23" s="49" t="n"/>
+      <c r="S23" s="49" t="n"/>
+      <c r="T23" s="49" t="n"/>
+      <c r="U23" s="49" t="n"/>
+      <c r="V23" s="49" t="n"/>
+      <c r="W23" s="50" t="n"/>
+      <c r="X23" s="50" t="n"/>
+      <c r="Y23" s="49" t="n"/>
+      <c r="Z23" s="49" t="n"/>
+      <c r="AA23" s="49" t="n"/>
+      <c r="AB23" s="49" t="n"/>
+      <c r="AC23" s="49" t="n"/>
+      <c r="AD23" s="49" t="n"/>
+      <c r="AE23" s="49" t="n"/>
+      <c r="AF23" s="49" t="n"/>
+      <c r="AH23" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 1</t>
         </is>
       </c>
-      <c r="AI23" s="51" t="n"/>
-      <c r="AK23" s="46" t="n"/>
-      <c r="AL23" s="46" t="n"/>
-      <c r="AN23" s="46" t="n"/>
-      <c r="AO23" s="46" t="n"/>
-      <c r="AQ23" s="46" t="n"/>
-      <c r="AS23" s="46" t="n"/>
+      <c r="AI23" s="52" t="n"/>
+      <c r="AK23" s="47" t="n"/>
+      <c r="AL23" s="47" t="n"/>
+      <c r="AN23" s="47" t="n"/>
+      <c r="AO23" s="47" t="n"/>
+      <c r="AQ23" s="47" t="n"/>
+      <c r="AS23" s="47" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="n"/>
-      <c r="C24" s="47" t="n"/>
-      <c r="D24" s="48" t="n"/>
-      <c r="E24" s="48" t="n"/>
-      <c r="F24" s="48" t="n"/>
-      <c r="G24" s="48" t="n"/>
-      <c r="H24" s="48" t="n"/>
-      <c r="I24" s="48" t="n"/>
-      <c r="J24" s="48" t="n"/>
-      <c r="K24" s="48" t="n"/>
-      <c r="L24" s="48" t="n"/>
-      <c r="M24" s="48" t="n"/>
-      <c r="N24" s="48" t="n"/>
-      <c r="O24" s="48" t="n"/>
-      <c r="P24" s="48" t="n"/>
-      <c r="Q24" s="48" t="n"/>
-      <c r="R24" s="48" t="n"/>
-      <c r="S24" s="48" t="n"/>
-      <c r="T24" s="48" t="n"/>
-      <c r="U24" s="48" t="n"/>
-      <c r="V24" s="48" t="n"/>
-      <c r="W24" s="49" t="n"/>
-      <c r="X24" s="49" t="n"/>
-      <c r="Y24" s="48" t="n"/>
-      <c r="Z24" s="48" t="n"/>
-      <c r="AA24" s="48" t="n"/>
-      <c r="AB24" s="48" t="n"/>
-      <c r="AC24" s="48" t="n"/>
-      <c r="AD24" s="48" t="n"/>
-      <c r="AE24" s="48" t="n"/>
-      <c r="AF24" s="48" t="n"/>
-      <c r="AH24" s="46" t="inlineStr">
+      <c r="A24" s="46" t="n"/>
+      <c r="B24" s="47" t="n"/>
+      <c r="C24" s="48" t="n"/>
+      <c r="D24" s="49" t="n"/>
+      <c r="E24" s="49" t="n"/>
+      <c r="F24" s="49" t="n"/>
+      <c r="G24" s="49" t="n"/>
+      <c r="H24" s="49" t="n"/>
+      <c r="I24" s="49" t="n"/>
+      <c r="J24" s="49" t="n"/>
+      <c r="K24" s="49" t="n"/>
+      <c r="L24" s="49" t="n"/>
+      <c r="M24" s="49" t="n"/>
+      <c r="N24" s="49" t="n"/>
+      <c r="O24" s="49" t="n"/>
+      <c r="P24" s="49" t="n"/>
+      <c r="Q24" s="49" t="n"/>
+      <c r="R24" s="49" t="n"/>
+      <c r="S24" s="49" t="n"/>
+      <c r="T24" s="49" t="n"/>
+      <c r="U24" s="49" t="n"/>
+      <c r="V24" s="49" t="n"/>
+      <c r="W24" s="50" t="n"/>
+      <c r="X24" s="50" t="n"/>
+      <c r="Y24" s="49" t="n"/>
+      <c r="Z24" s="49" t="n"/>
+      <c r="AA24" s="49" t="n"/>
+      <c r="AB24" s="49" t="n"/>
+      <c r="AC24" s="49" t="n"/>
+      <c r="AD24" s="49" t="n"/>
+      <c r="AE24" s="49" t="n"/>
+      <c r="AF24" s="49" t="n"/>
+      <c r="AH24" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 2</t>
         </is>
       </c>
-      <c r="AI24" s="51" t="n"/>
-      <c r="AK24" s="46" t="n"/>
-      <c r="AL24" s="46" t="n"/>
-      <c r="AN24" s="46" t="n"/>
-      <c r="AO24" s="46" t="n"/>
-      <c r="AQ24" s="46" t="n"/>
-      <c r="AS24" s="46" t="n"/>
+      <c r="AI24" s="52" t="n"/>
+      <c r="AK24" s="47" t="n"/>
+      <c r="AL24" s="47" t="n"/>
+      <c r="AN24" s="47" t="n"/>
+      <c r="AO24" s="47" t="n"/>
+      <c r="AQ24" s="47" t="n"/>
+      <c r="AS24" s="47" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="n"/>
-      <c r="C25" s="47" t="n"/>
-      <c r="D25" s="48" t="n"/>
-      <c r="E25" s="48" t="n"/>
-      <c r="F25" s="48" t="n"/>
-      <c r="G25" s="48" t="n"/>
-      <c r="H25" s="48" t="n"/>
-      <c r="I25" s="48" t="n"/>
-      <c r="J25" s="48" t="n"/>
-      <c r="K25" s="48" t="n"/>
-      <c r="L25" s="48" t="n"/>
-      <c r="M25" s="48" t="n"/>
-      <c r="N25" s="48" t="n"/>
-      <c r="O25" s="48" t="n"/>
-      <c r="P25" s="48" t="n"/>
-      <c r="Q25" s="48" t="n"/>
-      <c r="R25" s="48" t="n"/>
-      <c r="S25" s="48" t="n"/>
-      <c r="T25" s="48" t="n"/>
-      <c r="U25" s="48" t="n"/>
-      <c r="V25" s="48" t="n"/>
-      <c r="W25" s="49" t="n"/>
-      <c r="X25" s="49" t="n"/>
-      <c r="Y25" s="48" t="n"/>
-      <c r="Z25" s="48" t="n"/>
-      <c r="AA25" s="48" t="n"/>
-      <c r="AB25" s="48" t="n"/>
-      <c r="AC25" s="48" t="n"/>
-      <c r="AD25" s="48" t="n"/>
-      <c r="AE25" s="48" t="n"/>
-      <c r="AF25" s="48" t="n"/>
-      <c r="AH25" s="46" t="inlineStr">
+      <c r="A25" s="46" t="n"/>
+      <c r="B25" s="47" t="n"/>
+      <c r="C25" s="48" t="n"/>
+      <c r="D25" s="49" t="n"/>
+      <c r="E25" s="49" t="n"/>
+      <c r="F25" s="49" t="n"/>
+      <c r="G25" s="49" t="n"/>
+      <c r="H25" s="49" t="n"/>
+      <c r="I25" s="49" t="n"/>
+      <c r="J25" s="49" t="n"/>
+      <c r="K25" s="49" t="n"/>
+      <c r="L25" s="49" t="n"/>
+      <c r="M25" s="49" t="n"/>
+      <c r="N25" s="49" t="n"/>
+      <c r="O25" s="49" t="n"/>
+      <c r="P25" s="49" t="n"/>
+      <c r="Q25" s="49" t="n"/>
+      <c r="R25" s="49" t="n"/>
+      <c r="S25" s="49" t="n"/>
+      <c r="T25" s="49" t="n"/>
+      <c r="U25" s="49" t="n"/>
+      <c r="V25" s="49" t="n"/>
+      <c r="W25" s="50" t="n"/>
+      <c r="X25" s="50" t="n"/>
+      <c r="Y25" s="49" t="n"/>
+      <c r="Z25" s="49" t="n"/>
+      <c r="AA25" s="49" t="n"/>
+      <c r="AB25" s="49" t="n"/>
+      <c r="AC25" s="49" t="n"/>
+      <c r="AD25" s="49" t="n"/>
+      <c r="AE25" s="49" t="n"/>
+      <c r="AF25" s="49" t="n"/>
+      <c r="AH25" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 3</t>
         </is>
       </c>
-      <c r="AI25" s="51" t="n"/>
-      <c r="AK25" s="46" t="n"/>
-      <c r="AL25" s="46" t="n"/>
-      <c r="AN25" s="46" t="n"/>
-      <c r="AO25" s="46" t="n"/>
-      <c r="AQ25" s="46" t="n"/>
-      <c r="AS25" s="46" t="n"/>
+      <c r="AI25" s="52" t="n"/>
+      <c r="AK25" s="47" t="n"/>
+      <c r="AL25" s="47" t="n"/>
+      <c r="AN25" s="47" t="n"/>
+      <c r="AO25" s="47" t="n"/>
+      <c r="AQ25" s="47" t="n"/>
+      <c r="AS25" s="47" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="n"/>
-      <c r="C26" s="47" t="n"/>
-      <c r="D26" s="48" t="n"/>
-      <c r="E26" s="48" t="n"/>
-      <c r="F26" s="48" t="n"/>
-      <c r="G26" s="48" t="n"/>
-      <c r="H26" s="48" t="n"/>
-      <c r="I26" s="48" t="n"/>
-      <c r="J26" s="48" t="n"/>
-      <c r="K26" s="48" t="n"/>
-      <c r="L26" s="48" t="n"/>
-      <c r="M26" s="48" t="n"/>
-      <c r="N26" s="48" t="n"/>
-      <c r="O26" s="48" t="n"/>
-      <c r="P26" s="48" t="n"/>
-      <c r="Q26" s="48" t="n"/>
-      <c r="R26" s="48" t="n"/>
-      <c r="S26" s="48" t="n"/>
-      <c r="T26" s="48" t="n"/>
-      <c r="U26" s="48" t="n"/>
-      <c r="V26" s="48" t="n"/>
-      <c r="W26" s="49" t="n"/>
-      <c r="X26" s="49" t="n"/>
-      <c r="Y26" s="48" t="n"/>
-      <c r="Z26" s="48" t="n"/>
-      <c r="AA26" s="48" t="n"/>
-      <c r="AB26" s="48" t="n"/>
-      <c r="AC26" s="48" t="n"/>
-      <c r="AD26" s="48" t="n"/>
-      <c r="AE26" s="48" t="n"/>
-      <c r="AF26" s="48" t="n"/>
-      <c r="AH26" s="46" t="inlineStr">
+      <c r="A26" s="46" t="n"/>
+      <c r="B26" s="47" t="n"/>
+      <c r="C26" s="48" t="n"/>
+      <c r="D26" s="49" t="n"/>
+      <c r="E26" s="49" t="n"/>
+      <c r="F26" s="49" t="n"/>
+      <c r="G26" s="49" t="n"/>
+      <c r="H26" s="49" t="n"/>
+      <c r="I26" s="49" t="n"/>
+      <c r="J26" s="49" t="n"/>
+      <c r="K26" s="49" t="n"/>
+      <c r="L26" s="49" t="n"/>
+      <c r="M26" s="49" t="n"/>
+      <c r="N26" s="49" t="n"/>
+      <c r="O26" s="49" t="n"/>
+      <c r="P26" s="49" t="n"/>
+      <c r="Q26" s="49" t="n"/>
+      <c r="R26" s="49" t="n"/>
+      <c r="S26" s="49" t="n"/>
+      <c r="T26" s="49" t="n"/>
+      <c r="U26" s="49" t="n"/>
+      <c r="V26" s="49" t="n"/>
+      <c r="W26" s="50" t="n"/>
+      <c r="X26" s="50" t="n"/>
+      <c r="Y26" s="49" t="n"/>
+      <c r="Z26" s="49" t="n"/>
+      <c r="AA26" s="49" t="n"/>
+      <c r="AB26" s="49" t="n"/>
+      <c r="AC26" s="49" t="n"/>
+      <c r="AD26" s="49" t="n"/>
+      <c r="AE26" s="49" t="n"/>
+      <c r="AF26" s="49" t="n"/>
+      <c r="AH26" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 4</t>
         </is>
       </c>
-      <c r="AI26" s="51" t="n"/>
-      <c r="AK26" s="46" t="n"/>
-      <c r="AL26" s="46" t="n"/>
-      <c r="AN26" s="46" t="n"/>
-      <c r="AO26" s="46" t="n"/>
-      <c r="AQ26" s="46" t="n"/>
-      <c r="AS26" s="46" t="n"/>
+      <c r="AI26" s="52" t="n"/>
+      <c r="AK26" s="47" t="n"/>
+      <c r="AL26" s="47" t="n"/>
+      <c r="AN26" s="47" t="n"/>
+      <c r="AO26" s="47" t="n"/>
+      <c r="AQ26" s="47" t="n"/>
+      <c r="AS26" s="47" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="n"/>
-      <c r="C27" s="47" t="n"/>
-      <c r="D27" s="48" t="n"/>
-      <c r="E27" s="48" t="n"/>
-      <c r="F27" s="48" t="n"/>
-      <c r="G27" s="48" t="n"/>
-      <c r="H27" s="48" t="n"/>
-      <c r="I27" s="48" t="n"/>
-      <c r="J27" s="48" t="n"/>
-      <c r="K27" s="48" t="n"/>
-      <c r="L27" s="48" t="n"/>
-      <c r="M27" s="48" t="n"/>
-      <c r="N27" s="48" t="n"/>
-      <c r="O27" s="48" t="n"/>
-      <c r="P27" s="48" t="n"/>
-      <c r="Q27" s="48" t="n"/>
-      <c r="R27" s="48" t="n"/>
-      <c r="S27" s="48" t="n"/>
-      <c r="T27" s="48" t="n"/>
-      <c r="U27" s="48" t="n"/>
-      <c r="V27" s="48" t="n"/>
-      <c r="W27" s="49" t="n"/>
-      <c r="X27" s="49" t="n"/>
-      <c r="Y27" s="48" t="n"/>
-      <c r="Z27" s="48" t="n"/>
-      <c r="AA27" s="48" t="n"/>
-      <c r="AB27" s="48" t="n"/>
-      <c r="AC27" s="48" t="n"/>
-      <c r="AD27" s="48" t="n"/>
-      <c r="AE27" s="48" t="n"/>
-      <c r="AF27" s="48" t="n"/>
-      <c r="AH27" s="46" t="inlineStr">
+      <c r="A27" s="46" t="n"/>
+      <c r="B27" s="47" t="n"/>
+      <c r="C27" s="48" t="n"/>
+      <c r="D27" s="49" t="n"/>
+      <c r="E27" s="49" t="n"/>
+      <c r="F27" s="49" t="n"/>
+      <c r="G27" s="49" t="n"/>
+      <c r="H27" s="49" t="n"/>
+      <c r="I27" s="49" t="n"/>
+      <c r="J27" s="49" t="n"/>
+      <c r="K27" s="49" t="n"/>
+      <c r="L27" s="49" t="n"/>
+      <c r="M27" s="49" t="n"/>
+      <c r="N27" s="49" t="n"/>
+      <c r="O27" s="49" t="n"/>
+      <c r="P27" s="49" t="n"/>
+      <c r="Q27" s="49" t="n"/>
+      <c r="R27" s="49" t="n"/>
+      <c r="S27" s="49" t="n"/>
+      <c r="T27" s="49" t="n"/>
+      <c r="U27" s="49" t="n"/>
+      <c r="V27" s="49" t="n"/>
+      <c r="W27" s="50" t="n"/>
+      <c r="X27" s="50" t="n"/>
+      <c r="Y27" s="49" t="n"/>
+      <c r="Z27" s="49" t="n"/>
+      <c r="AA27" s="49" t="n"/>
+      <c r="AB27" s="49" t="n"/>
+      <c r="AC27" s="49" t="n"/>
+      <c r="AD27" s="49" t="n"/>
+      <c r="AE27" s="49" t="n"/>
+      <c r="AF27" s="49" t="n"/>
+      <c r="AH27" s="47" t="inlineStr">
         <is>
           <t>Grupos de clientes que compraram no ano</t>
         </is>
       </c>
-      <c r="AI27" s="47" t="n"/>
-      <c r="AK27" s="46" t="n"/>
-      <c r="AL27" s="46" t="n"/>
-      <c r="AN27" s="46" t="n"/>
-      <c r="AO27" s="46" t="n"/>
-      <c r="AQ27" s="46" t="n"/>
-      <c r="AS27" s="46" t="n"/>
+      <c r="AI27" s="48" t="n"/>
+      <c r="AK27" s="47" t="n"/>
+      <c r="AL27" s="47" t="n"/>
+      <c r="AN27" s="47" t="n"/>
+      <c r="AO27" s="47" t="n"/>
+      <c r="AQ27" s="47" t="n"/>
+      <c r="AS27" s="47" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="46" t="n"/>
-      <c r="C28" s="47" t="n"/>
-      <c r="D28" s="48" t="n"/>
-      <c r="E28" s="48" t="n"/>
-      <c r="F28" s="48" t="n"/>
-      <c r="G28" s="48" t="n"/>
-      <c r="H28" s="48" t="n"/>
-      <c r="I28" s="48" t="n"/>
-      <c r="J28" s="48" t="n"/>
-      <c r="K28" s="48" t="n"/>
-      <c r="L28" s="48" t="n"/>
-      <c r="M28" s="48" t="n"/>
-      <c r="N28" s="48" t="n"/>
-      <c r="O28" s="48" t="n"/>
-      <c r="P28" s="48" t="n"/>
-      <c r="Q28" s="48" t="n"/>
-      <c r="R28" s="48" t="n"/>
-      <c r="S28" s="48" t="n"/>
-      <c r="T28" s="48" t="n"/>
-      <c r="U28" s="48" t="n"/>
-      <c r="V28" s="48" t="n"/>
-      <c r="W28" s="49" t="n"/>
-      <c r="X28" s="49" t="n"/>
-      <c r="Y28" s="48" t="n"/>
-      <c r="Z28" s="48" t="n"/>
-      <c r="AA28" s="48" t="n"/>
-      <c r="AB28" s="48" t="n"/>
-      <c r="AC28" s="48" t="n"/>
-      <c r="AD28" s="48" t="n"/>
-      <c r="AE28" s="48" t="n"/>
-      <c r="AF28" s="48" t="n"/>
-      <c r="AH28" s="46" t="inlineStr">
+      <c r="A28" s="46" t="n"/>
+      <c r="B28" s="47" t="n"/>
+      <c r="C28" s="48" t="n"/>
+      <c r="D28" s="49" t="n"/>
+      <c r="E28" s="49" t="n"/>
+      <c r="F28" s="49" t="n"/>
+      <c r="G28" s="49" t="n"/>
+      <c r="H28" s="49" t="n"/>
+      <c r="I28" s="49" t="n"/>
+      <c r="J28" s="49" t="n"/>
+      <c r="K28" s="49" t="n"/>
+      <c r="L28" s="49" t="n"/>
+      <c r="M28" s="49" t="n"/>
+      <c r="N28" s="49" t="n"/>
+      <c r="O28" s="49" t="n"/>
+      <c r="P28" s="49" t="n"/>
+      <c r="Q28" s="49" t="n"/>
+      <c r="R28" s="49" t="n"/>
+      <c r="S28" s="49" t="n"/>
+      <c r="T28" s="49" t="n"/>
+      <c r="U28" s="49" t="n"/>
+      <c r="V28" s="49" t="n"/>
+      <c r="W28" s="50" t="n"/>
+      <c r="X28" s="50" t="n"/>
+      <c r="Y28" s="49" t="n"/>
+      <c r="Z28" s="49" t="n"/>
+      <c r="AA28" s="49" t="n"/>
+      <c r="AB28" s="49" t="n"/>
+      <c r="AC28" s="49" t="n"/>
+      <c r="AD28" s="49" t="n"/>
+      <c r="AE28" s="49" t="n"/>
+      <c r="AF28" s="49" t="n"/>
+      <c r="AH28" s="47" t="inlineStr">
         <is>
           <t>Grupos que compraram pela 1ª vez no ano</t>
         </is>
       </c>
-      <c r="AI28" s="47" t="n"/>
-      <c r="AK28" s="46" t="n"/>
-      <c r="AL28" s="46" t="n"/>
-      <c r="AN28" s="46" t="n"/>
-      <c r="AO28" s="46" t="n"/>
-      <c r="AQ28" s="46" t="n"/>
-      <c r="AS28" s="46" t="n"/>
+      <c r="AI28" s="48" t="n"/>
+      <c r="AK28" s="47" t="n"/>
+      <c r="AL28" s="47" t="n"/>
+      <c r="AN28" s="47" t="n"/>
+      <c r="AO28" s="47" t="n"/>
+      <c r="AQ28" s="47" t="n"/>
+      <c r="AS28" s="47" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="45" t="n"/>
-      <c r="B29" s="46" t="n"/>
-      <c r="C29" s="47" t="n"/>
-      <c r="D29" s="48" t="n"/>
-      <c r="E29" s="48" t="n"/>
-      <c r="F29" s="48" t="n"/>
-      <c r="G29" s="48" t="n"/>
-      <c r="H29" s="48" t="n"/>
-      <c r="I29" s="48" t="n"/>
-      <c r="J29" s="48" t="n"/>
-      <c r="K29" s="48" t="n"/>
-      <c r="L29" s="48" t="n"/>
-      <c r="M29" s="48" t="n"/>
-      <c r="N29" s="48" t="n"/>
-      <c r="O29" s="48" t="n"/>
-      <c r="P29" s="48" t="n"/>
-      <c r="Q29" s="48" t="n"/>
-      <c r="R29" s="48" t="n"/>
-      <c r="S29" s="48" t="n"/>
-      <c r="T29" s="48" t="n"/>
-      <c r="U29" s="48" t="n"/>
-      <c r="V29" s="48" t="n"/>
-      <c r="W29" s="49" t="n"/>
-      <c r="X29" s="49" t="n"/>
-      <c r="Y29" s="48" t="n"/>
-      <c r="Z29" s="48" t="n"/>
-      <c r="AA29" s="48" t="n"/>
-      <c r="AB29" s="48" t="n"/>
-      <c r="AC29" s="48" t="n"/>
-      <c r="AD29" s="48" t="n"/>
-      <c r="AE29" s="48" t="n"/>
-      <c r="AF29" s="48" t="n"/>
-      <c r="AK29" s="46" t="n"/>
-      <c r="AL29" s="46" t="n"/>
-      <c r="AN29" s="46" t="n"/>
-      <c r="AO29" s="46" t="n"/>
-      <c r="AQ29" s="46" t="n"/>
-      <c r="AS29" s="46" t="n"/>
+      <c r="A29" s="46" t="n"/>
+      <c r="B29" s="47" t="n"/>
+      <c r="C29" s="48" t="n"/>
+      <c r="D29" s="49" t="n"/>
+      <c r="E29" s="49" t="n"/>
+      <c r="F29" s="49" t="n"/>
+      <c r="G29" s="49" t="n"/>
+      <c r="H29" s="49" t="n"/>
+      <c r="I29" s="49" t="n"/>
+      <c r="J29" s="49" t="n"/>
+      <c r="K29" s="49" t="n"/>
+      <c r="L29" s="49" t="n"/>
+      <c r="M29" s="49" t="n"/>
+      <c r="N29" s="49" t="n"/>
+      <c r="O29" s="49" t="n"/>
+      <c r="P29" s="49" t="n"/>
+      <c r="Q29" s="49" t="n"/>
+      <c r="R29" s="49" t="n"/>
+      <c r="S29" s="49" t="n"/>
+      <c r="T29" s="49" t="n"/>
+      <c r="U29" s="49" t="n"/>
+      <c r="V29" s="49" t="n"/>
+      <c r="W29" s="50" t="n"/>
+      <c r="X29" s="50" t="n"/>
+      <c r="Y29" s="49" t="n"/>
+      <c r="Z29" s="49" t="n"/>
+      <c r="AA29" s="49" t="n"/>
+      <c r="AB29" s="49" t="n"/>
+      <c r="AC29" s="49" t="n"/>
+      <c r="AD29" s="49" t="n"/>
+      <c r="AE29" s="49" t="n"/>
+      <c r="AF29" s="49" t="n"/>
+      <c r="AK29" s="47" t="n"/>
+      <c r="AL29" s="47" t="n"/>
+      <c r="AN29" s="47" t="n"/>
+      <c r="AO29" s="47" t="n"/>
+      <c r="AQ29" s="47" t="n"/>
+      <c r="AS29" s="47" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="45" t="n"/>
-      <c r="B30" s="46" t="n"/>
-      <c r="C30" s="47" t="n"/>
-      <c r="D30" s="48" t="n"/>
-      <c r="E30" s="48" t="n"/>
-      <c r="F30" s="48" t="n"/>
-      <c r="G30" s="48" t="n"/>
-      <c r="H30" s="48" t="n"/>
-      <c r="I30" s="48" t="n"/>
-      <c r="J30" s="48" t="n"/>
-      <c r="K30" s="48" t="n"/>
-      <c r="L30" s="48" t="n"/>
-      <c r="M30" s="48" t="n"/>
-      <c r="N30" s="48" t="n"/>
-      <c r="O30" s="48" t="n"/>
-      <c r="P30" s="48" t="n"/>
-      <c r="Q30" s="48" t="n"/>
-      <c r="R30" s="48" t="n"/>
-      <c r="S30" s="48" t="n"/>
-      <c r="T30" s="48" t="n"/>
-      <c r="U30" s="48" t="n"/>
-      <c r="V30" s="48" t="n"/>
-      <c r="W30" s="49" t="n"/>
-      <c r="X30" s="49" t="n"/>
-      <c r="Y30" s="48" t="n"/>
-      <c r="Z30" s="48" t="n"/>
-      <c r="AA30" s="48" t="n"/>
-      <c r="AB30" s="48" t="n"/>
-      <c r="AC30" s="48" t="n"/>
-      <c r="AD30" s="48" t="n"/>
-      <c r="AE30" s="48" t="n"/>
-      <c r="AF30" s="48" t="n"/>
-      <c r="AK30" s="46" t="n"/>
-      <c r="AL30" s="46" t="n"/>
-      <c r="AN30" s="46" t="n"/>
-      <c r="AO30" s="46" t="n"/>
-      <c r="AQ30" s="46" t="n"/>
-      <c r="AS30" s="46" t="n"/>
+      <c r="A30" s="46" t="n"/>
+      <c r="B30" s="47" t="n"/>
+      <c r="C30" s="48" t="n"/>
+      <c r="D30" s="49" t="n"/>
+      <c r="E30" s="49" t="n"/>
+      <c r="F30" s="49" t="n"/>
+      <c r="G30" s="49" t="n"/>
+      <c r="H30" s="49" t="n"/>
+      <c r="I30" s="49" t="n"/>
+      <c r="J30" s="49" t="n"/>
+      <c r="K30" s="49" t="n"/>
+      <c r="L30" s="49" t="n"/>
+      <c r="M30" s="49" t="n"/>
+      <c r="N30" s="49" t="n"/>
+      <c r="O30" s="49" t="n"/>
+      <c r="P30" s="49" t="n"/>
+      <c r="Q30" s="49" t="n"/>
+      <c r="R30" s="49" t="n"/>
+      <c r="S30" s="49" t="n"/>
+      <c r="T30" s="49" t="n"/>
+      <c r="U30" s="49" t="n"/>
+      <c r="V30" s="49" t="n"/>
+      <c r="W30" s="50" t="n"/>
+      <c r="X30" s="50" t="n"/>
+      <c r="Y30" s="49" t="n"/>
+      <c r="Z30" s="49" t="n"/>
+      <c r="AA30" s="49" t="n"/>
+      <c r="AB30" s="49" t="n"/>
+      <c r="AC30" s="49" t="n"/>
+      <c r="AD30" s="49" t="n"/>
+      <c r="AE30" s="49" t="n"/>
+      <c r="AF30" s="49" t="n"/>
+      <c r="AK30" s="47" t="n"/>
+      <c r="AL30" s="47" t="n"/>
+      <c r="AN30" s="47" t="n"/>
+      <c r="AO30" s="47" t="n"/>
+      <c r="AQ30" s="47" t="n"/>
+      <c r="AS30" s="47" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="45" t="n"/>
-      <c r="B31" s="46" t="n"/>
-      <c r="C31" s="47" t="n"/>
-      <c r="D31" s="48" t="n"/>
-      <c r="E31" s="48" t="n"/>
-      <c r="F31" s="48" t="n"/>
-      <c r="G31" s="48" t="n"/>
-      <c r="H31" s="48" t="n"/>
-      <c r="I31" s="48" t="n"/>
-      <c r="J31" s="48" t="n"/>
-      <c r="K31" s="48" t="n"/>
-      <c r="L31" s="48" t="n"/>
-      <c r="M31" s="48" t="n"/>
-      <c r="N31" s="48" t="n"/>
-      <c r="O31" s="48" t="n"/>
-      <c r="P31" s="48" t="n"/>
-      <c r="Q31" s="48" t="n"/>
-      <c r="R31" s="48" t="n"/>
-      <c r="S31" s="48" t="n"/>
-      <c r="T31" s="48" t="n"/>
-      <c r="U31" s="48" t="n"/>
-      <c r="V31" s="48" t="n"/>
-      <c r="W31" s="49" t="n"/>
-      <c r="X31" s="49" t="n"/>
-      <c r="Y31" s="48" t="n"/>
-      <c r="Z31" s="48" t="n"/>
-      <c r="AA31" s="48" t="n"/>
-      <c r="AB31" s="48" t="n"/>
-      <c r="AC31" s="48" t="n"/>
-      <c r="AD31" s="48" t="n"/>
-      <c r="AE31" s="48" t="n"/>
-      <c r="AF31" s="48" t="n"/>
-      <c r="AK31" s="46" t="n"/>
-      <c r="AL31" s="46" t="n"/>
-      <c r="AN31" s="46" t="n"/>
-      <c r="AO31" s="46" t="n"/>
-      <c r="AQ31" s="46" t="n"/>
-      <c r="AS31" s="46" t="n"/>
+      <c r="A31" s="46" t="n"/>
+      <c r="B31" s="47" t="n"/>
+      <c r="C31" s="48" t="n"/>
+      <c r="D31" s="49" t="n"/>
+      <c r="E31" s="49" t="n"/>
+      <c r="F31" s="49" t="n"/>
+      <c r="G31" s="49" t="n"/>
+      <c r="H31" s="49" t="n"/>
+      <c r="I31" s="49" t="n"/>
+      <c r="J31" s="49" t="n"/>
+      <c r="K31" s="49" t="n"/>
+      <c r="L31" s="49" t="n"/>
+      <c r="M31" s="49" t="n"/>
+      <c r="N31" s="49" t="n"/>
+      <c r="O31" s="49" t="n"/>
+      <c r="P31" s="49" t="n"/>
+      <c r="Q31" s="49" t="n"/>
+      <c r="R31" s="49" t="n"/>
+      <c r="S31" s="49" t="n"/>
+      <c r="T31" s="49" t="n"/>
+      <c r="U31" s="49" t="n"/>
+      <c r="V31" s="49" t="n"/>
+      <c r="W31" s="50" t="n"/>
+      <c r="X31" s="50" t="n"/>
+      <c r="Y31" s="49" t="n"/>
+      <c r="Z31" s="49" t="n"/>
+      <c r="AA31" s="49" t="n"/>
+      <c r="AB31" s="49" t="n"/>
+      <c r="AC31" s="49" t="n"/>
+      <c r="AD31" s="49" t="n"/>
+      <c r="AE31" s="49" t="n"/>
+      <c r="AF31" s="49" t="n"/>
+      <c r="AK31" s="47" t="n"/>
+      <c r="AL31" s="47" t="n"/>
+      <c r="AN31" s="47" t="n"/>
+      <c r="AO31" s="47" t="n"/>
+      <c r="AQ31" s="47" t="n"/>
+      <c r="AS31" s="47" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="46" t="n"/>
-      <c r="C32" s="47" t="n"/>
-      <c r="D32" s="48" t="n"/>
-      <c r="E32" s="48" t="n"/>
-      <c r="F32" s="48" t="n"/>
-      <c r="G32" s="48" t="n"/>
-      <c r="H32" s="48" t="n"/>
-      <c r="I32" s="48" t="n"/>
-      <c r="J32" s="48" t="n"/>
-      <c r="K32" s="48" t="n"/>
-      <c r="L32" s="48" t="n"/>
-      <c r="M32" s="48" t="n"/>
-      <c r="N32" s="48" t="n"/>
-      <c r="O32" s="48" t="n"/>
-      <c r="P32" s="48" t="n"/>
-      <c r="Q32" s="48" t="n"/>
-      <c r="R32" s="48" t="n"/>
-      <c r="S32" s="48" t="n"/>
-      <c r="T32" s="48" t="n"/>
-      <c r="U32" s="48" t="n"/>
-      <c r="V32" s="48" t="n"/>
-      <c r="W32" s="49" t="n"/>
-      <c r="X32" s="49" t="n"/>
-      <c r="Y32" s="48" t="n"/>
-      <c r="Z32" s="48" t="n"/>
-      <c r="AA32" s="48" t="n"/>
-      <c r="AB32" s="48" t="n"/>
-      <c r="AC32" s="48" t="n"/>
-      <c r="AD32" s="48" t="n"/>
-      <c r="AE32" s="48" t="n"/>
-      <c r="AF32" s="48" t="n"/>
-      <c r="AK32" s="46" t="n"/>
-      <c r="AL32" s="46" t="n"/>
-      <c r="AN32" s="46" t="n"/>
-      <c r="AO32" s="46" t="n"/>
-      <c r="AQ32" s="46" t="n"/>
-      <c r="AS32" s="46" t="n"/>
+      <c r="A32" s="46" t="n"/>
+      <c r="B32" s="47" t="n"/>
+      <c r="C32" s="48" t="n"/>
+      <c r="D32" s="49" t="n"/>
+      <c r="E32" s="49" t="n"/>
+      <c r="F32" s="49" t="n"/>
+      <c r="G32" s="49" t="n"/>
+      <c r="H32" s="49" t="n"/>
+      <c r="I32" s="49" t="n"/>
+      <c r="J32" s="49" t="n"/>
+      <c r="K32" s="49" t="n"/>
+      <c r="L32" s="49" t="n"/>
+      <c r="M32" s="49" t="n"/>
+      <c r="N32" s="49" t="n"/>
+      <c r="O32" s="49" t="n"/>
+      <c r="P32" s="49" t="n"/>
+      <c r="Q32" s="49" t="n"/>
+      <c r="R32" s="49" t="n"/>
+      <c r="S32" s="49" t="n"/>
+      <c r="T32" s="49" t="n"/>
+      <c r="U32" s="49" t="n"/>
+      <c r="V32" s="49" t="n"/>
+      <c r="W32" s="50" t="n"/>
+      <c r="X32" s="50" t="n"/>
+      <c r="Y32" s="49" t="n"/>
+      <c r="Z32" s="49" t="n"/>
+      <c r="AA32" s="49" t="n"/>
+      <c r="AB32" s="49" t="n"/>
+      <c r="AC32" s="49" t="n"/>
+      <c r="AD32" s="49" t="n"/>
+      <c r="AE32" s="49" t="n"/>
+      <c r="AF32" s="49" t="n"/>
+      <c r="AK32" s="47" t="n"/>
+      <c r="AL32" s="47" t="n"/>
+      <c r="AN32" s="47" t="n"/>
+      <c r="AO32" s="47" t="n"/>
+      <c r="AQ32" s="47" t="n"/>
+      <c r="AS32" s="47" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="45" t="n"/>
-      <c r="B33" s="46" t="n"/>
-      <c r="C33" s="47" t="n"/>
-      <c r="D33" s="48" t="n"/>
-      <c r="E33" s="48" t="n"/>
-      <c r="F33" s="48" t="n"/>
-      <c r="G33" s="48" t="n"/>
-      <c r="H33" s="48" t="n"/>
-      <c r="I33" s="48" t="n"/>
-      <c r="J33" s="48" t="n"/>
-      <c r="K33" s="48" t="n"/>
-      <c r="L33" s="48" t="n"/>
-      <c r="M33" s="48" t="n"/>
-      <c r="N33" s="48" t="n"/>
-      <c r="O33" s="48" t="n"/>
-      <c r="P33" s="48" t="n"/>
-      <c r="Q33" s="48" t="n"/>
-      <c r="R33" s="48" t="n"/>
-      <c r="S33" s="48" t="n"/>
-      <c r="T33" s="48" t="n"/>
-      <c r="U33" s="48" t="n"/>
-      <c r="V33" s="48" t="n"/>
-      <c r="W33" s="49" t="n"/>
-      <c r="X33" s="49" t="n"/>
-      <c r="Y33" s="48" t="n"/>
-      <c r="Z33" s="48" t="n"/>
-      <c r="AA33" s="48" t="n"/>
-      <c r="AB33" s="48" t="n"/>
-      <c r="AC33" s="48" t="n"/>
-      <c r="AD33" s="48" t="n"/>
-      <c r="AE33" s="48" t="n"/>
-      <c r="AF33" s="48" t="n"/>
-      <c r="AK33" s="46" t="n"/>
-      <c r="AL33" s="46" t="n"/>
-      <c r="AN33" s="46" t="n"/>
-      <c r="AO33" s="46" t="n"/>
-      <c r="AQ33" s="46" t="n"/>
-      <c r="AS33" s="46" t="n"/>
+      <c r="A33" s="46" t="n"/>
+      <c r="B33" s="47" t="n"/>
+      <c r="C33" s="48" t="n"/>
+      <c r="D33" s="49" t="n"/>
+      <c r="E33" s="49" t="n"/>
+      <c r="F33" s="49" t="n"/>
+      <c r="G33" s="49" t="n"/>
+      <c r="H33" s="49" t="n"/>
+      <c r="I33" s="49" t="n"/>
+      <c r="J33" s="49" t="n"/>
+      <c r="K33" s="49" t="n"/>
+      <c r="L33" s="49" t="n"/>
+      <c r="M33" s="49" t="n"/>
+      <c r="N33" s="49" t="n"/>
+      <c r="O33" s="49" t="n"/>
+      <c r="P33" s="49" t="n"/>
+      <c r="Q33" s="49" t="n"/>
+      <c r="R33" s="49" t="n"/>
+      <c r="S33" s="49" t="n"/>
+      <c r="T33" s="49" t="n"/>
+      <c r="U33" s="49" t="n"/>
+      <c r="V33" s="49" t="n"/>
+      <c r="W33" s="50" t="n"/>
+      <c r="X33" s="50" t="n"/>
+      <c r="Y33" s="49" t="n"/>
+      <c r="Z33" s="49" t="n"/>
+      <c r="AA33" s="49" t="n"/>
+      <c r="AB33" s="49" t="n"/>
+      <c r="AC33" s="49" t="n"/>
+      <c r="AD33" s="49" t="n"/>
+      <c r="AE33" s="49" t="n"/>
+      <c r="AF33" s="49" t="n"/>
+      <c r="AK33" s="47" t="n"/>
+      <c r="AL33" s="47" t="n"/>
+      <c r="AN33" s="47" t="n"/>
+      <c r="AO33" s="47" t="n"/>
+      <c r="AQ33" s="47" t="n"/>
+      <c r="AS33" s="47" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="45" t="n"/>
-      <c r="B34" s="46" t="n"/>
-      <c r="C34" s="47" t="n"/>
-      <c r="D34" s="48" t="n"/>
-      <c r="E34" s="48" t="n"/>
-      <c r="F34" s="48" t="n"/>
-      <c r="G34" s="48" t="n"/>
-      <c r="H34" s="48" t="n"/>
-      <c r="I34" s="48" t="n"/>
-      <c r="J34" s="48" t="n"/>
-      <c r="K34" s="48" t="n"/>
-      <c r="L34" s="48" t="n"/>
-      <c r="M34" s="48" t="n"/>
-      <c r="N34" s="48" t="n"/>
-      <c r="O34" s="48" t="n"/>
-      <c r="P34" s="48" t="n"/>
-      <c r="Q34" s="48" t="n"/>
-      <c r="R34" s="48" t="n"/>
-      <c r="S34" s="48" t="n"/>
-      <c r="T34" s="48" t="n"/>
-      <c r="U34" s="48" t="n"/>
-      <c r="V34" s="48" t="n"/>
-      <c r="W34" s="49" t="n"/>
-      <c r="X34" s="49" t="n"/>
-      <c r="Y34" s="48" t="n"/>
-      <c r="Z34" s="48" t="n"/>
-      <c r="AA34" s="48" t="n"/>
-      <c r="AB34" s="48" t="n"/>
-      <c r="AC34" s="48" t="n"/>
-      <c r="AD34" s="48" t="n"/>
-      <c r="AE34" s="48" t="n"/>
-      <c r="AF34" s="48" t="n"/>
-      <c r="AK34" s="46" t="n"/>
-      <c r="AL34" s="46" t="n"/>
-      <c r="AN34" s="46" t="n"/>
-      <c r="AO34" s="46" t="n"/>
-      <c r="AQ34" s="46" t="n"/>
-      <c r="AS34" s="46" t="n"/>
+      <c r="A34" s="46" t="n"/>
+      <c r="B34" s="47" t="n"/>
+      <c r="C34" s="48" t="n"/>
+      <c r="D34" s="49" t="n"/>
+      <c r="E34" s="49" t="n"/>
+      <c r="F34" s="49" t="n"/>
+      <c r="G34" s="49" t="n"/>
+      <c r="H34" s="49" t="n"/>
+      <c r="I34" s="49" t="n"/>
+      <c r="J34" s="49" t="n"/>
+      <c r="K34" s="49" t="n"/>
+      <c r="L34" s="49" t="n"/>
+      <c r="M34" s="49" t="n"/>
+      <c r="N34" s="49" t="n"/>
+      <c r="O34" s="49" t="n"/>
+      <c r="P34" s="49" t="n"/>
+      <c r="Q34" s="49" t="n"/>
+      <c r="R34" s="49" t="n"/>
+      <c r="S34" s="49" t="n"/>
+      <c r="T34" s="49" t="n"/>
+      <c r="U34" s="49" t="n"/>
+      <c r="V34" s="49" t="n"/>
+      <c r="W34" s="50" t="n"/>
+      <c r="X34" s="50" t="n"/>
+      <c r="Y34" s="49" t="n"/>
+      <c r="Z34" s="49" t="n"/>
+      <c r="AA34" s="49" t="n"/>
+      <c r="AB34" s="49" t="n"/>
+      <c r="AC34" s="49" t="n"/>
+      <c r="AD34" s="49" t="n"/>
+      <c r="AE34" s="49" t="n"/>
+      <c r="AF34" s="49" t="n"/>
+      <c r="AK34" s="47" t="n"/>
+      <c r="AL34" s="47" t="n"/>
+      <c r="AN34" s="47" t="n"/>
+      <c r="AO34" s="47" t="n"/>
+      <c r="AQ34" s="47" t="n"/>
+      <c r="AS34" s="47" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="45" t="n"/>
-      <c r="B35" s="46" t="n"/>
-      <c r="C35" s="47" t="n"/>
-      <c r="D35" s="48" t="n"/>
-      <c r="E35" s="48" t="n"/>
-      <c r="F35" s="48" t="n"/>
-      <c r="G35" s="48" t="n"/>
-      <c r="H35" s="48" t="n"/>
-      <c r="I35" s="48" t="n"/>
-      <c r="J35" s="48" t="n"/>
-      <c r="K35" s="48" t="n"/>
-      <c r="L35" s="48" t="n"/>
-      <c r="M35" s="48" t="n"/>
-      <c r="N35" s="48" t="n"/>
-      <c r="O35" s="48" t="n"/>
-      <c r="P35" s="48" t="n"/>
-      <c r="Q35" s="48" t="n"/>
-      <c r="R35" s="48" t="n"/>
-      <c r="S35" s="48" t="n"/>
-      <c r="T35" s="48" t="n"/>
-      <c r="U35" s="48" t="n"/>
-      <c r="V35" s="48" t="n"/>
-      <c r="W35" s="49" t="n"/>
-      <c r="X35" s="49" t="n"/>
-      <c r="Y35" s="48" t="n"/>
-      <c r="Z35" s="48" t="n"/>
-      <c r="AA35" s="48" t="n"/>
-      <c r="AB35" s="48" t="n"/>
-      <c r="AC35" s="48" t="n"/>
-      <c r="AD35" s="48" t="n"/>
-      <c r="AE35" s="48" t="n"/>
-      <c r="AF35" s="48" t="n"/>
-      <c r="AK35" s="46" t="n"/>
-      <c r="AL35" s="46" t="n"/>
-      <c r="AN35" s="46" t="n"/>
-      <c r="AO35" s="46" t="n"/>
-      <c r="AQ35" s="46" t="n"/>
-      <c r="AS35" s="46" t="n"/>
+      <c r="A35" s="46" t="n"/>
+      <c r="B35" s="47" t="n"/>
+      <c r="C35" s="48" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="49" t="n"/>
+      <c r="I35" s="49" t="n"/>
+      <c r="J35" s="49" t="n"/>
+      <c r="K35" s="49" t="n"/>
+      <c r="L35" s="49" t="n"/>
+      <c r="M35" s="49" t="n"/>
+      <c r="N35" s="49" t="n"/>
+      <c r="O35" s="49" t="n"/>
+      <c r="P35" s="49" t="n"/>
+      <c r="Q35" s="49" t="n"/>
+      <c r="R35" s="49" t="n"/>
+      <c r="S35" s="49" t="n"/>
+      <c r="T35" s="49" t="n"/>
+      <c r="U35" s="49" t="n"/>
+      <c r="V35" s="49" t="n"/>
+      <c r="W35" s="50" t="n"/>
+      <c r="X35" s="50" t="n"/>
+      <c r="Y35" s="49" t="n"/>
+      <c r="Z35" s="49" t="n"/>
+      <c r="AA35" s="49" t="n"/>
+      <c r="AB35" s="49" t="n"/>
+      <c r="AC35" s="49" t="n"/>
+      <c r="AD35" s="49" t="n"/>
+      <c r="AE35" s="49" t="n"/>
+      <c r="AF35" s="49" t="n"/>
+      <c r="AK35" s="47" t="n"/>
+      <c r="AL35" s="47" t="n"/>
+      <c r="AN35" s="47" t="n"/>
+      <c r="AO35" s="47" t="n"/>
+      <c r="AQ35" s="47" t="n"/>
+      <c r="AS35" s="47" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="45" t="n"/>
-      <c r="B36" s="46" t="n"/>
-      <c r="C36" s="47" t="n"/>
-      <c r="D36" s="48" t="n"/>
-      <c r="E36" s="48" t="n"/>
-      <c r="F36" s="48" t="n"/>
-      <c r="G36" s="48" t="n"/>
-      <c r="H36" s="48" t="n"/>
-      <c r="I36" s="48" t="n"/>
-      <c r="J36" s="48" t="n"/>
-      <c r="K36" s="48" t="n"/>
-      <c r="L36" s="48" t="n"/>
-      <c r="M36" s="48" t="n"/>
-      <c r="N36" s="48" t="n"/>
-      <c r="O36" s="48" t="n"/>
-      <c r="P36" s="48" t="n"/>
-      <c r="Q36" s="48" t="n"/>
-      <c r="R36" s="48" t="n"/>
-      <c r="S36" s="48" t="n"/>
-      <c r="T36" s="48" t="n"/>
-      <c r="U36" s="48" t="n"/>
-      <c r="V36" s="48" t="n"/>
-      <c r="W36" s="49" t="n"/>
-      <c r="X36" s="49" t="n"/>
-      <c r="Y36" s="48" t="n"/>
-      <c r="Z36" s="48" t="n"/>
-      <c r="AA36" s="48" t="n"/>
-      <c r="AB36" s="48" t="n"/>
-      <c r="AC36" s="48" t="n"/>
-      <c r="AD36" s="48" t="n"/>
-      <c r="AE36" s="48" t="n"/>
-      <c r="AF36" s="48" t="n"/>
-      <c r="AK36" s="46" t="n"/>
-      <c r="AL36" s="46" t="n"/>
-      <c r="AN36" s="46" t="n"/>
-      <c r="AO36" s="46" t="n"/>
-      <c r="AQ36" s="46" t="n"/>
-      <c r="AS36" s="46" t="n"/>
+      <c r="A36" s="46" t="n"/>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="48" t="n"/>
+      <c r="D36" s="49" t="n"/>
+      <c r="E36" s="49" t="n"/>
+      <c r="F36" s="49" t="n"/>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="49" t="n"/>
+      <c r="I36" s="49" t="n"/>
+      <c r="J36" s="49" t="n"/>
+      <c r="K36" s="49" t="n"/>
+      <c r="L36" s="49" t="n"/>
+      <c r="M36" s="49" t="n"/>
+      <c r="N36" s="49" t="n"/>
+      <c r="O36" s="49" t="n"/>
+      <c r="P36" s="49" t="n"/>
+      <c r="Q36" s="49" t="n"/>
+      <c r="R36" s="49" t="n"/>
+      <c r="S36" s="49" t="n"/>
+      <c r="T36" s="49" t="n"/>
+      <c r="U36" s="49" t="n"/>
+      <c r="V36" s="49" t="n"/>
+      <c r="W36" s="50" t="n"/>
+      <c r="X36" s="50" t="n"/>
+      <c r="Y36" s="49" t="n"/>
+      <c r="Z36" s="49" t="n"/>
+      <c r="AA36" s="49" t="n"/>
+      <c r="AB36" s="49" t="n"/>
+      <c r="AC36" s="49" t="n"/>
+      <c r="AD36" s="49" t="n"/>
+      <c r="AE36" s="49" t="n"/>
+      <c r="AF36" s="49" t="n"/>
+      <c r="AK36" s="47" t="n"/>
+      <c r="AL36" s="47" t="n"/>
+      <c r="AN36" s="47" t="n"/>
+      <c r="AO36" s="47" t="n"/>
+      <c r="AQ36" s="47" t="n"/>
+      <c r="AS36" s="47" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="45" t="n"/>
-      <c r="B37" s="46" t="n"/>
-      <c r="C37" s="47" t="n"/>
-      <c r="D37" s="48" t="n"/>
-      <c r="E37" s="48" t="n"/>
-      <c r="F37" s="48" t="n"/>
-      <c r="G37" s="48" t="n"/>
-      <c r="H37" s="48" t="n"/>
-      <c r="I37" s="48" t="n"/>
-      <c r="J37" s="48" t="n"/>
-      <c r="K37" s="48" t="n"/>
-      <c r="L37" s="48" t="n"/>
-      <c r="M37" s="48" t="n"/>
-      <c r="N37" s="48" t="n"/>
-      <c r="O37" s="48" t="n"/>
-      <c r="P37" s="48" t="n"/>
-      <c r="Q37" s="48" t="n"/>
-      <c r="R37" s="48" t="n"/>
-      <c r="S37" s="48" t="n"/>
-      <c r="T37" s="48" t="n"/>
-      <c r="U37" s="48" t="n"/>
-      <c r="V37" s="48" t="n"/>
-      <c r="W37" s="49" t="n"/>
-      <c r="X37" s="49" t="n"/>
-      <c r="Y37" s="48" t="n"/>
-      <c r="Z37" s="48" t="n"/>
-      <c r="AA37" s="48" t="n"/>
-      <c r="AB37" s="48" t="n"/>
-      <c r="AC37" s="48" t="n"/>
-      <c r="AD37" s="48" t="n"/>
-      <c r="AE37" s="48" t="n"/>
-      <c r="AF37" s="48" t="n"/>
-      <c r="AK37" s="46" t="n"/>
-      <c r="AL37" s="46" t="n"/>
-      <c r="AN37" s="46" t="n"/>
-      <c r="AO37" s="46" t="n"/>
-      <c r="AQ37" s="46" t="n"/>
-      <c r="AS37" s="46" t="n"/>
+      <c r="A37" s="46" t="n"/>
+      <c r="B37" s="47" t="n"/>
+      <c r="C37" s="48" t="n"/>
+      <c r="D37" s="49" t="n"/>
+      <c r="E37" s="49" t="n"/>
+      <c r="F37" s="49" t="n"/>
+      <c r="G37" s="49" t="n"/>
+      <c r="H37" s="49" t="n"/>
+      <c r="I37" s="49" t="n"/>
+      <c r="J37" s="49" t="n"/>
+      <c r="K37" s="49" t="n"/>
+      <c r="L37" s="49" t="n"/>
+      <c r="M37" s="49" t="n"/>
+      <c r="N37" s="49" t="n"/>
+      <c r="O37" s="49" t="n"/>
+      <c r="P37" s="49" t="n"/>
+      <c r="Q37" s="49" t="n"/>
+      <c r="R37" s="49" t="n"/>
+      <c r="S37" s="49" t="n"/>
+      <c r="T37" s="49" t="n"/>
+      <c r="U37" s="49" t="n"/>
+      <c r="V37" s="49" t="n"/>
+      <c r="W37" s="50" t="n"/>
+      <c r="X37" s="50" t="n"/>
+      <c r="Y37" s="49" t="n"/>
+      <c r="Z37" s="49" t="n"/>
+      <c r="AA37" s="49" t="n"/>
+      <c r="AB37" s="49" t="n"/>
+      <c r="AC37" s="49" t="n"/>
+      <c r="AD37" s="49" t="n"/>
+      <c r="AE37" s="49" t="n"/>
+      <c r="AF37" s="49" t="n"/>
+      <c r="AK37" s="47" t="n"/>
+      <c r="AL37" s="47" t="n"/>
+      <c r="AN37" s="47" t="n"/>
+      <c r="AO37" s="47" t="n"/>
+      <c r="AQ37" s="47" t="n"/>
+      <c r="AS37" s="47" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="45" t="n"/>
-      <c r="B38" s="46" t="n"/>
-      <c r="C38" s="47" t="n"/>
-      <c r="D38" s="48" t="n"/>
-      <c r="E38" s="48" t="n"/>
-      <c r="F38" s="48" t="n"/>
-      <c r="G38" s="48" t="n"/>
-      <c r="H38" s="48" t="n"/>
-      <c r="I38" s="48" t="n"/>
-      <c r="J38" s="48" t="n"/>
-      <c r="K38" s="48" t="n"/>
-      <c r="L38" s="48" t="n"/>
-      <c r="M38" s="48" t="n"/>
-      <c r="N38" s="48" t="n"/>
-      <c r="O38" s="48" t="n"/>
-      <c r="P38" s="48" t="n"/>
-      <c r="Q38" s="48" t="n"/>
-      <c r="R38" s="48" t="n"/>
-      <c r="S38" s="48" t="n"/>
-      <c r="T38" s="48" t="n"/>
-      <c r="U38" s="48" t="n"/>
-      <c r="V38" s="48" t="n"/>
-      <c r="W38" s="49" t="n"/>
-      <c r="X38" s="49" t="n"/>
-      <c r="Y38" s="48" t="n"/>
-      <c r="Z38" s="48" t="n"/>
-      <c r="AA38" s="48" t="n"/>
-      <c r="AB38" s="48" t="n"/>
-      <c r="AC38" s="48" t="n"/>
-      <c r="AD38" s="48" t="n"/>
-      <c r="AE38" s="48" t="n"/>
-      <c r="AF38" s="48" t="n"/>
-      <c r="AK38" s="46" t="n"/>
-      <c r="AL38" s="46" t="n"/>
-      <c r="AN38" s="46" t="n"/>
-      <c r="AO38" s="46" t="n"/>
-      <c r="AQ38" s="46" t="n"/>
-      <c r="AS38" s="46" t="n"/>
+      <c r="A38" s="46" t="n"/>
+      <c r="B38" s="47" t="n"/>
+      <c r="C38" s="48" t="n"/>
+      <c r="D38" s="49" t="n"/>
+      <c r="E38" s="49" t="n"/>
+      <c r="F38" s="49" t="n"/>
+      <c r="G38" s="49" t="n"/>
+      <c r="H38" s="49" t="n"/>
+      <c r="I38" s="49" t="n"/>
+      <c r="J38" s="49" t="n"/>
+      <c r="K38" s="49" t="n"/>
+      <c r="L38" s="49" t="n"/>
+      <c r="M38" s="49" t="n"/>
+      <c r="N38" s="49" t="n"/>
+      <c r="O38" s="49" t="n"/>
+      <c r="P38" s="49" t="n"/>
+      <c r="Q38" s="49" t="n"/>
+      <c r="R38" s="49" t="n"/>
+      <c r="S38" s="49" t="n"/>
+      <c r="T38" s="49" t="n"/>
+      <c r="U38" s="49" t="n"/>
+      <c r="V38" s="49" t="n"/>
+      <c r="W38" s="50" t="n"/>
+      <c r="X38" s="50" t="n"/>
+      <c r="Y38" s="49" t="n"/>
+      <c r="Z38" s="49" t="n"/>
+      <c r="AA38" s="49" t="n"/>
+      <c r="AB38" s="49" t="n"/>
+      <c r="AC38" s="49" t="n"/>
+      <c r="AD38" s="49" t="n"/>
+      <c r="AE38" s="49" t="n"/>
+      <c r="AF38" s="49" t="n"/>
+      <c r="AK38" s="47" t="n"/>
+      <c r="AL38" s="47" t="n"/>
+      <c r="AN38" s="47" t="n"/>
+      <c r="AO38" s="47" t="n"/>
+      <c r="AQ38" s="47" t="n"/>
+      <c r="AS38" s="47" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="45" t="n"/>
-      <c r="B39" s="46" t="n"/>
-      <c r="C39" s="47" t="n"/>
-      <c r="D39" s="48" t="n"/>
-      <c r="E39" s="48" t="n"/>
-      <c r="F39" s="48" t="n"/>
-      <c r="G39" s="48" t="n"/>
-      <c r="H39" s="48" t="n"/>
-      <c r="I39" s="48" t="n"/>
-      <c r="J39" s="48" t="n"/>
-      <c r="K39" s="48" t="n"/>
-      <c r="L39" s="48" t="n"/>
-      <c r="M39" s="48" t="n"/>
-      <c r="N39" s="48" t="n"/>
-      <c r="O39" s="48" t="n"/>
-      <c r="P39" s="48" t="n"/>
-      <c r="Q39" s="48" t="n"/>
-      <c r="R39" s="48" t="n"/>
-      <c r="S39" s="48" t="n"/>
-      <c r="T39" s="48" t="n"/>
-      <c r="U39" s="48" t="n"/>
-      <c r="V39" s="48" t="n"/>
-      <c r="W39" s="49" t="n"/>
-      <c r="X39" s="49" t="n"/>
-      <c r="Y39" s="48" t="n"/>
-      <c r="Z39" s="48" t="n"/>
-      <c r="AA39" s="48" t="n"/>
-      <c r="AB39" s="48" t="n"/>
-      <c r="AC39" s="48" t="n"/>
-      <c r="AD39" s="48" t="n"/>
-      <c r="AE39" s="48" t="n"/>
-      <c r="AF39" s="48" t="n"/>
-      <c r="AK39" s="46" t="n"/>
-      <c r="AL39" s="46" t="n"/>
-      <c r="AN39" s="46" t="n"/>
-      <c r="AO39" s="46" t="n"/>
-      <c r="AQ39" s="46" t="n"/>
-      <c r="AS39" s="46" t="n"/>
+      <c r="A39" s="46" t="n"/>
+      <c r="B39" s="47" t="n"/>
+      <c r="C39" s="48" t="n"/>
+      <c r="D39" s="49" t="n"/>
+      <c r="E39" s="49" t="n"/>
+      <c r="F39" s="49" t="n"/>
+      <c r="G39" s="49" t="n"/>
+      <c r="H39" s="49" t="n"/>
+      <c r="I39" s="49" t="n"/>
+      <c r="J39" s="49" t="n"/>
+      <c r="K39" s="49" t="n"/>
+      <c r="L39" s="49" t="n"/>
+      <c r="M39" s="49" t="n"/>
+      <c r="N39" s="49" t="n"/>
+      <c r="O39" s="49" t="n"/>
+      <c r="P39" s="49" t="n"/>
+      <c r="Q39" s="49" t="n"/>
+      <c r="R39" s="49" t="n"/>
+      <c r="S39" s="49" t="n"/>
+      <c r="T39" s="49" t="n"/>
+      <c r="U39" s="49" t="n"/>
+      <c r="V39" s="49" t="n"/>
+      <c r="W39" s="50" t="n"/>
+      <c r="X39" s="50" t="n"/>
+      <c r="Y39" s="49" t="n"/>
+      <c r="Z39" s="49" t="n"/>
+      <c r="AA39" s="49" t="n"/>
+      <c r="AB39" s="49" t="n"/>
+      <c r="AC39" s="49" t="n"/>
+      <c r="AD39" s="49" t="n"/>
+      <c r="AE39" s="49" t="n"/>
+      <c r="AF39" s="49" t="n"/>
+      <c r="AK39" s="47" t="n"/>
+      <c r="AL39" s="47" t="n"/>
+      <c r="AN39" s="47" t="n"/>
+      <c r="AO39" s="47" t="n"/>
+      <c r="AQ39" s="47" t="n"/>
+      <c r="AS39" s="47" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="n"/>
-      <c r="C40" s="47" t="n"/>
-      <c r="D40" s="48" t="n"/>
-      <c r="E40" s="48" t="n"/>
-      <c r="F40" s="48" t="n"/>
-      <c r="G40" s="48" t="n"/>
-      <c r="H40" s="48" t="n"/>
-      <c r="I40" s="48" t="n"/>
-      <c r="J40" s="48" t="n"/>
-      <c r="K40" s="48" t="n"/>
-      <c r="L40" s="48" t="n"/>
-      <c r="M40" s="48" t="n"/>
-      <c r="N40" s="48" t="n"/>
-      <c r="O40" s="48" t="n"/>
-      <c r="P40" s="48" t="n"/>
-      <c r="Q40" s="48" t="n"/>
-      <c r="R40" s="48" t="n"/>
-      <c r="S40" s="48" t="n"/>
-      <c r="T40" s="48" t="n"/>
-      <c r="U40" s="48" t="n"/>
-      <c r="V40" s="48" t="n"/>
-      <c r="W40" s="49" t="n"/>
-      <c r="X40" s="49" t="n"/>
-      <c r="Y40" s="48" t="n"/>
-      <c r="Z40" s="48" t="n"/>
-      <c r="AA40" s="48" t="n"/>
-      <c r="AB40" s="48" t="n"/>
-      <c r="AC40" s="48" t="n"/>
-      <c r="AD40" s="48" t="n"/>
-      <c r="AE40" s="48" t="n"/>
-      <c r="AF40" s="48" t="n"/>
-      <c r="AK40" s="46" t="n"/>
-      <c r="AL40" s="46" t="n"/>
-      <c r="AN40" s="46" t="n"/>
-      <c r="AO40" s="46" t="n"/>
-      <c r="AQ40" s="46" t="n"/>
-      <c r="AS40" s="46" t="n"/>
+      <c r="A40" s="46" t="n"/>
+      <c r="B40" s="47" t="n"/>
+      <c r="C40" s="48" t="n"/>
+      <c r="D40" s="49" t="n"/>
+      <c r="E40" s="49" t="n"/>
+      <c r="F40" s="49" t="n"/>
+      <c r="G40" s="49" t="n"/>
+      <c r="H40" s="49" t="n"/>
+      <c r="I40" s="49" t="n"/>
+      <c r="J40" s="49" t="n"/>
+      <c r="K40" s="49" t="n"/>
+      <c r="L40" s="49" t="n"/>
+      <c r="M40" s="49" t="n"/>
+      <c r="N40" s="49" t="n"/>
+      <c r="O40" s="49" t="n"/>
+      <c r="P40" s="49" t="n"/>
+      <c r="Q40" s="49" t="n"/>
+      <c r="R40" s="49" t="n"/>
+      <c r="S40" s="49" t="n"/>
+      <c r="T40" s="49" t="n"/>
+      <c r="U40" s="49" t="n"/>
+      <c r="V40" s="49" t="n"/>
+      <c r="W40" s="50" t="n"/>
+      <c r="X40" s="50" t="n"/>
+      <c r="Y40" s="49" t="n"/>
+      <c r="Z40" s="49" t="n"/>
+      <c r="AA40" s="49" t="n"/>
+      <c r="AB40" s="49" t="n"/>
+      <c r="AC40" s="49" t="n"/>
+      <c r="AD40" s="49" t="n"/>
+      <c r="AE40" s="49" t="n"/>
+      <c r="AF40" s="49" t="n"/>
+      <c r="AK40" s="47" t="n"/>
+      <c r="AL40" s="47" t="n"/>
+      <c r="AN40" s="47" t="n"/>
+      <c r="AO40" s="47" t="n"/>
+      <c r="AQ40" s="47" t="n"/>
+      <c r="AS40" s="47" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="45" t="n"/>
-      <c r="B41" s="46" t="n"/>
-      <c r="C41" s="47" t="n"/>
-      <c r="D41" s="48" t="n"/>
-      <c r="E41" s="48" t="n"/>
-      <c r="F41" s="48" t="n"/>
-      <c r="G41" s="48" t="n"/>
-      <c r="H41" s="48" t="n"/>
-      <c r="I41" s="48" t="n"/>
-      <c r="J41" s="48" t="n"/>
-      <c r="K41" s="48" t="n"/>
-      <c r="L41" s="48" t="n"/>
-      <c r="M41" s="48" t="n"/>
-      <c r="N41" s="48" t="n"/>
-      <c r="O41" s="48" t="n"/>
-      <c r="P41" s="48" t="n"/>
-      <c r="Q41" s="48" t="n"/>
-      <c r="R41" s="48" t="n"/>
-      <c r="S41" s="48" t="n"/>
-      <c r="T41" s="48" t="n"/>
-      <c r="U41" s="48" t="n"/>
-      <c r="V41" s="48" t="n"/>
-      <c r="W41" s="49" t="n"/>
-      <c r="X41" s="49" t="n"/>
-      <c r="Y41" s="48" t="n"/>
-      <c r="Z41" s="48" t="n"/>
-      <c r="AA41" s="48" t="n"/>
-      <c r="AB41" s="48" t="n"/>
-      <c r="AC41" s="48" t="n"/>
-      <c r="AD41" s="48" t="n"/>
-      <c r="AE41" s="48" t="n"/>
-      <c r="AF41" s="48" t="n"/>
-      <c r="AK41" s="46" t="n"/>
-      <c r="AL41" s="46" t="n"/>
-      <c r="AN41" s="46" t="n"/>
-      <c r="AO41" s="46" t="n"/>
-      <c r="AQ41" s="46" t="n"/>
-      <c r="AS41" s="46" t="n"/>
+      <c r="A41" s="46" t="n"/>
+      <c r="B41" s="47" t="n"/>
+      <c r="C41" s="48" t="n"/>
+      <c r="D41" s="49" t="n"/>
+      <c r="E41" s="49" t="n"/>
+      <c r="F41" s="49" t="n"/>
+      <c r="G41" s="49" t="n"/>
+      <c r="H41" s="49" t="n"/>
+      <c r="I41" s="49" t="n"/>
+      <c r="J41" s="49" t="n"/>
+      <c r="K41" s="49" t="n"/>
+      <c r="L41" s="49" t="n"/>
+      <c r="M41" s="49" t="n"/>
+      <c r="N41" s="49" t="n"/>
+      <c r="O41" s="49" t="n"/>
+      <c r="P41" s="49" t="n"/>
+      <c r="Q41" s="49" t="n"/>
+      <c r="R41" s="49" t="n"/>
+      <c r="S41" s="49" t="n"/>
+      <c r="T41" s="49" t="n"/>
+      <c r="U41" s="49" t="n"/>
+      <c r="V41" s="49" t="n"/>
+      <c r="W41" s="50" t="n"/>
+      <c r="X41" s="50" t="n"/>
+      <c r="Y41" s="49" t="n"/>
+      <c r="Z41" s="49" t="n"/>
+      <c r="AA41" s="49" t="n"/>
+      <c r="AB41" s="49" t="n"/>
+      <c r="AC41" s="49" t="n"/>
+      <c r="AD41" s="49" t="n"/>
+      <c r="AE41" s="49" t="n"/>
+      <c r="AF41" s="49" t="n"/>
+      <c r="AK41" s="47" t="n"/>
+      <c r="AL41" s="47" t="n"/>
+      <c r="AN41" s="47" t="n"/>
+      <c r="AO41" s="47" t="n"/>
+      <c r="AQ41" s="47" t="n"/>
+      <c r="AS41" s="47" t="n"/>
     </row>
     <row r="42">
-      <c r="AK42" s="46" t="n"/>
-      <c r="AL42" s="46" t="n"/>
-      <c r="AN42" s="46" t="n"/>
-      <c r="AO42" s="46" t="n"/>
-      <c r="AQ42" s="46" t="n"/>
-      <c r="AS42" s="46" t="n"/>
+      <c r="AK42" s="47" t="n"/>
+      <c r="AL42" s="47" t="n"/>
+      <c r="AN42" s="47" t="n"/>
+      <c r="AO42" s="47" t="n"/>
+      <c r="AQ42" s="47" t="n"/>
+      <c r="AS42" s="47" t="n"/>
     </row>
     <row r="43">
-      <c r="AK43" s="46" t="n"/>
-      <c r="AL43" s="46" t="n"/>
-      <c r="AN43" s="46" t="n"/>
-      <c r="AO43" s="46" t="n"/>
-      <c r="AQ43" s="46" t="n"/>
-      <c r="AS43" s="46" t="n"/>
+      <c r="AK43" s="47" t="n"/>
+      <c r="AL43" s="47" t="n"/>
+      <c r="AN43" s="47" t="n"/>
+      <c r="AO43" s="47" t="n"/>
+      <c r="AQ43" s="47" t="n"/>
+      <c r="AS43" s="47" t="n"/>
     </row>
     <row r="44">
-      <c r="AK44" s="46" t="n"/>
-      <c r="AL44" s="46" t="n"/>
-      <c r="AN44" s="46" t="n"/>
-      <c r="AO44" s="46" t="n"/>
-      <c r="AQ44" s="46" t="n"/>
-      <c r="AS44" s="46" t="n"/>
+      <c r="AK44" s="47" t="n"/>
+      <c r="AL44" s="47" t="n"/>
+      <c r="AN44" s="47" t="n"/>
+      <c r="AO44" s="47" t="n"/>
+      <c r="AQ44" s="47" t="n"/>
+      <c r="AS44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
@@ -7610,50 +7716,50 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="44" t="inlineStr">
+      <c r="A46" s="45" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="B46" s="44" t="inlineStr">
+      <c r="B46" s="45" t="inlineStr">
         <is>
           <t>Rótulo</t>
         </is>
       </c>
-      <c r="C46" s="44" t="inlineStr">
+      <c r="C46" s="45" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D46" s="44" t="inlineStr">
+      <c r="D46" s="45" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="E46" s="44" t="inlineStr">
+      <c r="E46" s="45" t="inlineStr">
         <is>
           <t>Chave</t>
         </is>
       </c>
-      <c r="F46" s="44" t="inlineStr">
+      <c r="F46" s="45" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="G46" s="44" t="inlineStr">
+      <c r="G46" s="45" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="45" t="n"/>
-      <c r="B47" s="46" t="n"/>
-      <c r="C47" s="46" t="n"/>
-      <c r="D47" s="46" t="n"/>
-      <c r="E47" s="46" t="n"/>
-      <c r="F47" s="48" t="n"/>
-      <c r="G47" s="47" t="n"/>
+      <c r="A47" s="46" t="n"/>
+      <c r="B47" s="47" t="n"/>
+      <c r="C47" s="47" t="n"/>
+      <c r="D47" s="47" t="n"/>
+      <c r="E47" s="47" t="n"/>
+      <c r="F47" s="49" t="n"/>
+      <c r="G47" s="48" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10043,7 +10149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:Q46"/>
+  <dimension ref="B1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11960,7 +12066,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="18">
+      <c r="B35" s="36">
         <f>IF(Dados!$AS$5="","",Dados!$AS$5)</f>
         <v/>
       </c>
@@ -11974,7 +12080,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="18">
+      <c r="B36" s="36">
         <f>IF(Dados!$AS$6="","",Dados!$AS$6)</f>
         <v/>
       </c>
@@ -11988,7 +12094,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="18">
+      <c r="B37" s="36">
         <f>IF(Dados!$AS$7="","",Dados!$AS$7)</f>
         <v/>
       </c>
@@ -12002,7 +12108,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="18">
+      <c r="B38" s="36">
         <f>IF(Dados!$AS$8="","",Dados!$AS$8)</f>
         <v/>
       </c>
@@ -12016,7 +12122,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="18">
+      <c r="B39" s="36">
         <f>IF(Dados!$AS$9="","",Dados!$AS$9)</f>
         <v/>
       </c>
@@ -12030,7 +12136,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="18">
+      <c r="B40" s="36">
         <f>IF(Dados!$AS$10="","",Dados!$AS$10)</f>
         <v/>
       </c>
@@ -12044,7 +12150,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="18">
+      <c r="B41" s="36">
         <f>IF(Dados!$AS$11="","",Dados!$AS$11)</f>
         <v/>
       </c>
@@ -12058,7 +12164,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="18">
+      <c r="B42" s="36">
         <f>IF(Dados!$AS$12="","",Dados!$AS$12)</f>
         <v/>
       </c>
@@ -12072,7 +12178,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="18">
+      <c r="B43" s="36">
         <f>IF(Dados!$AS$13="","",Dados!$AS$13)</f>
         <v/>
       </c>
@@ -12086,7 +12192,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="18">
+      <c r="B44" s="36">
         <f>IF(Dados!$AS$14="","",Dados!$AS$14)</f>
         <v/>
       </c>
@@ -12102,7 +12208,14 @@
     <row r="46">
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>Inclui retiradas dos sócios e impostos, como no extrato. "sem detalhe": ano importado só com o total pago.</t>
+          <t>Inclui retiradas dos sócios e impostos, como no extrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>"sem detalhe": ano importado só com o total pago.</t>
         </is>
       </c>
     </row>
@@ -12333,7 +12446,7 @@
         <f>IF(N(O5)=0,"",IF(SUM($P$5:P5)-P5&lt;0.8,"A",IF(SUM($P$5:P5)-P5&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R5" s="36">
+      <c r="R5" s="37">
         <f>IF(Dados!$AL$5="","",Dados!$AL$5)</f>
         <v/>
       </c>
@@ -12407,7 +12520,7 @@
         <f>IF(N(O6)=0,"",IF(SUM($P$5:P6)-P6&lt;0.8,"A",IF(SUM($P$5:P6)-P6&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R6" s="36">
+      <c r="R6" s="37">
         <f>IF(Dados!$AL$6="","",Dados!$AL$6)</f>
         <v/>
       </c>
@@ -12481,7 +12594,7 @@
         <f>IF(N(O7)=0,"",IF(SUM($P$5:P7)-P7&lt;0.8,"A",IF(SUM($P$5:P7)-P7&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R7" s="36">
+      <c r="R7" s="37">
         <f>IF(Dados!$AL$7="","",Dados!$AL$7)</f>
         <v/>
       </c>
@@ -12555,7 +12668,7 @@
         <f>IF(N(O8)=0,"",IF(SUM($P$5:P8)-P8&lt;0.8,"A",IF(SUM($P$5:P8)-P8&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R8" s="36">
+      <c r="R8" s="37">
         <f>IF(Dados!$AL$8="","",Dados!$AL$8)</f>
         <v/>
       </c>
@@ -12629,7 +12742,7 @@
         <f>IF(N(O9)=0,"",IF(SUM($P$5:P9)-P9&lt;0.8,"A",IF(SUM($P$5:P9)-P9&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R9" s="36">
+      <c r="R9" s="37">
         <f>IF(Dados!$AL$9="","",Dados!$AL$9)</f>
         <v/>
       </c>
@@ -12703,7 +12816,7 @@
         <f>IF(N(O10)=0,"",IF(SUM($P$5:P10)-P10&lt;0.8,"A",IF(SUM($P$5:P10)-P10&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R10" s="36">
+      <c r="R10" s="37">
         <f>IF(Dados!$AL$10="","",Dados!$AL$10)</f>
         <v/>
       </c>
@@ -12777,7 +12890,7 @@
         <f>IF(N(O11)=0,"",IF(SUM($P$5:P11)-P11&lt;0.8,"A",IF(SUM($P$5:P11)-P11&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R11" s="36">
+      <c r="R11" s="37">
         <f>IF(Dados!$AL$11="","",Dados!$AL$11)</f>
         <v/>
       </c>
@@ -12851,7 +12964,7 @@
         <f>IF(N(O12)=0,"",IF(SUM($P$5:P12)-P12&lt;0.8,"A",IF(SUM($P$5:P12)-P12&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R12" s="36">
+      <c r="R12" s="37">
         <f>IF(Dados!$AL$12="","",Dados!$AL$12)</f>
         <v/>
       </c>
@@ -12925,7 +13038,7 @@
         <f>IF(N(O13)=0,"",IF(SUM($P$5:P13)-P13&lt;0.8,"A",IF(SUM($P$5:P13)-P13&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R13" s="36">
+      <c r="R13" s="37">
         <f>IF(Dados!$AL$13="","",Dados!$AL$13)</f>
         <v/>
       </c>
@@ -12999,7 +13112,7 @@
         <f>IF(N(O14)=0,"",IF(SUM($P$5:P14)-P14&lt;0.8,"A",IF(SUM($P$5:P14)-P14&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R14" s="36">
+      <c r="R14" s="37">
         <f>IF(Dados!$AL$14="","",Dados!$AL$14)</f>
         <v/>
       </c>
@@ -13073,7 +13186,7 @@
         <f>IF(N(O15)=0,"",IF(SUM($P$5:P15)-P15&lt;0.8,"A",IF(SUM($P$5:P15)-P15&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R15" s="36">
+      <c r="R15" s="37">
         <f>IF(Dados!$AL$15="","",Dados!$AL$15)</f>
         <v/>
       </c>
@@ -13147,7 +13260,7 @@
         <f>IF(N(O16)=0,"",IF(SUM($P$5:P16)-P16&lt;0.8,"A",IF(SUM($P$5:P16)-P16&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R16" s="36">
+      <c r="R16" s="37">
         <f>IF(Dados!$AL$16="","",Dados!$AL$16)</f>
         <v/>
       </c>
@@ -13221,7 +13334,7 @@
         <f>IF(N(O17)=0,"",IF(SUM($P$5:P17)-P17&lt;0.8,"A",IF(SUM($P$5:P17)-P17&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R17" s="36">
+      <c r="R17" s="37">
         <f>IF(Dados!$AL$17="","",Dados!$AL$17)</f>
         <v/>
       </c>
@@ -13295,7 +13408,7 @@
         <f>IF(N(O18)=0,"",IF(SUM($P$5:P18)-P18&lt;0.8,"A",IF(SUM($P$5:P18)-P18&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R18" s="36">
+      <c r="R18" s="37">
         <f>IF(Dados!$AL$18="","",Dados!$AL$18)</f>
         <v/>
       </c>
@@ -13369,7 +13482,7 @@
         <f>IF(N(O19)=0,"",IF(SUM($P$5:P19)-P19&lt;0.8,"A",IF(SUM($P$5:P19)-P19&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R19" s="36">
+      <c r="R19" s="37">
         <f>IF(Dados!$AL$19="","",Dados!$AL$19)</f>
         <v/>
       </c>
@@ -13443,7 +13556,7 @@
         <f>IF(N(O20)=0,"",IF(SUM($P$5:P20)-P20&lt;0.8,"A",IF(SUM($P$5:P20)-P20&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R20" s="36">
+      <c r="R20" s="37">
         <f>IF(Dados!$AL$20="","",Dados!$AL$20)</f>
         <v/>
       </c>
@@ -13517,7 +13630,7 @@
         <f>IF(N(O21)=0,"",IF(SUM($P$5:P21)-P21&lt;0.8,"A",IF(SUM($P$5:P21)-P21&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R21" s="36">
+      <c r="R21" s="37">
         <f>IF(Dados!$AL$21="","",Dados!$AL$21)</f>
         <v/>
       </c>
@@ -13591,7 +13704,7 @@
         <f>IF(N(O22)=0,"",IF(SUM($P$5:P22)-P22&lt;0.8,"A",IF(SUM($P$5:P22)-P22&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R22" s="36">
+      <c r="R22" s="37">
         <f>IF(Dados!$AL$22="","",Dados!$AL$22)</f>
         <v/>
       </c>
@@ -13665,7 +13778,7 @@
         <f>IF(N(O23)=0,"",IF(SUM($P$5:P23)-P23&lt;0.8,"A",IF(SUM($P$5:P23)-P23&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R23" s="36">
+      <c r="R23" s="37">
         <f>IF(Dados!$AL$23="","",Dados!$AL$23)</f>
         <v/>
       </c>
@@ -13739,7 +13852,7 @@
         <f>IF(N(O24)=0,"",IF(SUM($P$5:P24)-P24&lt;0.8,"A",IF(SUM($P$5:P24)-P24&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R24" s="36">
+      <c r="R24" s="37">
         <f>IF(Dados!$AL$24="","",Dados!$AL$24)</f>
         <v/>
       </c>
@@ -13813,7 +13926,7 @@
         <f>IF(N(O25)=0,"",IF(SUM($P$5:P25)-P25&lt;0.8,"A",IF(SUM($P$5:P25)-P25&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R25" s="36">
+      <c r="R25" s="37">
         <f>IF(Dados!$AL$25="","",Dados!$AL$25)</f>
         <v/>
       </c>
@@ -13887,7 +14000,7 @@
         <f>IF(N(O26)=0,"",IF(SUM($P$5:P26)-P26&lt;0.8,"A",IF(SUM($P$5:P26)-P26&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R26" s="36">
+      <c r="R26" s="37">
         <f>IF(Dados!$AL$26="","",Dados!$AL$26)</f>
         <v/>
       </c>
@@ -13961,7 +14074,7 @@
         <f>IF(N(O27)=0,"",IF(SUM($P$5:P27)-P27&lt;0.8,"A",IF(SUM($P$5:P27)-P27&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R27" s="36">
+      <c r="R27" s="37">
         <f>IF(Dados!$AL$27="","",Dados!$AL$27)</f>
         <v/>
       </c>
@@ -14035,7 +14148,7 @@
         <f>IF(N(O28)=0,"",IF(SUM($P$5:P28)-P28&lt;0.8,"A",IF(SUM($P$5:P28)-P28&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R28" s="36">
+      <c r="R28" s="37">
         <f>IF(Dados!$AL$28="","",Dados!$AL$28)</f>
         <v/>
       </c>
@@ -14109,7 +14222,7 @@
         <f>IF(N(O29)=0,"",IF(SUM($P$5:P29)-P29&lt;0.8,"A",IF(SUM($P$5:P29)-P29&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R29" s="36">
+      <c r="R29" s="37">
         <f>IF(Dados!$AL$29="","",Dados!$AL$29)</f>
         <v/>
       </c>
@@ -14183,7 +14296,7 @@
         <f>IF(N(O30)=0,"",IF(SUM($P$5:P30)-P30&lt;0.8,"A",IF(SUM($P$5:P30)-P30&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R30" s="36">
+      <c r="R30" s="37">
         <f>IF(Dados!$AL$30="","",Dados!$AL$30)</f>
         <v/>
       </c>
@@ -14257,7 +14370,7 @@
         <f>IF(N(O31)=0,"",IF(SUM($P$5:P31)-P31&lt;0.8,"A",IF(SUM($P$5:P31)-P31&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R31" s="36">
+      <c r="R31" s="37">
         <f>IF(Dados!$AL$31="","",Dados!$AL$31)</f>
         <v/>
       </c>
@@ -14331,7 +14444,7 @@
         <f>IF(N(O32)=0,"",IF(SUM($P$5:P32)-P32&lt;0.8,"A",IF(SUM($P$5:P32)-P32&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R32" s="36">
+      <c r="R32" s="37">
         <f>IF(Dados!$AL$32="","",Dados!$AL$32)</f>
         <v/>
       </c>
@@ -14405,7 +14518,7 @@
         <f>IF(N(O33)=0,"",IF(SUM($P$5:P33)-P33&lt;0.8,"A",IF(SUM($P$5:P33)-P33&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R33" s="36">
+      <c r="R33" s="37">
         <f>IF(Dados!$AL$33="","",Dados!$AL$33)</f>
         <v/>
       </c>
@@ -14479,7 +14592,7 @@
         <f>IF(N(O34)=0,"",IF(SUM($P$5:P34)-P34&lt;0.8,"A",IF(SUM($P$5:P34)-P34&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R34" s="36">
+      <c r="R34" s="37">
         <f>IF(Dados!$AL$34="","",Dados!$AL$34)</f>
         <v/>
       </c>
@@ -14553,7 +14666,7 @@
         <f>IF(N(O35)=0,"",IF(SUM($P$5:P35)-P35&lt;0.8,"A",IF(SUM($P$5:P35)-P35&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R35" s="36">
+      <c r="R35" s="37">
         <f>IF(Dados!$AL$35="","",Dados!$AL$35)</f>
         <v/>
       </c>
@@ -14627,7 +14740,7 @@
         <f>IF(N(O36)=0,"",IF(SUM($P$5:P36)-P36&lt;0.8,"A",IF(SUM($P$5:P36)-P36&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R36" s="36">
+      <c r="R36" s="37">
         <f>IF(Dados!$AL$36="","",Dados!$AL$36)</f>
         <v/>
       </c>
@@ -14701,7 +14814,7 @@
         <f>IF(N(O37)=0,"",IF(SUM($P$5:P37)-P37&lt;0.8,"A",IF(SUM($P$5:P37)-P37&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R37" s="36">
+      <c r="R37" s="37">
         <f>IF(Dados!$AL$37="","",Dados!$AL$37)</f>
         <v/>
       </c>
@@ -14775,7 +14888,7 @@
         <f>IF(N(O38)=0,"",IF(SUM($P$5:P38)-P38&lt;0.8,"A",IF(SUM($P$5:P38)-P38&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R38" s="36">
+      <c r="R38" s="37">
         <f>IF(Dados!$AL$38="","",Dados!$AL$38)</f>
         <v/>
       </c>
@@ -14849,7 +14962,7 @@
         <f>IF(N(O39)=0,"",IF(SUM($P$5:P39)-P39&lt;0.8,"A",IF(SUM($P$5:P39)-P39&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R39" s="36">
+      <c r="R39" s="37">
         <f>IF(Dados!$AL$39="","",Dados!$AL$39)</f>
         <v/>
       </c>
@@ -14923,7 +15036,7 @@
         <f>IF(N(O40)=0,"",IF(SUM($P$5:P40)-P40&lt;0.8,"A",IF(SUM($P$5:P40)-P40&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R40" s="36">
+      <c r="R40" s="37">
         <f>IF(Dados!$AL$40="","",Dados!$AL$40)</f>
         <v/>
       </c>
@@ -14997,7 +15110,7 @@
         <f>IF(N(O41)=0,"",IF(SUM($P$5:P41)-P41&lt;0.8,"A",IF(SUM($P$5:P41)-P41&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R41" s="36">
+      <c r="R41" s="37">
         <f>IF(Dados!$AL$41="","",Dados!$AL$41)</f>
         <v/>
       </c>
@@ -15071,7 +15184,7 @@
         <f>IF(N(O42)=0,"",IF(SUM($P$5:P42)-P42&lt;0.8,"A",IF(SUM($P$5:P42)-P42&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R42" s="36">
+      <c r="R42" s="37">
         <f>IF(Dados!$AL$42="","",Dados!$AL$42)</f>
         <v/>
       </c>
@@ -15145,7 +15258,7 @@
         <f>IF(N(O43)=0,"",IF(SUM($P$5:P43)-P43&lt;0.8,"A",IF(SUM($P$5:P43)-P43&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R43" s="36">
+      <c r="R43" s="37">
         <f>IF(Dados!$AL$43="","",Dados!$AL$43)</f>
         <v/>
       </c>
@@ -15219,7 +15332,7 @@
         <f>IF(N(O44)=0,"",IF(SUM($P$5:P44)-P44&lt;0.8,"A",IF(SUM($P$5:P44)-P44&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R44" s="36">
+      <c r="R44" s="37">
         <f>IF(Dados!$AL$44="","",Dados!$AL$44)</f>
         <v/>
       </c>
@@ -17145,7 +17258,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>Vencido há até 30 dias</t>
         </is>
@@ -17200,7 +17313,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Vencido há mais de 30 dias</t>
         </is>
@@ -17482,7 +17595,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>Vencido há até 30 dias</t>
         </is>
@@ -17537,7 +17650,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="37" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Vencido há mais de 30 dias</t>
         </is>
@@ -17921,7 +18034,7 @@
         <f>VLOOKUP($B5,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="39">
         <f>C5+D5</f>
         <v/>
       </c>
@@ -17951,7 +18064,7 @@
         <f>VLOOKUP($B6,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="39">
         <f>C6+D6</f>
         <v/>
       </c>
@@ -17981,7 +18094,7 @@
         <f>VLOOKUP($B7,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="39">
         <f>C7+D7</f>
         <v/>
       </c>
@@ -18011,7 +18124,7 @@
         <f>VLOOKUP($B8,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="39">
         <f>C8+D8</f>
         <v/>
       </c>
@@ -18041,7 +18154,7 @@
         <f>VLOOKUP($B9,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="39">
         <f>C9+D9</f>
         <v/>
       </c>
@@ -18071,7 +18184,7 @@
         <f>VLOOKUP($B10,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E10" s="38">
+      <c r="E10" s="39">
         <f>C10+D10</f>
         <v/>
       </c>
@@ -18101,7 +18214,7 @@
         <f>VLOOKUP($B11,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="39">
         <f>C11+D11</f>
         <v/>
       </c>
@@ -18131,7 +18244,7 @@
         <f>VLOOKUP($B12,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E12" s="38">
+      <c r="E12" s="39">
         <f>C12+D12</f>
         <v/>
       </c>
@@ -18161,7 +18274,7 @@
         <f>VLOOKUP($B13,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E13" s="38">
+      <c r="E13" s="39">
         <f>C13+D13</f>
         <v/>
       </c>
@@ -18191,7 +18304,7 @@
         <f>VLOOKUP($B14,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E14" s="38">
+      <c r="E14" s="39">
         <f>C14+D14</f>
         <v/>
       </c>
@@ -18221,7 +18334,7 @@
         <f>VLOOKUP($B15,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E15" s="38">
+      <c r="E15" s="39">
         <f>C15+D15</f>
         <v/>
       </c>
@@ -18251,7 +18364,7 @@
         <f>VLOOKUP($B16,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E16" s="38">
+      <c r="E16" s="39">
         <f>C16+D16</f>
         <v/>
       </c>
@@ -18281,7 +18394,7 @@
         <f>VLOOKUP($B17,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E17" s="38">
+      <c r="E17" s="39">
         <f>C17+D17</f>
         <v/>
       </c>
@@ -18311,7 +18424,7 @@
         <f>VLOOKUP($B18,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E18" s="38">
+      <c r="E18" s="39">
         <f>C18+D18</f>
         <v/>
       </c>
@@ -18341,7 +18454,7 @@
         <f>VLOOKUP($B19,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E19" s="38">
+      <c r="E19" s="39">
         <f>C19+D19</f>
         <v/>
       </c>
@@ -18371,7 +18484,7 @@
         <f>VLOOKUP($B20,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E20" s="38">
+      <c r="E20" s="39">
         <f>C20+D20</f>
         <v/>
       </c>
@@ -18401,7 +18514,7 @@
         <f>VLOOKUP($B21,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E21" s="38">
+      <c r="E21" s="39">
         <f>C21+D21</f>
         <v/>
       </c>
@@ -18431,7 +18544,7 @@
         <f>VLOOKUP($B22,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E22" s="38">
+      <c r="E22" s="39">
         <f>C22+D22</f>
         <v/>
       </c>
@@ -18461,7 +18574,7 @@
         <f>VLOOKUP($B23,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E23" s="38">
+      <c r="E23" s="39">
         <f>C23+D23</f>
         <v/>
       </c>
@@ -18491,7 +18604,7 @@
         <f>VLOOKUP($B24,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E24" s="38">
+      <c r="E24" s="39">
         <f>C24+D24</f>
         <v/>
       </c>
@@ -18521,7 +18634,7 @@
         <f>VLOOKUP($B25,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E25" s="38">
+      <c r="E25" s="39">
         <f>C25+D25</f>
         <v/>
       </c>
@@ -18551,7 +18664,7 @@
         <f>VLOOKUP($B26,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E26" s="38">
+      <c r="E26" s="39">
         <f>C26+D26</f>
         <v/>
       </c>
@@ -18581,7 +18694,7 @@
         <f>VLOOKUP($B27,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E27" s="38">
+      <c r="E27" s="39">
         <f>C27+D27</f>
         <v/>
       </c>
@@ -18599,31 +18712,31 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="39">
+      <c r="B28" s="40">
         <f>VLOOKUP(EOMONTH(Dados!$AI$5,-1)+1,Dados!$A$5:$B$41,2,FALSE)</f>
         <v/>
       </c>
-      <c r="C28" s="40">
+      <c r="C28" s="41">
         <f>VLOOKUP($B28,Dados!$B$5:$AF$41,10,FALSE)</f>
         <v/>
       </c>
-      <c r="D28" s="40">
+      <c r="D28" s="41">
         <f>VLOOKUP($B28,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E28" s="40">
+      <c r="E28" s="41">
         <f>C28+D28</f>
         <v/>
       </c>
-      <c r="F28" s="41">
+      <c r="F28" s="42">
         <f>E28-E27</f>
         <v/>
       </c>
-      <c r="G28" s="41">
+      <c r="G28" s="42">
         <f>VLOOKUP($B28,Dados!$B$5:$AF$41,5,FALSE)</f>
         <v/>
       </c>
-      <c r="H28" s="42">
+      <c r="H28" s="43">
         <f>IFERROR(E28/AVERAGE(G26:G28),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix(workbook): gráficos sem texto sobreposto no Excel (#117)
- Título e legenda com overlay desligado: o Excel desenhava os dois por cima
  da área do gráfico e dos rótulos do eixo.
- Barras negativas (pago) sem inversão de cor: saíam brancas.
- Rankings (categorias, clientes, estados) com o valor na ponta da barra e
  sem eixo de valores, que ia para o topo e encostava no título.
- Rótulos das categorias como texto (strRef).
- O cache dos gráficos agora é gravado também no XML sem prefixo "c:"
  (openpyxl): o arquivo abre com os gráficos preenchidos sem recálculo.
- Nomes longos de fornecedor reduzem a fonte em vez de cortar; nota da aba
  Despesas em duas linhas para não passar por baixo do gráfico.


Claude-Session: https://claude.ai/code/session_01NefkA2otxn5XifgkSQBnwE

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v2.xlsx
+++ b/public/workbook_fechamento_v2.xlsx
@@ -209,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -307,6 +307,9 @@
     </xf>
     <xf numFmtId="166" fontId="13" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" shrinkToFit="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -481,6 +484,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -503,10 +507,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resultado'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -531,10 +536,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resultado'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -580,6 +586,11 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <strRef>
+              <f>'Resultado'!$C$4:$N$4</f>
+            </strRef>
+          </cat>
           <val>
             <numRef>
               <f>'Resultado'!$C$90:$N$90</f>
@@ -686,6 +697,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -744,6 +756,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -780,9 +793,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Redes'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -823,9 +836,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Redes'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -933,6 +946,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -991,6 +1005,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1013,10 +1028,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1041,10 +1057,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1151,6 +1168,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1209,6 +1227,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <lineChart>
@@ -1245,9 +1264,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1288,9 +1307,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1331,9 +1350,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Faturamento'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1440,6 +1459,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1498,6 +1518,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1520,10 +1541,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Caixa'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1548,10 +1570,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Caixa'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1597,6 +1620,11 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <strRef>
+              <f>'Caixa'!$C$4:$N$4</f>
+            </strRef>
+          </cat>
           <val>
             <numRef>
               <f>'Caixa'!$C$13:$N$13</f>
@@ -1702,6 +1730,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -1760,6 +1789,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1782,10 +1812,42 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="800" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="1B1411"/>
+                    </a:solidFill>
+                    <a:latin typeface="Montserrat"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="1B1411"/>
+                  </a:solidFill>
+                  <a:latin typeface="Montserrat"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Despesas'!$B$5:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1844,18 +1906,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="E4DCD2"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -1925,6 +1977,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -1947,10 +2000,42 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="800" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="1B1411"/>
+                    </a:solidFill>
+                    <a:latin typeface="Montserrat"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="1B1411"/>
+                  </a:solidFill>
+                  <a:latin typeface="Montserrat"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Clientes'!$B$5:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2009,18 +2094,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="E4DCD2"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -2090,6 +2165,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2112,10 +2188,42 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="800" b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="1B1411"/>
+                    </a:solidFill>
+                    <a:latin typeface="Montserrat"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+                <a:endParaRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="1B1411"/>
+                  </a:solidFill>
+                  <a:latin typeface="Montserrat"/>
+                </a:endParaRPr>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Estados'!$B$5:$B$14</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2174,18 +2282,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="E4DCD2"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -2255,6 +2353,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2277,10 +2376,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Capital de giro'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2305,10 +2405,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Capital de giro'!$C$4:$N$4</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2415,6 +2516,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -2473,6 +2575,7 @@
           </a:p>
         </rich>
       </tx>
+      <overlay val="0"/>
     </title>
     <plotArea>
       <barChart>
@@ -2495,10 +2598,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Estoque'!$B$5:$B$28</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2523,10 +2627,11 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Estoque'!$B$5:$B$28</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -2634,6 +2739,7 @@
     </plotArea>
     <legend>
       <legendPos val="b"/>
+      <overlay val="0"/>
       <txPr>
         <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -5257,51 +5363,51 @@
           <t>ganho no mês</t>
         </is>
       </c>
-      <c r="C6" s="43">
+      <c r="C6" s="44">
         <f>IF(AND(ISNUMBER(C5),ISNUMBER(Dados!$W$29)),C5-Dados!$W$29,"")</f>
         <v/>
       </c>
-      <c r="D6" s="43">
+      <c r="D6" s="44">
         <f>IF(AND(ISNUMBER(D5),ISNUMBER(C5)),D5-C5,"")</f>
         <v/>
       </c>
-      <c r="E6" s="43">
+      <c r="E6" s="44">
         <f>IF(AND(ISNUMBER(E5),ISNUMBER(D5)),E5-D5,"")</f>
         <v/>
       </c>
-      <c r="F6" s="43">
+      <c r="F6" s="44">
         <f>IF(AND(ISNUMBER(F5),ISNUMBER(E5)),F5-E5,"")</f>
         <v/>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="44">
         <f>IF(AND(ISNUMBER(G5),ISNUMBER(F5)),G5-F5,"")</f>
         <v/>
       </c>
-      <c r="H6" s="43">
+      <c r="H6" s="44">
         <f>IF(AND(ISNUMBER(H5),ISNUMBER(G5)),H5-G5,"")</f>
         <v/>
       </c>
-      <c r="I6" s="43">
+      <c r="I6" s="44">
         <f>IF(AND(ISNUMBER(I5),ISNUMBER(H5)),I5-H5,"")</f>
         <v/>
       </c>
-      <c r="J6" s="43">
+      <c r="J6" s="44">
         <f>IF(AND(ISNUMBER(J5),ISNUMBER(I5)),J5-I5,"")</f>
         <v/>
       </c>
-      <c r="K6" s="43">
+      <c r="K6" s="44">
         <f>IF(AND(ISNUMBER(K5),ISNUMBER(J5)),K5-J5,"")</f>
         <v/>
       </c>
-      <c r="L6" s="43">
+      <c r="L6" s="44">
         <f>IF(AND(ISNUMBER(L5),ISNUMBER(K5)),L5-K5,"")</f>
         <v/>
       </c>
-      <c r="M6" s="43">
+      <c r="M6" s="44">
         <f>IF(AND(ISNUMBER(M5),ISNUMBER(L5)),M5-L5,"")</f>
         <v/>
       </c>
-      <c r="N6" s="43">
+      <c r="N6" s="44">
         <f>IF(AND(ISNUMBER(N5),ISNUMBER(M5)),N5-M5,"")</f>
         <v/>
       </c>
@@ -5372,51 +5478,51 @@
           <t>ganho no mês</t>
         </is>
       </c>
-      <c r="C8" s="43">
+      <c r="C8" s="44">
         <f>IF(AND(ISNUMBER(C7),ISNUMBER(Dados!$X$29)),C7-Dados!$X$29,"")</f>
         <v/>
       </c>
-      <c r="D8" s="43">
+      <c r="D8" s="44">
         <f>IF(AND(ISNUMBER(D7),ISNUMBER(C7)),D7-C7,"")</f>
         <v/>
       </c>
-      <c r="E8" s="43">
+      <c r="E8" s="44">
         <f>IF(AND(ISNUMBER(E7),ISNUMBER(D7)),E7-D7,"")</f>
         <v/>
       </c>
-      <c r="F8" s="43">
+      <c r="F8" s="44">
         <f>IF(AND(ISNUMBER(F7),ISNUMBER(E7)),F7-E7,"")</f>
         <v/>
       </c>
-      <c r="G8" s="43">
+      <c r="G8" s="44">
         <f>IF(AND(ISNUMBER(G7),ISNUMBER(F7)),G7-F7,"")</f>
         <v/>
       </c>
-      <c r="H8" s="43">
+      <c r="H8" s="44">
         <f>IF(AND(ISNUMBER(H7),ISNUMBER(G7)),H7-G7,"")</f>
         <v/>
       </c>
-      <c r="I8" s="43">
+      <c r="I8" s="44">
         <f>IF(AND(ISNUMBER(I7),ISNUMBER(H7)),I7-H7,"")</f>
         <v/>
       </c>
-      <c r="J8" s="43">
+      <c r="J8" s="44">
         <f>IF(AND(ISNUMBER(J7),ISNUMBER(I7)),J7-I7,"")</f>
         <v/>
       </c>
-      <c r="K8" s="43">
+      <c r="K8" s="44">
         <f>IF(AND(ISNUMBER(K7),ISNUMBER(J7)),K7-J7,"")</f>
         <v/>
       </c>
-      <c r="L8" s="43">
+      <c r="L8" s="44">
         <f>IF(AND(ISNUMBER(L7),ISNUMBER(K7)),L7-K7,"")</f>
         <v/>
       </c>
-      <c r="M8" s="43">
+      <c r="M8" s="44">
         <f>IF(AND(ISNUMBER(M7),ISNUMBER(L7)),M7-L7,"")</f>
         <v/>
       </c>
-      <c r="N8" s="43">
+      <c r="N8" s="44">
         <f>IF(AND(ISNUMBER(N7),ISNUMBER(M7)),N7-M7,"")</f>
         <v/>
       </c>
@@ -5753,1854 +5859,1854 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="B4" s="44" t="inlineStr">
+      <c r="B4" s="45" t="inlineStr">
         <is>
           <t>Rótulo</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="45" t="inlineStr">
         <is>
           <t>Fechado</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
+      <c r="D4" s="45" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="E4" s="44" t="inlineStr">
+      <c r="E4" s="45" t="inlineStr">
         <is>
           <t>Pago</t>
         </is>
       </c>
-      <c r="F4" s="44" t="inlineStr">
+      <c r="F4" s="45" t="inlineStr">
         <is>
           <t>Faturamento</t>
         </is>
       </c>
-      <c r="G4" s="44" t="inlineStr">
+      <c r="G4" s="45" t="inlineStr">
         <is>
           <t>Caixa final</t>
         </is>
       </c>
-      <c r="H4" s="44" t="inlineStr">
+      <c r="H4" s="45" t="inlineStr">
         <is>
           <t>Caixa calculado (ERP)</t>
         </is>
       </c>
-      <c r="I4" s="44" t="inlineStr">
+      <c r="I4" s="45" t="inlineStr">
         <is>
           <t>Ajuste ao extrato</t>
         </is>
       </c>
-      <c r="J4" s="44" t="inlineStr">
+      <c r="J4" s="45" t="inlineStr">
         <is>
           <t>Bloqueado</t>
         </is>
       </c>
-      <c r="K4" s="44" t="inlineStr">
+      <c r="K4" s="45" t="inlineStr">
         <is>
           <t>Estoque produtos</t>
         </is>
       </c>
-      <c r="L4" s="44" t="inlineStr">
+      <c r="L4" s="45" t="inlineStr">
         <is>
           <t>Estoque materiais</t>
         </is>
       </c>
-      <c r="M4" s="44" t="inlineStr">
+      <c r="M4" s="45" t="inlineStr">
         <is>
           <t>Receber a vencer 0-30</t>
         </is>
       </c>
-      <c r="N4" s="44" t="inlineStr">
+      <c r="N4" s="45" t="inlineStr">
         <is>
           <t>Receber a vencer 31-90</t>
         </is>
       </c>
-      <c r="O4" s="44" t="inlineStr">
+      <c r="O4" s="45" t="inlineStr">
         <is>
           <t>Receber a vencer &gt;90</t>
         </is>
       </c>
-      <c r="P4" s="44" t="inlineStr">
+      <c r="P4" s="45" t="inlineStr">
         <is>
           <t>Receber vencido 0-30</t>
         </is>
       </c>
-      <c r="Q4" s="44" t="inlineStr">
+      <c r="Q4" s="45" t="inlineStr">
         <is>
           <t>Receber vencido &gt;30</t>
         </is>
       </c>
-      <c r="R4" s="44" t="inlineStr">
+      <c r="R4" s="45" t="inlineStr">
         <is>
           <t>Pagar a vencer 0-30</t>
         </is>
       </c>
-      <c r="S4" s="44" t="inlineStr">
+      <c r="S4" s="45" t="inlineStr">
         <is>
           <t>Pagar a vencer 31-90</t>
         </is>
       </c>
-      <c r="T4" s="44" t="inlineStr">
+      <c r="T4" s="45" t="inlineStr">
         <is>
           <t>Pagar a vencer &gt;90</t>
         </is>
       </c>
-      <c r="U4" s="44" t="inlineStr">
+      <c r="U4" s="45" t="inlineStr">
         <is>
           <t>Pagar vencido 0-30</t>
         </is>
       </c>
-      <c r="V4" s="44" t="inlineStr">
+      <c r="V4" s="45" t="inlineStr">
         <is>
           <t>Pagar vencido &gt;30</t>
         </is>
       </c>
-      <c r="W4" s="44" t="inlineStr">
+      <c r="W4" s="45" t="inlineStr">
         <is>
           <t>Seguidores LinkedIn</t>
         </is>
       </c>
-      <c r="X4" s="44" t="inlineStr">
+      <c r="X4" s="45" t="inlineStr">
         <is>
           <t>Seguidores Instagram</t>
         </is>
       </c>
-      <c r="Y4" s="44" t="inlineStr">
+      <c r="Y4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 1</t>
         </is>
       </c>
-      <c r="Z4" s="44" t="inlineStr">
+      <c r="Z4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 2</t>
         </is>
       </c>
-      <c r="AA4" s="44" t="inlineStr">
+      <c r="AA4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 3</t>
         </is>
       </c>
-      <c r="AB4" s="44" t="inlineStr">
+      <c r="AB4" s="45" t="inlineStr">
         <is>
           <t>Retirada sócio 4</t>
         </is>
       </c>
-      <c r="AC4" s="44" t="inlineStr">
+      <c r="AC4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 1</t>
         </is>
       </c>
-      <c r="AD4" s="44" t="inlineStr">
+      <c r="AD4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 2</t>
         </is>
       </c>
-      <c r="AE4" s="44" t="inlineStr">
+      <c r="AE4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 3</t>
         </is>
       </c>
-      <c r="AF4" s="44" t="inlineStr">
+      <c r="AF4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 4</t>
         </is>
       </c>
-      <c r="AH4" s="44" t="inlineStr">
+      <c r="AH4" s="45" t="inlineStr">
         <is>
           <t>Parâmetro</t>
         </is>
       </c>
-      <c r="AI4" s="44" t="inlineStr">
+      <c r="AI4" s="45" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="AK4" s="44" t="inlineStr">
+      <c r="AK4" s="45" t="inlineStr">
         <is>
           <t>Cliente (grupo)</t>
         </is>
       </c>
-      <c r="AL4" s="44" t="inlineStr">
+      <c r="AL4" s="45" t="inlineStr">
         <is>
           <t>1ª compra</t>
         </is>
       </c>
-      <c r="AN4" s="44" t="inlineStr">
+      <c r="AN4" s="45" t="inlineStr">
         <is>
           <t>UF</t>
         </is>
       </c>
-      <c r="AO4" s="44" t="inlineStr">
+      <c r="AO4" s="45" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="AQ4" s="44" t="inlineStr">
+      <c r="AQ4" s="45" t="inlineStr">
         <is>
           <t>Categoria de despesa</t>
         </is>
       </c>
-      <c r="AS4" s="44" t="inlineStr">
+      <c r="AS4" s="45" t="inlineStr">
         <is>
           <t>Fornecedor do mês</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="45" t="n"/>
-      <c r="B5" s="46" t="n"/>
-      <c r="C5" s="47" t="n"/>
-      <c r="D5" s="48" t="n"/>
-      <c r="E5" s="48" t="n"/>
-      <c r="F5" s="48" t="n"/>
-      <c r="G5" s="48" t="n"/>
-      <c r="H5" s="48" t="n"/>
-      <c r="I5" s="48" t="n"/>
-      <c r="J5" s="48" t="n"/>
-      <c r="K5" s="48" t="n"/>
-      <c r="L5" s="48" t="n"/>
-      <c r="M5" s="48" t="n"/>
-      <c r="N5" s="48" t="n"/>
-      <c r="O5" s="48" t="n"/>
-      <c r="P5" s="48" t="n"/>
-      <c r="Q5" s="48" t="n"/>
-      <c r="R5" s="48" t="n"/>
-      <c r="S5" s="48" t="n"/>
-      <c r="T5" s="48" t="n"/>
-      <c r="U5" s="48" t="n"/>
-      <c r="V5" s="48" t="n"/>
-      <c r="W5" s="49" t="n"/>
-      <c r="X5" s="49" t="n"/>
-      <c r="Y5" s="48" t="n"/>
-      <c r="Z5" s="48" t="n"/>
-      <c r="AA5" s="48" t="n"/>
-      <c r="AB5" s="48" t="n"/>
-      <c r="AC5" s="48" t="n"/>
-      <c r="AD5" s="48" t="n"/>
-      <c r="AE5" s="48" t="n"/>
-      <c r="AF5" s="48" t="n"/>
-      <c r="AH5" s="46" t="inlineStr">
+      <c r="A5" s="46" t="n"/>
+      <c r="B5" s="47" t="n"/>
+      <c r="C5" s="48" t="n"/>
+      <c r="D5" s="49" t="n"/>
+      <c r="E5" s="49" t="n"/>
+      <c r="F5" s="49" t="n"/>
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="49" t="n"/>
+      <c r="I5" s="49" t="n"/>
+      <c r="J5" s="49" t="n"/>
+      <c r="K5" s="49" t="n"/>
+      <c r="L5" s="49" t="n"/>
+      <c r="M5" s="49" t="n"/>
+      <c r="N5" s="49" t="n"/>
+      <c r="O5" s="49" t="n"/>
+      <c r="P5" s="49" t="n"/>
+      <c r="Q5" s="49" t="n"/>
+      <c r="R5" s="49" t="n"/>
+      <c r="S5" s="49" t="n"/>
+      <c r="T5" s="49" t="n"/>
+      <c r="U5" s="49" t="n"/>
+      <c r="V5" s="49" t="n"/>
+      <c r="W5" s="50" t="n"/>
+      <c r="X5" s="50" t="n"/>
+      <c r="Y5" s="49" t="n"/>
+      <c r="Z5" s="49" t="n"/>
+      <c r="AA5" s="49" t="n"/>
+      <c r="AB5" s="49" t="n"/>
+      <c r="AC5" s="49" t="n"/>
+      <c r="AD5" s="49" t="n"/>
+      <c r="AE5" s="49" t="n"/>
+      <c r="AF5" s="49" t="n"/>
+      <c r="AH5" s="47" t="inlineStr">
         <is>
           <t>Competência</t>
         </is>
       </c>
-      <c r="AI5" s="45" t="n"/>
-      <c r="AK5" s="46" t="n"/>
-      <c r="AL5" s="46" t="n"/>
-      <c r="AN5" s="46" t="n"/>
-      <c r="AO5" s="46" t="n"/>
-      <c r="AQ5" s="46" t="n"/>
-      <c r="AS5" s="46" t="n"/>
+      <c r="AI5" s="46" t="n"/>
+      <c r="AK5" s="47" t="n"/>
+      <c r="AL5" s="47" t="n"/>
+      <c r="AN5" s="47" t="n"/>
+      <c r="AO5" s="47" t="n"/>
+      <c r="AQ5" s="47" t="n"/>
+      <c r="AS5" s="47" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="45" t="n"/>
-      <c r="B6" s="46" t="n"/>
-      <c r="C6" s="47" t="n"/>
-      <c r="D6" s="48" t="n"/>
-      <c r="E6" s="48" t="n"/>
-      <c r="F6" s="48" t="n"/>
-      <c r="G6" s="48" t="n"/>
-      <c r="H6" s="48" t="n"/>
-      <c r="I6" s="48" t="n"/>
-      <c r="J6" s="48" t="n"/>
-      <c r="K6" s="48" t="n"/>
-      <c r="L6" s="48" t="n"/>
-      <c r="M6" s="48" t="n"/>
-      <c r="N6" s="48" t="n"/>
-      <c r="O6" s="48" t="n"/>
-      <c r="P6" s="48" t="n"/>
-      <c r="Q6" s="48" t="n"/>
-      <c r="R6" s="48" t="n"/>
-      <c r="S6" s="48" t="n"/>
-      <c r="T6" s="48" t="n"/>
-      <c r="U6" s="48" t="n"/>
-      <c r="V6" s="48" t="n"/>
-      <c r="W6" s="49" t="n"/>
-      <c r="X6" s="49" t="n"/>
-      <c r="Y6" s="48" t="n"/>
-      <c r="Z6" s="48" t="n"/>
-      <c r="AA6" s="48" t="n"/>
-      <c r="AB6" s="48" t="n"/>
-      <c r="AC6" s="48" t="n"/>
-      <c r="AD6" s="48" t="n"/>
-      <c r="AE6" s="48" t="n"/>
-      <c r="AF6" s="48" t="n"/>
-      <c r="AH6" s="46" t="inlineStr">
+      <c r="A6" s="46" t="n"/>
+      <c r="B6" s="47" t="n"/>
+      <c r="C6" s="48" t="n"/>
+      <c r="D6" s="49" t="n"/>
+      <c r="E6" s="49" t="n"/>
+      <c r="F6" s="49" t="n"/>
+      <c r="G6" s="49" t="n"/>
+      <c r="H6" s="49" t="n"/>
+      <c r="I6" s="49" t="n"/>
+      <c r="J6" s="49" t="n"/>
+      <c r="K6" s="49" t="n"/>
+      <c r="L6" s="49" t="n"/>
+      <c r="M6" s="49" t="n"/>
+      <c r="N6" s="49" t="n"/>
+      <c r="O6" s="49" t="n"/>
+      <c r="P6" s="49" t="n"/>
+      <c r="Q6" s="49" t="n"/>
+      <c r="R6" s="49" t="n"/>
+      <c r="S6" s="49" t="n"/>
+      <c r="T6" s="49" t="n"/>
+      <c r="U6" s="49" t="n"/>
+      <c r="V6" s="49" t="n"/>
+      <c r="W6" s="50" t="n"/>
+      <c r="X6" s="50" t="n"/>
+      <c r="Y6" s="49" t="n"/>
+      <c r="Z6" s="49" t="n"/>
+      <c r="AA6" s="49" t="n"/>
+      <c r="AB6" s="49" t="n"/>
+      <c r="AC6" s="49" t="n"/>
+      <c r="AD6" s="49" t="n"/>
+      <c r="AE6" s="49" t="n"/>
+      <c r="AF6" s="49" t="n"/>
+      <c r="AH6" s="47" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="AI6" s="47" t="n"/>
-      <c r="AK6" s="46" t="n"/>
-      <c r="AL6" s="46" t="n"/>
-      <c r="AN6" s="46" t="n"/>
-      <c r="AO6" s="46" t="n"/>
-      <c r="AQ6" s="46" t="n"/>
-      <c r="AS6" s="46" t="n"/>
+      <c r="AI6" s="48" t="n"/>
+      <c r="AK6" s="47" t="n"/>
+      <c r="AL6" s="47" t="n"/>
+      <c r="AN6" s="47" t="n"/>
+      <c r="AO6" s="47" t="n"/>
+      <c r="AQ6" s="47" t="n"/>
+      <c r="AS6" s="47" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="45" t="n"/>
-      <c r="B7" s="46" t="n"/>
-      <c r="C7" s="47" t="n"/>
-      <c r="D7" s="48" t="n"/>
-      <c r="E7" s="48" t="n"/>
-      <c r="F7" s="48" t="n"/>
-      <c r="G7" s="48" t="n"/>
-      <c r="H7" s="48" t="n"/>
-      <c r="I7" s="48" t="n"/>
-      <c r="J7" s="48" t="n"/>
-      <c r="K7" s="48" t="n"/>
-      <c r="L7" s="48" t="n"/>
-      <c r="M7" s="48" t="n"/>
-      <c r="N7" s="48" t="n"/>
-      <c r="O7" s="48" t="n"/>
-      <c r="P7" s="48" t="n"/>
-      <c r="Q7" s="48" t="n"/>
-      <c r="R7" s="48" t="n"/>
-      <c r="S7" s="48" t="n"/>
-      <c r="T7" s="48" t="n"/>
-      <c r="U7" s="48" t="n"/>
-      <c r="V7" s="48" t="n"/>
-      <c r="W7" s="49" t="n"/>
-      <c r="X7" s="49" t="n"/>
-      <c r="Y7" s="48" t="n"/>
-      <c r="Z7" s="48" t="n"/>
-      <c r="AA7" s="48" t="n"/>
-      <c r="AB7" s="48" t="n"/>
-      <c r="AC7" s="48" t="n"/>
-      <c r="AD7" s="48" t="n"/>
-      <c r="AE7" s="48" t="n"/>
-      <c r="AF7" s="48" t="n"/>
-      <c r="AH7" s="46" t="inlineStr">
+      <c r="A7" s="46" t="n"/>
+      <c r="B7" s="47" t="n"/>
+      <c r="C7" s="48" t="n"/>
+      <c r="D7" s="49" t="n"/>
+      <c r="E7" s="49" t="n"/>
+      <c r="F7" s="49" t="n"/>
+      <c r="G7" s="49" t="n"/>
+      <c r="H7" s="49" t="n"/>
+      <c r="I7" s="49" t="n"/>
+      <c r="J7" s="49" t="n"/>
+      <c r="K7" s="49" t="n"/>
+      <c r="L7" s="49" t="n"/>
+      <c r="M7" s="49" t="n"/>
+      <c r="N7" s="49" t="n"/>
+      <c r="O7" s="49" t="n"/>
+      <c r="P7" s="49" t="n"/>
+      <c r="Q7" s="49" t="n"/>
+      <c r="R7" s="49" t="n"/>
+      <c r="S7" s="49" t="n"/>
+      <c r="T7" s="49" t="n"/>
+      <c r="U7" s="49" t="n"/>
+      <c r="V7" s="49" t="n"/>
+      <c r="W7" s="50" t="n"/>
+      <c r="X7" s="50" t="n"/>
+      <c r="Y7" s="49" t="n"/>
+      <c r="Z7" s="49" t="n"/>
+      <c r="AA7" s="49" t="n"/>
+      <c r="AB7" s="49" t="n"/>
+      <c r="AC7" s="49" t="n"/>
+      <c r="AD7" s="49" t="n"/>
+      <c r="AE7" s="49" t="n"/>
+      <c r="AF7" s="49" t="n"/>
+      <c r="AH7" s="47" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="AI7" s="47" t="n"/>
-      <c r="AK7" s="46" t="n"/>
-      <c r="AL7" s="46" t="n"/>
-      <c r="AN7" s="46" t="n"/>
-      <c r="AO7" s="46" t="n"/>
-      <c r="AQ7" s="46" t="n"/>
-      <c r="AS7" s="46" t="n"/>
+      <c r="AI7" s="48" t="n"/>
+      <c r="AK7" s="47" t="n"/>
+      <c r="AL7" s="47" t="n"/>
+      <c r="AN7" s="47" t="n"/>
+      <c r="AO7" s="47" t="n"/>
+      <c r="AQ7" s="47" t="n"/>
+      <c r="AS7" s="47" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="45" t="n"/>
-      <c r="B8" s="46" t="n"/>
-      <c r="C8" s="47" t="n"/>
-      <c r="D8" s="48" t="n"/>
-      <c r="E8" s="48" t="n"/>
-      <c r="F8" s="48" t="n"/>
-      <c r="G8" s="48" t="n"/>
-      <c r="H8" s="48" t="n"/>
-      <c r="I8" s="48" t="n"/>
-      <c r="J8" s="48" t="n"/>
-      <c r="K8" s="48" t="n"/>
-      <c r="L8" s="48" t="n"/>
-      <c r="M8" s="48" t="n"/>
-      <c r="N8" s="48" t="n"/>
-      <c r="O8" s="48" t="n"/>
-      <c r="P8" s="48" t="n"/>
-      <c r="Q8" s="48" t="n"/>
-      <c r="R8" s="48" t="n"/>
-      <c r="S8" s="48" t="n"/>
-      <c r="T8" s="48" t="n"/>
-      <c r="U8" s="48" t="n"/>
-      <c r="V8" s="48" t="n"/>
-      <c r="W8" s="49" t="n"/>
-      <c r="X8" s="49" t="n"/>
-      <c r="Y8" s="48" t="n"/>
-      <c r="Z8" s="48" t="n"/>
-      <c r="AA8" s="48" t="n"/>
-      <c r="AB8" s="48" t="n"/>
-      <c r="AC8" s="48" t="n"/>
-      <c r="AD8" s="48" t="n"/>
-      <c r="AE8" s="48" t="n"/>
-      <c r="AF8" s="48" t="n"/>
-      <c r="AH8" s="46" t="inlineStr">
+      <c r="A8" s="46" t="n"/>
+      <c r="B8" s="47" t="n"/>
+      <c r="C8" s="48" t="n"/>
+      <c r="D8" s="49" t="n"/>
+      <c r="E8" s="49" t="n"/>
+      <c r="F8" s="49" t="n"/>
+      <c r="G8" s="49" t="n"/>
+      <c r="H8" s="49" t="n"/>
+      <c r="I8" s="49" t="n"/>
+      <c r="J8" s="49" t="n"/>
+      <c r="K8" s="49" t="n"/>
+      <c r="L8" s="49" t="n"/>
+      <c r="M8" s="49" t="n"/>
+      <c r="N8" s="49" t="n"/>
+      <c r="O8" s="49" t="n"/>
+      <c r="P8" s="49" t="n"/>
+      <c r="Q8" s="49" t="n"/>
+      <c r="R8" s="49" t="n"/>
+      <c r="S8" s="49" t="n"/>
+      <c r="T8" s="49" t="n"/>
+      <c r="U8" s="49" t="n"/>
+      <c r="V8" s="49" t="n"/>
+      <c r="W8" s="50" t="n"/>
+      <c r="X8" s="50" t="n"/>
+      <c r="Y8" s="49" t="n"/>
+      <c r="Z8" s="49" t="n"/>
+      <c r="AA8" s="49" t="n"/>
+      <c r="AB8" s="49" t="n"/>
+      <c r="AC8" s="49" t="n"/>
+      <c r="AD8" s="49" t="n"/>
+      <c r="AE8" s="49" t="n"/>
+      <c r="AF8" s="49" t="n"/>
+      <c r="AH8" s="47" t="inlineStr">
         <is>
           <t>Período</t>
         </is>
       </c>
-      <c r="AI8" s="46" t="n"/>
-      <c r="AK8" s="46" t="n"/>
-      <c r="AL8" s="46" t="n"/>
-      <c r="AN8" s="46" t="n"/>
-      <c r="AO8" s="46" t="n"/>
-      <c r="AQ8" s="46" t="n"/>
-      <c r="AS8" s="46" t="n"/>
+      <c r="AI8" s="47" t="n"/>
+      <c r="AK8" s="47" t="n"/>
+      <c r="AL8" s="47" t="n"/>
+      <c r="AN8" s="47" t="n"/>
+      <c r="AO8" s="47" t="n"/>
+      <c r="AQ8" s="47" t="n"/>
+      <c r="AS8" s="47" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="45" t="n"/>
-      <c r="B9" s="46" t="n"/>
-      <c r="C9" s="47" t="n"/>
-      <c r="D9" s="48" t="n"/>
-      <c r="E9" s="48" t="n"/>
-      <c r="F9" s="48" t="n"/>
-      <c r="G9" s="48" t="n"/>
-      <c r="H9" s="48" t="n"/>
-      <c r="I9" s="48" t="n"/>
-      <c r="J9" s="48" t="n"/>
-      <c r="K9" s="48" t="n"/>
-      <c r="L9" s="48" t="n"/>
-      <c r="M9" s="48" t="n"/>
-      <c r="N9" s="48" t="n"/>
-      <c r="O9" s="48" t="n"/>
-      <c r="P9" s="48" t="n"/>
-      <c r="Q9" s="48" t="n"/>
-      <c r="R9" s="48" t="n"/>
-      <c r="S9" s="48" t="n"/>
-      <c r="T9" s="48" t="n"/>
-      <c r="U9" s="48" t="n"/>
-      <c r="V9" s="48" t="n"/>
-      <c r="W9" s="49" t="n"/>
-      <c r="X9" s="49" t="n"/>
-      <c r="Y9" s="48" t="n"/>
-      <c r="Z9" s="48" t="n"/>
-      <c r="AA9" s="48" t="n"/>
-      <c r="AB9" s="48" t="n"/>
-      <c r="AC9" s="48" t="n"/>
-      <c r="AD9" s="48" t="n"/>
-      <c r="AE9" s="48" t="n"/>
-      <c r="AF9" s="48" t="n"/>
-      <c r="AH9" s="46" t="inlineStr">
+      <c r="A9" s="46" t="n"/>
+      <c r="B9" s="47" t="n"/>
+      <c r="C9" s="48" t="n"/>
+      <c r="D9" s="49" t="n"/>
+      <c r="E9" s="49" t="n"/>
+      <c r="F9" s="49" t="n"/>
+      <c r="G9" s="49" t="n"/>
+      <c r="H9" s="49" t="n"/>
+      <c r="I9" s="49" t="n"/>
+      <c r="J9" s="49" t="n"/>
+      <c r="K9" s="49" t="n"/>
+      <c r="L9" s="49" t="n"/>
+      <c r="M9" s="49" t="n"/>
+      <c r="N9" s="49" t="n"/>
+      <c r="O9" s="49" t="n"/>
+      <c r="P9" s="49" t="n"/>
+      <c r="Q9" s="49" t="n"/>
+      <c r="R9" s="49" t="n"/>
+      <c r="S9" s="49" t="n"/>
+      <c r="T9" s="49" t="n"/>
+      <c r="U9" s="49" t="n"/>
+      <c r="V9" s="49" t="n"/>
+      <c r="W9" s="50" t="n"/>
+      <c r="X9" s="50" t="n"/>
+      <c r="Y9" s="49" t="n"/>
+      <c r="Z9" s="49" t="n"/>
+      <c r="AA9" s="49" t="n"/>
+      <c r="AB9" s="49" t="n"/>
+      <c r="AC9" s="49" t="n"/>
+      <c r="AD9" s="49" t="n"/>
+      <c r="AE9" s="49" t="n"/>
+      <c r="AF9" s="49" t="n"/>
+      <c r="AH9" s="47" t="inlineStr">
         <is>
           <t>Data-base</t>
         </is>
       </c>
-      <c r="AI9" s="50" t="n"/>
-      <c r="AK9" s="46" t="n"/>
-      <c r="AL9" s="46" t="n"/>
-      <c r="AN9" s="46" t="n"/>
-      <c r="AO9" s="46" t="n"/>
-      <c r="AQ9" s="46" t="n"/>
-      <c r="AS9" s="46" t="n"/>
+      <c r="AI9" s="51" t="n"/>
+      <c r="AK9" s="47" t="n"/>
+      <c r="AL9" s="47" t="n"/>
+      <c r="AN9" s="47" t="n"/>
+      <c r="AO9" s="47" t="n"/>
+      <c r="AQ9" s="47" t="n"/>
+      <c r="AS9" s="47" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="45" t="n"/>
-      <c r="B10" s="46" t="n"/>
-      <c r="C10" s="47" t="n"/>
-      <c r="D10" s="48" t="n"/>
-      <c r="E10" s="48" t="n"/>
-      <c r="F10" s="48" t="n"/>
-      <c r="G10" s="48" t="n"/>
-      <c r="H10" s="48" t="n"/>
-      <c r="I10" s="48" t="n"/>
-      <c r="J10" s="48" t="n"/>
-      <c r="K10" s="48" t="n"/>
-      <c r="L10" s="48" t="n"/>
-      <c r="M10" s="48" t="n"/>
-      <c r="N10" s="48" t="n"/>
-      <c r="O10" s="48" t="n"/>
-      <c r="P10" s="48" t="n"/>
-      <c r="Q10" s="48" t="n"/>
-      <c r="R10" s="48" t="n"/>
-      <c r="S10" s="48" t="n"/>
-      <c r="T10" s="48" t="n"/>
-      <c r="U10" s="48" t="n"/>
-      <c r="V10" s="48" t="n"/>
-      <c r="W10" s="49" t="n"/>
-      <c r="X10" s="49" t="n"/>
-      <c r="Y10" s="48" t="n"/>
-      <c r="Z10" s="48" t="n"/>
-      <c r="AA10" s="48" t="n"/>
-      <c r="AB10" s="48" t="n"/>
-      <c r="AC10" s="48" t="n"/>
-      <c r="AD10" s="48" t="n"/>
-      <c r="AE10" s="48" t="n"/>
-      <c r="AF10" s="48" t="n"/>
-      <c r="AH10" s="46" t="inlineStr">
+      <c r="A10" s="46" t="n"/>
+      <c r="B10" s="47" t="n"/>
+      <c r="C10" s="48" t="n"/>
+      <c r="D10" s="49" t="n"/>
+      <c r="E10" s="49" t="n"/>
+      <c r="F10" s="49" t="n"/>
+      <c r="G10" s="49" t="n"/>
+      <c r="H10" s="49" t="n"/>
+      <c r="I10" s="49" t="n"/>
+      <c r="J10" s="49" t="n"/>
+      <c r="K10" s="49" t="n"/>
+      <c r="L10" s="49" t="n"/>
+      <c r="M10" s="49" t="n"/>
+      <c r="N10" s="49" t="n"/>
+      <c r="O10" s="49" t="n"/>
+      <c r="P10" s="49" t="n"/>
+      <c r="Q10" s="49" t="n"/>
+      <c r="R10" s="49" t="n"/>
+      <c r="S10" s="49" t="n"/>
+      <c r="T10" s="49" t="n"/>
+      <c r="U10" s="49" t="n"/>
+      <c r="V10" s="49" t="n"/>
+      <c r="W10" s="50" t="n"/>
+      <c r="X10" s="50" t="n"/>
+      <c r="Y10" s="49" t="n"/>
+      <c r="Z10" s="49" t="n"/>
+      <c r="AA10" s="49" t="n"/>
+      <c r="AB10" s="49" t="n"/>
+      <c r="AC10" s="49" t="n"/>
+      <c r="AD10" s="49" t="n"/>
+      <c r="AE10" s="49" t="n"/>
+      <c r="AF10" s="49" t="n"/>
+      <c r="AH10" s="47" t="inlineStr">
         <is>
           <t>Gerado em</t>
         </is>
       </c>
-      <c r="AI10" s="50" t="n"/>
-      <c r="AK10" s="46" t="n"/>
-      <c r="AL10" s="46" t="n"/>
-      <c r="AN10" s="46" t="n"/>
-      <c r="AO10" s="46" t="n"/>
-      <c r="AQ10" s="46" t="n"/>
-      <c r="AS10" s="46" t="n"/>
+      <c r="AI10" s="51" t="n"/>
+      <c r="AK10" s="47" t="n"/>
+      <c r="AL10" s="47" t="n"/>
+      <c r="AN10" s="47" t="n"/>
+      <c r="AO10" s="47" t="n"/>
+      <c r="AQ10" s="47" t="n"/>
+      <c r="AS10" s="47" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="45" t="n"/>
-      <c r="B11" s="46" t="n"/>
-      <c r="C11" s="47" t="n"/>
-      <c r="D11" s="48" t="n"/>
-      <c r="E11" s="48" t="n"/>
-      <c r="F11" s="48" t="n"/>
-      <c r="G11" s="48" t="n"/>
-      <c r="H11" s="48" t="n"/>
-      <c r="I11" s="48" t="n"/>
-      <c r="J11" s="48" t="n"/>
-      <c r="K11" s="48" t="n"/>
-      <c r="L11" s="48" t="n"/>
-      <c r="M11" s="48" t="n"/>
-      <c r="N11" s="48" t="n"/>
-      <c r="O11" s="48" t="n"/>
-      <c r="P11" s="48" t="n"/>
-      <c r="Q11" s="48" t="n"/>
-      <c r="R11" s="48" t="n"/>
-      <c r="S11" s="48" t="n"/>
-      <c r="T11" s="48" t="n"/>
-      <c r="U11" s="48" t="n"/>
-      <c r="V11" s="48" t="n"/>
-      <c r="W11" s="49" t="n"/>
-      <c r="X11" s="49" t="n"/>
-      <c r="Y11" s="48" t="n"/>
-      <c r="Z11" s="48" t="n"/>
-      <c r="AA11" s="48" t="n"/>
-      <c r="AB11" s="48" t="n"/>
-      <c r="AC11" s="48" t="n"/>
-      <c r="AD11" s="48" t="n"/>
-      <c r="AE11" s="48" t="n"/>
-      <c r="AF11" s="48" t="n"/>
-      <c r="AH11" s="46" t="inlineStr">
+      <c r="A11" s="46" t="n"/>
+      <c r="B11" s="47" t="n"/>
+      <c r="C11" s="48" t="n"/>
+      <c r="D11" s="49" t="n"/>
+      <c r="E11" s="49" t="n"/>
+      <c r="F11" s="49" t="n"/>
+      <c r="G11" s="49" t="n"/>
+      <c r="H11" s="49" t="n"/>
+      <c r="I11" s="49" t="n"/>
+      <c r="J11" s="49" t="n"/>
+      <c r="K11" s="49" t="n"/>
+      <c r="L11" s="49" t="n"/>
+      <c r="M11" s="49" t="n"/>
+      <c r="N11" s="49" t="n"/>
+      <c r="O11" s="49" t="n"/>
+      <c r="P11" s="49" t="n"/>
+      <c r="Q11" s="49" t="n"/>
+      <c r="R11" s="49" t="n"/>
+      <c r="S11" s="49" t="n"/>
+      <c r="T11" s="49" t="n"/>
+      <c r="U11" s="49" t="n"/>
+      <c r="V11" s="49" t="n"/>
+      <c r="W11" s="50" t="n"/>
+      <c r="X11" s="50" t="n"/>
+      <c r="Y11" s="49" t="n"/>
+      <c r="Z11" s="49" t="n"/>
+      <c r="AA11" s="49" t="n"/>
+      <c r="AB11" s="49" t="n"/>
+      <c r="AC11" s="49" t="n"/>
+      <c r="AD11" s="49" t="n"/>
+      <c r="AE11" s="49" t="n"/>
+      <c r="AF11" s="49" t="n"/>
+      <c r="AH11" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano</t>
         </is>
       </c>
-      <c r="AI11" s="51" t="n"/>
-      <c r="AK11" s="46" t="n"/>
-      <c r="AL11" s="46" t="n"/>
-      <c r="AN11" s="46" t="n"/>
-      <c r="AO11" s="46" t="n"/>
-      <c r="AQ11" s="46" t="n"/>
-      <c r="AS11" s="46" t="n"/>
+      <c r="AI11" s="52" t="n"/>
+      <c r="AK11" s="47" t="n"/>
+      <c r="AL11" s="47" t="n"/>
+      <c r="AN11" s="47" t="n"/>
+      <c r="AO11" s="47" t="n"/>
+      <c r="AQ11" s="47" t="n"/>
+      <c r="AS11" s="47" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="45" t="n"/>
-      <c r="B12" s="46" t="n"/>
-      <c r="C12" s="47" t="n"/>
-      <c r="D12" s="48" t="n"/>
-      <c r="E12" s="48" t="n"/>
-      <c r="F12" s="48" t="n"/>
-      <c r="G12" s="48" t="n"/>
-      <c r="H12" s="48" t="n"/>
-      <c r="I12" s="48" t="n"/>
-      <c r="J12" s="48" t="n"/>
-      <c r="K12" s="48" t="n"/>
-      <c r="L12" s="48" t="n"/>
-      <c r="M12" s="48" t="n"/>
-      <c r="N12" s="48" t="n"/>
-      <c r="O12" s="48" t="n"/>
-      <c r="P12" s="48" t="n"/>
-      <c r="Q12" s="48" t="n"/>
-      <c r="R12" s="48" t="n"/>
-      <c r="S12" s="48" t="n"/>
-      <c r="T12" s="48" t="n"/>
-      <c r="U12" s="48" t="n"/>
-      <c r="V12" s="48" t="n"/>
-      <c r="W12" s="49" t="n"/>
-      <c r="X12" s="49" t="n"/>
-      <c r="Y12" s="48" t="n"/>
-      <c r="Z12" s="48" t="n"/>
-      <c r="AA12" s="48" t="n"/>
-      <c r="AB12" s="48" t="n"/>
-      <c r="AC12" s="48" t="n"/>
-      <c r="AD12" s="48" t="n"/>
-      <c r="AE12" s="48" t="n"/>
-      <c r="AF12" s="48" t="n"/>
-      <c r="AH12" s="46" t="inlineStr">
+      <c r="A12" s="46" t="n"/>
+      <c r="B12" s="47" t="n"/>
+      <c r="C12" s="48" t="n"/>
+      <c r="D12" s="49" t="n"/>
+      <c r="E12" s="49" t="n"/>
+      <c r="F12" s="49" t="n"/>
+      <c r="G12" s="49" t="n"/>
+      <c r="H12" s="49" t="n"/>
+      <c r="I12" s="49" t="n"/>
+      <c r="J12" s="49" t="n"/>
+      <c r="K12" s="49" t="n"/>
+      <c r="L12" s="49" t="n"/>
+      <c r="M12" s="49" t="n"/>
+      <c r="N12" s="49" t="n"/>
+      <c r="O12" s="49" t="n"/>
+      <c r="P12" s="49" t="n"/>
+      <c r="Q12" s="49" t="n"/>
+      <c r="R12" s="49" t="n"/>
+      <c r="S12" s="49" t="n"/>
+      <c r="T12" s="49" t="n"/>
+      <c r="U12" s="49" t="n"/>
+      <c r="V12" s="49" t="n"/>
+      <c r="W12" s="50" t="n"/>
+      <c r="X12" s="50" t="n"/>
+      <c r="Y12" s="49" t="n"/>
+      <c r="Z12" s="49" t="n"/>
+      <c r="AA12" s="49" t="n"/>
+      <c r="AB12" s="49" t="n"/>
+      <c r="AC12" s="49" t="n"/>
+      <c r="AD12" s="49" t="n"/>
+      <c r="AE12" s="49" t="n"/>
+      <c r="AF12" s="49" t="n"/>
+      <c r="AH12" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano anterior</t>
         </is>
       </c>
-      <c r="AI12" s="51" t="n"/>
-      <c r="AK12" s="46" t="n"/>
-      <c r="AL12" s="46" t="n"/>
-      <c r="AN12" s="46" t="n"/>
-      <c r="AO12" s="46" t="n"/>
-      <c r="AQ12" s="46" t="n"/>
-      <c r="AS12" s="46" t="n"/>
+      <c r="AI12" s="52" t="n"/>
+      <c r="AK12" s="47" t="n"/>
+      <c r="AL12" s="47" t="n"/>
+      <c r="AN12" s="47" t="n"/>
+      <c r="AO12" s="47" t="n"/>
+      <c r="AQ12" s="47" t="n"/>
+      <c r="AS12" s="47" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="45" t="n"/>
-      <c r="B13" s="46" t="n"/>
-      <c r="C13" s="47" t="n"/>
-      <c r="D13" s="48" t="n"/>
-      <c r="E13" s="48" t="n"/>
-      <c r="F13" s="48" t="n"/>
-      <c r="G13" s="48" t="n"/>
-      <c r="H13" s="48" t="n"/>
-      <c r="I13" s="48" t="n"/>
-      <c r="J13" s="48" t="n"/>
-      <c r="K13" s="48" t="n"/>
-      <c r="L13" s="48" t="n"/>
-      <c r="M13" s="48" t="n"/>
-      <c r="N13" s="48" t="n"/>
-      <c r="O13" s="48" t="n"/>
-      <c r="P13" s="48" t="n"/>
-      <c r="Q13" s="48" t="n"/>
-      <c r="R13" s="48" t="n"/>
-      <c r="S13" s="48" t="n"/>
-      <c r="T13" s="48" t="n"/>
-      <c r="U13" s="48" t="n"/>
-      <c r="V13" s="48" t="n"/>
-      <c r="W13" s="49" t="n"/>
-      <c r="X13" s="49" t="n"/>
-      <c r="Y13" s="48" t="n"/>
-      <c r="Z13" s="48" t="n"/>
-      <c r="AA13" s="48" t="n"/>
-      <c r="AB13" s="48" t="n"/>
-      <c r="AC13" s="48" t="n"/>
-      <c r="AD13" s="48" t="n"/>
-      <c r="AE13" s="48" t="n"/>
-      <c r="AF13" s="48" t="n"/>
-      <c r="AH13" s="46" t="inlineStr">
+      <c r="A13" s="46" t="n"/>
+      <c r="B13" s="47" t="n"/>
+      <c r="C13" s="48" t="n"/>
+      <c r="D13" s="49" t="n"/>
+      <c r="E13" s="49" t="n"/>
+      <c r="F13" s="49" t="n"/>
+      <c r="G13" s="49" t="n"/>
+      <c r="H13" s="49" t="n"/>
+      <c r="I13" s="49" t="n"/>
+      <c r="J13" s="49" t="n"/>
+      <c r="K13" s="49" t="n"/>
+      <c r="L13" s="49" t="n"/>
+      <c r="M13" s="49" t="n"/>
+      <c r="N13" s="49" t="n"/>
+      <c r="O13" s="49" t="n"/>
+      <c r="P13" s="49" t="n"/>
+      <c r="Q13" s="49" t="n"/>
+      <c r="R13" s="49" t="n"/>
+      <c r="S13" s="49" t="n"/>
+      <c r="T13" s="49" t="n"/>
+      <c r="U13" s="49" t="n"/>
+      <c r="V13" s="49" t="n"/>
+      <c r="W13" s="50" t="n"/>
+      <c r="X13" s="50" t="n"/>
+      <c r="Y13" s="49" t="n"/>
+      <c r="Z13" s="49" t="n"/>
+      <c r="AA13" s="49" t="n"/>
+      <c r="AB13" s="49" t="n"/>
+      <c r="AC13" s="49" t="n"/>
+      <c r="AD13" s="49" t="n"/>
+      <c r="AE13" s="49" t="n"/>
+      <c r="AF13" s="49" t="n"/>
+      <c r="AH13" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-2)</t>
         </is>
       </c>
-      <c r="AI13" s="48" t="n"/>
-      <c r="AK13" s="46" t="n"/>
-      <c r="AL13" s="46" t="n"/>
-      <c r="AN13" s="46" t="n"/>
-      <c r="AO13" s="46" t="n"/>
-      <c r="AQ13" s="46" t="n"/>
-      <c r="AS13" s="46" t="n"/>
+      <c r="AI13" s="49" t="n"/>
+      <c r="AK13" s="47" t="n"/>
+      <c r="AL13" s="47" t="n"/>
+      <c r="AN13" s="47" t="n"/>
+      <c r="AO13" s="47" t="n"/>
+      <c r="AQ13" s="47" t="n"/>
+      <c r="AS13" s="47" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="45" t="n"/>
-      <c r="B14" s="46" t="n"/>
-      <c r="C14" s="47" t="n"/>
-      <c r="D14" s="48" t="n"/>
-      <c r="E14" s="48" t="n"/>
-      <c r="F14" s="48" t="n"/>
-      <c r="G14" s="48" t="n"/>
-      <c r="H14" s="48" t="n"/>
-      <c r="I14" s="48" t="n"/>
-      <c r="J14" s="48" t="n"/>
-      <c r="K14" s="48" t="n"/>
-      <c r="L14" s="48" t="n"/>
-      <c r="M14" s="48" t="n"/>
-      <c r="N14" s="48" t="n"/>
-      <c r="O14" s="48" t="n"/>
-      <c r="P14" s="48" t="n"/>
-      <c r="Q14" s="48" t="n"/>
-      <c r="R14" s="48" t="n"/>
-      <c r="S14" s="48" t="n"/>
-      <c r="T14" s="48" t="n"/>
-      <c r="U14" s="48" t="n"/>
-      <c r="V14" s="48" t="n"/>
-      <c r="W14" s="49" t="n"/>
-      <c r="X14" s="49" t="n"/>
-      <c r="Y14" s="48" t="n"/>
-      <c r="Z14" s="48" t="n"/>
-      <c r="AA14" s="48" t="n"/>
-      <c r="AB14" s="48" t="n"/>
-      <c r="AC14" s="48" t="n"/>
-      <c r="AD14" s="48" t="n"/>
-      <c r="AE14" s="48" t="n"/>
-      <c r="AF14" s="48" t="n"/>
-      <c r="AH14" s="46" t="inlineStr">
+      <c r="A14" s="46" t="n"/>
+      <c r="B14" s="47" t="n"/>
+      <c r="C14" s="48" t="n"/>
+      <c r="D14" s="49" t="n"/>
+      <c r="E14" s="49" t="n"/>
+      <c r="F14" s="49" t="n"/>
+      <c r="G14" s="49" t="n"/>
+      <c r="H14" s="49" t="n"/>
+      <c r="I14" s="49" t="n"/>
+      <c r="J14" s="49" t="n"/>
+      <c r="K14" s="49" t="n"/>
+      <c r="L14" s="49" t="n"/>
+      <c r="M14" s="49" t="n"/>
+      <c r="N14" s="49" t="n"/>
+      <c r="O14" s="49" t="n"/>
+      <c r="P14" s="49" t="n"/>
+      <c r="Q14" s="49" t="n"/>
+      <c r="R14" s="49" t="n"/>
+      <c r="S14" s="49" t="n"/>
+      <c r="T14" s="49" t="n"/>
+      <c r="U14" s="49" t="n"/>
+      <c r="V14" s="49" t="n"/>
+      <c r="W14" s="50" t="n"/>
+      <c r="X14" s="50" t="n"/>
+      <c r="Y14" s="49" t="n"/>
+      <c r="Z14" s="49" t="n"/>
+      <c r="AA14" s="49" t="n"/>
+      <c r="AB14" s="49" t="n"/>
+      <c r="AC14" s="49" t="n"/>
+      <c r="AD14" s="49" t="n"/>
+      <c r="AE14" s="49" t="n"/>
+      <c r="AF14" s="49" t="n"/>
+      <c r="AH14" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-1)</t>
         </is>
       </c>
-      <c r="AI14" s="48" t="n"/>
-      <c r="AK14" s="46" t="n"/>
-      <c r="AL14" s="46" t="n"/>
-      <c r="AN14" s="46" t="n"/>
-      <c r="AO14" s="46" t="n"/>
-      <c r="AQ14" s="46" t="n"/>
-      <c r="AS14" s="46" t="n"/>
+      <c r="AI14" s="49" t="n"/>
+      <c r="AK14" s="47" t="n"/>
+      <c r="AL14" s="47" t="n"/>
+      <c r="AN14" s="47" t="n"/>
+      <c r="AO14" s="47" t="n"/>
+      <c r="AQ14" s="47" t="n"/>
+      <c r="AS14" s="47" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="45" t="n"/>
-      <c r="B15" s="46" t="n"/>
-      <c r="C15" s="47" t="n"/>
-      <c r="D15" s="48" t="n"/>
-      <c r="E15" s="48" t="n"/>
-      <c r="F15" s="48" t="n"/>
-      <c r="G15" s="48" t="n"/>
-      <c r="H15" s="48" t="n"/>
-      <c r="I15" s="48" t="n"/>
-      <c r="J15" s="48" t="n"/>
-      <c r="K15" s="48" t="n"/>
-      <c r="L15" s="48" t="n"/>
-      <c r="M15" s="48" t="n"/>
-      <c r="N15" s="48" t="n"/>
-      <c r="O15" s="48" t="n"/>
-      <c r="P15" s="48" t="n"/>
-      <c r="Q15" s="48" t="n"/>
-      <c r="R15" s="48" t="n"/>
-      <c r="S15" s="48" t="n"/>
-      <c r="T15" s="48" t="n"/>
-      <c r="U15" s="48" t="n"/>
-      <c r="V15" s="48" t="n"/>
-      <c r="W15" s="49" t="n"/>
-      <c r="X15" s="49" t="n"/>
-      <c r="Y15" s="48" t="n"/>
-      <c r="Z15" s="48" t="n"/>
-      <c r="AA15" s="48" t="n"/>
-      <c r="AB15" s="48" t="n"/>
-      <c r="AC15" s="48" t="n"/>
-      <c r="AD15" s="48" t="n"/>
-      <c r="AE15" s="48" t="n"/>
-      <c r="AF15" s="48" t="n"/>
-      <c r="AH15" s="46" t="inlineStr">
+      <c r="A15" s="46" t="n"/>
+      <c r="B15" s="47" t="n"/>
+      <c r="C15" s="48" t="n"/>
+      <c r="D15" s="49" t="n"/>
+      <c r="E15" s="49" t="n"/>
+      <c r="F15" s="49" t="n"/>
+      <c r="G15" s="49" t="n"/>
+      <c r="H15" s="49" t="n"/>
+      <c r="I15" s="49" t="n"/>
+      <c r="J15" s="49" t="n"/>
+      <c r="K15" s="49" t="n"/>
+      <c r="L15" s="49" t="n"/>
+      <c r="M15" s="49" t="n"/>
+      <c r="N15" s="49" t="n"/>
+      <c r="O15" s="49" t="n"/>
+      <c r="P15" s="49" t="n"/>
+      <c r="Q15" s="49" t="n"/>
+      <c r="R15" s="49" t="n"/>
+      <c r="S15" s="49" t="n"/>
+      <c r="T15" s="49" t="n"/>
+      <c r="U15" s="49" t="n"/>
+      <c r="V15" s="49" t="n"/>
+      <c r="W15" s="50" t="n"/>
+      <c r="X15" s="50" t="n"/>
+      <c r="Y15" s="49" t="n"/>
+      <c r="Z15" s="49" t="n"/>
+      <c r="AA15" s="49" t="n"/>
+      <c r="AB15" s="49" t="n"/>
+      <c r="AC15" s="49" t="n"/>
+      <c r="AD15" s="49" t="n"/>
+      <c r="AE15" s="49" t="n"/>
+      <c r="AF15" s="49" t="n"/>
+      <c r="AH15" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano)</t>
         </is>
       </c>
-      <c r="AI15" s="48" t="n"/>
-      <c r="AK15" s="46" t="n"/>
-      <c r="AL15" s="46" t="n"/>
-      <c r="AN15" s="46" t="n"/>
-      <c r="AO15" s="46" t="n"/>
-      <c r="AQ15" s="46" t="n"/>
-      <c r="AS15" s="46" t="n"/>
+      <c r="AI15" s="49" t="n"/>
+      <c r="AK15" s="47" t="n"/>
+      <c r="AL15" s="47" t="n"/>
+      <c r="AN15" s="47" t="n"/>
+      <c r="AO15" s="47" t="n"/>
+      <c r="AQ15" s="47" t="n"/>
+      <c r="AS15" s="47" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="45" t="n"/>
-      <c r="B16" s="46" t="n"/>
-      <c r="C16" s="47" t="n"/>
-      <c r="D16" s="48" t="n"/>
-      <c r="E16" s="48" t="n"/>
-      <c r="F16" s="48" t="n"/>
-      <c r="G16" s="48" t="n"/>
-      <c r="H16" s="48" t="n"/>
-      <c r="I16" s="48" t="n"/>
-      <c r="J16" s="48" t="n"/>
-      <c r="K16" s="48" t="n"/>
-      <c r="L16" s="48" t="n"/>
-      <c r="M16" s="48" t="n"/>
-      <c r="N16" s="48" t="n"/>
-      <c r="O16" s="48" t="n"/>
-      <c r="P16" s="48" t="n"/>
-      <c r="Q16" s="48" t="n"/>
-      <c r="R16" s="48" t="n"/>
-      <c r="S16" s="48" t="n"/>
-      <c r="T16" s="48" t="n"/>
-      <c r="U16" s="48" t="n"/>
-      <c r="V16" s="48" t="n"/>
-      <c r="W16" s="49" t="n"/>
-      <c r="X16" s="49" t="n"/>
-      <c r="Y16" s="48" t="n"/>
-      <c r="Z16" s="48" t="n"/>
-      <c r="AA16" s="48" t="n"/>
-      <c r="AB16" s="48" t="n"/>
-      <c r="AC16" s="48" t="n"/>
-      <c r="AD16" s="48" t="n"/>
-      <c r="AE16" s="48" t="n"/>
-      <c r="AF16" s="48" t="n"/>
-      <c r="AH16" s="46" t="inlineStr">
+      <c r="A16" s="46" t="n"/>
+      <c r="B16" s="47" t="n"/>
+      <c r="C16" s="48" t="n"/>
+      <c r="D16" s="49" t="n"/>
+      <c r="E16" s="49" t="n"/>
+      <c r="F16" s="49" t="n"/>
+      <c r="G16" s="49" t="n"/>
+      <c r="H16" s="49" t="n"/>
+      <c r="I16" s="49" t="n"/>
+      <c r="J16" s="49" t="n"/>
+      <c r="K16" s="49" t="n"/>
+      <c r="L16" s="49" t="n"/>
+      <c r="M16" s="49" t="n"/>
+      <c r="N16" s="49" t="n"/>
+      <c r="O16" s="49" t="n"/>
+      <c r="P16" s="49" t="n"/>
+      <c r="Q16" s="49" t="n"/>
+      <c r="R16" s="49" t="n"/>
+      <c r="S16" s="49" t="n"/>
+      <c r="T16" s="49" t="n"/>
+      <c r="U16" s="49" t="n"/>
+      <c r="V16" s="49" t="n"/>
+      <c r="W16" s="50" t="n"/>
+      <c r="X16" s="50" t="n"/>
+      <c r="Y16" s="49" t="n"/>
+      <c r="Z16" s="49" t="n"/>
+      <c r="AA16" s="49" t="n"/>
+      <c r="AB16" s="49" t="n"/>
+      <c r="AC16" s="49" t="n"/>
+      <c r="AD16" s="49" t="n"/>
+      <c r="AE16" s="49" t="n"/>
+      <c r="AF16" s="49" t="n"/>
+      <c r="AH16" s="47" t="inlineStr">
         <is>
           <t>Linhas do extrato pendentes</t>
         </is>
       </c>
-      <c r="AI16" s="47" t="n"/>
-      <c r="AK16" s="46" t="n"/>
-      <c r="AL16" s="46" t="n"/>
-      <c r="AN16" s="46" t="n"/>
-      <c r="AO16" s="46" t="n"/>
-      <c r="AQ16" s="46" t="n"/>
-      <c r="AS16" s="46" t="n"/>
+      <c r="AI16" s="48" t="n"/>
+      <c r="AK16" s="47" t="n"/>
+      <c r="AL16" s="47" t="n"/>
+      <c r="AN16" s="47" t="n"/>
+      <c r="AO16" s="47" t="n"/>
+      <c r="AQ16" s="47" t="n"/>
+      <c r="AS16" s="47" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="45" t="n"/>
-      <c r="B17" s="46" t="n"/>
-      <c r="C17" s="47" t="n"/>
-      <c r="D17" s="48" t="n"/>
-      <c r="E17" s="48" t="n"/>
-      <c r="F17" s="48" t="n"/>
-      <c r="G17" s="48" t="n"/>
-      <c r="H17" s="48" t="n"/>
-      <c r="I17" s="48" t="n"/>
-      <c r="J17" s="48" t="n"/>
-      <c r="K17" s="48" t="n"/>
-      <c r="L17" s="48" t="n"/>
-      <c r="M17" s="48" t="n"/>
-      <c r="N17" s="48" t="n"/>
-      <c r="O17" s="48" t="n"/>
-      <c r="P17" s="48" t="n"/>
-      <c r="Q17" s="48" t="n"/>
-      <c r="R17" s="48" t="n"/>
-      <c r="S17" s="48" t="n"/>
-      <c r="T17" s="48" t="n"/>
-      <c r="U17" s="48" t="n"/>
-      <c r="V17" s="48" t="n"/>
-      <c r="W17" s="49" t="n"/>
-      <c r="X17" s="49" t="n"/>
-      <c r="Y17" s="48" t="n"/>
-      <c r="Z17" s="48" t="n"/>
-      <c r="AA17" s="48" t="n"/>
-      <c r="AB17" s="48" t="n"/>
-      <c r="AC17" s="48" t="n"/>
-      <c r="AD17" s="48" t="n"/>
-      <c r="AE17" s="48" t="n"/>
-      <c r="AF17" s="48" t="n"/>
-      <c r="AH17" s="46" t="inlineStr">
+      <c r="A17" s="46" t="n"/>
+      <c r="B17" s="47" t="n"/>
+      <c r="C17" s="48" t="n"/>
+      <c r="D17" s="49" t="n"/>
+      <c r="E17" s="49" t="n"/>
+      <c r="F17" s="49" t="n"/>
+      <c r="G17" s="49" t="n"/>
+      <c r="H17" s="49" t="n"/>
+      <c r="I17" s="49" t="n"/>
+      <c r="J17" s="49" t="n"/>
+      <c r="K17" s="49" t="n"/>
+      <c r="L17" s="49" t="n"/>
+      <c r="M17" s="49" t="n"/>
+      <c r="N17" s="49" t="n"/>
+      <c r="O17" s="49" t="n"/>
+      <c r="P17" s="49" t="n"/>
+      <c r="Q17" s="49" t="n"/>
+      <c r="R17" s="49" t="n"/>
+      <c r="S17" s="49" t="n"/>
+      <c r="T17" s="49" t="n"/>
+      <c r="U17" s="49" t="n"/>
+      <c r="V17" s="49" t="n"/>
+      <c r="W17" s="50" t="n"/>
+      <c r="X17" s="50" t="n"/>
+      <c r="Y17" s="49" t="n"/>
+      <c r="Z17" s="49" t="n"/>
+      <c r="AA17" s="49" t="n"/>
+      <c r="AB17" s="49" t="n"/>
+      <c r="AC17" s="49" t="n"/>
+      <c r="AD17" s="49" t="n"/>
+      <c r="AE17" s="49" t="n"/>
+      <c r="AF17" s="49" t="n"/>
+      <c r="AH17" s="47" t="inlineStr">
         <is>
           <t>Último extrato importado</t>
         </is>
       </c>
-      <c r="AI17" s="50" t="n"/>
-      <c r="AK17" s="46" t="n"/>
-      <c r="AL17" s="46" t="n"/>
-      <c r="AN17" s="46" t="n"/>
-      <c r="AO17" s="46" t="n"/>
-      <c r="AQ17" s="46" t="n"/>
-      <c r="AS17" s="46" t="n"/>
+      <c r="AI17" s="51" t="n"/>
+      <c r="AK17" s="47" t="n"/>
+      <c r="AL17" s="47" t="n"/>
+      <c r="AN17" s="47" t="n"/>
+      <c r="AO17" s="47" t="n"/>
+      <c r="AQ17" s="47" t="n"/>
+      <c r="AS17" s="47" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="45" t="n"/>
-      <c r="B18" s="46" t="n"/>
-      <c r="C18" s="47" t="n"/>
-      <c r="D18" s="48" t="n"/>
-      <c r="E18" s="48" t="n"/>
-      <c r="F18" s="48" t="n"/>
-      <c r="G18" s="48" t="n"/>
-      <c r="H18" s="48" t="n"/>
-      <c r="I18" s="48" t="n"/>
-      <c r="J18" s="48" t="n"/>
-      <c r="K18" s="48" t="n"/>
-      <c r="L18" s="48" t="n"/>
-      <c r="M18" s="48" t="n"/>
-      <c r="N18" s="48" t="n"/>
-      <c r="O18" s="48" t="n"/>
-      <c r="P18" s="48" t="n"/>
-      <c r="Q18" s="48" t="n"/>
-      <c r="R18" s="48" t="n"/>
-      <c r="S18" s="48" t="n"/>
-      <c r="T18" s="48" t="n"/>
-      <c r="U18" s="48" t="n"/>
-      <c r="V18" s="48" t="n"/>
-      <c r="W18" s="49" t="n"/>
-      <c r="X18" s="49" t="n"/>
-      <c r="Y18" s="48" t="n"/>
-      <c r="Z18" s="48" t="n"/>
-      <c r="AA18" s="48" t="n"/>
-      <c r="AB18" s="48" t="n"/>
-      <c r="AC18" s="48" t="n"/>
-      <c r="AD18" s="48" t="n"/>
-      <c r="AE18" s="48" t="n"/>
-      <c r="AF18" s="48" t="n"/>
-      <c r="AH18" s="46" t="inlineStr">
+      <c r="A18" s="46" t="n"/>
+      <c r="B18" s="47" t="n"/>
+      <c r="C18" s="48" t="n"/>
+      <c r="D18" s="49" t="n"/>
+      <c r="E18" s="49" t="n"/>
+      <c r="F18" s="49" t="n"/>
+      <c r="G18" s="49" t="n"/>
+      <c r="H18" s="49" t="n"/>
+      <c r="I18" s="49" t="n"/>
+      <c r="J18" s="49" t="n"/>
+      <c r="K18" s="49" t="n"/>
+      <c r="L18" s="49" t="n"/>
+      <c r="M18" s="49" t="n"/>
+      <c r="N18" s="49" t="n"/>
+      <c r="O18" s="49" t="n"/>
+      <c r="P18" s="49" t="n"/>
+      <c r="Q18" s="49" t="n"/>
+      <c r="R18" s="49" t="n"/>
+      <c r="S18" s="49" t="n"/>
+      <c r="T18" s="49" t="n"/>
+      <c r="U18" s="49" t="n"/>
+      <c r="V18" s="49" t="n"/>
+      <c r="W18" s="50" t="n"/>
+      <c r="X18" s="50" t="n"/>
+      <c r="Y18" s="49" t="n"/>
+      <c r="Z18" s="49" t="n"/>
+      <c r="AA18" s="49" t="n"/>
+      <c r="AB18" s="49" t="n"/>
+      <c r="AC18" s="49" t="n"/>
+      <c r="AD18" s="49" t="n"/>
+      <c r="AE18" s="49" t="n"/>
+      <c r="AF18" s="49" t="n"/>
+      <c r="AH18" s="47" t="inlineStr">
         <is>
           <t>Notas de saída no mês</t>
         </is>
       </c>
-      <c r="AI18" s="47" t="n"/>
-      <c r="AK18" s="46" t="n"/>
-      <c r="AL18" s="46" t="n"/>
-      <c r="AN18" s="46" t="n"/>
-      <c r="AO18" s="46" t="n"/>
-      <c r="AQ18" s="46" t="n"/>
-      <c r="AS18" s="46" t="n"/>
+      <c r="AI18" s="48" t="n"/>
+      <c r="AK18" s="47" t="n"/>
+      <c r="AL18" s="47" t="n"/>
+      <c r="AN18" s="47" t="n"/>
+      <c r="AO18" s="47" t="n"/>
+      <c r="AQ18" s="47" t="n"/>
+      <c r="AS18" s="47" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="45" t="n"/>
-      <c r="B19" s="46" t="n"/>
-      <c r="C19" s="47" t="n"/>
-      <c r="D19" s="48" t="n"/>
-      <c r="E19" s="48" t="n"/>
-      <c r="F19" s="48" t="n"/>
-      <c r="G19" s="48" t="n"/>
-      <c r="H19" s="48" t="n"/>
-      <c r="I19" s="48" t="n"/>
-      <c r="J19" s="48" t="n"/>
-      <c r="K19" s="48" t="n"/>
-      <c r="L19" s="48" t="n"/>
-      <c r="M19" s="48" t="n"/>
-      <c r="N19" s="48" t="n"/>
-      <c r="O19" s="48" t="n"/>
-      <c r="P19" s="48" t="n"/>
-      <c r="Q19" s="48" t="n"/>
-      <c r="R19" s="48" t="n"/>
-      <c r="S19" s="48" t="n"/>
-      <c r="T19" s="48" t="n"/>
-      <c r="U19" s="48" t="n"/>
-      <c r="V19" s="48" t="n"/>
-      <c r="W19" s="49" t="n"/>
-      <c r="X19" s="49" t="n"/>
-      <c r="Y19" s="48" t="n"/>
-      <c r="Z19" s="48" t="n"/>
-      <c r="AA19" s="48" t="n"/>
-      <c r="AB19" s="48" t="n"/>
-      <c r="AC19" s="48" t="n"/>
-      <c r="AD19" s="48" t="n"/>
-      <c r="AE19" s="48" t="n"/>
-      <c r="AF19" s="48" t="n"/>
-      <c r="AH19" s="46" t="inlineStr">
+      <c r="A19" s="46" t="n"/>
+      <c r="B19" s="47" t="n"/>
+      <c r="C19" s="48" t="n"/>
+      <c r="D19" s="49" t="n"/>
+      <c r="E19" s="49" t="n"/>
+      <c r="F19" s="49" t="n"/>
+      <c r="G19" s="49" t="n"/>
+      <c r="H19" s="49" t="n"/>
+      <c r="I19" s="49" t="n"/>
+      <c r="J19" s="49" t="n"/>
+      <c r="K19" s="49" t="n"/>
+      <c r="L19" s="49" t="n"/>
+      <c r="M19" s="49" t="n"/>
+      <c r="N19" s="49" t="n"/>
+      <c r="O19" s="49" t="n"/>
+      <c r="P19" s="49" t="n"/>
+      <c r="Q19" s="49" t="n"/>
+      <c r="R19" s="49" t="n"/>
+      <c r="S19" s="49" t="n"/>
+      <c r="T19" s="49" t="n"/>
+      <c r="U19" s="49" t="n"/>
+      <c r="V19" s="49" t="n"/>
+      <c r="W19" s="50" t="n"/>
+      <c r="X19" s="50" t="n"/>
+      <c r="Y19" s="49" t="n"/>
+      <c r="Z19" s="49" t="n"/>
+      <c r="AA19" s="49" t="n"/>
+      <c r="AB19" s="49" t="n"/>
+      <c r="AC19" s="49" t="n"/>
+      <c r="AD19" s="49" t="n"/>
+      <c r="AE19" s="49" t="n"/>
+      <c r="AF19" s="49" t="n"/>
+      <c r="AH19" s="47" t="inlineStr">
         <is>
           <t>Sócio 1</t>
         </is>
       </c>
-      <c r="AI19" s="46" t="n"/>
-      <c r="AK19" s="46" t="n"/>
-      <c r="AL19" s="46" t="n"/>
-      <c r="AN19" s="46" t="n"/>
-      <c r="AO19" s="46" t="n"/>
-      <c r="AQ19" s="46" t="n"/>
-      <c r="AS19" s="46" t="n"/>
+      <c r="AI19" s="47" t="n"/>
+      <c r="AK19" s="47" t="n"/>
+      <c r="AL19" s="47" t="n"/>
+      <c r="AN19" s="47" t="n"/>
+      <c r="AO19" s="47" t="n"/>
+      <c r="AQ19" s="47" t="n"/>
+      <c r="AS19" s="47" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="45" t="n"/>
-      <c r="B20" s="46" t="n"/>
-      <c r="C20" s="47" t="n"/>
-      <c r="D20" s="48" t="n"/>
-      <c r="E20" s="48" t="n"/>
-      <c r="F20" s="48" t="n"/>
-      <c r="G20" s="48" t="n"/>
-      <c r="H20" s="48" t="n"/>
-      <c r="I20" s="48" t="n"/>
-      <c r="J20" s="48" t="n"/>
-      <c r="K20" s="48" t="n"/>
-      <c r="L20" s="48" t="n"/>
-      <c r="M20" s="48" t="n"/>
-      <c r="N20" s="48" t="n"/>
-      <c r="O20" s="48" t="n"/>
-      <c r="P20" s="48" t="n"/>
-      <c r="Q20" s="48" t="n"/>
-      <c r="R20" s="48" t="n"/>
-      <c r="S20" s="48" t="n"/>
-      <c r="T20" s="48" t="n"/>
-      <c r="U20" s="48" t="n"/>
-      <c r="V20" s="48" t="n"/>
-      <c r="W20" s="49" t="n"/>
-      <c r="X20" s="49" t="n"/>
-      <c r="Y20" s="48" t="n"/>
-      <c r="Z20" s="48" t="n"/>
-      <c r="AA20" s="48" t="n"/>
-      <c r="AB20" s="48" t="n"/>
-      <c r="AC20" s="48" t="n"/>
-      <c r="AD20" s="48" t="n"/>
-      <c r="AE20" s="48" t="n"/>
-      <c r="AF20" s="48" t="n"/>
-      <c r="AH20" s="46" t="inlineStr">
+      <c r="A20" s="46" t="n"/>
+      <c r="B20" s="47" t="n"/>
+      <c r="C20" s="48" t="n"/>
+      <c r="D20" s="49" t="n"/>
+      <c r="E20" s="49" t="n"/>
+      <c r="F20" s="49" t="n"/>
+      <c r="G20" s="49" t="n"/>
+      <c r="H20" s="49" t="n"/>
+      <c r="I20" s="49" t="n"/>
+      <c r="J20" s="49" t="n"/>
+      <c r="K20" s="49" t="n"/>
+      <c r="L20" s="49" t="n"/>
+      <c r="M20" s="49" t="n"/>
+      <c r="N20" s="49" t="n"/>
+      <c r="O20" s="49" t="n"/>
+      <c r="P20" s="49" t="n"/>
+      <c r="Q20" s="49" t="n"/>
+      <c r="R20" s="49" t="n"/>
+      <c r="S20" s="49" t="n"/>
+      <c r="T20" s="49" t="n"/>
+      <c r="U20" s="49" t="n"/>
+      <c r="V20" s="49" t="n"/>
+      <c r="W20" s="50" t="n"/>
+      <c r="X20" s="50" t="n"/>
+      <c r="Y20" s="49" t="n"/>
+      <c r="Z20" s="49" t="n"/>
+      <c r="AA20" s="49" t="n"/>
+      <c r="AB20" s="49" t="n"/>
+      <c r="AC20" s="49" t="n"/>
+      <c r="AD20" s="49" t="n"/>
+      <c r="AE20" s="49" t="n"/>
+      <c r="AF20" s="49" t="n"/>
+      <c r="AH20" s="47" t="inlineStr">
         <is>
           <t>Sócio 2</t>
         </is>
       </c>
-      <c r="AI20" s="46" t="n"/>
-      <c r="AK20" s="46" t="n"/>
-      <c r="AL20" s="46" t="n"/>
-      <c r="AN20" s="46" t="n"/>
-      <c r="AO20" s="46" t="n"/>
-      <c r="AQ20" s="46" t="n"/>
-      <c r="AS20" s="46" t="n"/>
+      <c r="AI20" s="47" t="n"/>
+      <c r="AK20" s="47" t="n"/>
+      <c r="AL20" s="47" t="n"/>
+      <c r="AN20" s="47" t="n"/>
+      <c r="AO20" s="47" t="n"/>
+      <c r="AQ20" s="47" t="n"/>
+      <c r="AS20" s="47" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="45" t="n"/>
-      <c r="B21" s="46" t="n"/>
-      <c r="C21" s="47" t="n"/>
-      <c r="D21" s="48" t="n"/>
-      <c r="E21" s="48" t="n"/>
-      <c r="F21" s="48" t="n"/>
-      <c r="G21" s="48" t="n"/>
-      <c r="H21" s="48" t="n"/>
-      <c r="I21" s="48" t="n"/>
-      <c r="J21" s="48" t="n"/>
-      <c r="K21" s="48" t="n"/>
-      <c r="L21" s="48" t="n"/>
-      <c r="M21" s="48" t="n"/>
-      <c r="N21" s="48" t="n"/>
-      <c r="O21" s="48" t="n"/>
-      <c r="P21" s="48" t="n"/>
-      <c r="Q21" s="48" t="n"/>
-      <c r="R21" s="48" t="n"/>
-      <c r="S21" s="48" t="n"/>
-      <c r="T21" s="48" t="n"/>
-      <c r="U21" s="48" t="n"/>
-      <c r="V21" s="48" t="n"/>
-      <c r="W21" s="49" t="n"/>
-      <c r="X21" s="49" t="n"/>
-      <c r="Y21" s="48" t="n"/>
-      <c r="Z21" s="48" t="n"/>
-      <c r="AA21" s="48" t="n"/>
-      <c r="AB21" s="48" t="n"/>
-      <c r="AC21" s="48" t="n"/>
-      <c r="AD21" s="48" t="n"/>
-      <c r="AE21" s="48" t="n"/>
-      <c r="AF21" s="48" t="n"/>
-      <c r="AH21" s="46" t="inlineStr">
+      <c r="A21" s="46" t="n"/>
+      <c r="B21" s="47" t="n"/>
+      <c r="C21" s="48" t="n"/>
+      <c r="D21" s="49" t="n"/>
+      <c r="E21" s="49" t="n"/>
+      <c r="F21" s="49" t="n"/>
+      <c r="G21" s="49" t="n"/>
+      <c r="H21" s="49" t="n"/>
+      <c r="I21" s="49" t="n"/>
+      <c r="J21" s="49" t="n"/>
+      <c r="K21" s="49" t="n"/>
+      <c r="L21" s="49" t="n"/>
+      <c r="M21" s="49" t="n"/>
+      <c r="N21" s="49" t="n"/>
+      <c r="O21" s="49" t="n"/>
+      <c r="P21" s="49" t="n"/>
+      <c r="Q21" s="49" t="n"/>
+      <c r="R21" s="49" t="n"/>
+      <c r="S21" s="49" t="n"/>
+      <c r="T21" s="49" t="n"/>
+      <c r="U21" s="49" t="n"/>
+      <c r="V21" s="49" t="n"/>
+      <c r="W21" s="50" t="n"/>
+      <c r="X21" s="50" t="n"/>
+      <c r="Y21" s="49" t="n"/>
+      <c r="Z21" s="49" t="n"/>
+      <c r="AA21" s="49" t="n"/>
+      <c r="AB21" s="49" t="n"/>
+      <c r="AC21" s="49" t="n"/>
+      <c r="AD21" s="49" t="n"/>
+      <c r="AE21" s="49" t="n"/>
+      <c r="AF21" s="49" t="n"/>
+      <c r="AH21" s="47" t="inlineStr">
         <is>
           <t>Sócio 3</t>
         </is>
       </c>
-      <c r="AI21" s="46" t="n"/>
-      <c r="AK21" s="46" t="n"/>
-      <c r="AL21" s="46" t="n"/>
-      <c r="AN21" s="46" t="n"/>
-      <c r="AO21" s="46" t="n"/>
-      <c r="AQ21" s="46" t="n"/>
-      <c r="AS21" s="46" t="n"/>
+      <c r="AI21" s="47" t="n"/>
+      <c r="AK21" s="47" t="n"/>
+      <c r="AL21" s="47" t="n"/>
+      <c r="AN21" s="47" t="n"/>
+      <c r="AO21" s="47" t="n"/>
+      <c r="AQ21" s="47" t="n"/>
+      <c r="AS21" s="47" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="45" t="n"/>
-      <c r="B22" s="46" t="n"/>
-      <c r="C22" s="47" t="n"/>
-      <c r="D22" s="48" t="n"/>
-      <c r="E22" s="48" t="n"/>
-      <c r="F22" s="48" t="n"/>
-      <c r="G22" s="48" t="n"/>
-      <c r="H22" s="48" t="n"/>
-      <c r="I22" s="48" t="n"/>
-      <c r="J22" s="48" t="n"/>
-      <c r="K22" s="48" t="n"/>
-      <c r="L22" s="48" t="n"/>
-      <c r="M22" s="48" t="n"/>
-      <c r="N22" s="48" t="n"/>
-      <c r="O22" s="48" t="n"/>
-      <c r="P22" s="48" t="n"/>
-      <c r="Q22" s="48" t="n"/>
-      <c r="R22" s="48" t="n"/>
-      <c r="S22" s="48" t="n"/>
-      <c r="T22" s="48" t="n"/>
-      <c r="U22" s="48" t="n"/>
-      <c r="V22" s="48" t="n"/>
-      <c r="W22" s="49" t="n"/>
-      <c r="X22" s="49" t="n"/>
-      <c r="Y22" s="48" t="n"/>
-      <c r="Z22" s="48" t="n"/>
-      <c r="AA22" s="48" t="n"/>
-      <c r="AB22" s="48" t="n"/>
-      <c r="AC22" s="48" t="n"/>
-      <c r="AD22" s="48" t="n"/>
-      <c r="AE22" s="48" t="n"/>
-      <c r="AF22" s="48" t="n"/>
-      <c r="AH22" s="46" t="inlineStr">
+      <c r="A22" s="46" t="n"/>
+      <c r="B22" s="47" t="n"/>
+      <c r="C22" s="48" t="n"/>
+      <c r="D22" s="49" t="n"/>
+      <c r="E22" s="49" t="n"/>
+      <c r="F22" s="49" t="n"/>
+      <c r="G22" s="49" t="n"/>
+      <c r="H22" s="49" t="n"/>
+      <c r="I22" s="49" t="n"/>
+      <c r="J22" s="49" t="n"/>
+      <c r="K22" s="49" t="n"/>
+      <c r="L22" s="49" t="n"/>
+      <c r="M22" s="49" t="n"/>
+      <c r="N22" s="49" t="n"/>
+      <c r="O22" s="49" t="n"/>
+      <c r="P22" s="49" t="n"/>
+      <c r="Q22" s="49" t="n"/>
+      <c r="R22" s="49" t="n"/>
+      <c r="S22" s="49" t="n"/>
+      <c r="T22" s="49" t="n"/>
+      <c r="U22" s="49" t="n"/>
+      <c r="V22" s="49" t="n"/>
+      <c r="W22" s="50" t="n"/>
+      <c r="X22" s="50" t="n"/>
+      <c r="Y22" s="49" t="n"/>
+      <c r="Z22" s="49" t="n"/>
+      <c r="AA22" s="49" t="n"/>
+      <c r="AB22" s="49" t="n"/>
+      <c r="AC22" s="49" t="n"/>
+      <c r="AD22" s="49" t="n"/>
+      <c r="AE22" s="49" t="n"/>
+      <c r="AF22" s="49" t="n"/>
+      <c r="AH22" s="47" t="inlineStr">
         <is>
           <t>Sócio 4</t>
         </is>
       </c>
-      <c r="AI22" s="46" t="n"/>
-      <c r="AK22" s="46" t="n"/>
-      <c r="AL22" s="46" t="n"/>
-      <c r="AN22" s="46" t="n"/>
-      <c r="AO22" s="46" t="n"/>
-      <c r="AQ22" s="46" t="n"/>
-      <c r="AS22" s="46" t="n"/>
+      <c r="AI22" s="47" t="n"/>
+      <c r="AK22" s="47" t="n"/>
+      <c r="AL22" s="47" t="n"/>
+      <c r="AN22" s="47" t="n"/>
+      <c r="AO22" s="47" t="n"/>
+      <c r="AQ22" s="47" t="n"/>
+      <c r="AS22" s="47" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="45" t="n"/>
-      <c r="B23" s="46" t="n"/>
-      <c r="C23" s="47" t="n"/>
-      <c r="D23" s="48" t="n"/>
-      <c r="E23" s="48" t="n"/>
-      <c r="F23" s="48" t="n"/>
-      <c r="G23" s="48" t="n"/>
-      <c r="H23" s="48" t="n"/>
-      <c r="I23" s="48" t="n"/>
-      <c r="J23" s="48" t="n"/>
-      <c r="K23" s="48" t="n"/>
-      <c r="L23" s="48" t="n"/>
-      <c r="M23" s="48" t="n"/>
-      <c r="N23" s="48" t="n"/>
-      <c r="O23" s="48" t="n"/>
-      <c r="P23" s="48" t="n"/>
-      <c r="Q23" s="48" t="n"/>
-      <c r="R23" s="48" t="n"/>
-      <c r="S23" s="48" t="n"/>
-      <c r="T23" s="48" t="n"/>
-      <c r="U23" s="48" t="n"/>
-      <c r="V23" s="48" t="n"/>
-      <c r="W23" s="49" t="n"/>
-      <c r="X23" s="49" t="n"/>
-      <c r="Y23" s="48" t="n"/>
-      <c r="Z23" s="48" t="n"/>
-      <c r="AA23" s="48" t="n"/>
-      <c r="AB23" s="48" t="n"/>
-      <c r="AC23" s="48" t="n"/>
-      <c r="AD23" s="48" t="n"/>
-      <c r="AE23" s="48" t="n"/>
-      <c r="AF23" s="48" t="n"/>
-      <c r="AH23" s="46" t="inlineStr">
+      <c r="A23" s="46" t="n"/>
+      <c r="B23" s="47" t="n"/>
+      <c r="C23" s="48" t="n"/>
+      <c r="D23" s="49" t="n"/>
+      <c r="E23" s="49" t="n"/>
+      <c r="F23" s="49" t="n"/>
+      <c r="G23" s="49" t="n"/>
+      <c r="H23" s="49" t="n"/>
+      <c r="I23" s="49" t="n"/>
+      <c r="J23" s="49" t="n"/>
+      <c r="K23" s="49" t="n"/>
+      <c r="L23" s="49" t="n"/>
+      <c r="M23" s="49" t="n"/>
+      <c r="N23" s="49" t="n"/>
+      <c r="O23" s="49" t="n"/>
+      <c r="P23" s="49" t="n"/>
+      <c r="Q23" s="49" t="n"/>
+      <c r="R23" s="49" t="n"/>
+      <c r="S23" s="49" t="n"/>
+      <c r="T23" s="49" t="n"/>
+      <c r="U23" s="49" t="n"/>
+      <c r="V23" s="49" t="n"/>
+      <c r="W23" s="50" t="n"/>
+      <c r="X23" s="50" t="n"/>
+      <c r="Y23" s="49" t="n"/>
+      <c r="Z23" s="49" t="n"/>
+      <c r="AA23" s="49" t="n"/>
+      <c r="AB23" s="49" t="n"/>
+      <c r="AC23" s="49" t="n"/>
+      <c r="AD23" s="49" t="n"/>
+      <c r="AE23" s="49" t="n"/>
+      <c r="AF23" s="49" t="n"/>
+      <c r="AH23" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 1</t>
         </is>
       </c>
-      <c r="AI23" s="51" t="n"/>
-      <c r="AK23" s="46" t="n"/>
-      <c r="AL23" s="46" t="n"/>
-      <c r="AN23" s="46" t="n"/>
-      <c r="AO23" s="46" t="n"/>
-      <c r="AQ23" s="46" t="n"/>
-      <c r="AS23" s="46" t="n"/>
+      <c r="AI23" s="52" t="n"/>
+      <c r="AK23" s="47" t="n"/>
+      <c r="AL23" s="47" t="n"/>
+      <c r="AN23" s="47" t="n"/>
+      <c r="AO23" s="47" t="n"/>
+      <c r="AQ23" s="47" t="n"/>
+      <c r="AS23" s="47" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="45" t="n"/>
-      <c r="B24" s="46" t="n"/>
-      <c r="C24" s="47" t="n"/>
-      <c r="D24" s="48" t="n"/>
-      <c r="E24" s="48" t="n"/>
-      <c r="F24" s="48" t="n"/>
-      <c r="G24" s="48" t="n"/>
-      <c r="H24" s="48" t="n"/>
-      <c r="I24" s="48" t="n"/>
-      <c r="J24" s="48" t="n"/>
-      <c r="K24" s="48" t="n"/>
-      <c r="L24" s="48" t="n"/>
-      <c r="M24" s="48" t="n"/>
-      <c r="N24" s="48" t="n"/>
-      <c r="O24" s="48" t="n"/>
-      <c r="P24" s="48" t="n"/>
-      <c r="Q24" s="48" t="n"/>
-      <c r="R24" s="48" t="n"/>
-      <c r="S24" s="48" t="n"/>
-      <c r="T24" s="48" t="n"/>
-      <c r="U24" s="48" t="n"/>
-      <c r="V24" s="48" t="n"/>
-      <c r="W24" s="49" t="n"/>
-      <c r="X24" s="49" t="n"/>
-      <c r="Y24" s="48" t="n"/>
-      <c r="Z24" s="48" t="n"/>
-      <c r="AA24" s="48" t="n"/>
-      <c r="AB24" s="48" t="n"/>
-      <c r="AC24" s="48" t="n"/>
-      <c r="AD24" s="48" t="n"/>
-      <c r="AE24" s="48" t="n"/>
-      <c r="AF24" s="48" t="n"/>
-      <c r="AH24" s="46" t="inlineStr">
+      <c r="A24" s="46" t="n"/>
+      <c r="B24" s="47" t="n"/>
+      <c r="C24" s="48" t="n"/>
+      <c r="D24" s="49" t="n"/>
+      <c r="E24" s="49" t="n"/>
+      <c r="F24" s="49" t="n"/>
+      <c r="G24" s="49" t="n"/>
+      <c r="H24" s="49" t="n"/>
+      <c r="I24" s="49" t="n"/>
+      <c r="J24" s="49" t="n"/>
+      <c r="K24" s="49" t="n"/>
+      <c r="L24" s="49" t="n"/>
+      <c r="M24" s="49" t="n"/>
+      <c r="N24" s="49" t="n"/>
+      <c r="O24" s="49" t="n"/>
+      <c r="P24" s="49" t="n"/>
+      <c r="Q24" s="49" t="n"/>
+      <c r="R24" s="49" t="n"/>
+      <c r="S24" s="49" t="n"/>
+      <c r="T24" s="49" t="n"/>
+      <c r="U24" s="49" t="n"/>
+      <c r="V24" s="49" t="n"/>
+      <c r="W24" s="50" t="n"/>
+      <c r="X24" s="50" t="n"/>
+      <c r="Y24" s="49" t="n"/>
+      <c r="Z24" s="49" t="n"/>
+      <c r="AA24" s="49" t="n"/>
+      <c r="AB24" s="49" t="n"/>
+      <c r="AC24" s="49" t="n"/>
+      <c r="AD24" s="49" t="n"/>
+      <c r="AE24" s="49" t="n"/>
+      <c r="AF24" s="49" t="n"/>
+      <c r="AH24" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 2</t>
         </is>
       </c>
-      <c r="AI24" s="51" t="n"/>
-      <c r="AK24" s="46" t="n"/>
-      <c r="AL24" s="46" t="n"/>
-      <c r="AN24" s="46" t="n"/>
-      <c r="AO24" s="46" t="n"/>
-      <c r="AQ24" s="46" t="n"/>
-      <c r="AS24" s="46" t="n"/>
+      <c r="AI24" s="52" t="n"/>
+      <c r="AK24" s="47" t="n"/>
+      <c r="AL24" s="47" t="n"/>
+      <c r="AN24" s="47" t="n"/>
+      <c r="AO24" s="47" t="n"/>
+      <c r="AQ24" s="47" t="n"/>
+      <c r="AS24" s="47" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="45" t="n"/>
-      <c r="B25" s="46" t="n"/>
-      <c r="C25" s="47" t="n"/>
-      <c r="D25" s="48" t="n"/>
-      <c r="E25" s="48" t="n"/>
-      <c r="F25" s="48" t="n"/>
-      <c r="G25" s="48" t="n"/>
-      <c r="H25" s="48" t="n"/>
-      <c r="I25" s="48" t="n"/>
-      <c r="J25" s="48" t="n"/>
-      <c r="K25" s="48" t="n"/>
-      <c r="L25" s="48" t="n"/>
-      <c r="M25" s="48" t="n"/>
-      <c r="N25" s="48" t="n"/>
-      <c r="O25" s="48" t="n"/>
-      <c r="P25" s="48" t="n"/>
-      <c r="Q25" s="48" t="n"/>
-      <c r="R25" s="48" t="n"/>
-      <c r="S25" s="48" t="n"/>
-      <c r="T25" s="48" t="n"/>
-      <c r="U25" s="48" t="n"/>
-      <c r="V25" s="48" t="n"/>
-      <c r="W25" s="49" t="n"/>
-      <c r="X25" s="49" t="n"/>
-      <c r="Y25" s="48" t="n"/>
-      <c r="Z25" s="48" t="n"/>
-      <c r="AA25" s="48" t="n"/>
-      <c r="AB25" s="48" t="n"/>
-      <c r="AC25" s="48" t="n"/>
-      <c r="AD25" s="48" t="n"/>
-      <c r="AE25" s="48" t="n"/>
-      <c r="AF25" s="48" t="n"/>
-      <c r="AH25" s="46" t="inlineStr">
+      <c r="A25" s="46" t="n"/>
+      <c r="B25" s="47" t="n"/>
+      <c r="C25" s="48" t="n"/>
+      <c r="D25" s="49" t="n"/>
+      <c r="E25" s="49" t="n"/>
+      <c r="F25" s="49" t="n"/>
+      <c r="G25" s="49" t="n"/>
+      <c r="H25" s="49" t="n"/>
+      <c r="I25" s="49" t="n"/>
+      <c r="J25" s="49" t="n"/>
+      <c r="K25" s="49" t="n"/>
+      <c r="L25" s="49" t="n"/>
+      <c r="M25" s="49" t="n"/>
+      <c r="N25" s="49" t="n"/>
+      <c r="O25" s="49" t="n"/>
+      <c r="P25" s="49" t="n"/>
+      <c r="Q25" s="49" t="n"/>
+      <c r="R25" s="49" t="n"/>
+      <c r="S25" s="49" t="n"/>
+      <c r="T25" s="49" t="n"/>
+      <c r="U25" s="49" t="n"/>
+      <c r="V25" s="49" t="n"/>
+      <c r="W25" s="50" t="n"/>
+      <c r="X25" s="50" t="n"/>
+      <c r="Y25" s="49" t="n"/>
+      <c r="Z25" s="49" t="n"/>
+      <c r="AA25" s="49" t="n"/>
+      <c r="AB25" s="49" t="n"/>
+      <c r="AC25" s="49" t="n"/>
+      <c r="AD25" s="49" t="n"/>
+      <c r="AE25" s="49" t="n"/>
+      <c r="AF25" s="49" t="n"/>
+      <c r="AH25" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 3</t>
         </is>
       </c>
-      <c r="AI25" s="51" t="n"/>
-      <c r="AK25" s="46" t="n"/>
-      <c r="AL25" s="46" t="n"/>
-      <c r="AN25" s="46" t="n"/>
-      <c r="AO25" s="46" t="n"/>
-      <c r="AQ25" s="46" t="n"/>
-      <c r="AS25" s="46" t="n"/>
+      <c r="AI25" s="52" t="n"/>
+      <c r="AK25" s="47" t="n"/>
+      <c r="AL25" s="47" t="n"/>
+      <c r="AN25" s="47" t="n"/>
+      <c r="AO25" s="47" t="n"/>
+      <c r="AQ25" s="47" t="n"/>
+      <c r="AS25" s="47" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="45" t="n"/>
-      <c r="B26" s="46" t="n"/>
-      <c r="C26" s="47" t="n"/>
-      <c r="D26" s="48" t="n"/>
-      <c r="E26" s="48" t="n"/>
-      <c r="F26" s="48" t="n"/>
-      <c r="G26" s="48" t="n"/>
-      <c r="H26" s="48" t="n"/>
-      <c r="I26" s="48" t="n"/>
-      <c r="J26" s="48" t="n"/>
-      <c r="K26" s="48" t="n"/>
-      <c r="L26" s="48" t="n"/>
-      <c r="M26" s="48" t="n"/>
-      <c r="N26" s="48" t="n"/>
-      <c r="O26" s="48" t="n"/>
-      <c r="P26" s="48" t="n"/>
-      <c r="Q26" s="48" t="n"/>
-      <c r="R26" s="48" t="n"/>
-      <c r="S26" s="48" t="n"/>
-      <c r="T26" s="48" t="n"/>
-      <c r="U26" s="48" t="n"/>
-      <c r="V26" s="48" t="n"/>
-      <c r="W26" s="49" t="n"/>
-      <c r="X26" s="49" t="n"/>
-      <c r="Y26" s="48" t="n"/>
-      <c r="Z26" s="48" t="n"/>
-      <c r="AA26" s="48" t="n"/>
-      <c r="AB26" s="48" t="n"/>
-      <c r="AC26" s="48" t="n"/>
-      <c r="AD26" s="48" t="n"/>
-      <c r="AE26" s="48" t="n"/>
-      <c r="AF26" s="48" t="n"/>
-      <c r="AH26" s="46" t="inlineStr">
+      <c r="A26" s="46" t="n"/>
+      <c r="B26" s="47" t="n"/>
+      <c r="C26" s="48" t="n"/>
+      <c r="D26" s="49" t="n"/>
+      <c r="E26" s="49" t="n"/>
+      <c r="F26" s="49" t="n"/>
+      <c r="G26" s="49" t="n"/>
+      <c r="H26" s="49" t="n"/>
+      <c r="I26" s="49" t="n"/>
+      <c r="J26" s="49" t="n"/>
+      <c r="K26" s="49" t="n"/>
+      <c r="L26" s="49" t="n"/>
+      <c r="M26" s="49" t="n"/>
+      <c r="N26" s="49" t="n"/>
+      <c r="O26" s="49" t="n"/>
+      <c r="P26" s="49" t="n"/>
+      <c r="Q26" s="49" t="n"/>
+      <c r="R26" s="49" t="n"/>
+      <c r="S26" s="49" t="n"/>
+      <c r="T26" s="49" t="n"/>
+      <c r="U26" s="49" t="n"/>
+      <c r="V26" s="49" t="n"/>
+      <c r="W26" s="50" t="n"/>
+      <c r="X26" s="50" t="n"/>
+      <c r="Y26" s="49" t="n"/>
+      <c r="Z26" s="49" t="n"/>
+      <c r="AA26" s="49" t="n"/>
+      <c r="AB26" s="49" t="n"/>
+      <c r="AC26" s="49" t="n"/>
+      <c r="AD26" s="49" t="n"/>
+      <c r="AE26" s="49" t="n"/>
+      <c r="AF26" s="49" t="n"/>
+      <c r="AH26" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 4</t>
         </is>
       </c>
-      <c r="AI26" s="51" t="n"/>
-      <c r="AK26" s="46" t="n"/>
-      <c r="AL26" s="46" t="n"/>
-      <c r="AN26" s="46" t="n"/>
-      <c r="AO26" s="46" t="n"/>
-      <c r="AQ26" s="46" t="n"/>
-      <c r="AS26" s="46" t="n"/>
+      <c r="AI26" s="52" t="n"/>
+      <c r="AK26" s="47" t="n"/>
+      <c r="AL26" s="47" t="n"/>
+      <c r="AN26" s="47" t="n"/>
+      <c r="AO26" s="47" t="n"/>
+      <c r="AQ26" s="47" t="n"/>
+      <c r="AS26" s="47" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="45" t="n"/>
-      <c r="B27" s="46" t="n"/>
-      <c r="C27" s="47" t="n"/>
-      <c r="D27" s="48" t="n"/>
-      <c r="E27" s="48" t="n"/>
-      <c r="F27" s="48" t="n"/>
-      <c r="G27" s="48" t="n"/>
-      <c r="H27" s="48" t="n"/>
-      <c r="I27" s="48" t="n"/>
-      <c r="J27" s="48" t="n"/>
-      <c r="K27" s="48" t="n"/>
-      <c r="L27" s="48" t="n"/>
-      <c r="M27" s="48" t="n"/>
-      <c r="N27" s="48" t="n"/>
-      <c r="O27" s="48" t="n"/>
-      <c r="P27" s="48" t="n"/>
-      <c r="Q27" s="48" t="n"/>
-      <c r="R27" s="48" t="n"/>
-      <c r="S27" s="48" t="n"/>
-      <c r="T27" s="48" t="n"/>
-      <c r="U27" s="48" t="n"/>
-      <c r="V27" s="48" t="n"/>
-      <c r="W27" s="49" t="n"/>
-      <c r="X27" s="49" t="n"/>
-      <c r="Y27" s="48" t="n"/>
-      <c r="Z27" s="48" t="n"/>
-      <c r="AA27" s="48" t="n"/>
-      <c r="AB27" s="48" t="n"/>
-      <c r="AC27" s="48" t="n"/>
-      <c r="AD27" s="48" t="n"/>
-      <c r="AE27" s="48" t="n"/>
-      <c r="AF27" s="48" t="n"/>
-      <c r="AH27" s="46" t="inlineStr">
+      <c r="A27" s="46" t="n"/>
+      <c r="B27" s="47" t="n"/>
+      <c r="C27" s="48" t="n"/>
+      <c r="D27" s="49" t="n"/>
+      <c r="E27" s="49" t="n"/>
+      <c r="F27" s="49" t="n"/>
+      <c r="G27" s="49" t="n"/>
+      <c r="H27" s="49" t="n"/>
+      <c r="I27" s="49" t="n"/>
+      <c r="J27" s="49" t="n"/>
+      <c r="K27" s="49" t="n"/>
+      <c r="L27" s="49" t="n"/>
+      <c r="M27" s="49" t="n"/>
+      <c r="N27" s="49" t="n"/>
+      <c r="O27" s="49" t="n"/>
+      <c r="P27" s="49" t="n"/>
+      <c r="Q27" s="49" t="n"/>
+      <c r="R27" s="49" t="n"/>
+      <c r="S27" s="49" t="n"/>
+      <c r="T27" s="49" t="n"/>
+      <c r="U27" s="49" t="n"/>
+      <c r="V27" s="49" t="n"/>
+      <c r="W27" s="50" t="n"/>
+      <c r="X27" s="50" t="n"/>
+      <c r="Y27" s="49" t="n"/>
+      <c r="Z27" s="49" t="n"/>
+      <c r="AA27" s="49" t="n"/>
+      <c r="AB27" s="49" t="n"/>
+      <c r="AC27" s="49" t="n"/>
+      <c r="AD27" s="49" t="n"/>
+      <c r="AE27" s="49" t="n"/>
+      <c r="AF27" s="49" t="n"/>
+      <c r="AH27" s="47" t="inlineStr">
         <is>
           <t>Grupos de clientes que compraram no ano</t>
         </is>
       </c>
-      <c r="AI27" s="47" t="n"/>
-      <c r="AK27" s="46" t="n"/>
-      <c r="AL27" s="46" t="n"/>
-      <c r="AN27" s="46" t="n"/>
-      <c r="AO27" s="46" t="n"/>
-      <c r="AQ27" s="46" t="n"/>
-      <c r="AS27" s="46" t="n"/>
+      <c r="AI27" s="48" t="n"/>
+      <c r="AK27" s="47" t="n"/>
+      <c r="AL27" s="47" t="n"/>
+      <c r="AN27" s="47" t="n"/>
+      <c r="AO27" s="47" t="n"/>
+      <c r="AQ27" s="47" t="n"/>
+      <c r="AS27" s="47" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="45" t="n"/>
-      <c r="B28" s="46" t="n"/>
-      <c r="C28" s="47" t="n"/>
-      <c r="D28" s="48" t="n"/>
-      <c r="E28" s="48" t="n"/>
-      <c r="F28" s="48" t="n"/>
-      <c r="G28" s="48" t="n"/>
-      <c r="H28" s="48" t="n"/>
-      <c r="I28" s="48" t="n"/>
-      <c r="J28" s="48" t="n"/>
-      <c r="K28" s="48" t="n"/>
-      <c r="L28" s="48" t="n"/>
-      <c r="M28" s="48" t="n"/>
-      <c r="N28" s="48" t="n"/>
-      <c r="O28" s="48" t="n"/>
-      <c r="P28" s="48" t="n"/>
-      <c r="Q28" s="48" t="n"/>
-      <c r="R28" s="48" t="n"/>
-      <c r="S28" s="48" t="n"/>
-      <c r="T28" s="48" t="n"/>
-      <c r="U28" s="48" t="n"/>
-      <c r="V28" s="48" t="n"/>
-      <c r="W28" s="49" t="n"/>
-      <c r="X28" s="49" t="n"/>
-      <c r="Y28" s="48" t="n"/>
-      <c r="Z28" s="48" t="n"/>
-      <c r="AA28" s="48" t="n"/>
-      <c r="AB28" s="48" t="n"/>
-      <c r="AC28" s="48" t="n"/>
-      <c r="AD28" s="48" t="n"/>
-      <c r="AE28" s="48" t="n"/>
-      <c r="AF28" s="48" t="n"/>
-      <c r="AH28" s="46" t="inlineStr">
+      <c r="A28" s="46" t="n"/>
+      <c r="B28" s="47" t="n"/>
+      <c r="C28" s="48" t="n"/>
+      <c r="D28" s="49" t="n"/>
+      <c r="E28" s="49" t="n"/>
+      <c r="F28" s="49" t="n"/>
+      <c r="G28" s="49" t="n"/>
+      <c r="H28" s="49" t="n"/>
+      <c r="I28" s="49" t="n"/>
+      <c r="J28" s="49" t="n"/>
+      <c r="K28" s="49" t="n"/>
+      <c r="L28" s="49" t="n"/>
+      <c r="M28" s="49" t="n"/>
+      <c r="N28" s="49" t="n"/>
+      <c r="O28" s="49" t="n"/>
+      <c r="P28" s="49" t="n"/>
+      <c r="Q28" s="49" t="n"/>
+      <c r="R28" s="49" t="n"/>
+      <c r="S28" s="49" t="n"/>
+      <c r="T28" s="49" t="n"/>
+      <c r="U28" s="49" t="n"/>
+      <c r="V28" s="49" t="n"/>
+      <c r="W28" s="50" t="n"/>
+      <c r="X28" s="50" t="n"/>
+      <c r="Y28" s="49" t="n"/>
+      <c r="Z28" s="49" t="n"/>
+      <c r="AA28" s="49" t="n"/>
+      <c r="AB28" s="49" t="n"/>
+      <c r="AC28" s="49" t="n"/>
+      <c r="AD28" s="49" t="n"/>
+      <c r="AE28" s="49" t="n"/>
+      <c r="AF28" s="49" t="n"/>
+      <c r="AH28" s="47" t="inlineStr">
         <is>
           <t>Grupos que compraram pela 1ª vez no ano</t>
         </is>
       </c>
-      <c r="AI28" s="47" t="n"/>
-      <c r="AK28" s="46" t="n"/>
-      <c r="AL28" s="46" t="n"/>
-      <c r="AN28" s="46" t="n"/>
-      <c r="AO28" s="46" t="n"/>
-      <c r="AQ28" s="46" t="n"/>
-      <c r="AS28" s="46" t="n"/>
+      <c r="AI28" s="48" t="n"/>
+      <c r="AK28" s="47" t="n"/>
+      <c r="AL28" s="47" t="n"/>
+      <c r="AN28" s="47" t="n"/>
+      <c r="AO28" s="47" t="n"/>
+      <c r="AQ28" s="47" t="n"/>
+      <c r="AS28" s="47" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="45" t="n"/>
-      <c r="B29" s="46" t="n"/>
-      <c r="C29" s="47" t="n"/>
-      <c r="D29" s="48" t="n"/>
-      <c r="E29" s="48" t="n"/>
-      <c r="F29" s="48" t="n"/>
-      <c r="G29" s="48" t="n"/>
-      <c r="H29" s="48" t="n"/>
-      <c r="I29" s="48" t="n"/>
-      <c r="J29" s="48" t="n"/>
-      <c r="K29" s="48" t="n"/>
-      <c r="L29" s="48" t="n"/>
-      <c r="M29" s="48" t="n"/>
-      <c r="N29" s="48" t="n"/>
-      <c r="O29" s="48" t="n"/>
-      <c r="P29" s="48" t="n"/>
-      <c r="Q29" s="48" t="n"/>
-      <c r="R29" s="48" t="n"/>
-      <c r="S29" s="48" t="n"/>
-      <c r="T29" s="48" t="n"/>
-      <c r="U29" s="48" t="n"/>
-      <c r="V29" s="48" t="n"/>
-      <c r="W29" s="49" t="n"/>
-      <c r="X29" s="49" t="n"/>
-      <c r="Y29" s="48" t="n"/>
-      <c r="Z29" s="48" t="n"/>
-      <c r="AA29" s="48" t="n"/>
-      <c r="AB29" s="48" t="n"/>
-      <c r="AC29" s="48" t="n"/>
-      <c r="AD29" s="48" t="n"/>
-      <c r="AE29" s="48" t="n"/>
-      <c r="AF29" s="48" t="n"/>
-      <c r="AK29" s="46" t="n"/>
-      <c r="AL29" s="46" t="n"/>
-      <c r="AN29" s="46" t="n"/>
-      <c r="AO29" s="46" t="n"/>
-      <c r="AQ29" s="46" t="n"/>
-      <c r="AS29" s="46" t="n"/>
+      <c r="A29" s="46" t="n"/>
+      <c r="B29" s="47" t="n"/>
+      <c r="C29" s="48" t="n"/>
+      <c r="D29" s="49" t="n"/>
+      <c r="E29" s="49" t="n"/>
+      <c r="F29" s="49" t="n"/>
+      <c r="G29" s="49" t="n"/>
+      <c r="H29" s="49" t="n"/>
+      <c r="I29" s="49" t="n"/>
+      <c r="J29" s="49" t="n"/>
+      <c r="K29" s="49" t="n"/>
+      <c r="L29" s="49" t="n"/>
+      <c r="M29" s="49" t="n"/>
+      <c r="N29" s="49" t="n"/>
+      <c r="O29" s="49" t="n"/>
+      <c r="P29" s="49" t="n"/>
+      <c r="Q29" s="49" t="n"/>
+      <c r="R29" s="49" t="n"/>
+      <c r="S29" s="49" t="n"/>
+      <c r="T29" s="49" t="n"/>
+      <c r="U29" s="49" t="n"/>
+      <c r="V29" s="49" t="n"/>
+      <c r="W29" s="50" t="n"/>
+      <c r="X29" s="50" t="n"/>
+      <c r="Y29" s="49" t="n"/>
+      <c r="Z29" s="49" t="n"/>
+      <c r="AA29" s="49" t="n"/>
+      <c r="AB29" s="49" t="n"/>
+      <c r="AC29" s="49" t="n"/>
+      <c r="AD29" s="49" t="n"/>
+      <c r="AE29" s="49" t="n"/>
+      <c r="AF29" s="49" t="n"/>
+      <c r="AK29" s="47" t="n"/>
+      <c r="AL29" s="47" t="n"/>
+      <c r="AN29" s="47" t="n"/>
+      <c r="AO29" s="47" t="n"/>
+      <c r="AQ29" s="47" t="n"/>
+      <c r="AS29" s="47" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="45" t="n"/>
-      <c r="B30" s="46" t="n"/>
-      <c r="C30" s="47" t="n"/>
-      <c r="D30" s="48" t="n"/>
-      <c r="E30" s="48" t="n"/>
-      <c r="F30" s="48" t="n"/>
-      <c r="G30" s="48" t="n"/>
-      <c r="H30" s="48" t="n"/>
-      <c r="I30" s="48" t="n"/>
-      <c r="J30" s="48" t="n"/>
-      <c r="K30" s="48" t="n"/>
-      <c r="L30" s="48" t="n"/>
-      <c r="M30" s="48" t="n"/>
-      <c r="N30" s="48" t="n"/>
-      <c r="O30" s="48" t="n"/>
-      <c r="P30" s="48" t="n"/>
-      <c r="Q30" s="48" t="n"/>
-      <c r="R30" s="48" t="n"/>
-      <c r="S30" s="48" t="n"/>
-      <c r="T30" s="48" t="n"/>
-      <c r="U30" s="48" t="n"/>
-      <c r="V30" s="48" t="n"/>
-      <c r="W30" s="49" t="n"/>
-      <c r="X30" s="49" t="n"/>
-      <c r="Y30" s="48" t="n"/>
-      <c r="Z30" s="48" t="n"/>
-      <c r="AA30" s="48" t="n"/>
-      <c r="AB30" s="48" t="n"/>
-      <c r="AC30" s="48" t="n"/>
-      <c r="AD30" s="48" t="n"/>
-      <c r="AE30" s="48" t="n"/>
-      <c r="AF30" s="48" t="n"/>
-      <c r="AK30" s="46" t="n"/>
-      <c r="AL30" s="46" t="n"/>
-      <c r="AN30" s="46" t="n"/>
-      <c r="AO30" s="46" t="n"/>
-      <c r="AQ30" s="46" t="n"/>
-      <c r="AS30" s="46" t="n"/>
+      <c r="A30" s="46" t="n"/>
+      <c r="B30" s="47" t="n"/>
+      <c r="C30" s="48" t="n"/>
+      <c r="D30" s="49" t="n"/>
+      <c r="E30" s="49" t="n"/>
+      <c r="F30" s="49" t="n"/>
+      <c r="G30" s="49" t="n"/>
+      <c r="H30" s="49" t="n"/>
+      <c r="I30" s="49" t="n"/>
+      <c r="J30" s="49" t="n"/>
+      <c r="K30" s="49" t="n"/>
+      <c r="L30" s="49" t="n"/>
+      <c r="M30" s="49" t="n"/>
+      <c r="N30" s="49" t="n"/>
+      <c r="O30" s="49" t="n"/>
+      <c r="P30" s="49" t="n"/>
+      <c r="Q30" s="49" t="n"/>
+      <c r="R30" s="49" t="n"/>
+      <c r="S30" s="49" t="n"/>
+      <c r="T30" s="49" t="n"/>
+      <c r="U30" s="49" t="n"/>
+      <c r="V30" s="49" t="n"/>
+      <c r="W30" s="50" t="n"/>
+      <c r="X30" s="50" t="n"/>
+      <c r="Y30" s="49" t="n"/>
+      <c r="Z30" s="49" t="n"/>
+      <c r="AA30" s="49" t="n"/>
+      <c r="AB30" s="49" t="n"/>
+      <c r="AC30" s="49" t="n"/>
+      <c r="AD30" s="49" t="n"/>
+      <c r="AE30" s="49" t="n"/>
+      <c r="AF30" s="49" t="n"/>
+      <c r="AK30" s="47" t="n"/>
+      <c r="AL30" s="47" t="n"/>
+      <c r="AN30" s="47" t="n"/>
+      <c r="AO30" s="47" t="n"/>
+      <c r="AQ30" s="47" t="n"/>
+      <c r="AS30" s="47" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="45" t="n"/>
-      <c r="B31" s="46" t="n"/>
-      <c r="C31" s="47" t="n"/>
-      <c r="D31" s="48" t="n"/>
-      <c r="E31" s="48" t="n"/>
-      <c r="F31" s="48" t="n"/>
-      <c r="G31" s="48" t="n"/>
-      <c r="H31" s="48" t="n"/>
-      <c r="I31" s="48" t="n"/>
-      <c r="J31" s="48" t="n"/>
-      <c r="K31" s="48" t="n"/>
-      <c r="L31" s="48" t="n"/>
-      <c r="M31" s="48" t="n"/>
-      <c r="N31" s="48" t="n"/>
-      <c r="O31" s="48" t="n"/>
-      <c r="P31" s="48" t="n"/>
-      <c r="Q31" s="48" t="n"/>
-      <c r="R31" s="48" t="n"/>
-      <c r="S31" s="48" t="n"/>
-      <c r="T31" s="48" t="n"/>
-      <c r="U31" s="48" t="n"/>
-      <c r="V31" s="48" t="n"/>
-      <c r="W31" s="49" t="n"/>
-      <c r="X31" s="49" t="n"/>
-      <c r="Y31" s="48" t="n"/>
-      <c r="Z31" s="48" t="n"/>
-      <c r="AA31" s="48" t="n"/>
-      <c r="AB31" s="48" t="n"/>
-      <c r="AC31" s="48" t="n"/>
-      <c r="AD31" s="48" t="n"/>
-      <c r="AE31" s="48" t="n"/>
-      <c r="AF31" s="48" t="n"/>
-      <c r="AK31" s="46" t="n"/>
-      <c r="AL31" s="46" t="n"/>
-      <c r="AN31" s="46" t="n"/>
-      <c r="AO31" s="46" t="n"/>
-      <c r="AQ31" s="46" t="n"/>
-      <c r="AS31" s="46" t="n"/>
+      <c r="A31" s="46" t="n"/>
+      <c r="B31" s="47" t="n"/>
+      <c r="C31" s="48" t="n"/>
+      <c r="D31" s="49" t="n"/>
+      <c r="E31" s="49" t="n"/>
+      <c r="F31" s="49" t="n"/>
+      <c r="G31" s="49" t="n"/>
+      <c r="H31" s="49" t="n"/>
+      <c r="I31" s="49" t="n"/>
+      <c r="J31" s="49" t="n"/>
+      <c r="K31" s="49" t="n"/>
+      <c r="L31" s="49" t="n"/>
+      <c r="M31" s="49" t="n"/>
+      <c r="N31" s="49" t="n"/>
+      <c r="O31" s="49" t="n"/>
+      <c r="P31" s="49" t="n"/>
+      <c r="Q31" s="49" t="n"/>
+      <c r="R31" s="49" t="n"/>
+      <c r="S31" s="49" t="n"/>
+      <c r="T31" s="49" t="n"/>
+      <c r="U31" s="49" t="n"/>
+      <c r="V31" s="49" t="n"/>
+      <c r="W31" s="50" t="n"/>
+      <c r="X31" s="50" t="n"/>
+      <c r="Y31" s="49" t="n"/>
+      <c r="Z31" s="49" t="n"/>
+      <c r="AA31" s="49" t="n"/>
+      <c r="AB31" s="49" t="n"/>
+      <c r="AC31" s="49" t="n"/>
+      <c r="AD31" s="49" t="n"/>
+      <c r="AE31" s="49" t="n"/>
+      <c r="AF31" s="49" t="n"/>
+      <c r="AK31" s="47" t="n"/>
+      <c r="AL31" s="47" t="n"/>
+      <c r="AN31" s="47" t="n"/>
+      <c r="AO31" s="47" t="n"/>
+      <c r="AQ31" s="47" t="n"/>
+      <c r="AS31" s="47" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="45" t="n"/>
-      <c r="B32" s="46" t="n"/>
-      <c r="C32" s="47" t="n"/>
-      <c r="D32" s="48" t="n"/>
-      <c r="E32" s="48" t="n"/>
-      <c r="F32" s="48" t="n"/>
-      <c r="G32" s="48" t="n"/>
-      <c r="H32" s="48" t="n"/>
-      <c r="I32" s="48" t="n"/>
-      <c r="J32" s="48" t="n"/>
-      <c r="K32" s="48" t="n"/>
-      <c r="L32" s="48" t="n"/>
-      <c r="M32" s="48" t="n"/>
-      <c r="N32" s="48" t="n"/>
-      <c r="O32" s="48" t="n"/>
-      <c r="P32" s="48" t="n"/>
-      <c r="Q32" s="48" t="n"/>
-      <c r="R32" s="48" t="n"/>
-      <c r="S32" s="48" t="n"/>
-      <c r="T32" s="48" t="n"/>
-      <c r="U32" s="48" t="n"/>
-      <c r="V32" s="48" t="n"/>
-      <c r="W32" s="49" t="n"/>
-      <c r="X32" s="49" t="n"/>
-      <c r="Y32" s="48" t="n"/>
-      <c r="Z32" s="48" t="n"/>
-      <c r="AA32" s="48" t="n"/>
-      <c r="AB32" s="48" t="n"/>
-      <c r="AC32" s="48" t="n"/>
-      <c r="AD32" s="48" t="n"/>
-      <c r="AE32" s="48" t="n"/>
-      <c r="AF32" s="48" t="n"/>
-      <c r="AK32" s="46" t="n"/>
-      <c r="AL32" s="46" t="n"/>
-      <c r="AN32" s="46" t="n"/>
-      <c r="AO32" s="46" t="n"/>
-      <c r="AQ32" s="46" t="n"/>
-      <c r="AS32" s="46" t="n"/>
+      <c r="A32" s="46" t="n"/>
+      <c r="B32" s="47" t="n"/>
+      <c r="C32" s="48" t="n"/>
+      <c r="D32" s="49" t="n"/>
+      <c r="E32" s="49" t="n"/>
+      <c r="F32" s="49" t="n"/>
+      <c r="G32" s="49" t="n"/>
+      <c r="H32" s="49" t="n"/>
+      <c r="I32" s="49" t="n"/>
+      <c r="J32" s="49" t="n"/>
+      <c r="K32" s="49" t="n"/>
+      <c r="L32" s="49" t="n"/>
+      <c r="M32" s="49" t="n"/>
+      <c r="N32" s="49" t="n"/>
+      <c r="O32" s="49" t="n"/>
+      <c r="P32" s="49" t="n"/>
+      <c r="Q32" s="49" t="n"/>
+      <c r="R32" s="49" t="n"/>
+      <c r="S32" s="49" t="n"/>
+      <c r="T32" s="49" t="n"/>
+      <c r="U32" s="49" t="n"/>
+      <c r="V32" s="49" t="n"/>
+      <c r="W32" s="50" t="n"/>
+      <c r="X32" s="50" t="n"/>
+      <c r="Y32" s="49" t="n"/>
+      <c r="Z32" s="49" t="n"/>
+      <c r="AA32" s="49" t="n"/>
+      <c r="AB32" s="49" t="n"/>
+      <c r="AC32" s="49" t="n"/>
+      <c r="AD32" s="49" t="n"/>
+      <c r="AE32" s="49" t="n"/>
+      <c r="AF32" s="49" t="n"/>
+      <c r="AK32" s="47" t="n"/>
+      <c r="AL32" s="47" t="n"/>
+      <c r="AN32" s="47" t="n"/>
+      <c r="AO32" s="47" t="n"/>
+      <c r="AQ32" s="47" t="n"/>
+      <c r="AS32" s="47" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="45" t="n"/>
-      <c r="B33" s="46" t="n"/>
-      <c r="C33" s="47" t="n"/>
-      <c r="D33" s="48" t="n"/>
-      <c r="E33" s="48" t="n"/>
-      <c r="F33" s="48" t="n"/>
-      <c r="G33" s="48" t="n"/>
-      <c r="H33" s="48" t="n"/>
-      <c r="I33" s="48" t="n"/>
-      <c r="J33" s="48" t="n"/>
-      <c r="K33" s="48" t="n"/>
-      <c r="L33" s="48" t="n"/>
-      <c r="M33" s="48" t="n"/>
-      <c r="N33" s="48" t="n"/>
-      <c r="O33" s="48" t="n"/>
-      <c r="P33" s="48" t="n"/>
-      <c r="Q33" s="48" t="n"/>
-      <c r="R33" s="48" t="n"/>
-      <c r="S33" s="48" t="n"/>
-      <c r="T33" s="48" t="n"/>
-      <c r="U33" s="48" t="n"/>
-      <c r="V33" s="48" t="n"/>
-      <c r="W33" s="49" t="n"/>
-      <c r="X33" s="49" t="n"/>
-      <c r="Y33" s="48" t="n"/>
-      <c r="Z33" s="48" t="n"/>
-      <c r="AA33" s="48" t="n"/>
-      <c r="AB33" s="48" t="n"/>
-      <c r="AC33" s="48" t="n"/>
-      <c r="AD33" s="48" t="n"/>
-      <c r="AE33" s="48" t="n"/>
-      <c r="AF33" s="48" t="n"/>
-      <c r="AK33" s="46" t="n"/>
-      <c r="AL33" s="46" t="n"/>
-      <c r="AN33" s="46" t="n"/>
-      <c r="AO33" s="46" t="n"/>
-      <c r="AQ33" s="46" t="n"/>
-      <c r="AS33" s="46" t="n"/>
+      <c r="A33" s="46" t="n"/>
+      <c r="B33" s="47" t="n"/>
+      <c r="C33" s="48" t="n"/>
+      <c r="D33" s="49" t="n"/>
+      <c r="E33" s="49" t="n"/>
+      <c r="F33" s="49" t="n"/>
+      <c r="G33" s="49" t="n"/>
+      <c r="H33" s="49" t="n"/>
+      <c r="I33" s="49" t="n"/>
+      <c r="J33" s="49" t="n"/>
+      <c r="K33" s="49" t="n"/>
+      <c r="L33" s="49" t="n"/>
+      <c r="M33" s="49" t="n"/>
+      <c r="N33" s="49" t="n"/>
+      <c r="O33" s="49" t="n"/>
+      <c r="P33" s="49" t="n"/>
+      <c r="Q33" s="49" t="n"/>
+      <c r="R33" s="49" t="n"/>
+      <c r="S33" s="49" t="n"/>
+      <c r="T33" s="49" t="n"/>
+      <c r="U33" s="49" t="n"/>
+      <c r="V33" s="49" t="n"/>
+      <c r="W33" s="50" t="n"/>
+      <c r="X33" s="50" t="n"/>
+      <c r="Y33" s="49" t="n"/>
+      <c r="Z33" s="49" t="n"/>
+      <c r="AA33" s="49" t="n"/>
+      <c r="AB33" s="49" t="n"/>
+      <c r="AC33" s="49" t="n"/>
+      <c r="AD33" s="49" t="n"/>
+      <c r="AE33" s="49" t="n"/>
+      <c r="AF33" s="49" t="n"/>
+      <c r="AK33" s="47" t="n"/>
+      <c r="AL33" s="47" t="n"/>
+      <c r="AN33" s="47" t="n"/>
+      <c r="AO33" s="47" t="n"/>
+      <c r="AQ33" s="47" t="n"/>
+      <c r="AS33" s="47" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="45" t="n"/>
-      <c r="B34" s="46" t="n"/>
-      <c r="C34" s="47" t="n"/>
-      <c r="D34" s="48" t="n"/>
-      <c r="E34" s="48" t="n"/>
-      <c r="F34" s="48" t="n"/>
-      <c r="G34" s="48" t="n"/>
-      <c r="H34" s="48" t="n"/>
-      <c r="I34" s="48" t="n"/>
-      <c r="J34" s="48" t="n"/>
-      <c r="K34" s="48" t="n"/>
-      <c r="L34" s="48" t="n"/>
-      <c r="M34" s="48" t="n"/>
-      <c r="N34" s="48" t="n"/>
-      <c r="O34" s="48" t="n"/>
-      <c r="P34" s="48" t="n"/>
-      <c r="Q34" s="48" t="n"/>
-      <c r="R34" s="48" t="n"/>
-      <c r="S34" s="48" t="n"/>
-      <c r="T34" s="48" t="n"/>
-      <c r="U34" s="48" t="n"/>
-      <c r="V34" s="48" t="n"/>
-      <c r="W34" s="49" t="n"/>
-      <c r="X34" s="49" t="n"/>
-      <c r="Y34" s="48" t="n"/>
-      <c r="Z34" s="48" t="n"/>
-      <c r="AA34" s="48" t="n"/>
-      <c r="AB34" s="48" t="n"/>
-      <c r="AC34" s="48" t="n"/>
-      <c r="AD34" s="48" t="n"/>
-      <c r="AE34" s="48" t="n"/>
-      <c r="AF34" s="48" t="n"/>
-      <c r="AK34" s="46" t="n"/>
-      <c r="AL34" s="46" t="n"/>
-      <c r="AN34" s="46" t="n"/>
-      <c r="AO34" s="46" t="n"/>
-      <c r="AQ34" s="46" t="n"/>
-      <c r="AS34" s="46" t="n"/>
+      <c r="A34" s="46" t="n"/>
+      <c r="B34" s="47" t="n"/>
+      <c r="C34" s="48" t="n"/>
+      <c r="D34" s="49" t="n"/>
+      <c r="E34" s="49" t="n"/>
+      <c r="F34" s="49" t="n"/>
+      <c r="G34" s="49" t="n"/>
+      <c r="H34" s="49" t="n"/>
+      <c r="I34" s="49" t="n"/>
+      <c r="J34" s="49" t="n"/>
+      <c r="K34" s="49" t="n"/>
+      <c r="L34" s="49" t="n"/>
+      <c r="M34" s="49" t="n"/>
+      <c r="N34" s="49" t="n"/>
+      <c r="O34" s="49" t="n"/>
+      <c r="P34" s="49" t="n"/>
+      <c r="Q34" s="49" t="n"/>
+      <c r="R34" s="49" t="n"/>
+      <c r="S34" s="49" t="n"/>
+      <c r="T34" s="49" t="n"/>
+      <c r="U34" s="49" t="n"/>
+      <c r="V34" s="49" t="n"/>
+      <c r="W34" s="50" t="n"/>
+      <c r="X34" s="50" t="n"/>
+      <c r="Y34" s="49" t="n"/>
+      <c r="Z34" s="49" t="n"/>
+      <c r="AA34" s="49" t="n"/>
+      <c r="AB34" s="49" t="n"/>
+      <c r="AC34" s="49" t="n"/>
+      <c r="AD34" s="49" t="n"/>
+      <c r="AE34" s="49" t="n"/>
+      <c r="AF34" s="49" t="n"/>
+      <c r="AK34" s="47" t="n"/>
+      <c r="AL34" s="47" t="n"/>
+      <c r="AN34" s="47" t="n"/>
+      <c r="AO34" s="47" t="n"/>
+      <c r="AQ34" s="47" t="n"/>
+      <c r="AS34" s="47" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="45" t="n"/>
-      <c r="B35" s="46" t="n"/>
-      <c r="C35" s="47" t="n"/>
-      <c r="D35" s="48" t="n"/>
-      <c r="E35" s="48" t="n"/>
-      <c r="F35" s="48" t="n"/>
-      <c r="G35" s="48" t="n"/>
-      <c r="H35" s="48" t="n"/>
-      <c r="I35" s="48" t="n"/>
-      <c r="J35" s="48" t="n"/>
-      <c r="K35" s="48" t="n"/>
-      <c r="L35" s="48" t="n"/>
-      <c r="M35" s="48" t="n"/>
-      <c r="N35" s="48" t="n"/>
-      <c r="O35" s="48" t="n"/>
-      <c r="P35" s="48" t="n"/>
-      <c r="Q35" s="48" t="n"/>
-      <c r="R35" s="48" t="n"/>
-      <c r="S35" s="48" t="n"/>
-      <c r="T35" s="48" t="n"/>
-      <c r="U35" s="48" t="n"/>
-      <c r="V35" s="48" t="n"/>
-      <c r="W35" s="49" t="n"/>
-      <c r="X35" s="49" t="n"/>
-      <c r="Y35" s="48" t="n"/>
-      <c r="Z35" s="48" t="n"/>
-      <c r="AA35" s="48" t="n"/>
-      <c r="AB35" s="48" t="n"/>
-      <c r="AC35" s="48" t="n"/>
-      <c r="AD35" s="48" t="n"/>
-      <c r="AE35" s="48" t="n"/>
-      <c r="AF35" s="48" t="n"/>
-      <c r="AK35" s="46" t="n"/>
-      <c r="AL35" s="46" t="n"/>
-      <c r="AN35" s="46" t="n"/>
-      <c r="AO35" s="46" t="n"/>
-      <c r="AQ35" s="46" t="n"/>
-      <c r="AS35" s="46" t="n"/>
+      <c r="A35" s="46" t="n"/>
+      <c r="B35" s="47" t="n"/>
+      <c r="C35" s="48" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="49" t="n"/>
+      <c r="I35" s="49" t="n"/>
+      <c r="J35" s="49" t="n"/>
+      <c r="K35" s="49" t="n"/>
+      <c r="L35" s="49" t="n"/>
+      <c r="M35" s="49" t="n"/>
+      <c r="N35" s="49" t="n"/>
+      <c r="O35" s="49" t="n"/>
+      <c r="P35" s="49" t="n"/>
+      <c r="Q35" s="49" t="n"/>
+      <c r="R35" s="49" t="n"/>
+      <c r="S35" s="49" t="n"/>
+      <c r="T35" s="49" t="n"/>
+      <c r="U35" s="49" t="n"/>
+      <c r="V35" s="49" t="n"/>
+      <c r="W35" s="50" t="n"/>
+      <c r="X35" s="50" t="n"/>
+      <c r="Y35" s="49" t="n"/>
+      <c r="Z35" s="49" t="n"/>
+      <c r="AA35" s="49" t="n"/>
+      <c r="AB35" s="49" t="n"/>
+      <c r="AC35" s="49" t="n"/>
+      <c r="AD35" s="49" t="n"/>
+      <c r="AE35" s="49" t="n"/>
+      <c r="AF35" s="49" t="n"/>
+      <c r="AK35" s="47" t="n"/>
+      <c r="AL35" s="47" t="n"/>
+      <c r="AN35" s="47" t="n"/>
+      <c r="AO35" s="47" t="n"/>
+      <c r="AQ35" s="47" t="n"/>
+      <c r="AS35" s="47" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="45" t="n"/>
-      <c r="B36" s="46" t="n"/>
-      <c r="C36" s="47" t="n"/>
-      <c r="D36" s="48" t="n"/>
-      <c r="E36" s="48" t="n"/>
-      <c r="F36" s="48" t="n"/>
-      <c r="G36" s="48" t="n"/>
-      <c r="H36" s="48" t="n"/>
-      <c r="I36" s="48" t="n"/>
-      <c r="J36" s="48" t="n"/>
-      <c r="K36" s="48" t="n"/>
-      <c r="L36" s="48" t="n"/>
-      <c r="M36" s="48" t="n"/>
-      <c r="N36" s="48" t="n"/>
-      <c r="O36" s="48" t="n"/>
-      <c r="P36" s="48" t="n"/>
-      <c r="Q36" s="48" t="n"/>
-      <c r="R36" s="48" t="n"/>
-      <c r="S36" s="48" t="n"/>
-      <c r="T36" s="48" t="n"/>
-      <c r="U36" s="48" t="n"/>
-      <c r="V36" s="48" t="n"/>
-      <c r="W36" s="49" t="n"/>
-      <c r="X36" s="49" t="n"/>
-      <c r="Y36" s="48" t="n"/>
-      <c r="Z36" s="48" t="n"/>
-      <c r="AA36" s="48" t="n"/>
-      <c r="AB36" s="48" t="n"/>
-      <c r="AC36" s="48" t="n"/>
-      <c r="AD36" s="48" t="n"/>
-      <c r="AE36" s="48" t="n"/>
-      <c r="AF36" s="48" t="n"/>
-      <c r="AK36" s="46" t="n"/>
-      <c r="AL36" s="46" t="n"/>
-      <c r="AN36" s="46" t="n"/>
-      <c r="AO36" s="46" t="n"/>
-      <c r="AQ36" s="46" t="n"/>
-      <c r="AS36" s="46" t="n"/>
+      <c r="A36" s="46" t="n"/>
+      <c r="B36" s="47" t="n"/>
+      <c r="C36" s="48" t="n"/>
+      <c r="D36" s="49" t="n"/>
+      <c r="E36" s="49" t="n"/>
+      <c r="F36" s="49" t="n"/>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="49" t="n"/>
+      <c r="I36" s="49" t="n"/>
+      <c r="J36" s="49" t="n"/>
+      <c r="K36" s="49" t="n"/>
+      <c r="L36" s="49" t="n"/>
+      <c r="M36" s="49" t="n"/>
+      <c r="N36" s="49" t="n"/>
+      <c r="O36" s="49" t="n"/>
+      <c r="P36" s="49" t="n"/>
+      <c r="Q36" s="49" t="n"/>
+      <c r="R36" s="49" t="n"/>
+      <c r="S36" s="49" t="n"/>
+      <c r="T36" s="49" t="n"/>
+      <c r="U36" s="49" t="n"/>
+      <c r="V36" s="49" t="n"/>
+      <c r="W36" s="50" t="n"/>
+      <c r="X36" s="50" t="n"/>
+      <c r="Y36" s="49" t="n"/>
+      <c r="Z36" s="49" t="n"/>
+      <c r="AA36" s="49" t="n"/>
+      <c r="AB36" s="49" t="n"/>
+      <c r="AC36" s="49" t="n"/>
+      <c r="AD36" s="49" t="n"/>
+      <c r="AE36" s="49" t="n"/>
+      <c r="AF36" s="49" t="n"/>
+      <c r="AK36" s="47" t="n"/>
+      <c r="AL36" s="47" t="n"/>
+      <c r="AN36" s="47" t="n"/>
+      <c r="AO36" s="47" t="n"/>
+      <c r="AQ36" s="47" t="n"/>
+      <c r="AS36" s="47" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="45" t="n"/>
-      <c r="B37" s="46" t="n"/>
-      <c r="C37" s="47" t="n"/>
-      <c r="D37" s="48" t="n"/>
-      <c r="E37" s="48" t="n"/>
-      <c r="F37" s="48" t="n"/>
-      <c r="G37" s="48" t="n"/>
-      <c r="H37" s="48" t="n"/>
-      <c r="I37" s="48" t="n"/>
-      <c r="J37" s="48" t="n"/>
-      <c r="K37" s="48" t="n"/>
-      <c r="L37" s="48" t="n"/>
-      <c r="M37" s="48" t="n"/>
-      <c r="N37" s="48" t="n"/>
-      <c r="O37" s="48" t="n"/>
-      <c r="P37" s="48" t="n"/>
-      <c r="Q37" s="48" t="n"/>
-      <c r="R37" s="48" t="n"/>
-      <c r="S37" s="48" t="n"/>
-      <c r="T37" s="48" t="n"/>
-      <c r="U37" s="48" t="n"/>
-      <c r="V37" s="48" t="n"/>
-      <c r="W37" s="49" t="n"/>
-      <c r="X37" s="49" t="n"/>
-      <c r="Y37" s="48" t="n"/>
-      <c r="Z37" s="48" t="n"/>
-      <c r="AA37" s="48" t="n"/>
-      <c r="AB37" s="48" t="n"/>
-      <c r="AC37" s="48" t="n"/>
-      <c r="AD37" s="48" t="n"/>
-      <c r="AE37" s="48" t="n"/>
-      <c r="AF37" s="48" t="n"/>
-      <c r="AK37" s="46" t="n"/>
-      <c r="AL37" s="46" t="n"/>
-      <c r="AN37" s="46" t="n"/>
-      <c r="AO37" s="46" t="n"/>
-      <c r="AQ37" s="46" t="n"/>
-      <c r="AS37" s="46" t="n"/>
+      <c r="A37" s="46" t="n"/>
+      <c r="B37" s="47" t="n"/>
+      <c r="C37" s="48" t="n"/>
+      <c r="D37" s="49" t="n"/>
+      <c r="E37" s="49" t="n"/>
+      <c r="F37" s="49" t="n"/>
+      <c r="G37" s="49" t="n"/>
+      <c r="H37" s="49" t="n"/>
+      <c r="I37" s="49" t="n"/>
+      <c r="J37" s="49" t="n"/>
+      <c r="K37" s="49" t="n"/>
+      <c r="L37" s="49" t="n"/>
+      <c r="M37" s="49" t="n"/>
+      <c r="N37" s="49" t="n"/>
+      <c r="O37" s="49" t="n"/>
+      <c r="P37" s="49" t="n"/>
+      <c r="Q37" s="49" t="n"/>
+      <c r="R37" s="49" t="n"/>
+      <c r="S37" s="49" t="n"/>
+      <c r="T37" s="49" t="n"/>
+      <c r="U37" s="49" t="n"/>
+      <c r="V37" s="49" t="n"/>
+      <c r="W37" s="50" t="n"/>
+      <c r="X37" s="50" t="n"/>
+      <c r="Y37" s="49" t="n"/>
+      <c r="Z37" s="49" t="n"/>
+      <c r="AA37" s="49" t="n"/>
+      <c r="AB37" s="49" t="n"/>
+      <c r="AC37" s="49" t="n"/>
+      <c r="AD37" s="49" t="n"/>
+      <c r="AE37" s="49" t="n"/>
+      <c r="AF37" s="49" t="n"/>
+      <c r="AK37" s="47" t="n"/>
+      <c r="AL37" s="47" t="n"/>
+      <c r="AN37" s="47" t="n"/>
+      <c r="AO37" s="47" t="n"/>
+      <c r="AQ37" s="47" t="n"/>
+      <c r="AS37" s="47" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="45" t="n"/>
-      <c r="B38" s="46" t="n"/>
-      <c r="C38" s="47" t="n"/>
-      <c r="D38" s="48" t="n"/>
-      <c r="E38" s="48" t="n"/>
-      <c r="F38" s="48" t="n"/>
-      <c r="G38" s="48" t="n"/>
-      <c r="H38" s="48" t="n"/>
-      <c r="I38" s="48" t="n"/>
-      <c r="J38" s="48" t="n"/>
-      <c r="K38" s="48" t="n"/>
-      <c r="L38" s="48" t="n"/>
-      <c r="M38" s="48" t="n"/>
-      <c r="N38" s="48" t="n"/>
-      <c r="O38" s="48" t="n"/>
-      <c r="P38" s="48" t="n"/>
-      <c r="Q38" s="48" t="n"/>
-      <c r="R38" s="48" t="n"/>
-      <c r="S38" s="48" t="n"/>
-      <c r="T38" s="48" t="n"/>
-      <c r="U38" s="48" t="n"/>
-      <c r="V38" s="48" t="n"/>
-      <c r="W38" s="49" t="n"/>
-      <c r="X38" s="49" t="n"/>
-      <c r="Y38" s="48" t="n"/>
-      <c r="Z38" s="48" t="n"/>
-      <c r="AA38" s="48" t="n"/>
-      <c r="AB38" s="48" t="n"/>
-      <c r="AC38" s="48" t="n"/>
-      <c r="AD38" s="48" t="n"/>
-      <c r="AE38" s="48" t="n"/>
-      <c r="AF38" s="48" t="n"/>
-      <c r="AK38" s="46" t="n"/>
-      <c r="AL38" s="46" t="n"/>
-      <c r="AN38" s="46" t="n"/>
-      <c r="AO38" s="46" t="n"/>
-      <c r="AQ38" s="46" t="n"/>
-      <c r="AS38" s="46" t="n"/>
+      <c r="A38" s="46" t="n"/>
+      <c r="B38" s="47" t="n"/>
+      <c r="C38" s="48" t="n"/>
+      <c r="D38" s="49" t="n"/>
+      <c r="E38" s="49" t="n"/>
+      <c r="F38" s="49" t="n"/>
+      <c r="G38" s="49" t="n"/>
+      <c r="H38" s="49" t="n"/>
+      <c r="I38" s="49" t="n"/>
+      <c r="J38" s="49" t="n"/>
+      <c r="K38" s="49" t="n"/>
+      <c r="L38" s="49" t="n"/>
+      <c r="M38" s="49" t="n"/>
+      <c r="N38" s="49" t="n"/>
+      <c r="O38" s="49" t="n"/>
+      <c r="P38" s="49" t="n"/>
+      <c r="Q38" s="49" t="n"/>
+      <c r="R38" s="49" t="n"/>
+      <c r="S38" s="49" t="n"/>
+      <c r="T38" s="49" t="n"/>
+      <c r="U38" s="49" t="n"/>
+      <c r="V38" s="49" t="n"/>
+      <c r="W38" s="50" t="n"/>
+      <c r="X38" s="50" t="n"/>
+      <c r="Y38" s="49" t="n"/>
+      <c r="Z38" s="49" t="n"/>
+      <c r="AA38" s="49" t="n"/>
+      <c r="AB38" s="49" t="n"/>
+      <c r="AC38" s="49" t="n"/>
+      <c r="AD38" s="49" t="n"/>
+      <c r="AE38" s="49" t="n"/>
+      <c r="AF38" s="49" t="n"/>
+      <c r="AK38" s="47" t="n"/>
+      <c r="AL38" s="47" t="n"/>
+      <c r="AN38" s="47" t="n"/>
+      <c r="AO38" s="47" t="n"/>
+      <c r="AQ38" s="47" t="n"/>
+      <c r="AS38" s="47" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="45" t="n"/>
-      <c r="B39" s="46" t="n"/>
-      <c r="C39" s="47" t="n"/>
-      <c r="D39" s="48" t="n"/>
-      <c r="E39" s="48" t="n"/>
-      <c r="F39" s="48" t="n"/>
-      <c r="G39" s="48" t="n"/>
-      <c r="H39" s="48" t="n"/>
-      <c r="I39" s="48" t="n"/>
-      <c r="J39" s="48" t="n"/>
-      <c r="K39" s="48" t="n"/>
-      <c r="L39" s="48" t="n"/>
-      <c r="M39" s="48" t="n"/>
-      <c r="N39" s="48" t="n"/>
-      <c r="O39" s="48" t="n"/>
-      <c r="P39" s="48" t="n"/>
-      <c r="Q39" s="48" t="n"/>
-      <c r="R39" s="48" t="n"/>
-      <c r="S39" s="48" t="n"/>
-      <c r="T39" s="48" t="n"/>
-      <c r="U39" s="48" t="n"/>
-      <c r="V39" s="48" t="n"/>
-      <c r="W39" s="49" t="n"/>
-      <c r="X39" s="49" t="n"/>
-      <c r="Y39" s="48" t="n"/>
-      <c r="Z39" s="48" t="n"/>
-      <c r="AA39" s="48" t="n"/>
-      <c r="AB39" s="48" t="n"/>
-      <c r="AC39" s="48" t="n"/>
-      <c r="AD39" s="48" t="n"/>
-      <c r="AE39" s="48" t="n"/>
-      <c r="AF39" s="48" t="n"/>
-      <c r="AK39" s="46" t="n"/>
-      <c r="AL39" s="46" t="n"/>
-      <c r="AN39" s="46" t="n"/>
-      <c r="AO39" s="46" t="n"/>
-      <c r="AQ39" s="46" t="n"/>
-      <c r="AS39" s="46" t="n"/>
+      <c r="A39" s="46" t="n"/>
+      <c r="B39" s="47" t="n"/>
+      <c r="C39" s="48" t="n"/>
+      <c r="D39" s="49" t="n"/>
+      <c r="E39" s="49" t="n"/>
+      <c r="F39" s="49" t="n"/>
+      <c r="G39" s="49" t="n"/>
+      <c r="H39" s="49" t="n"/>
+      <c r="I39" s="49" t="n"/>
+      <c r="J39" s="49" t="n"/>
+      <c r="K39" s="49" t="n"/>
+      <c r="L39" s="49" t="n"/>
+      <c r="M39" s="49" t="n"/>
+      <c r="N39" s="49" t="n"/>
+      <c r="O39" s="49" t="n"/>
+      <c r="P39" s="49" t="n"/>
+      <c r="Q39" s="49" t="n"/>
+      <c r="R39" s="49" t="n"/>
+      <c r="S39" s="49" t="n"/>
+      <c r="T39" s="49" t="n"/>
+      <c r="U39" s="49" t="n"/>
+      <c r="V39" s="49" t="n"/>
+      <c r="W39" s="50" t="n"/>
+      <c r="X39" s="50" t="n"/>
+      <c r="Y39" s="49" t="n"/>
+      <c r="Z39" s="49" t="n"/>
+      <c r="AA39" s="49" t="n"/>
+      <c r="AB39" s="49" t="n"/>
+      <c r="AC39" s="49" t="n"/>
+      <c r="AD39" s="49" t="n"/>
+      <c r="AE39" s="49" t="n"/>
+      <c r="AF39" s="49" t="n"/>
+      <c r="AK39" s="47" t="n"/>
+      <c r="AL39" s="47" t="n"/>
+      <c r="AN39" s="47" t="n"/>
+      <c r="AO39" s="47" t="n"/>
+      <c r="AQ39" s="47" t="n"/>
+      <c r="AS39" s="47" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="45" t="n"/>
-      <c r="B40" s="46" t="n"/>
-      <c r="C40" s="47" t="n"/>
-      <c r="D40" s="48" t="n"/>
-      <c r="E40" s="48" t="n"/>
-      <c r="F40" s="48" t="n"/>
-      <c r="G40" s="48" t="n"/>
-      <c r="H40" s="48" t="n"/>
-      <c r="I40" s="48" t="n"/>
-      <c r="J40" s="48" t="n"/>
-      <c r="K40" s="48" t="n"/>
-      <c r="L40" s="48" t="n"/>
-      <c r="M40" s="48" t="n"/>
-      <c r="N40" s="48" t="n"/>
-      <c r="O40" s="48" t="n"/>
-      <c r="P40" s="48" t="n"/>
-      <c r="Q40" s="48" t="n"/>
-      <c r="R40" s="48" t="n"/>
-      <c r="S40" s="48" t="n"/>
-      <c r="T40" s="48" t="n"/>
-      <c r="U40" s="48" t="n"/>
-      <c r="V40" s="48" t="n"/>
-      <c r="W40" s="49" t="n"/>
-      <c r="X40" s="49" t="n"/>
-      <c r="Y40" s="48" t="n"/>
-      <c r="Z40" s="48" t="n"/>
-      <c r="AA40" s="48" t="n"/>
-      <c r="AB40" s="48" t="n"/>
-      <c r="AC40" s="48" t="n"/>
-      <c r="AD40" s="48" t="n"/>
-      <c r="AE40" s="48" t="n"/>
-      <c r="AF40" s="48" t="n"/>
-      <c r="AK40" s="46" t="n"/>
-      <c r="AL40" s="46" t="n"/>
-      <c r="AN40" s="46" t="n"/>
-      <c r="AO40" s="46" t="n"/>
-      <c r="AQ40" s="46" t="n"/>
-      <c r="AS40" s="46" t="n"/>
+      <c r="A40" s="46" t="n"/>
+      <c r="B40" s="47" t="n"/>
+      <c r="C40" s="48" t="n"/>
+      <c r="D40" s="49" t="n"/>
+      <c r="E40" s="49" t="n"/>
+      <c r="F40" s="49" t="n"/>
+      <c r="G40" s="49" t="n"/>
+      <c r="H40" s="49" t="n"/>
+      <c r="I40" s="49" t="n"/>
+      <c r="J40" s="49" t="n"/>
+      <c r="K40" s="49" t="n"/>
+      <c r="L40" s="49" t="n"/>
+      <c r="M40" s="49" t="n"/>
+      <c r="N40" s="49" t="n"/>
+      <c r="O40" s="49" t="n"/>
+      <c r="P40" s="49" t="n"/>
+      <c r="Q40" s="49" t="n"/>
+      <c r="R40" s="49" t="n"/>
+      <c r="S40" s="49" t="n"/>
+      <c r="T40" s="49" t="n"/>
+      <c r="U40" s="49" t="n"/>
+      <c r="V40" s="49" t="n"/>
+      <c r="W40" s="50" t="n"/>
+      <c r="X40" s="50" t="n"/>
+      <c r="Y40" s="49" t="n"/>
+      <c r="Z40" s="49" t="n"/>
+      <c r="AA40" s="49" t="n"/>
+      <c r="AB40" s="49" t="n"/>
+      <c r="AC40" s="49" t="n"/>
+      <c r="AD40" s="49" t="n"/>
+      <c r="AE40" s="49" t="n"/>
+      <c r="AF40" s="49" t="n"/>
+      <c r="AK40" s="47" t="n"/>
+      <c r="AL40" s="47" t="n"/>
+      <c r="AN40" s="47" t="n"/>
+      <c r="AO40" s="47" t="n"/>
+      <c r="AQ40" s="47" t="n"/>
+      <c r="AS40" s="47" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="45" t="n"/>
-      <c r="B41" s="46" t="n"/>
-      <c r="C41" s="47" t="n"/>
-      <c r="D41" s="48" t="n"/>
-      <c r="E41" s="48" t="n"/>
-      <c r="F41" s="48" t="n"/>
-      <c r="G41" s="48" t="n"/>
-      <c r="H41" s="48" t="n"/>
-      <c r="I41" s="48" t="n"/>
-      <c r="J41" s="48" t="n"/>
-      <c r="K41" s="48" t="n"/>
-      <c r="L41" s="48" t="n"/>
-      <c r="M41" s="48" t="n"/>
-      <c r="N41" s="48" t="n"/>
-      <c r="O41" s="48" t="n"/>
-      <c r="P41" s="48" t="n"/>
-      <c r="Q41" s="48" t="n"/>
-      <c r="R41" s="48" t="n"/>
-      <c r="S41" s="48" t="n"/>
-      <c r="T41" s="48" t="n"/>
-      <c r="U41" s="48" t="n"/>
-      <c r="V41" s="48" t="n"/>
-      <c r="W41" s="49" t="n"/>
-      <c r="X41" s="49" t="n"/>
-      <c r="Y41" s="48" t="n"/>
-      <c r="Z41" s="48" t="n"/>
-      <c r="AA41" s="48" t="n"/>
-      <c r="AB41" s="48" t="n"/>
-      <c r="AC41" s="48" t="n"/>
-      <c r="AD41" s="48" t="n"/>
-      <c r="AE41" s="48" t="n"/>
-      <c r="AF41" s="48" t="n"/>
-      <c r="AK41" s="46" t="n"/>
-      <c r="AL41" s="46" t="n"/>
-      <c r="AN41" s="46" t="n"/>
-      <c r="AO41" s="46" t="n"/>
-      <c r="AQ41" s="46" t="n"/>
-      <c r="AS41" s="46" t="n"/>
+      <c r="A41" s="46" t="n"/>
+      <c r="B41" s="47" t="n"/>
+      <c r="C41" s="48" t="n"/>
+      <c r="D41" s="49" t="n"/>
+      <c r="E41" s="49" t="n"/>
+      <c r="F41" s="49" t="n"/>
+      <c r="G41" s="49" t="n"/>
+      <c r="H41" s="49" t="n"/>
+      <c r="I41" s="49" t="n"/>
+      <c r="J41" s="49" t="n"/>
+      <c r="K41" s="49" t="n"/>
+      <c r="L41" s="49" t="n"/>
+      <c r="M41" s="49" t="n"/>
+      <c r="N41" s="49" t="n"/>
+      <c r="O41" s="49" t="n"/>
+      <c r="P41" s="49" t="n"/>
+      <c r="Q41" s="49" t="n"/>
+      <c r="R41" s="49" t="n"/>
+      <c r="S41" s="49" t="n"/>
+      <c r="T41" s="49" t="n"/>
+      <c r="U41" s="49" t="n"/>
+      <c r="V41" s="49" t="n"/>
+      <c r="W41" s="50" t="n"/>
+      <c r="X41" s="50" t="n"/>
+      <c r="Y41" s="49" t="n"/>
+      <c r="Z41" s="49" t="n"/>
+      <c r="AA41" s="49" t="n"/>
+      <c r="AB41" s="49" t="n"/>
+      <c r="AC41" s="49" t="n"/>
+      <c r="AD41" s="49" t="n"/>
+      <c r="AE41" s="49" t="n"/>
+      <c r="AF41" s="49" t="n"/>
+      <c r="AK41" s="47" t="n"/>
+      <c r="AL41" s="47" t="n"/>
+      <c r="AN41" s="47" t="n"/>
+      <c r="AO41" s="47" t="n"/>
+      <c r="AQ41" s="47" t="n"/>
+      <c r="AS41" s="47" t="n"/>
     </row>
     <row r="42">
-      <c r="AK42" s="46" t="n"/>
-      <c r="AL42" s="46" t="n"/>
-      <c r="AN42" s="46" t="n"/>
-      <c r="AO42" s="46" t="n"/>
-      <c r="AQ42" s="46" t="n"/>
-      <c r="AS42" s="46" t="n"/>
+      <c r="AK42" s="47" t="n"/>
+      <c r="AL42" s="47" t="n"/>
+      <c r="AN42" s="47" t="n"/>
+      <c r="AO42" s="47" t="n"/>
+      <c r="AQ42" s="47" t="n"/>
+      <c r="AS42" s="47" t="n"/>
     </row>
     <row r="43">
-      <c r="AK43" s="46" t="n"/>
-      <c r="AL43" s="46" t="n"/>
-      <c r="AN43" s="46" t="n"/>
-      <c r="AO43" s="46" t="n"/>
-      <c r="AQ43" s="46" t="n"/>
-      <c r="AS43" s="46" t="n"/>
+      <c r="AK43" s="47" t="n"/>
+      <c r="AL43" s="47" t="n"/>
+      <c r="AN43" s="47" t="n"/>
+      <c r="AO43" s="47" t="n"/>
+      <c r="AQ43" s="47" t="n"/>
+      <c r="AS43" s="47" t="n"/>
     </row>
     <row r="44">
-      <c r="AK44" s="46" t="n"/>
-      <c r="AL44" s="46" t="n"/>
-      <c r="AN44" s="46" t="n"/>
-      <c r="AO44" s="46" t="n"/>
-      <c r="AQ44" s="46" t="n"/>
-      <c r="AS44" s="46" t="n"/>
+      <c r="AK44" s="47" t="n"/>
+      <c r="AL44" s="47" t="n"/>
+      <c r="AN44" s="47" t="n"/>
+      <c r="AO44" s="47" t="n"/>
+      <c r="AQ44" s="47" t="n"/>
+      <c r="AS44" s="47" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr">
@@ -7610,50 +7716,50 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="44" t="inlineStr">
+      <c r="A46" s="45" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="B46" s="44" t="inlineStr">
+      <c r="B46" s="45" t="inlineStr">
         <is>
           <t>Rótulo</t>
         </is>
       </c>
-      <c r="C46" s="44" t="inlineStr">
+      <c r="C46" s="45" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D46" s="44" t="inlineStr">
+      <c r="D46" s="45" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="E46" s="44" t="inlineStr">
+      <c r="E46" s="45" t="inlineStr">
         <is>
           <t>Chave</t>
         </is>
       </c>
-      <c r="F46" s="44" t="inlineStr">
+      <c r="F46" s="45" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="G46" s="44" t="inlineStr">
+      <c r="G46" s="45" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="45" t="n"/>
-      <c r="B47" s="46" t="n"/>
-      <c r="C47" s="46" t="n"/>
-      <c r="D47" s="46" t="n"/>
-      <c r="E47" s="46" t="n"/>
-      <c r="F47" s="48" t="n"/>
-      <c r="G47" s="47" t="n"/>
+      <c r="A47" s="46" t="n"/>
+      <c r="B47" s="47" t="n"/>
+      <c r="C47" s="47" t="n"/>
+      <c r="D47" s="47" t="n"/>
+      <c r="E47" s="47" t="n"/>
+      <c r="F47" s="49" t="n"/>
+      <c r="G47" s="48" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10043,7 +10149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:Q46"/>
+  <dimension ref="B1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -11960,7 +12066,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="18">
+      <c r="B35" s="36">
         <f>IF(Dados!$AS$5="","",Dados!$AS$5)</f>
         <v/>
       </c>
@@ -11974,7 +12080,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="18">
+      <c r="B36" s="36">
         <f>IF(Dados!$AS$6="","",Dados!$AS$6)</f>
         <v/>
       </c>
@@ -11988,7 +12094,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="18">
+      <c r="B37" s="36">
         <f>IF(Dados!$AS$7="","",Dados!$AS$7)</f>
         <v/>
       </c>
@@ -12002,7 +12108,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="18">
+      <c r="B38" s="36">
         <f>IF(Dados!$AS$8="","",Dados!$AS$8)</f>
         <v/>
       </c>
@@ -12016,7 +12122,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="18">
+      <c r="B39" s="36">
         <f>IF(Dados!$AS$9="","",Dados!$AS$9)</f>
         <v/>
       </c>
@@ -12030,7 +12136,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="18">
+      <c r="B40" s="36">
         <f>IF(Dados!$AS$10="","",Dados!$AS$10)</f>
         <v/>
       </c>
@@ -12044,7 +12150,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="18">
+      <c r="B41" s="36">
         <f>IF(Dados!$AS$11="","",Dados!$AS$11)</f>
         <v/>
       </c>
@@ -12058,7 +12164,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="18">
+      <c r="B42" s="36">
         <f>IF(Dados!$AS$12="","",Dados!$AS$12)</f>
         <v/>
       </c>
@@ -12072,7 +12178,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="18">
+      <c r="B43" s="36">
         <f>IF(Dados!$AS$13="","",Dados!$AS$13)</f>
         <v/>
       </c>
@@ -12086,7 +12192,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="18">
+      <c r="B44" s="36">
         <f>IF(Dados!$AS$14="","",Dados!$AS$14)</f>
         <v/>
       </c>
@@ -12102,7 +12208,14 @@
     <row r="46">
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>Inclui retiradas dos sócios e impostos, como no extrato. "sem detalhe": ano importado só com o total pago.</t>
+          <t>Inclui retiradas dos sócios e impostos, como no extrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>"sem detalhe": ano importado só com o total pago.</t>
         </is>
       </c>
     </row>
@@ -12333,7 +12446,7 @@
         <f>IF(N(O5)=0,"",IF(SUM($P$5:P5)-P5&lt;0.8,"A",IF(SUM($P$5:P5)-P5&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R5" s="36">
+      <c r="R5" s="37">
         <f>IF(Dados!$AL$5="","",Dados!$AL$5)</f>
         <v/>
       </c>
@@ -12407,7 +12520,7 @@
         <f>IF(N(O6)=0,"",IF(SUM($P$5:P6)-P6&lt;0.8,"A",IF(SUM($P$5:P6)-P6&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R6" s="36">
+      <c r="R6" s="37">
         <f>IF(Dados!$AL$6="","",Dados!$AL$6)</f>
         <v/>
       </c>
@@ -12481,7 +12594,7 @@
         <f>IF(N(O7)=0,"",IF(SUM($P$5:P7)-P7&lt;0.8,"A",IF(SUM($P$5:P7)-P7&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R7" s="36">
+      <c r="R7" s="37">
         <f>IF(Dados!$AL$7="","",Dados!$AL$7)</f>
         <v/>
       </c>
@@ -12555,7 +12668,7 @@
         <f>IF(N(O8)=0,"",IF(SUM($P$5:P8)-P8&lt;0.8,"A",IF(SUM($P$5:P8)-P8&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R8" s="36">
+      <c r="R8" s="37">
         <f>IF(Dados!$AL$8="","",Dados!$AL$8)</f>
         <v/>
       </c>
@@ -12629,7 +12742,7 @@
         <f>IF(N(O9)=0,"",IF(SUM($P$5:P9)-P9&lt;0.8,"A",IF(SUM($P$5:P9)-P9&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R9" s="36">
+      <c r="R9" s="37">
         <f>IF(Dados!$AL$9="","",Dados!$AL$9)</f>
         <v/>
       </c>
@@ -12703,7 +12816,7 @@
         <f>IF(N(O10)=0,"",IF(SUM($P$5:P10)-P10&lt;0.8,"A",IF(SUM($P$5:P10)-P10&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R10" s="36">
+      <c r="R10" s="37">
         <f>IF(Dados!$AL$10="","",Dados!$AL$10)</f>
         <v/>
       </c>
@@ -12777,7 +12890,7 @@
         <f>IF(N(O11)=0,"",IF(SUM($P$5:P11)-P11&lt;0.8,"A",IF(SUM($P$5:P11)-P11&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R11" s="36">
+      <c r="R11" s="37">
         <f>IF(Dados!$AL$11="","",Dados!$AL$11)</f>
         <v/>
       </c>
@@ -12851,7 +12964,7 @@
         <f>IF(N(O12)=0,"",IF(SUM($P$5:P12)-P12&lt;0.8,"A",IF(SUM($P$5:P12)-P12&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R12" s="36">
+      <c r="R12" s="37">
         <f>IF(Dados!$AL$12="","",Dados!$AL$12)</f>
         <v/>
       </c>
@@ -12925,7 +13038,7 @@
         <f>IF(N(O13)=0,"",IF(SUM($P$5:P13)-P13&lt;0.8,"A",IF(SUM($P$5:P13)-P13&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R13" s="36">
+      <c r="R13" s="37">
         <f>IF(Dados!$AL$13="","",Dados!$AL$13)</f>
         <v/>
       </c>
@@ -12999,7 +13112,7 @@
         <f>IF(N(O14)=0,"",IF(SUM($P$5:P14)-P14&lt;0.8,"A",IF(SUM($P$5:P14)-P14&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R14" s="36">
+      <c r="R14" s="37">
         <f>IF(Dados!$AL$14="","",Dados!$AL$14)</f>
         <v/>
       </c>
@@ -13073,7 +13186,7 @@
         <f>IF(N(O15)=0,"",IF(SUM($P$5:P15)-P15&lt;0.8,"A",IF(SUM($P$5:P15)-P15&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R15" s="36">
+      <c r="R15" s="37">
         <f>IF(Dados!$AL$15="","",Dados!$AL$15)</f>
         <v/>
       </c>
@@ -13147,7 +13260,7 @@
         <f>IF(N(O16)=0,"",IF(SUM($P$5:P16)-P16&lt;0.8,"A",IF(SUM($P$5:P16)-P16&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R16" s="36">
+      <c r="R16" s="37">
         <f>IF(Dados!$AL$16="","",Dados!$AL$16)</f>
         <v/>
       </c>
@@ -13221,7 +13334,7 @@
         <f>IF(N(O17)=0,"",IF(SUM($P$5:P17)-P17&lt;0.8,"A",IF(SUM($P$5:P17)-P17&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R17" s="36">
+      <c r="R17" s="37">
         <f>IF(Dados!$AL$17="","",Dados!$AL$17)</f>
         <v/>
       </c>
@@ -13295,7 +13408,7 @@
         <f>IF(N(O18)=0,"",IF(SUM($P$5:P18)-P18&lt;0.8,"A",IF(SUM($P$5:P18)-P18&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R18" s="36">
+      <c r="R18" s="37">
         <f>IF(Dados!$AL$18="","",Dados!$AL$18)</f>
         <v/>
       </c>
@@ -13369,7 +13482,7 @@
         <f>IF(N(O19)=0,"",IF(SUM($P$5:P19)-P19&lt;0.8,"A",IF(SUM($P$5:P19)-P19&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R19" s="36">
+      <c r="R19" s="37">
         <f>IF(Dados!$AL$19="","",Dados!$AL$19)</f>
         <v/>
       </c>
@@ -13443,7 +13556,7 @@
         <f>IF(N(O20)=0,"",IF(SUM($P$5:P20)-P20&lt;0.8,"A",IF(SUM($P$5:P20)-P20&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R20" s="36">
+      <c r="R20" s="37">
         <f>IF(Dados!$AL$20="","",Dados!$AL$20)</f>
         <v/>
       </c>
@@ -13517,7 +13630,7 @@
         <f>IF(N(O21)=0,"",IF(SUM($P$5:P21)-P21&lt;0.8,"A",IF(SUM($P$5:P21)-P21&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R21" s="36">
+      <c r="R21" s="37">
         <f>IF(Dados!$AL$21="","",Dados!$AL$21)</f>
         <v/>
       </c>
@@ -13591,7 +13704,7 @@
         <f>IF(N(O22)=0,"",IF(SUM($P$5:P22)-P22&lt;0.8,"A",IF(SUM($P$5:P22)-P22&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R22" s="36">
+      <c r="R22" s="37">
         <f>IF(Dados!$AL$22="","",Dados!$AL$22)</f>
         <v/>
       </c>
@@ -13665,7 +13778,7 @@
         <f>IF(N(O23)=0,"",IF(SUM($P$5:P23)-P23&lt;0.8,"A",IF(SUM($P$5:P23)-P23&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R23" s="36">
+      <c r="R23" s="37">
         <f>IF(Dados!$AL$23="","",Dados!$AL$23)</f>
         <v/>
       </c>
@@ -13739,7 +13852,7 @@
         <f>IF(N(O24)=0,"",IF(SUM($P$5:P24)-P24&lt;0.8,"A",IF(SUM($P$5:P24)-P24&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R24" s="36">
+      <c r="R24" s="37">
         <f>IF(Dados!$AL$24="","",Dados!$AL$24)</f>
         <v/>
       </c>
@@ -13813,7 +13926,7 @@
         <f>IF(N(O25)=0,"",IF(SUM($P$5:P25)-P25&lt;0.8,"A",IF(SUM($P$5:P25)-P25&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R25" s="36">
+      <c r="R25" s="37">
         <f>IF(Dados!$AL$25="","",Dados!$AL$25)</f>
         <v/>
       </c>
@@ -13887,7 +14000,7 @@
         <f>IF(N(O26)=0,"",IF(SUM($P$5:P26)-P26&lt;0.8,"A",IF(SUM($P$5:P26)-P26&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R26" s="36">
+      <c r="R26" s="37">
         <f>IF(Dados!$AL$26="","",Dados!$AL$26)</f>
         <v/>
       </c>
@@ -13961,7 +14074,7 @@
         <f>IF(N(O27)=0,"",IF(SUM($P$5:P27)-P27&lt;0.8,"A",IF(SUM($P$5:P27)-P27&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R27" s="36">
+      <c r="R27" s="37">
         <f>IF(Dados!$AL$27="","",Dados!$AL$27)</f>
         <v/>
       </c>
@@ -14035,7 +14148,7 @@
         <f>IF(N(O28)=0,"",IF(SUM($P$5:P28)-P28&lt;0.8,"A",IF(SUM($P$5:P28)-P28&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R28" s="36">
+      <c r="R28" s="37">
         <f>IF(Dados!$AL$28="","",Dados!$AL$28)</f>
         <v/>
       </c>
@@ -14109,7 +14222,7 @@
         <f>IF(N(O29)=0,"",IF(SUM($P$5:P29)-P29&lt;0.8,"A",IF(SUM($P$5:P29)-P29&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R29" s="36">
+      <c r="R29" s="37">
         <f>IF(Dados!$AL$29="","",Dados!$AL$29)</f>
         <v/>
       </c>
@@ -14183,7 +14296,7 @@
         <f>IF(N(O30)=0,"",IF(SUM($P$5:P30)-P30&lt;0.8,"A",IF(SUM($P$5:P30)-P30&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R30" s="36">
+      <c r="R30" s="37">
         <f>IF(Dados!$AL$30="","",Dados!$AL$30)</f>
         <v/>
       </c>
@@ -14257,7 +14370,7 @@
         <f>IF(N(O31)=0,"",IF(SUM($P$5:P31)-P31&lt;0.8,"A",IF(SUM($P$5:P31)-P31&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R31" s="36">
+      <c r="R31" s="37">
         <f>IF(Dados!$AL$31="","",Dados!$AL$31)</f>
         <v/>
       </c>
@@ -14331,7 +14444,7 @@
         <f>IF(N(O32)=0,"",IF(SUM($P$5:P32)-P32&lt;0.8,"A",IF(SUM($P$5:P32)-P32&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R32" s="36">
+      <c r="R32" s="37">
         <f>IF(Dados!$AL$32="","",Dados!$AL$32)</f>
         <v/>
       </c>
@@ -14405,7 +14518,7 @@
         <f>IF(N(O33)=0,"",IF(SUM($P$5:P33)-P33&lt;0.8,"A",IF(SUM($P$5:P33)-P33&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R33" s="36">
+      <c r="R33" s="37">
         <f>IF(Dados!$AL$33="","",Dados!$AL$33)</f>
         <v/>
       </c>
@@ -14479,7 +14592,7 @@
         <f>IF(N(O34)=0,"",IF(SUM($P$5:P34)-P34&lt;0.8,"A",IF(SUM($P$5:P34)-P34&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R34" s="36">
+      <c r="R34" s="37">
         <f>IF(Dados!$AL$34="","",Dados!$AL$34)</f>
         <v/>
       </c>
@@ -14553,7 +14666,7 @@
         <f>IF(N(O35)=0,"",IF(SUM($P$5:P35)-P35&lt;0.8,"A",IF(SUM($P$5:P35)-P35&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R35" s="36">
+      <c r="R35" s="37">
         <f>IF(Dados!$AL$35="","",Dados!$AL$35)</f>
         <v/>
       </c>
@@ -14627,7 +14740,7 @@
         <f>IF(N(O36)=0,"",IF(SUM($P$5:P36)-P36&lt;0.8,"A",IF(SUM($P$5:P36)-P36&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R36" s="36">
+      <c r="R36" s="37">
         <f>IF(Dados!$AL$36="","",Dados!$AL$36)</f>
         <v/>
       </c>
@@ -14701,7 +14814,7 @@
         <f>IF(N(O37)=0,"",IF(SUM($P$5:P37)-P37&lt;0.8,"A",IF(SUM($P$5:P37)-P37&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R37" s="36">
+      <c r="R37" s="37">
         <f>IF(Dados!$AL$37="","",Dados!$AL$37)</f>
         <v/>
       </c>
@@ -14775,7 +14888,7 @@
         <f>IF(N(O38)=0,"",IF(SUM($P$5:P38)-P38&lt;0.8,"A",IF(SUM($P$5:P38)-P38&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R38" s="36">
+      <c r="R38" s="37">
         <f>IF(Dados!$AL$38="","",Dados!$AL$38)</f>
         <v/>
       </c>
@@ -14849,7 +14962,7 @@
         <f>IF(N(O39)=0,"",IF(SUM($P$5:P39)-P39&lt;0.8,"A",IF(SUM($P$5:P39)-P39&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R39" s="36">
+      <c r="R39" s="37">
         <f>IF(Dados!$AL$39="","",Dados!$AL$39)</f>
         <v/>
       </c>
@@ -14923,7 +15036,7 @@
         <f>IF(N(O40)=0,"",IF(SUM($P$5:P40)-P40&lt;0.8,"A",IF(SUM($P$5:P40)-P40&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R40" s="36">
+      <c r="R40" s="37">
         <f>IF(Dados!$AL$40="","",Dados!$AL$40)</f>
         <v/>
       </c>
@@ -14997,7 +15110,7 @@
         <f>IF(N(O41)=0,"",IF(SUM($P$5:P41)-P41&lt;0.8,"A",IF(SUM($P$5:P41)-P41&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R41" s="36">
+      <c r="R41" s="37">
         <f>IF(Dados!$AL$41="","",Dados!$AL$41)</f>
         <v/>
       </c>
@@ -15071,7 +15184,7 @@
         <f>IF(N(O42)=0,"",IF(SUM($P$5:P42)-P42&lt;0.8,"A",IF(SUM($P$5:P42)-P42&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R42" s="36">
+      <c r="R42" s="37">
         <f>IF(Dados!$AL$42="","",Dados!$AL$42)</f>
         <v/>
       </c>
@@ -15145,7 +15258,7 @@
         <f>IF(N(O43)=0,"",IF(SUM($P$5:P43)-P43&lt;0.8,"A",IF(SUM($P$5:P43)-P43&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R43" s="36">
+      <c r="R43" s="37">
         <f>IF(Dados!$AL$43="","",Dados!$AL$43)</f>
         <v/>
       </c>
@@ -15219,7 +15332,7 @@
         <f>IF(N(O44)=0,"",IF(SUM($P$5:P44)-P44&lt;0.8,"A",IF(SUM($P$5:P44)-P44&lt;0.95,"B","C")))</f>
         <v/>
       </c>
-      <c r="R44" s="36">
+      <c r="R44" s="37">
         <f>IF(Dados!$AL$44="","",Dados!$AL$44)</f>
         <v/>
       </c>
@@ -17145,7 +17258,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="38" t="inlineStr">
         <is>
           <t>Vencido há até 30 dias</t>
         </is>
@@ -17200,7 +17313,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Vencido há mais de 30 dias</t>
         </is>
@@ -17482,7 +17595,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B17" s="38" t="inlineStr">
         <is>
           <t>Vencido há até 30 dias</t>
         </is>
@@ -17537,7 +17650,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="37" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Vencido há mais de 30 dias</t>
         </is>
@@ -17921,7 +18034,7 @@
         <f>VLOOKUP($B5,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="39">
         <f>C5+D5</f>
         <v/>
       </c>
@@ -17951,7 +18064,7 @@
         <f>VLOOKUP($B6,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="39">
         <f>C6+D6</f>
         <v/>
       </c>
@@ -17981,7 +18094,7 @@
         <f>VLOOKUP($B7,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="39">
         <f>C7+D7</f>
         <v/>
       </c>
@@ -18011,7 +18124,7 @@
         <f>VLOOKUP($B8,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="39">
         <f>C8+D8</f>
         <v/>
       </c>
@@ -18041,7 +18154,7 @@
         <f>VLOOKUP($B9,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="39">
         <f>C9+D9</f>
         <v/>
       </c>
@@ -18071,7 +18184,7 @@
         <f>VLOOKUP($B10,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E10" s="38">
+      <c r="E10" s="39">
         <f>C10+D10</f>
         <v/>
       </c>
@@ -18101,7 +18214,7 @@
         <f>VLOOKUP($B11,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="39">
         <f>C11+D11</f>
         <v/>
       </c>
@@ -18131,7 +18244,7 @@
         <f>VLOOKUP($B12,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E12" s="38">
+      <c r="E12" s="39">
         <f>C12+D12</f>
         <v/>
       </c>
@@ -18161,7 +18274,7 @@
         <f>VLOOKUP($B13,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E13" s="38">
+      <c r="E13" s="39">
         <f>C13+D13</f>
         <v/>
       </c>
@@ -18191,7 +18304,7 @@
         <f>VLOOKUP($B14,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E14" s="38">
+      <c r="E14" s="39">
         <f>C14+D14</f>
         <v/>
       </c>
@@ -18221,7 +18334,7 @@
         <f>VLOOKUP($B15,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E15" s="38">
+      <c r="E15" s="39">
         <f>C15+D15</f>
         <v/>
       </c>
@@ -18251,7 +18364,7 @@
         <f>VLOOKUP($B16,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E16" s="38">
+      <c r="E16" s="39">
         <f>C16+D16</f>
         <v/>
       </c>
@@ -18281,7 +18394,7 @@
         <f>VLOOKUP($B17,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E17" s="38">
+      <c r="E17" s="39">
         <f>C17+D17</f>
         <v/>
       </c>
@@ -18311,7 +18424,7 @@
         <f>VLOOKUP($B18,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E18" s="38">
+      <c r="E18" s="39">
         <f>C18+D18</f>
         <v/>
       </c>
@@ -18341,7 +18454,7 @@
         <f>VLOOKUP($B19,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E19" s="38">
+      <c r="E19" s="39">
         <f>C19+D19</f>
         <v/>
       </c>
@@ -18371,7 +18484,7 @@
         <f>VLOOKUP($B20,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E20" s="38">
+      <c r="E20" s="39">
         <f>C20+D20</f>
         <v/>
       </c>
@@ -18401,7 +18514,7 @@
         <f>VLOOKUP($B21,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E21" s="38">
+      <c r="E21" s="39">
         <f>C21+D21</f>
         <v/>
       </c>
@@ -18431,7 +18544,7 @@
         <f>VLOOKUP($B22,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E22" s="38">
+      <c r="E22" s="39">
         <f>C22+D22</f>
         <v/>
       </c>
@@ -18461,7 +18574,7 @@
         <f>VLOOKUP($B23,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E23" s="38">
+      <c r="E23" s="39">
         <f>C23+D23</f>
         <v/>
       </c>
@@ -18491,7 +18604,7 @@
         <f>VLOOKUP($B24,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E24" s="38">
+      <c r="E24" s="39">
         <f>C24+D24</f>
         <v/>
       </c>
@@ -18521,7 +18634,7 @@
         <f>VLOOKUP($B25,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E25" s="38">
+      <c r="E25" s="39">
         <f>C25+D25</f>
         <v/>
       </c>
@@ -18551,7 +18664,7 @@
         <f>VLOOKUP($B26,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E26" s="38">
+      <c r="E26" s="39">
         <f>C26+D26</f>
         <v/>
       </c>
@@ -18581,7 +18694,7 @@
         <f>VLOOKUP($B27,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E27" s="38">
+      <c r="E27" s="39">
         <f>C27+D27</f>
         <v/>
       </c>
@@ -18599,31 +18712,31 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="39">
+      <c r="B28" s="40">
         <f>VLOOKUP(EOMONTH(Dados!$AI$5,-1)+1,Dados!$A$5:$B$41,2,FALSE)</f>
         <v/>
       </c>
-      <c r="C28" s="40">
+      <c r="C28" s="41">
         <f>VLOOKUP($B28,Dados!$B$5:$AF$41,10,FALSE)</f>
         <v/>
       </c>
-      <c r="D28" s="40">
+      <c r="D28" s="41">
         <f>VLOOKUP($B28,Dados!$B$5:$AF$41,11,FALSE)</f>
         <v/>
       </c>
-      <c r="E28" s="40">
+      <c r="E28" s="41">
         <f>C28+D28</f>
         <v/>
       </c>
-      <c r="F28" s="41">
+      <c r="F28" s="42">
         <f>E28-E27</f>
         <v/>
       </c>
-      <c r="G28" s="41">
+      <c r="G28" s="42">
         <f>VLOOKUP($B28,Dados!$B$5:$AF$41,5,FALSE)</f>
         <v/>
       </c>
-      <c r="H28" s="42">
+      <c r="H28" s="43">
         <f>IFERROR(E28/AVERAGE(G26:G28),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
fix(workbook): ajuste ao extrato aparece como "Ajustado", não "Verificar"
O caixa informado do extrato é o valor certo do mês; a diferença para o
calculado pelo ERP é o ajuste ao extrato, e a conferência da ponte do caixa
já garante que ele fecha. A linha do Resumo passa a mostrar "Ajustado" em
destaque neutro (com o valor do ajuste) em vez de "Verificar".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NefkA2otxn5XifgkSQBnwE
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v2.xlsx
+++ b/public/workbook_fechamento_v2.xlsx
@@ -349,7 +349,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <font>
         <b val="1"/>
@@ -365,6 +365,18 @@
         <patternFill patternType="solid">
           <fgColor rgb="00B2592C"/>
           <bgColor rgb="00B2592C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B2592C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFAED"/>
+          <bgColor rgb="00FFFAED"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4045,11 +4057,11 @@
     <row r="22">
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Caixa do extrato = caixa calculado pelo ERP</t>
+          <t>Ajuste ao extrato: caixa informado − calculado pelo ERP</t>
         </is>
       </c>
       <c r="F22" s="19">
-        <f>IF(ABS(I22)&lt;1,"OK","Verificar")</f>
+        <f>IF(ABS(I22)&lt;1,"OK","Ajustado")</f>
         <v/>
       </c>
       <c r="G22" s="20">
@@ -4388,6 +4400,9 @@
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>F19="Verificar"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>F19="Ajustado"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -5166,7 +5181,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:N17">
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C6)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5763,12 +5778,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N12">
-    <cfRule type="expression" priority="2" dxfId="4">
+    <cfRule type="expression" priority="2" dxfId="5">
       <formula>C5="s/d"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N8">
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8638,7 +8653,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N9">
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9433,7 +9448,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N16">
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10123,7 +10138,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N14">
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12226,7 +12241,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N30">
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15506,12 +15521,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5:Q44">
-    <cfRule type="expression" priority="2" dxfId="3">
+    <cfRule type="expression" priority="2" dxfId="4">
       <formula>Q5="A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:N46">
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17931,7 +17946,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:N23">
-    <cfRule type="expression" priority="2" dxfId="2">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
feat(fechamento): rendimentos de aplicações no fechamento do mês
Os rendimentos (CDB, reserva remunerada, CDI das carteiras) ficavam dentro
do ajuste ao extrato. Agora:

- conta 6.1.2.01.001 "Rendimentos de Aplicações Financeiras";
- RPC registrar_rendimentos_mes: o total informado no fechamento vira um
  recebimento no último dia do mês (completa o que já estiver lançado no
  Financeiro; 0 cancela);
- workbook_fechamento_dados devolve "rendimentos" por mês;
- Entradas do fechamento: campo "Rendimentos de aplicações no mês";
- Workbook: coluna AG na aba Dados e linha própria na ponte da aba Caixa;
- apresentação: passo "Rendimentos" na ponte do caixa.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NefkA2otxn5XifgkSQBnwE
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v2.xlsx
+++ b/public/workbook_fechamento_v2.xlsx
@@ -1541,7 +1541,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Caixa'!$B$11</f>
+              <f>'Caixa'!$B$12</f>
             </strRef>
           </tx>
           <spPr>
@@ -1561,7 +1561,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Caixa'!$C$11:$N$11</f>
+              <f>'Caixa'!$C$12:$N$12</f>
             </numRef>
           </val>
         </ser>
@@ -1570,7 +1570,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Caixa'!$B$10</f>
+              <f>'Caixa'!$B$11</f>
             </strRef>
           </tx>
           <spPr>
@@ -1590,7 +1590,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Caixa'!$C$10:$N$10</f>
+              <f>'Caixa'!$C$11:$N$11</f>
             </numRef>
           </val>
         </ser>
@@ -1606,7 +1606,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Caixa'!$B$13</f>
+              <f>'Caixa'!$B$14</f>
             </strRef>
           </tx>
           <spPr>
@@ -1639,7 +1639,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Caixa'!$C$13:$N$13</f>
+              <f>'Caixa'!$C$14:$N$14</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -3031,7 +3031,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9360000" cy="3060000"/>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>Ponte do caixa mês a mês, bloqueado, disponível e meses de despesa cobertos</t>
+          <t>Ponte do caixa mês a mês (com rendimentos), bloqueado, disponível e meses de despesa cobertos</t>
         </is>
       </c>
       <c r="D30" s="18" t="n"/>
@@ -5844,7 +5844,7 @@
     <col width="11" customWidth="1" min="30" max="30"/>
     <col width="11" customWidth="1" min="31" max="31"/>
     <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="3" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
     <col width="34" customWidth="1" min="34" max="34"/>
     <col width="16" customWidth="1" min="35" max="35"/>
     <col width="3" customWidth="1" min="36" max="36"/>
@@ -6032,6 +6032,11 @@
       <c r="AF4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 4</t>
+        </is>
+      </c>
+      <c r="AG4" s="45" t="inlineStr">
+        <is>
+          <t>Rendimentos de aplicações</t>
         </is>
       </c>
       <c r="AH4" s="45" t="inlineStr">
@@ -6108,6 +6113,7 @@
       <c r="AD5" s="49" t="n"/>
       <c r="AE5" s="49" t="n"/>
       <c r="AF5" s="49" t="n"/>
+      <c r="AG5" s="49" t="n"/>
       <c r="AH5" s="47" t="inlineStr">
         <is>
           <t>Competência</t>
@@ -6154,6 +6160,7 @@
       <c r="AD6" s="49" t="n"/>
       <c r="AE6" s="49" t="n"/>
       <c r="AF6" s="49" t="n"/>
+      <c r="AG6" s="49" t="n"/>
       <c r="AH6" s="47" t="inlineStr">
         <is>
           <t>Mês</t>
@@ -6200,6 +6207,7 @@
       <c r="AD7" s="49" t="n"/>
       <c r="AE7" s="49" t="n"/>
       <c r="AF7" s="49" t="n"/>
+      <c r="AG7" s="49" t="n"/>
       <c r="AH7" s="47" t="inlineStr">
         <is>
           <t>Ano</t>
@@ -6246,6 +6254,7 @@
       <c r="AD8" s="49" t="n"/>
       <c r="AE8" s="49" t="n"/>
       <c r="AF8" s="49" t="n"/>
+      <c r="AG8" s="49" t="n"/>
       <c r="AH8" s="47" t="inlineStr">
         <is>
           <t>Período</t>
@@ -6292,6 +6301,7 @@
       <c r="AD9" s="49" t="n"/>
       <c r="AE9" s="49" t="n"/>
       <c r="AF9" s="49" t="n"/>
+      <c r="AG9" s="49" t="n"/>
       <c r="AH9" s="47" t="inlineStr">
         <is>
           <t>Data-base</t>
@@ -6338,6 +6348,7 @@
       <c r="AD10" s="49" t="n"/>
       <c r="AE10" s="49" t="n"/>
       <c r="AF10" s="49" t="n"/>
+      <c r="AG10" s="49" t="n"/>
       <c r="AH10" s="47" t="inlineStr">
         <is>
           <t>Gerado em</t>
@@ -6384,6 +6395,7 @@
       <c r="AD11" s="49" t="n"/>
       <c r="AE11" s="49" t="n"/>
       <c r="AF11" s="49" t="n"/>
+      <c r="AG11" s="49" t="n"/>
       <c r="AH11" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano</t>
@@ -6430,6 +6442,7 @@
       <c r="AD12" s="49" t="n"/>
       <c r="AE12" s="49" t="n"/>
       <c r="AF12" s="49" t="n"/>
+      <c r="AG12" s="49" t="n"/>
       <c r="AH12" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano anterior</t>
@@ -6476,6 +6489,7 @@
       <c r="AD13" s="49" t="n"/>
       <c r="AE13" s="49" t="n"/>
       <c r="AF13" s="49" t="n"/>
+      <c r="AG13" s="49" t="n"/>
       <c r="AH13" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-2)</t>
@@ -6522,6 +6536,7 @@
       <c r="AD14" s="49" t="n"/>
       <c r="AE14" s="49" t="n"/>
       <c r="AF14" s="49" t="n"/>
+      <c r="AG14" s="49" t="n"/>
       <c r="AH14" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-1)</t>
@@ -6568,6 +6583,7 @@
       <c r="AD15" s="49" t="n"/>
       <c r="AE15" s="49" t="n"/>
       <c r="AF15" s="49" t="n"/>
+      <c r="AG15" s="49" t="n"/>
       <c r="AH15" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano)</t>
@@ -6614,6 +6630,7 @@
       <c r="AD16" s="49" t="n"/>
       <c r="AE16" s="49" t="n"/>
       <c r="AF16" s="49" t="n"/>
+      <c r="AG16" s="49" t="n"/>
       <c r="AH16" s="47" t="inlineStr">
         <is>
           <t>Linhas do extrato pendentes</t>
@@ -6660,6 +6677,7 @@
       <c r="AD17" s="49" t="n"/>
       <c r="AE17" s="49" t="n"/>
       <c r="AF17" s="49" t="n"/>
+      <c r="AG17" s="49" t="n"/>
       <c r="AH17" s="47" t="inlineStr">
         <is>
           <t>Último extrato importado</t>
@@ -6706,6 +6724,7 @@
       <c r="AD18" s="49" t="n"/>
       <c r="AE18" s="49" t="n"/>
       <c r="AF18" s="49" t="n"/>
+      <c r="AG18" s="49" t="n"/>
       <c r="AH18" s="47" t="inlineStr">
         <is>
           <t>Notas de saída no mês</t>
@@ -6752,6 +6771,7 @@
       <c r="AD19" s="49" t="n"/>
       <c r="AE19" s="49" t="n"/>
       <c r="AF19" s="49" t="n"/>
+      <c r="AG19" s="49" t="n"/>
       <c r="AH19" s="47" t="inlineStr">
         <is>
           <t>Sócio 1</t>
@@ -6798,6 +6818,7 @@
       <c r="AD20" s="49" t="n"/>
       <c r="AE20" s="49" t="n"/>
       <c r="AF20" s="49" t="n"/>
+      <c r="AG20" s="49" t="n"/>
       <c r="AH20" s="47" t="inlineStr">
         <is>
           <t>Sócio 2</t>
@@ -6844,6 +6865,7 @@
       <c r="AD21" s="49" t="n"/>
       <c r="AE21" s="49" t="n"/>
       <c r="AF21" s="49" t="n"/>
+      <c r="AG21" s="49" t="n"/>
       <c r="AH21" s="47" t="inlineStr">
         <is>
           <t>Sócio 3</t>
@@ -6890,6 +6912,7 @@
       <c r="AD22" s="49" t="n"/>
       <c r="AE22" s="49" t="n"/>
       <c r="AF22" s="49" t="n"/>
+      <c r="AG22" s="49" t="n"/>
       <c r="AH22" s="47" t="inlineStr">
         <is>
           <t>Sócio 4</t>
@@ -6936,6 +6959,7 @@
       <c r="AD23" s="49" t="n"/>
       <c r="AE23" s="49" t="n"/>
       <c r="AF23" s="49" t="n"/>
+      <c r="AG23" s="49" t="n"/>
       <c r="AH23" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 1</t>
@@ -6982,6 +7006,7 @@
       <c r="AD24" s="49" t="n"/>
       <c r="AE24" s="49" t="n"/>
       <c r="AF24" s="49" t="n"/>
+      <c r="AG24" s="49" t="n"/>
       <c r="AH24" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 2</t>
@@ -7028,6 +7053,7 @@
       <c r="AD25" s="49" t="n"/>
       <c r="AE25" s="49" t="n"/>
       <c r="AF25" s="49" t="n"/>
+      <c r="AG25" s="49" t="n"/>
       <c r="AH25" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 3</t>
@@ -7074,6 +7100,7 @@
       <c r="AD26" s="49" t="n"/>
       <c r="AE26" s="49" t="n"/>
       <c r="AF26" s="49" t="n"/>
+      <c r="AG26" s="49" t="n"/>
       <c r="AH26" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 4</t>
@@ -7120,6 +7147,7 @@
       <c r="AD27" s="49" t="n"/>
       <c r="AE27" s="49" t="n"/>
       <c r="AF27" s="49" t="n"/>
+      <c r="AG27" s="49" t="n"/>
       <c r="AH27" s="47" t="inlineStr">
         <is>
           <t>Grupos de clientes que compraram no ano</t>
@@ -7166,6 +7194,7 @@
       <c r="AD28" s="49" t="n"/>
       <c r="AE28" s="49" t="n"/>
       <c r="AF28" s="49" t="n"/>
+      <c r="AG28" s="49" t="n"/>
       <c r="AH28" s="47" t="inlineStr">
         <is>
           <t>Grupos que compraram pela 1ª vez no ano</t>
@@ -7212,6 +7241,7 @@
       <c r="AD29" s="49" t="n"/>
       <c r="AE29" s="49" t="n"/>
       <c r="AF29" s="49" t="n"/>
+      <c r="AG29" s="49" t="n"/>
       <c r="AK29" s="47" t="n"/>
       <c r="AL29" s="47" t="n"/>
       <c r="AN29" s="47" t="n"/>
@@ -7252,6 +7282,7 @@
       <c r="AD30" s="49" t="n"/>
       <c r="AE30" s="49" t="n"/>
       <c r="AF30" s="49" t="n"/>
+      <c r="AG30" s="49" t="n"/>
       <c r="AK30" s="47" t="n"/>
       <c r="AL30" s="47" t="n"/>
       <c r="AN30" s="47" t="n"/>
@@ -7292,6 +7323,7 @@
       <c r="AD31" s="49" t="n"/>
       <c r="AE31" s="49" t="n"/>
       <c r="AF31" s="49" t="n"/>
+      <c r="AG31" s="49" t="n"/>
       <c r="AK31" s="47" t="n"/>
       <c r="AL31" s="47" t="n"/>
       <c r="AN31" s="47" t="n"/>
@@ -7332,6 +7364,7 @@
       <c r="AD32" s="49" t="n"/>
       <c r="AE32" s="49" t="n"/>
       <c r="AF32" s="49" t="n"/>
+      <c r="AG32" s="49" t="n"/>
       <c r="AK32" s="47" t="n"/>
       <c r="AL32" s="47" t="n"/>
       <c r="AN32" s="47" t="n"/>
@@ -7372,6 +7405,7 @@
       <c r="AD33" s="49" t="n"/>
       <c r="AE33" s="49" t="n"/>
       <c r="AF33" s="49" t="n"/>
+      <c r="AG33" s="49" t="n"/>
       <c r="AK33" s="47" t="n"/>
       <c r="AL33" s="47" t="n"/>
       <c r="AN33" s="47" t="n"/>
@@ -7412,6 +7446,7 @@
       <c r="AD34" s="49" t="n"/>
       <c r="AE34" s="49" t="n"/>
       <c r="AF34" s="49" t="n"/>
+      <c r="AG34" s="49" t="n"/>
       <c r="AK34" s="47" t="n"/>
       <c r="AL34" s="47" t="n"/>
       <c r="AN34" s="47" t="n"/>
@@ -7452,6 +7487,7 @@
       <c r="AD35" s="49" t="n"/>
       <c r="AE35" s="49" t="n"/>
       <c r="AF35" s="49" t="n"/>
+      <c r="AG35" s="49" t="n"/>
       <c r="AK35" s="47" t="n"/>
       <c r="AL35" s="47" t="n"/>
       <c r="AN35" s="47" t="n"/>
@@ -7492,6 +7528,7 @@
       <c r="AD36" s="49" t="n"/>
       <c r="AE36" s="49" t="n"/>
       <c r="AF36" s="49" t="n"/>
+      <c r="AG36" s="49" t="n"/>
       <c r="AK36" s="47" t="n"/>
       <c r="AL36" s="47" t="n"/>
       <c r="AN36" s="47" t="n"/>
@@ -7532,6 +7569,7 @@
       <c r="AD37" s="49" t="n"/>
       <c r="AE37" s="49" t="n"/>
       <c r="AF37" s="49" t="n"/>
+      <c r="AG37" s="49" t="n"/>
       <c r="AK37" s="47" t="n"/>
       <c r="AL37" s="47" t="n"/>
       <c r="AN37" s="47" t="n"/>
@@ -7572,6 +7610,7 @@
       <c r="AD38" s="49" t="n"/>
       <c r="AE38" s="49" t="n"/>
       <c r="AF38" s="49" t="n"/>
+      <c r="AG38" s="49" t="n"/>
       <c r="AK38" s="47" t="n"/>
       <c r="AL38" s="47" t="n"/>
       <c r="AN38" s="47" t="n"/>
@@ -7612,6 +7651,7 @@
       <c r="AD39" s="49" t="n"/>
       <c r="AE39" s="49" t="n"/>
       <c r="AF39" s="49" t="n"/>
+      <c r="AG39" s="49" t="n"/>
       <c r="AK39" s="47" t="n"/>
       <c r="AL39" s="47" t="n"/>
       <c r="AN39" s="47" t="n"/>
@@ -7652,6 +7692,7 @@
       <c r="AD40" s="49" t="n"/>
       <c r="AE40" s="49" t="n"/>
       <c r="AF40" s="49" t="n"/>
+      <c r="AG40" s="49" t="n"/>
       <c r="AK40" s="47" t="n"/>
       <c r="AL40" s="47" t="n"/>
       <c r="AN40" s="47" t="n"/>
@@ -7692,6 +7733,7 @@
       <c r="AD41" s="49" t="n"/>
       <c r="AE41" s="49" t="n"/>
       <c r="AF41" s="49" t="n"/>
+      <c r="AG41" s="49" t="n"/>
       <c r="AK41" s="47" t="n"/>
       <c r="AL41" s="47" t="n"/>
       <c r="AN41" s="47" t="n"/>
@@ -9474,7 +9516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:N15"/>
+  <dimension ref="B1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9632,502 +9674,557 @@
     <row r="6">
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>+ Recebido</t>
+          <t>+ Recebimentos</t>
         </is>
       </c>
       <c r="C6" s="20">
-        <f>IF(Dados!$C$30=1,Dados!$D$30,"")</f>
+        <f>IF(Dados!$C$30=1,Dados!$D$30-Dados!$AG$30,"")</f>
         <v/>
       </c>
       <c r="D6" s="20">
-        <f>IF(Dados!$C$31=1,Dados!$D$31,"")</f>
+        <f>IF(Dados!$C$31=1,Dados!$D$31-Dados!$AG$31,"")</f>
         <v/>
       </c>
       <c r="E6" s="20">
-        <f>IF(Dados!$C$32=1,Dados!$D$32,"")</f>
+        <f>IF(Dados!$C$32=1,Dados!$D$32-Dados!$AG$32,"")</f>
         <v/>
       </c>
       <c r="F6" s="20">
-        <f>IF(Dados!$C$33=1,Dados!$D$33,"")</f>
+        <f>IF(Dados!$C$33=1,Dados!$D$33-Dados!$AG$33,"")</f>
         <v/>
       </c>
       <c r="G6" s="20">
-        <f>IF(Dados!$C$34=1,Dados!$D$34,"")</f>
+        <f>IF(Dados!$C$34=1,Dados!$D$34-Dados!$AG$34,"")</f>
         <v/>
       </c>
       <c r="H6" s="20">
-        <f>IF(Dados!$C$35=1,Dados!$D$35,"")</f>
+        <f>IF(Dados!$C$35=1,Dados!$D$35-Dados!$AG$35,"")</f>
         <v/>
       </c>
       <c r="I6" s="20">
-        <f>IF(Dados!$C$36=1,Dados!$D$36,"")</f>
+        <f>IF(Dados!$C$36=1,Dados!$D$36-Dados!$AG$36,"")</f>
         <v/>
       </c>
       <c r="J6" s="20">
-        <f>IF(Dados!$C$37=1,Dados!$D$37,"")</f>
+        <f>IF(Dados!$C$37=1,Dados!$D$37-Dados!$AG$37,"")</f>
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>IF(Dados!$C$38=1,Dados!$D$38,"")</f>
+        <f>IF(Dados!$C$38=1,Dados!$D$38-Dados!$AG$38,"")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>IF(Dados!$C$39=1,Dados!$D$39,"")</f>
+        <f>IF(Dados!$C$39=1,Dados!$D$39-Dados!$AG$39,"")</f>
         <v/>
       </c>
       <c r="M6" s="20">
-        <f>IF(Dados!$C$40=1,Dados!$D$40,"")</f>
+        <f>IF(Dados!$C$40=1,Dados!$D$40-Dados!$AG$40,"")</f>
         <v/>
       </c>
       <c r="N6" s="20">
-        <f>IF(Dados!$C$41=1,Dados!$D$41,"")</f>
+        <f>IF(Dados!$C$41=1,Dados!$D$41-Dados!$AG$41,"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>− Pago</t>
+          <t>+ Rendimentos de aplicações</t>
         </is>
       </c>
       <c r="C7" s="20">
-        <f>IF(Dados!$C$30=1,-Dados!$E$30,"")</f>
+        <f>IF(Dados!$C$30=1,Dados!$AG$30,"")</f>
         <v/>
       </c>
       <c r="D7" s="20">
-        <f>IF(Dados!$C$31=1,-Dados!$E$31,"")</f>
+        <f>IF(Dados!$C$31=1,Dados!$AG$31,"")</f>
         <v/>
       </c>
       <c r="E7" s="20">
-        <f>IF(Dados!$C$32=1,-Dados!$E$32,"")</f>
+        <f>IF(Dados!$C$32=1,Dados!$AG$32,"")</f>
         <v/>
       </c>
       <c r="F7" s="20">
-        <f>IF(Dados!$C$33=1,-Dados!$E$33,"")</f>
+        <f>IF(Dados!$C$33=1,Dados!$AG$33,"")</f>
         <v/>
       </c>
       <c r="G7" s="20">
-        <f>IF(Dados!$C$34=1,-Dados!$E$34,"")</f>
+        <f>IF(Dados!$C$34=1,Dados!$AG$34,"")</f>
         <v/>
       </c>
       <c r="H7" s="20">
-        <f>IF(Dados!$C$35=1,-Dados!$E$35,"")</f>
+        <f>IF(Dados!$C$35=1,Dados!$AG$35,"")</f>
         <v/>
       </c>
       <c r="I7" s="20">
-        <f>IF(Dados!$C$36=1,-Dados!$E$36,"")</f>
+        <f>IF(Dados!$C$36=1,Dados!$AG$36,"")</f>
         <v/>
       </c>
       <c r="J7" s="20">
-        <f>IF(Dados!$C$37=1,-Dados!$E$37,"")</f>
+        <f>IF(Dados!$C$37=1,Dados!$AG$37,"")</f>
         <v/>
       </c>
       <c r="K7" s="20">
-        <f>IF(Dados!$C$38=1,-Dados!$E$38,"")</f>
+        <f>IF(Dados!$C$38=1,Dados!$AG$38,"")</f>
         <v/>
       </c>
       <c r="L7" s="20">
-        <f>IF(Dados!$C$39=1,-Dados!$E$39,"")</f>
+        <f>IF(Dados!$C$39=1,Dados!$AG$39,"")</f>
         <v/>
       </c>
       <c r="M7" s="20">
-        <f>IF(Dados!$C$40=1,-Dados!$E$40,"")</f>
+        <f>IF(Dados!$C$40=1,Dados!$AG$40,"")</f>
         <v/>
       </c>
       <c r="N7" s="20">
-        <f>IF(Dados!$C$41=1,-Dados!$E$41,"")</f>
+        <f>IF(Dados!$C$41=1,Dados!$AG$41,"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="18" t="inlineStr">
         <is>
+          <t>− Pago</t>
+        </is>
+      </c>
+      <c r="C8" s="20">
+        <f>IF(Dados!$C$30=1,-Dados!$E$30,"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="20">
+        <f>IF(Dados!$C$31=1,-Dados!$E$31,"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="20">
+        <f>IF(Dados!$C$32=1,-Dados!$E$32,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="20">
+        <f>IF(Dados!$C$33=1,-Dados!$E$33,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="20">
+        <f>IF(Dados!$C$34=1,-Dados!$E$34,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="20">
+        <f>IF(Dados!$C$35=1,-Dados!$E$35,"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="20">
+        <f>IF(Dados!$C$36=1,-Dados!$E$36,"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="20">
+        <f>IF(Dados!$C$37=1,-Dados!$E$37,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="20">
+        <f>IF(Dados!$C$38=1,-Dados!$E$38,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="20">
+        <f>IF(Dados!$C$39=1,-Dados!$E$39,"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="20">
+        <f>IF(Dados!$C$40=1,-Dados!$E$40,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="20">
+        <f>IF(Dados!$C$41=1,-Dados!$E$41,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
           <t>± Ajuste ao extrato</t>
         </is>
       </c>
-      <c r="C8" s="20">
+      <c r="C9" s="20">
         <f>IF(Dados!$C$30=1,Dados!$I$30,"")</f>
         <v/>
       </c>
-      <c r="D8" s="20">
+      <c r="D9" s="20">
         <f>IF(Dados!$C$31=1,Dados!$I$31,"")</f>
         <v/>
       </c>
-      <c r="E8" s="20">
+      <c r="E9" s="20">
         <f>IF(Dados!$C$32=1,Dados!$I$32,"")</f>
         <v/>
       </c>
-      <c r="F8" s="20">
+      <c r="F9" s="20">
         <f>IF(Dados!$C$33=1,Dados!$I$33,"")</f>
         <v/>
       </c>
-      <c r="G8" s="20">
+      <c r="G9" s="20">
         <f>IF(Dados!$C$34=1,Dados!$I$34,"")</f>
         <v/>
       </c>
-      <c r="H8" s="20">
+      <c r="H9" s="20">
         <f>IF(Dados!$C$35=1,Dados!$I$35,"")</f>
         <v/>
       </c>
-      <c r="I8" s="20">
+      <c r="I9" s="20">
         <f>IF(Dados!$C$36=1,Dados!$I$36,"")</f>
         <v/>
       </c>
-      <c r="J8" s="20">
+      <c r="J9" s="20">
         <f>IF(Dados!$C$37=1,Dados!$I$37,"")</f>
         <v/>
       </c>
-      <c r="K8" s="20">
+      <c r="K9" s="20">
         <f>IF(Dados!$C$38=1,Dados!$I$38,"")</f>
         <v/>
       </c>
-      <c r="L8" s="20">
+      <c r="L9" s="20">
         <f>IF(Dados!$C$39=1,Dados!$I$39,"")</f>
         <v/>
       </c>
-      <c r="M8" s="20">
+      <c r="M9" s="20">
         <f>IF(Dados!$C$40=1,Dados!$I$40,"")</f>
         <v/>
       </c>
-      <c r="N8" s="20">
+      <c r="N9" s="20">
         <f>IF(Dados!$C$41=1,Dados!$I$41,"")</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="26" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Caixa final</t>
         </is>
       </c>
-      <c r="C9" s="27">
+      <c r="C10" s="27">
         <f>IF(Dados!$C$30=1,Dados!$G$30,"")</f>
         <v/>
       </c>
-      <c r="D9" s="27">
+      <c r="D10" s="27">
         <f>IF(Dados!$C$31=1,Dados!$G$31,"")</f>
         <v/>
       </c>
-      <c r="E9" s="27">
+      <c r="E10" s="27">
         <f>IF(Dados!$C$32=1,Dados!$G$32,"")</f>
         <v/>
       </c>
-      <c r="F9" s="27">
+      <c r="F10" s="27">
         <f>IF(Dados!$C$33=1,Dados!$G$33,"")</f>
         <v/>
       </c>
-      <c r="G9" s="27">
+      <c r="G10" s="27">
         <f>IF(Dados!$C$34=1,Dados!$G$34,"")</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H10" s="27">
         <f>IF(Dados!$C$35=1,Dados!$G$35,"")</f>
         <v/>
       </c>
-      <c r="I9" s="27">
+      <c r="I10" s="27">
         <f>IF(Dados!$C$36=1,Dados!$G$36,"")</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J10" s="27">
         <f>IF(Dados!$C$37=1,Dados!$G$37,"")</f>
         <v/>
       </c>
-      <c r="K9" s="27">
+      <c r="K10" s="27">
         <f>IF(Dados!$C$38=1,Dados!$G$38,"")</f>
         <v/>
       </c>
-      <c r="L9" s="27">
+      <c r="L10" s="27">
         <f>IF(Dados!$C$39=1,Dados!$G$39,"")</f>
         <v/>
       </c>
-      <c r="M9" s="27">
+      <c r="M10" s="27">
         <f>IF(Dados!$C$40=1,Dados!$G$40,"")</f>
         <v/>
       </c>
-      <c r="N9" s="27">
+      <c r="N10" s="27">
         <f>IF(Dados!$C$41=1,Dados!$G$41,"")</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="28" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>bloqueado em garantia</t>
         </is>
       </c>
-      <c r="C10" s="29">
+      <c r="C11" s="29">
         <f>IF(Dados!$C$30=1,Dados!$J$30,"")</f>
         <v/>
       </c>
-      <c r="D10" s="29">
+      <c r="D11" s="29">
         <f>IF(Dados!$C$31=1,Dados!$J$31,"")</f>
         <v/>
       </c>
-      <c r="E10" s="29">
+      <c r="E11" s="29">
         <f>IF(Dados!$C$32=1,Dados!$J$32,"")</f>
         <v/>
       </c>
-      <c r="F10" s="29">
+      <c r="F11" s="29">
         <f>IF(Dados!$C$33=1,Dados!$J$33,"")</f>
         <v/>
       </c>
-      <c r="G10" s="29">
+      <c r="G11" s="29">
         <f>IF(Dados!$C$34=1,Dados!$J$34,"")</f>
         <v/>
       </c>
-      <c r="H10" s="29">
+      <c r="H11" s="29">
         <f>IF(Dados!$C$35=1,Dados!$J$35,"")</f>
         <v/>
       </c>
-      <c r="I10" s="29">
+      <c r="I11" s="29">
         <f>IF(Dados!$C$36=1,Dados!$J$36,"")</f>
         <v/>
       </c>
-      <c r="J10" s="29">
+      <c r="J11" s="29">
         <f>IF(Dados!$C$37=1,Dados!$J$37,"")</f>
         <v/>
       </c>
-      <c r="K10" s="29">
+      <c r="K11" s="29">
         <f>IF(Dados!$C$38=1,Dados!$J$38,"")</f>
         <v/>
       </c>
-      <c r="L10" s="29">
+      <c r="L11" s="29">
         <f>IF(Dados!$C$39=1,Dados!$J$39,"")</f>
         <v/>
       </c>
-      <c r="M10" s="29">
+      <c r="M11" s="29">
         <f>IF(Dados!$C$40=1,Dados!$J$40,"")</f>
         <v/>
       </c>
-      <c r="N10" s="29">
+      <c r="N11" s="29">
         <f>IF(Dados!$C$41=1,Dados!$J$41,"")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="33" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>disponível</t>
         </is>
       </c>
-      <c r="C11" s="20">
+      <c r="C12" s="20">
         <f>IF(Dados!$C$30=1,Dados!$G$30-Dados!$J$30,"")</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D12" s="20">
         <f>IF(Dados!$C$31=1,Dados!$G$31-Dados!$J$31,"")</f>
         <v/>
       </c>
-      <c r="E11" s="20">
+      <c r="E12" s="20">
         <f>IF(Dados!$C$32=1,Dados!$G$32-Dados!$J$32,"")</f>
         <v/>
       </c>
-      <c r="F11" s="20">
+      <c r="F12" s="20">
         <f>IF(Dados!$C$33=1,Dados!$G$33-Dados!$J$33,"")</f>
         <v/>
       </c>
-      <c r="G11" s="20">
+      <c r="G12" s="20">
         <f>IF(Dados!$C$34=1,Dados!$G$34-Dados!$J$34,"")</f>
         <v/>
       </c>
-      <c r="H11" s="20">
+      <c r="H12" s="20">
         <f>IF(Dados!$C$35=1,Dados!$G$35-Dados!$J$35,"")</f>
         <v/>
       </c>
-      <c r="I11" s="20">
+      <c r="I12" s="20">
         <f>IF(Dados!$C$36=1,Dados!$G$36-Dados!$J$36,"")</f>
         <v/>
       </c>
-      <c r="J11" s="20">
+      <c r="J12" s="20">
         <f>IF(Dados!$C$37=1,Dados!$G$37-Dados!$J$37,"")</f>
         <v/>
       </c>
-      <c r="K11" s="20">
+      <c r="K12" s="20">
         <f>IF(Dados!$C$38=1,Dados!$G$38-Dados!$J$38,"")</f>
         <v/>
       </c>
-      <c r="L11" s="20">
+      <c r="L12" s="20">
         <f>IF(Dados!$C$39=1,Dados!$G$39-Dados!$J$39,"")</f>
         <v/>
       </c>
-      <c r="M11" s="20">
+      <c r="M12" s="20">
         <f>IF(Dados!$C$40=1,Dados!$G$40-Dados!$J$40,"")</f>
         <v/>
       </c>
-      <c r="N11" s="20">
+      <c r="N12" s="20">
         <f>IF(Dados!$C$41=1,Dados!$G$41-Dados!$J$41,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t>Meses de despesa cobertos</t>
-        </is>
-      </c>
-      <c r="C12" s="34">
-        <f>IF(Dados!$C$30=1,IFERROR(C11/AVERAGE(Dados!$E$28:$E$30),""),"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="34">
-        <f>IF(Dados!$C$31=1,IFERROR(D11/AVERAGE(Dados!$E$29:$E$31),""),"")</f>
-        <v/>
-      </c>
-      <c r="E12" s="34">
-        <f>IF(Dados!$C$32=1,IFERROR(E11/AVERAGE(Dados!$E$30:$E$32),""),"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="34">
-        <f>IF(Dados!$C$33=1,IFERROR(F11/AVERAGE(Dados!$E$31:$E$33),""),"")</f>
-        <v/>
-      </c>
-      <c r="G12" s="34">
-        <f>IF(Dados!$C$34=1,IFERROR(G11/AVERAGE(Dados!$E$32:$E$34),""),"")</f>
-        <v/>
-      </c>
-      <c r="H12" s="34">
-        <f>IF(Dados!$C$35=1,IFERROR(H11/AVERAGE(Dados!$E$33:$E$35),""),"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="34">
-        <f>IF(Dados!$C$36=1,IFERROR(I11/AVERAGE(Dados!$E$34:$E$36),""),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="34">
-        <f>IF(Dados!$C$37=1,IFERROR(J11/AVERAGE(Dados!$E$35:$E$37),""),"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="34">
-        <f>IF(Dados!$C$38=1,IFERROR(K11/AVERAGE(Dados!$E$36:$E$38),""),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="34">
-        <f>IF(Dados!$C$39=1,IFERROR(L11/AVERAGE(Dados!$E$37:$E$39),""),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="34">
-        <f>IF(Dados!$C$40=1,IFERROR(M11/AVERAGE(Dados!$E$38:$E$40),""),"")</f>
-        <v/>
-      </c>
-      <c r="N12" s="34">
-        <f>IF(Dados!$C$41=1,IFERROR(N11/AVERAGE(Dados!$E$39:$E$41),""),"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="28" t="inlineStr">
         <is>
-          <t>Caixa final do ano anterior</t>
-        </is>
-      </c>
-      <c r="C13" s="29">
-        <f>IF(Dados!$C$18=1,Dados!$G$18,"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="29">
-        <f>IF(Dados!$C$19=1,Dados!$G$19,"")</f>
-        <v/>
-      </c>
-      <c r="E13" s="29">
-        <f>IF(Dados!$C$20=1,Dados!$G$20,"")</f>
-        <v/>
-      </c>
-      <c r="F13" s="29">
-        <f>IF(Dados!$C$21=1,Dados!$G$21,"")</f>
-        <v/>
-      </c>
-      <c r="G13" s="29">
-        <f>IF(Dados!$C$22=1,Dados!$G$22,"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="29">
-        <f>IF(Dados!$C$23=1,Dados!$G$23,"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="29">
-        <f>IF(Dados!$C$24=1,Dados!$G$24,"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="29">
-        <f>IF(Dados!$C$25=1,Dados!$G$25,"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="29">
-        <f>IF(Dados!$C$26=1,Dados!$G$26,"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="29">
-        <f>IF(Dados!$C$27=1,Dados!$G$27,"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="29">
-        <f>IF(Dados!$C$28=1,Dados!$G$28,"")</f>
-        <v/>
-      </c>
-      <c r="N13" s="29">
-        <f>IF(Dados!$C$29=1,Dados!$G$29,"")</f>
+          <t>Meses de despesa cobertos</t>
+        </is>
+      </c>
+      <c r="C13" s="34">
+        <f>IF(Dados!$C$30=1,IFERROR(C12/AVERAGE(Dados!$E$28:$E$30),""),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="34">
+        <f>IF(Dados!$C$31=1,IFERROR(D12/AVERAGE(Dados!$E$29:$E$31),""),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="34">
+        <f>IF(Dados!$C$32=1,IFERROR(E12/AVERAGE(Dados!$E$30:$E$32),""),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="34">
+        <f>IF(Dados!$C$33=1,IFERROR(F12/AVERAGE(Dados!$E$31:$E$33),""),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="34">
+        <f>IF(Dados!$C$34=1,IFERROR(G12/AVERAGE(Dados!$E$32:$E$34),""),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="34">
+        <f>IF(Dados!$C$35=1,IFERROR(H12/AVERAGE(Dados!$E$33:$E$35),""),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="34">
+        <f>IF(Dados!$C$36=1,IFERROR(I12/AVERAGE(Dados!$E$34:$E$36),""),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="34">
+        <f>IF(Dados!$C$37=1,IFERROR(J12/AVERAGE(Dados!$E$35:$E$37),""),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="34">
+        <f>IF(Dados!$C$38=1,IFERROR(K12/AVERAGE(Dados!$E$36:$E$38),""),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="34">
+        <f>IF(Dados!$C$39=1,IFERROR(L12/AVERAGE(Dados!$E$37:$E$39),""),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="34">
+        <f>IF(Dados!$C$40=1,IFERROR(M12/AVERAGE(Dados!$E$38:$E$40),""),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="34">
+        <f>IF(Dados!$C$41=1,IFERROR(N12/AVERAGE(Dados!$E$39:$E$41),""),"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="28" t="inlineStr">
         <is>
+          <t>Caixa final do ano anterior</t>
+        </is>
+      </c>
+      <c r="C14" s="29">
+        <f>IF(Dados!$C$18=1,Dados!$G$18,"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="29">
+        <f>IF(Dados!$C$19=1,Dados!$G$19,"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>IF(Dados!$C$20=1,Dados!$G$20,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="29">
+        <f>IF(Dados!$C$21=1,Dados!$G$21,"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>IF(Dados!$C$22=1,Dados!$G$22,"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="29">
+        <f>IF(Dados!$C$23=1,Dados!$G$23,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="29">
+        <f>IF(Dados!$C$24=1,Dados!$G$24,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="29">
+        <f>IF(Dados!$C$25=1,Dados!$G$25,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="29">
+        <f>IF(Dados!$C$26=1,Dados!$G$26,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="29">
+        <f>IF(Dados!$C$27=1,Dados!$G$27,"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="29">
+        <f>IF(Dados!$C$28=1,Dados!$G$28,"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="29">
+        <f>IF(Dados!$C$29=1,Dados!$G$29,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
           <t>Diferença na ponte (deve ser zero)</t>
         </is>
       </c>
-      <c r="C14" s="29">
-        <f>IF(C9="","",ROUND(C5+C6+C7+C8-C9,2))</f>
-        <v/>
-      </c>
-      <c r="D14" s="29">
-        <f>IF(D9="","",ROUND(D5+D6+D7+D8-D9,2))</f>
-        <v/>
-      </c>
-      <c r="E14" s="29">
-        <f>IF(E9="","",ROUND(E5+E6+E7+E8-E9,2))</f>
-        <v/>
-      </c>
-      <c r="F14" s="29">
-        <f>IF(F9="","",ROUND(F5+F6+F7+F8-F9,2))</f>
-        <v/>
-      </c>
-      <c r="G14" s="29">
-        <f>IF(G9="","",ROUND(G5+G6+G7+G8-G9,2))</f>
-        <v/>
-      </c>
-      <c r="H14" s="29">
-        <f>IF(H9="","",ROUND(H5+H6+H7+H8-H9,2))</f>
-        <v/>
-      </c>
-      <c r="I14" s="29">
-        <f>IF(I9="","",ROUND(I5+I6+I7+I8-I9,2))</f>
-        <v/>
-      </c>
-      <c r="J14" s="29">
-        <f>IF(J9="","",ROUND(J5+J6+J7+J8-J9,2))</f>
-        <v/>
-      </c>
-      <c r="K14" s="29">
-        <f>IF(K9="","",ROUND(K5+K6+K7+K8-K9,2))</f>
-        <v/>
-      </c>
-      <c r="L14" s="29">
-        <f>IF(L9="","",ROUND(L5+L6+L7+L8-L9,2))</f>
-        <v/>
-      </c>
-      <c r="M14" s="29">
-        <f>IF(M9="","",ROUND(M5+M6+M7+M8-M9,2))</f>
-        <v/>
-      </c>
-      <c r="N14" s="29">
-        <f>IF(N9="","",ROUND(N5+N6+N7+N8-N9,2))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>Meses de despesa cobertos: caixa disponível ÷ média do pago nos últimos 3 meses.</t>
+      <c r="C15" s="29">
+        <f>IF(C10="","",ROUND(C5+C6+C7+C8+C9-C10,2))</f>
+        <v/>
+      </c>
+      <c r="D15" s="29">
+        <f>IF(D10="","",ROUND(D5+D6+D7+D8+D9-D10,2))</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>IF(E10="","",ROUND(E5+E6+E7+E8+E9-E10,2))</f>
+        <v/>
+      </c>
+      <c r="F15" s="29">
+        <f>IF(F10="","",ROUND(F5+F6+F7+F8+F9-F10,2))</f>
+        <v/>
+      </c>
+      <c r="G15" s="29">
+        <f>IF(G10="","",ROUND(G5+G6+G7+G8+G9-G10,2))</f>
+        <v/>
+      </c>
+      <c r="H15" s="29">
+        <f>IF(H10="","",ROUND(H5+H6+H7+H8+H9-H10,2))</f>
+        <v/>
+      </c>
+      <c r="I15" s="29">
+        <f>IF(I10="","",ROUND(I5+I6+I7+I8+I9-I10,2))</f>
+        <v/>
+      </c>
+      <c r="J15" s="29">
+        <f>IF(J10="","",ROUND(J5+J6+J7+J8+J9-J10,2))</f>
+        <v/>
+      </c>
+      <c r="K15" s="29">
+        <f>IF(K10="","",ROUND(K5+K6+K7+K8+K9-K10,2))</f>
+        <v/>
+      </c>
+      <c r="L15" s="29">
+        <f>IF(L10="","",ROUND(L5+L6+L7+L8+L9-L10,2))</f>
+        <v/>
+      </c>
+      <c r="M15" s="29">
+        <f>IF(M10="","",ROUND(M5+M6+M7+M8+M9-M10,2))</f>
+        <v/>
+      </c>
+      <c r="N15" s="29">
+        <f>IF(N10="","",ROUND(N5+N6+N7+N8+N9-N10,2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Meses de despesa cobertos: caixa disponível ÷ média do pago nos últimos 3 meses. Rendimentos: CDB, reserva remunerada e CDI informados no fechamento.</t>
         </is>
       </c>
     </row>
@@ -10137,7 +10234,7 @@
       <formula>COLUMN(C4)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:N14">
+  <conditionalFormatting sqref="C5:N15">
     <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat(fechamento): rendimentos de aplicações no fechamento do mês (#120)
Os rendimentos (CDB, reserva remunerada, CDI das carteiras) ficavam dentro
do ajuste ao extrato. Agora:

- conta 6.1.2.01.001 "Rendimentos de Aplicações Financeiras";
- RPC registrar_rendimentos_mes: o total informado no fechamento vira um
  recebimento no último dia do mês (completa o que já estiver lançado no
  Financeiro; 0 cancela);
- workbook_fechamento_dados devolve "rendimentos" por mês;
- Entradas do fechamento: campo "Rendimentos de aplicações no mês";
- Workbook: coluna AG na aba Dados e linha própria na ponte da aba Caixa;
- apresentação: passo "Rendimentos" na ponte do caixa.


Claude-Session: https://claude.ai/code/session_01NefkA2otxn5XifgkSQBnwE

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/workbook_fechamento_v2.xlsx
+++ b/public/workbook_fechamento_v2.xlsx
@@ -1541,7 +1541,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Caixa'!$B$11</f>
+              <f>'Caixa'!$B$12</f>
             </strRef>
           </tx>
           <spPr>
@@ -1561,7 +1561,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Caixa'!$C$11:$N$11</f>
+              <f>'Caixa'!$C$12:$N$12</f>
             </numRef>
           </val>
         </ser>
@@ -1570,7 +1570,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Caixa'!$B$10</f>
+              <f>'Caixa'!$B$11</f>
             </strRef>
           </tx>
           <spPr>
@@ -1590,7 +1590,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Caixa'!$C$10:$N$10</f>
+              <f>'Caixa'!$C$11:$N$11</f>
             </numRef>
           </val>
         </ser>
@@ -1606,7 +1606,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Caixa'!$B$13</f>
+              <f>'Caixa'!$B$14</f>
             </strRef>
           </tx>
           <spPr>
@@ -1639,7 +1639,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Caixa'!$C$13:$N$13</f>
+              <f>'Caixa'!$C$14:$N$14</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -3031,7 +3031,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>17</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9360000" cy="3060000"/>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>Ponte do caixa mês a mês, bloqueado, disponível e meses de despesa cobertos</t>
+          <t>Ponte do caixa mês a mês (com rendimentos), bloqueado, disponível e meses de despesa cobertos</t>
         </is>
       </c>
       <c r="D30" s="18" t="n"/>
@@ -5844,7 +5844,7 @@
     <col width="11" customWidth="1" min="30" max="30"/>
     <col width="11" customWidth="1" min="31" max="31"/>
     <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="3" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
     <col width="34" customWidth="1" min="34" max="34"/>
     <col width="16" customWidth="1" min="35" max="35"/>
     <col width="3" customWidth="1" min="36" max="36"/>
@@ -6032,6 +6032,11 @@
       <c r="AF4" s="45" t="inlineStr">
         <is>
           <t>Resultado atribuído sócio 4</t>
+        </is>
+      </c>
+      <c r="AG4" s="45" t="inlineStr">
+        <is>
+          <t>Rendimentos de aplicações</t>
         </is>
       </c>
       <c r="AH4" s="45" t="inlineStr">
@@ -6108,6 +6113,7 @@
       <c r="AD5" s="49" t="n"/>
       <c r="AE5" s="49" t="n"/>
       <c r="AF5" s="49" t="n"/>
+      <c r="AG5" s="49" t="n"/>
       <c r="AH5" s="47" t="inlineStr">
         <is>
           <t>Competência</t>
@@ -6154,6 +6160,7 @@
       <c r="AD6" s="49" t="n"/>
       <c r="AE6" s="49" t="n"/>
       <c r="AF6" s="49" t="n"/>
+      <c r="AG6" s="49" t="n"/>
       <c r="AH6" s="47" t="inlineStr">
         <is>
           <t>Mês</t>
@@ -6200,6 +6207,7 @@
       <c r="AD7" s="49" t="n"/>
       <c r="AE7" s="49" t="n"/>
       <c r="AF7" s="49" t="n"/>
+      <c r="AG7" s="49" t="n"/>
       <c r="AH7" s="47" t="inlineStr">
         <is>
           <t>Ano</t>
@@ -6246,6 +6254,7 @@
       <c r="AD8" s="49" t="n"/>
       <c r="AE8" s="49" t="n"/>
       <c r="AF8" s="49" t="n"/>
+      <c r="AG8" s="49" t="n"/>
       <c r="AH8" s="47" t="inlineStr">
         <is>
           <t>Período</t>
@@ -6292,6 +6301,7 @@
       <c r="AD9" s="49" t="n"/>
       <c r="AE9" s="49" t="n"/>
       <c r="AF9" s="49" t="n"/>
+      <c r="AG9" s="49" t="n"/>
       <c r="AH9" s="47" t="inlineStr">
         <is>
           <t>Data-base</t>
@@ -6338,6 +6348,7 @@
       <c r="AD10" s="49" t="n"/>
       <c r="AE10" s="49" t="n"/>
       <c r="AF10" s="49" t="n"/>
+      <c r="AG10" s="49" t="n"/>
       <c r="AH10" s="47" t="inlineStr">
         <is>
           <t>Gerado em</t>
@@ -6384,6 +6395,7 @@
       <c r="AD11" s="49" t="n"/>
       <c r="AE11" s="49" t="n"/>
       <c r="AF11" s="49" t="n"/>
+      <c r="AG11" s="49" t="n"/>
       <c r="AH11" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano</t>
@@ -6430,6 +6442,7 @@
       <c r="AD12" s="49" t="n"/>
       <c r="AE12" s="49" t="n"/>
       <c r="AF12" s="49" t="n"/>
+      <c r="AG12" s="49" t="n"/>
       <c r="AH12" s="47" t="inlineStr">
         <is>
           <t>Meta de crescimento do ano anterior</t>
@@ -6476,6 +6489,7 @@
       <c r="AD13" s="49" t="n"/>
       <c r="AE13" s="49" t="n"/>
       <c r="AF13" s="49" t="n"/>
+      <c r="AG13" s="49" t="n"/>
       <c r="AH13" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-2)</t>
@@ -6522,6 +6536,7 @@
       <c r="AD14" s="49" t="n"/>
       <c r="AE14" s="49" t="n"/>
       <c r="AF14" s="49" t="n"/>
+      <c r="AG14" s="49" t="n"/>
       <c r="AH14" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano-1)</t>
@@ -6568,6 +6583,7 @@
       <c r="AD15" s="49" t="n"/>
       <c r="AE15" s="49" t="n"/>
       <c r="AF15" s="49" t="n"/>
+      <c r="AG15" s="49" t="n"/>
       <c r="AH15" s="47" t="inlineStr">
         <is>
           <t>Limite de faturamento (ano)</t>
@@ -6614,6 +6630,7 @@
       <c r="AD16" s="49" t="n"/>
       <c r="AE16" s="49" t="n"/>
       <c r="AF16" s="49" t="n"/>
+      <c r="AG16" s="49" t="n"/>
       <c r="AH16" s="47" t="inlineStr">
         <is>
           <t>Linhas do extrato pendentes</t>
@@ -6660,6 +6677,7 @@
       <c r="AD17" s="49" t="n"/>
       <c r="AE17" s="49" t="n"/>
       <c r="AF17" s="49" t="n"/>
+      <c r="AG17" s="49" t="n"/>
       <c r="AH17" s="47" t="inlineStr">
         <is>
           <t>Último extrato importado</t>
@@ -6706,6 +6724,7 @@
       <c r="AD18" s="49" t="n"/>
       <c r="AE18" s="49" t="n"/>
       <c r="AF18" s="49" t="n"/>
+      <c r="AG18" s="49" t="n"/>
       <c r="AH18" s="47" t="inlineStr">
         <is>
           <t>Notas de saída no mês</t>
@@ -6752,6 +6771,7 @@
       <c r="AD19" s="49" t="n"/>
       <c r="AE19" s="49" t="n"/>
       <c r="AF19" s="49" t="n"/>
+      <c r="AG19" s="49" t="n"/>
       <c r="AH19" s="47" t="inlineStr">
         <is>
           <t>Sócio 1</t>
@@ -6798,6 +6818,7 @@
       <c r="AD20" s="49" t="n"/>
       <c r="AE20" s="49" t="n"/>
       <c r="AF20" s="49" t="n"/>
+      <c r="AG20" s="49" t="n"/>
       <c r="AH20" s="47" t="inlineStr">
         <is>
           <t>Sócio 2</t>
@@ -6844,6 +6865,7 @@
       <c r="AD21" s="49" t="n"/>
       <c r="AE21" s="49" t="n"/>
       <c r="AF21" s="49" t="n"/>
+      <c r="AG21" s="49" t="n"/>
       <c r="AH21" s="47" t="inlineStr">
         <is>
           <t>Sócio 3</t>
@@ -6890,6 +6912,7 @@
       <c r="AD22" s="49" t="n"/>
       <c r="AE22" s="49" t="n"/>
       <c r="AF22" s="49" t="n"/>
+      <c r="AG22" s="49" t="n"/>
       <c r="AH22" s="47" t="inlineStr">
         <is>
           <t>Sócio 4</t>
@@ -6936,6 +6959,7 @@
       <c r="AD23" s="49" t="n"/>
       <c r="AE23" s="49" t="n"/>
       <c r="AF23" s="49" t="n"/>
+      <c r="AG23" s="49" t="n"/>
       <c r="AH23" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 1</t>
@@ -6982,6 +7006,7 @@
       <c r="AD24" s="49" t="n"/>
       <c r="AE24" s="49" t="n"/>
       <c r="AF24" s="49" t="n"/>
+      <c r="AG24" s="49" t="n"/>
       <c r="AH24" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 2</t>
@@ -7028,6 +7053,7 @@
       <c r="AD25" s="49" t="n"/>
       <c r="AE25" s="49" t="n"/>
       <c r="AF25" s="49" t="n"/>
+      <c r="AG25" s="49" t="n"/>
       <c r="AH25" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 3</t>
@@ -7074,6 +7100,7 @@
       <c r="AD26" s="49" t="n"/>
       <c r="AE26" s="49" t="n"/>
       <c r="AF26" s="49" t="n"/>
+      <c r="AG26" s="49" t="n"/>
       <c r="AH26" s="47" t="inlineStr">
         <is>
           <t>Participação sócio 4</t>
@@ -7120,6 +7147,7 @@
       <c r="AD27" s="49" t="n"/>
       <c r="AE27" s="49" t="n"/>
       <c r="AF27" s="49" t="n"/>
+      <c r="AG27" s="49" t="n"/>
       <c r="AH27" s="47" t="inlineStr">
         <is>
           <t>Grupos de clientes que compraram no ano</t>
@@ -7166,6 +7194,7 @@
       <c r="AD28" s="49" t="n"/>
       <c r="AE28" s="49" t="n"/>
       <c r="AF28" s="49" t="n"/>
+      <c r="AG28" s="49" t="n"/>
       <c r="AH28" s="47" t="inlineStr">
         <is>
           <t>Grupos que compraram pela 1ª vez no ano</t>
@@ -7212,6 +7241,7 @@
       <c r="AD29" s="49" t="n"/>
       <c r="AE29" s="49" t="n"/>
       <c r="AF29" s="49" t="n"/>
+      <c r="AG29" s="49" t="n"/>
       <c r="AK29" s="47" t="n"/>
       <c r="AL29" s="47" t="n"/>
       <c r="AN29" s="47" t="n"/>
@@ -7252,6 +7282,7 @@
       <c r="AD30" s="49" t="n"/>
       <c r="AE30" s="49" t="n"/>
       <c r="AF30" s="49" t="n"/>
+      <c r="AG30" s="49" t="n"/>
       <c r="AK30" s="47" t="n"/>
       <c r="AL30" s="47" t="n"/>
       <c r="AN30" s="47" t="n"/>
@@ -7292,6 +7323,7 @@
       <c r="AD31" s="49" t="n"/>
       <c r="AE31" s="49" t="n"/>
       <c r="AF31" s="49" t="n"/>
+      <c r="AG31" s="49" t="n"/>
       <c r="AK31" s="47" t="n"/>
       <c r="AL31" s="47" t="n"/>
       <c r="AN31" s="47" t="n"/>
@@ -7332,6 +7364,7 @@
       <c r="AD32" s="49" t="n"/>
       <c r="AE32" s="49" t="n"/>
       <c r="AF32" s="49" t="n"/>
+      <c r="AG32" s="49" t="n"/>
       <c r="AK32" s="47" t="n"/>
       <c r="AL32" s="47" t="n"/>
       <c r="AN32" s="47" t="n"/>
@@ -7372,6 +7405,7 @@
       <c r="AD33" s="49" t="n"/>
       <c r="AE33" s="49" t="n"/>
       <c r="AF33" s="49" t="n"/>
+      <c r="AG33" s="49" t="n"/>
       <c r="AK33" s="47" t="n"/>
       <c r="AL33" s="47" t="n"/>
       <c r="AN33" s="47" t="n"/>
@@ -7412,6 +7446,7 @@
       <c r="AD34" s="49" t="n"/>
       <c r="AE34" s="49" t="n"/>
       <c r="AF34" s="49" t="n"/>
+      <c r="AG34" s="49" t="n"/>
       <c r="AK34" s="47" t="n"/>
       <c r="AL34" s="47" t="n"/>
       <c r="AN34" s="47" t="n"/>
@@ -7452,6 +7487,7 @@
       <c r="AD35" s="49" t="n"/>
       <c r="AE35" s="49" t="n"/>
       <c r="AF35" s="49" t="n"/>
+      <c r="AG35" s="49" t="n"/>
       <c r="AK35" s="47" t="n"/>
       <c r="AL35" s="47" t="n"/>
       <c r="AN35" s="47" t="n"/>
@@ -7492,6 +7528,7 @@
       <c r="AD36" s="49" t="n"/>
       <c r="AE36" s="49" t="n"/>
       <c r="AF36" s="49" t="n"/>
+      <c r="AG36" s="49" t="n"/>
       <c r="AK36" s="47" t="n"/>
       <c r="AL36" s="47" t="n"/>
       <c r="AN36" s="47" t="n"/>
@@ -7532,6 +7569,7 @@
       <c r="AD37" s="49" t="n"/>
       <c r="AE37" s="49" t="n"/>
       <c r="AF37" s="49" t="n"/>
+      <c r="AG37" s="49" t="n"/>
       <c r="AK37" s="47" t="n"/>
       <c r="AL37" s="47" t="n"/>
       <c r="AN37" s="47" t="n"/>
@@ -7572,6 +7610,7 @@
       <c r="AD38" s="49" t="n"/>
       <c r="AE38" s="49" t="n"/>
       <c r="AF38" s="49" t="n"/>
+      <c r="AG38" s="49" t="n"/>
       <c r="AK38" s="47" t="n"/>
       <c r="AL38" s="47" t="n"/>
       <c r="AN38" s="47" t="n"/>
@@ -7612,6 +7651,7 @@
       <c r="AD39" s="49" t="n"/>
       <c r="AE39" s="49" t="n"/>
       <c r="AF39" s="49" t="n"/>
+      <c r="AG39" s="49" t="n"/>
       <c r="AK39" s="47" t="n"/>
       <c r="AL39" s="47" t="n"/>
       <c r="AN39" s="47" t="n"/>
@@ -7652,6 +7692,7 @@
       <c r="AD40" s="49" t="n"/>
       <c r="AE40" s="49" t="n"/>
       <c r="AF40" s="49" t="n"/>
+      <c r="AG40" s="49" t="n"/>
       <c r="AK40" s="47" t="n"/>
       <c r="AL40" s="47" t="n"/>
       <c r="AN40" s="47" t="n"/>
@@ -7692,6 +7733,7 @@
       <c r="AD41" s="49" t="n"/>
       <c r="AE41" s="49" t="n"/>
       <c r="AF41" s="49" t="n"/>
+      <c r="AG41" s="49" t="n"/>
       <c r="AK41" s="47" t="n"/>
       <c r="AL41" s="47" t="n"/>
       <c r="AN41" s="47" t="n"/>
@@ -9474,7 +9516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:N15"/>
+  <dimension ref="B1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -9632,502 +9674,557 @@
     <row r="6">
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>+ Recebido</t>
+          <t>+ Recebimentos</t>
         </is>
       </c>
       <c r="C6" s="20">
-        <f>IF(Dados!$C$30=1,Dados!$D$30,"")</f>
+        <f>IF(Dados!$C$30=1,Dados!$D$30-Dados!$AG$30,"")</f>
         <v/>
       </c>
       <c r="D6" s="20">
-        <f>IF(Dados!$C$31=1,Dados!$D$31,"")</f>
+        <f>IF(Dados!$C$31=1,Dados!$D$31-Dados!$AG$31,"")</f>
         <v/>
       </c>
       <c r="E6" s="20">
-        <f>IF(Dados!$C$32=1,Dados!$D$32,"")</f>
+        <f>IF(Dados!$C$32=1,Dados!$D$32-Dados!$AG$32,"")</f>
         <v/>
       </c>
       <c r="F6" s="20">
-        <f>IF(Dados!$C$33=1,Dados!$D$33,"")</f>
+        <f>IF(Dados!$C$33=1,Dados!$D$33-Dados!$AG$33,"")</f>
         <v/>
       </c>
       <c r="G6" s="20">
-        <f>IF(Dados!$C$34=1,Dados!$D$34,"")</f>
+        <f>IF(Dados!$C$34=1,Dados!$D$34-Dados!$AG$34,"")</f>
         <v/>
       </c>
       <c r="H6" s="20">
-        <f>IF(Dados!$C$35=1,Dados!$D$35,"")</f>
+        <f>IF(Dados!$C$35=1,Dados!$D$35-Dados!$AG$35,"")</f>
         <v/>
       </c>
       <c r="I6" s="20">
-        <f>IF(Dados!$C$36=1,Dados!$D$36,"")</f>
+        <f>IF(Dados!$C$36=1,Dados!$D$36-Dados!$AG$36,"")</f>
         <v/>
       </c>
       <c r="J6" s="20">
-        <f>IF(Dados!$C$37=1,Dados!$D$37,"")</f>
+        <f>IF(Dados!$C$37=1,Dados!$D$37-Dados!$AG$37,"")</f>
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>IF(Dados!$C$38=1,Dados!$D$38,"")</f>
+        <f>IF(Dados!$C$38=1,Dados!$D$38-Dados!$AG$38,"")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>IF(Dados!$C$39=1,Dados!$D$39,"")</f>
+        <f>IF(Dados!$C$39=1,Dados!$D$39-Dados!$AG$39,"")</f>
         <v/>
       </c>
       <c r="M6" s="20">
-        <f>IF(Dados!$C$40=1,Dados!$D$40,"")</f>
+        <f>IF(Dados!$C$40=1,Dados!$D$40-Dados!$AG$40,"")</f>
         <v/>
       </c>
       <c r="N6" s="20">
-        <f>IF(Dados!$C$41=1,Dados!$D$41,"")</f>
+        <f>IF(Dados!$C$41=1,Dados!$D$41-Dados!$AG$41,"")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>− Pago</t>
+          <t>+ Rendimentos de aplicações</t>
         </is>
       </c>
       <c r="C7" s="20">
-        <f>IF(Dados!$C$30=1,-Dados!$E$30,"")</f>
+        <f>IF(Dados!$C$30=1,Dados!$AG$30,"")</f>
         <v/>
       </c>
       <c r="D7" s="20">
-        <f>IF(Dados!$C$31=1,-Dados!$E$31,"")</f>
+        <f>IF(Dados!$C$31=1,Dados!$AG$31,"")</f>
         <v/>
       </c>
       <c r="E7" s="20">
-        <f>IF(Dados!$C$32=1,-Dados!$E$32,"")</f>
+        <f>IF(Dados!$C$32=1,Dados!$AG$32,"")</f>
         <v/>
       </c>
       <c r="F7" s="20">
-        <f>IF(Dados!$C$33=1,-Dados!$E$33,"")</f>
+        <f>IF(Dados!$C$33=1,Dados!$AG$33,"")</f>
         <v/>
       </c>
       <c r="G7" s="20">
-        <f>IF(Dados!$C$34=1,-Dados!$E$34,"")</f>
+        <f>IF(Dados!$C$34=1,Dados!$AG$34,"")</f>
         <v/>
       </c>
       <c r="H7" s="20">
-        <f>IF(Dados!$C$35=1,-Dados!$E$35,"")</f>
+        <f>IF(Dados!$C$35=1,Dados!$AG$35,"")</f>
         <v/>
       </c>
       <c r="I7" s="20">
-        <f>IF(Dados!$C$36=1,-Dados!$E$36,"")</f>
+        <f>IF(Dados!$C$36=1,Dados!$AG$36,"")</f>
         <v/>
       </c>
       <c r="J7" s="20">
-        <f>IF(Dados!$C$37=1,-Dados!$E$37,"")</f>
+        <f>IF(Dados!$C$37=1,Dados!$AG$37,"")</f>
         <v/>
       </c>
       <c r="K7" s="20">
-        <f>IF(Dados!$C$38=1,-Dados!$E$38,"")</f>
+        <f>IF(Dados!$C$38=1,Dados!$AG$38,"")</f>
         <v/>
       </c>
       <c r="L7" s="20">
-        <f>IF(Dados!$C$39=1,-Dados!$E$39,"")</f>
+        <f>IF(Dados!$C$39=1,Dados!$AG$39,"")</f>
         <v/>
       </c>
       <c r="M7" s="20">
-        <f>IF(Dados!$C$40=1,-Dados!$E$40,"")</f>
+        <f>IF(Dados!$C$40=1,Dados!$AG$40,"")</f>
         <v/>
       </c>
       <c r="N7" s="20">
-        <f>IF(Dados!$C$41=1,-Dados!$E$41,"")</f>
+        <f>IF(Dados!$C$41=1,Dados!$AG$41,"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="18" t="inlineStr">
         <is>
+          <t>− Pago</t>
+        </is>
+      </c>
+      <c r="C8" s="20">
+        <f>IF(Dados!$C$30=1,-Dados!$E$30,"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="20">
+        <f>IF(Dados!$C$31=1,-Dados!$E$31,"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="20">
+        <f>IF(Dados!$C$32=1,-Dados!$E$32,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="20">
+        <f>IF(Dados!$C$33=1,-Dados!$E$33,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="20">
+        <f>IF(Dados!$C$34=1,-Dados!$E$34,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="20">
+        <f>IF(Dados!$C$35=1,-Dados!$E$35,"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="20">
+        <f>IF(Dados!$C$36=1,-Dados!$E$36,"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="20">
+        <f>IF(Dados!$C$37=1,-Dados!$E$37,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="20">
+        <f>IF(Dados!$C$38=1,-Dados!$E$38,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="20">
+        <f>IF(Dados!$C$39=1,-Dados!$E$39,"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="20">
+        <f>IF(Dados!$C$40=1,-Dados!$E$40,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="20">
+        <f>IF(Dados!$C$41=1,-Dados!$E$41,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
           <t>± Ajuste ao extrato</t>
         </is>
       </c>
-      <c r="C8" s="20">
+      <c r="C9" s="20">
         <f>IF(Dados!$C$30=1,Dados!$I$30,"")</f>
         <v/>
       </c>
-      <c r="D8" s="20">
+      <c r="D9" s="20">
         <f>IF(Dados!$C$31=1,Dados!$I$31,"")</f>
         <v/>
       </c>
-      <c r="E8" s="20">
+      <c r="E9" s="20">
         <f>IF(Dados!$C$32=1,Dados!$I$32,"")</f>
         <v/>
       </c>
-      <c r="F8" s="20">
+      <c r="F9" s="20">
         <f>IF(Dados!$C$33=1,Dados!$I$33,"")</f>
         <v/>
       </c>
-      <c r="G8" s="20">
+      <c r="G9" s="20">
         <f>IF(Dados!$C$34=1,Dados!$I$34,"")</f>
         <v/>
       </c>
-      <c r="H8" s="20">
+      <c r="H9" s="20">
         <f>IF(Dados!$C$35=1,Dados!$I$35,"")</f>
         <v/>
       </c>
-      <c r="I8" s="20">
+      <c r="I9" s="20">
         <f>IF(Dados!$C$36=1,Dados!$I$36,"")</f>
         <v/>
       </c>
-      <c r="J8" s="20">
+      <c r="J9" s="20">
         <f>IF(Dados!$C$37=1,Dados!$I$37,"")</f>
         <v/>
       </c>
-      <c r="K8" s="20">
+      <c r="K9" s="20">
         <f>IF(Dados!$C$38=1,Dados!$I$38,"")</f>
         <v/>
       </c>
-      <c r="L8" s="20">
+      <c r="L9" s="20">
         <f>IF(Dados!$C$39=1,Dados!$I$39,"")</f>
         <v/>
       </c>
-      <c r="M8" s="20">
+      <c r="M9" s="20">
         <f>IF(Dados!$C$40=1,Dados!$I$40,"")</f>
         <v/>
       </c>
-      <c r="N8" s="20">
+      <c r="N9" s="20">
         <f>IF(Dados!$C$41=1,Dados!$I$41,"")</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="26" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Caixa final</t>
         </is>
       </c>
-      <c r="C9" s="27">
+      <c r="C10" s="27">
         <f>IF(Dados!$C$30=1,Dados!$G$30,"")</f>
         <v/>
       </c>
-      <c r="D9" s="27">
+      <c r="D10" s="27">
         <f>IF(Dados!$C$31=1,Dados!$G$31,"")</f>
         <v/>
       </c>
-      <c r="E9" s="27">
+      <c r="E10" s="27">
         <f>IF(Dados!$C$32=1,Dados!$G$32,"")</f>
         <v/>
       </c>
-      <c r="F9" s="27">
+      <c r="F10" s="27">
         <f>IF(Dados!$C$33=1,Dados!$G$33,"")</f>
         <v/>
       </c>
-      <c r="G9" s="27">
+      <c r="G10" s="27">
         <f>IF(Dados!$C$34=1,Dados!$G$34,"")</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H10" s="27">
         <f>IF(Dados!$C$35=1,Dados!$G$35,"")</f>
         <v/>
       </c>
-      <c r="I9" s="27">
+      <c r="I10" s="27">
         <f>IF(Dados!$C$36=1,Dados!$G$36,"")</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J10" s="27">
         <f>IF(Dados!$C$37=1,Dados!$G$37,"")</f>
         <v/>
       </c>
-      <c r="K9" s="27">
+      <c r="K10" s="27">
         <f>IF(Dados!$C$38=1,Dados!$G$38,"")</f>
         <v/>
       </c>
-      <c r="L9" s="27">
+      <c r="L10" s="27">
         <f>IF(Dados!$C$39=1,Dados!$G$39,"")</f>
         <v/>
       </c>
-      <c r="M9" s="27">
+      <c r="M10" s="27">
         <f>IF(Dados!$C$40=1,Dados!$G$40,"")</f>
         <v/>
       </c>
-      <c r="N9" s="27">
+      <c r="N10" s="27">
         <f>IF(Dados!$C$41=1,Dados!$G$41,"")</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="28" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="28" t="inlineStr">
         <is>
           <t>bloqueado em garantia</t>
         </is>
       </c>
-      <c r="C10" s="29">
+      <c r="C11" s="29">
         <f>IF(Dados!$C$30=1,Dados!$J$30,"")</f>
         <v/>
       </c>
-      <c r="D10" s="29">
+      <c r="D11" s="29">
         <f>IF(Dados!$C$31=1,Dados!$J$31,"")</f>
         <v/>
       </c>
-      <c r="E10" s="29">
+      <c r="E11" s="29">
         <f>IF(Dados!$C$32=1,Dados!$J$32,"")</f>
         <v/>
       </c>
-      <c r="F10" s="29">
+      <c r="F11" s="29">
         <f>IF(Dados!$C$33=1,Dados!$J$33,"")</f>
         <v/>
       </c>
-      <c r="G10" s="29">
+      <c r="G11" s="29">
         <f>IF(Dados!$C$34=1,Dados!$J$34,"")</f>
         <v/>
       </c>
-      <c r="H10" s="29">
+      <c r="H11" s="29">
         <f>IF(Dados!$C$35=1,Dados!$J$35,"")</f>
         <v/>
       </c>
-      <c r="I10" s="29">
+      <c r="I11" s="29">
         <f>IF(Dados!$C$36=1,Dados!$J$36,"")</f>
         <v/>
       </c>
-      <c r="J10" s="29">
+      <c r="J11" s="29">
         <f>IF(Dados!$C$37=1,Dados!$J$37,"")</f>
         <v/>
       </c>
-      <c r="K10" s="29">
+      <c r="K11" s="29">
         <f>IF(Dados!$C$38=1,Dados!$J$38,"")</f>
         <v/>
       </c>
-      <c r="L10" s="29">
+      <c r="L11" s="29">
         <f>IF(Dados!$C$39=1,Dados!$J$39,"")</f>
         <v/>
       </c>
-      <c r="M10" s="29">
+      <c r="M11" s="29">
         <f>IF(Dados!$C$40=1,Dados!$J$40,"")</f>
         <v/>
       </c>
-      <c r="N10" s="29">
+      <c r="N11" s="29">
         <f>IF(Dados!$C$41=1,Dados!$J$41,"")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="33" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>disponível</t>
         </is>
       </c>
-      <c r="C11" s="20">
+      <c r="C12" s="20">
         <f>IF(Dados!$C$30=1,Dados!$G$30-Dados!$J$30,"")</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D12" s="20">
         <f>IF(Dados!$C$31=1,Dados!$G$31-Dados!$J$31,"")</f>
         <v/>
       </c>
-      <c r="E11" s="20">
+      <c r="E12" s="20">
         <f>IF(Dados!$C$32=1,Dados!$G$32-Dados!$J$32,"")</f>
         <v/>
       </c>
-      <c r="F11" s="20">
+      <c r="F12" s="20">
         <f>IF(Dados!$C$33=1,Dados!$G$33-Dados!$J$33,"")</f>
         <v/>
       </c>
-      <c r="G11" s="20">
+      <c r="G12" s="20">
         <f>IF(Dados!$C$34=1,Dados!$G$34-Dados!$J$34,"")</f>
         <v/>
       </c>
-      <c r="H11" s="20">
+      <c r="H12" s="20">
         <f>IF(Dados!$C$35=1,Dados!$G$35-Dados!$J$35,"")</f>
         <v/>
       </c>
-      <c r="I11" s="20">
+      <c r="I12" s="20">
         <f>IF(Dados!$C$36=1,Dados!$G$36-Dados!$J$36,"")</f>
         <v/>
       </c>
-      <c r="J11" s="20">
+      <c r="J12" s="20">
         <f>IF(Dados!$C$37=1,Dados!$G$37-Dados!$J$37,"")</f>
         <v/>
       </c>
-      <c r="K11" s="20">
+      <c r="K12" s="20">
         <f>IF(Dados!$C$38=1,Dados!$G$38-Dados!$J$38,"")</f>
         <v/>
       </c>
-      <c r="L11" s="20">
+      <c r="L12" s="20">
         <f>IF(Dados!$C$39=1,Dados!$G$39-Dados!$J$39,"")</f>
         <v/>
       </c>
-      <c r="M11" s="20">
+      <c r="M12" s="20">
         <f>IF(Dados!$C$40=1,Dados!$G$40-Dados!$J$40,"")</f>
         <v/>
       </c>
-      <c r="N11" s="20">
+      <c r="N12" s="20">
         <f>IF(Dados!$C$41=1,Dados!$G$41-Dados!$J$41,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="28" t="inlineStr">
-        <is>
-          <t>Meses de despesa cobertos</t>
-        </is>
-      </c>
-      <c r="C12" s="34">
-        <f>IF(Dados!$C$30=1,IFERROR(C11/AVERAGE(Dados!$E$28:$E$30),""),"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="34">
-        <f>IF(Dados!$C$31=1,IFERROR(D11/AVERAGE(Dados!$E$29:$E$31),""),"")</f>
-        <v/>
-      </c>
-      <c r="E12" s="34">
-        <f>IF(Dados!$C$32=1,IFERROR(E11/AVERAGE(Dados!$E$30:$E$32),""),"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="34">
-        <f>IF(Dados!$C$33=1,IFERROR(F11/AVERAGE(Dados!$E$31:$E$33),""),"")</f>
-        <v/>
-      </c>
-      <c r="G12" s="34">
-        <f>IF(Dados!$C$34=1,IFERROR(G11/AVERAGE(Dados!$E$32:$E$34),""),"")</f>
-        <v/>
-      </c>
-      <c r="H12" s="34">
-        <f>IF(Dados!$C$35=1,IFERROR(H11/AVERAGE(Dados!$E$33:$E$35),""),"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="34">
-        <f>IF(Dados!$C$36=1,IFERROR(I11/AVERAGE(Dados!$E$34:$E$36),""),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="34">
-        <f>IF(Dados!$C$37=1,IFERROR(J11/AVERAGE(Dados!$E$35:$E$37),""),"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="34">
-        <f>IF(Dados!$C$38=1,IFERROR(K11/AVERAGE(Dados!$E$36:$E$38),""),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="34">
-        <f>IF(Dados!$C$39=1,IFERROR(L11/AVERAGE(Dados!$E$37:$E$39),""),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="34">
-        <f>IF(Dados!$C$40=1,IFERROR(M11/AVERAGE(Dados!$E$38:$E$40),""),"")</f>
-        <v/>
-      </c>
-      <c r="N12" s="34">
-        <f>IF(Dados!$C$41=1,IFERROR(N11/AVERAGE(Dados!$E$39:$E$41),""),"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="28" t="inlineStr">
         <is>
-          <t>Caixa final do ano anterior</t>
-        </is>
-      </c>
-      <c r="C13" s="29">
-        <f>IF(Dados!$C$18=1,Dados!$G$18,"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="29">
-        <f>IF(Dados!$C$19=1,Dados!$G$19,"")</f>
-        <v/>
-      </c>
-      <c r="E13" s="29">
-        <f>IF(Dados!$C$20=1,Dados!$G$20,"")</f>
-        <v/>
-      </c>
-      <c r="F13" s="29">
-        <f>IF(Dados!$C$21=1,Dados!$G$21,"")</f>
-        <v/>
-      </c>
-      <c r="G13" s="29">
-        <f>IF(Dados!$C$22=1,Dados!$G$22,"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="29">
-        <f>IF(Dados!$C$23=1,Dados!$G$23,"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="29">
-        <f>IF(Dados!$C$24=1,Dados!$G$24,"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="29">
-        <f>IF(Dados!$C$25=1,Dados!$G$25,"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="29">
-        <f>IF(Dados!$C$26=1,Dados!$G$26,"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="29">
-        <f>IF(Dados!$C$27=1,Dados!$G$27,"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="29">
-        <f>IF(Dados!$C$28=1,Dados!$G$28,"")</f>
-        <v/>
-      </c>
-      <c r="N13" s="29">
-        <f>IF(Dados!$C$29=1,Dados!$G$29,"")</f>
+          <t>Meses de despesa cobertos</t>
+        </is>
+      </c>
+      <c r="C13" s="34">
+        <f>IF(Dados!$C$30=1,IFERROR(C12/AVERAGE(Dados!$E$28:$E$30),""),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="34">
+        <f>IF(Dados!$C$31=1,IFERROR(D12/AVERAGE(Dados!$E$29:$E$31),""),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="34">
+        <f>IF(Dados!$C$32=1,IFERROR(E12/AVERAGE(Dados!$E$30:$E$32),""),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="34">
+        <f>IF(Dados!$C$33=1,IFERROR(F12/AVERAGE(Dados!$E$31:$E$33),""),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="34">
+        <f>IF(Dados!$C$34=1,IFERROR(G12/AVERAGE(Dados!$E$32:$E$34),""),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="34">
+        <f>IF(Dados!$C$35=1,IFERROR(H12/AVERAGE(Dados!$E$33:$E$35),""),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="34">
+        <f>IF(Dados!$C$36=1,IFERROR(I12/AVERAGE(Dados!$E$34:$E$36),""),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="34">
+        <f>IF(Dados!$C$37=1,IFERROR(J12/AVERAGE(Dados!$E$35:$E$37),""),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="34">
+        <f>IF(Dados!$C$38=1,IFERROR(K12/AVERAGE(Dados!$E$36:$E$38),""),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="34">
+        <f>IF(Dados!$C$39=1,IFERROR(L12/AVERAGE(Dados!$E$37:$E$39),""),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="34">
+        <f>IF(Dados!$C$40=1,IFERROR(M12/AVERAGE(Dados!$E$38:$E$40),""),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="34">
+        <f>IF(Dados!$C$41=1,IFERROR(N12/AVERAGE(Dados!$E$39:$E$41),""),"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="28" t="inlineStr">
         <is>
+          <t>Caixa final do ano anterior</t>
+        </is>
+      </c>
+      <c r="C14" s="29">
+        <f>IF(Dados!$C$18=1,Dados!$G$18,"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="29">
+        <f>IF(Dados!$C$19=1,Dados!$G$19,"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>IF(Dados!$C$20=1,Dados!$G$20,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="29">
+        <f>IF(Dados!$C$21=1,Dados!$G$21,"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="29">
+        <f>IF(Dados!$C$22=1,Dados!$G$22,"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="29">
+        <f>IF(Dados!$C$23=1,Dados!$G$23,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="29">
+        <f>IF(Dados!$C$24=1,Dados!$G$24,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="29">
+        <f>IF(Dados!$C$25=1,Dados!$G$25,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="29">
+        <f>IF(Dados!$C$26=1,Dados!$G$26,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="29">
+        <f>IF(Dados!$C$27=1,Dados!$G$27,"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="29">
+        <f>IF(Dados!$C$28=1,Dados!$G$28,"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="29">
+        <f>IF(Dados!$C$29=1,Dados!$G$29,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
           <t>Diferença na ponte (deve ser zero)</t>
         </is>
       </c>
-      <c r="C14" s="29">
-        <f>IF(C9="","",ROUND(C5+C6+C7+C8-C9,2))</f>
-        <v/>
-      </c>
-      <c r="D14" s="29">
-        <f>IF(D9="","",ROUND(D5+D6+D7+D8-D9,2))</f>
-        <v/>
-      </c>
-      <c r="E14" s="29">
-        <f>IF(E9="","",ROUND(E5+E6+E7+E8-E9,2))</f>
-        <v/>
-      </c>
-      <c r="F14" s="29">
-        <f>IF(F9="","",ROUND(F5+F6+F7+F8-F9,2))</f>
-        <v/>
-      </c>
-      <c r="G14" s="29">
-        <f>IF(G9="","",ROUND(G5+G6+G7+G8-G9,2))</f>
-        <v/>
-      </c>
-      <c r="H14" s="29">
-        <f>IF(H9="","",ROUND(H5+H6+H7+H8-H9,2))</f>
-        <v/>
-      </c>
-      <c r="I14" s="29">
-        <f>IF(I9="","",ROUND(I5+I6+I7+I8-I9,2))</f>
-        <v/>
-      </c>
-      <c r="J14" s="29">
-        <f>IF(J9="","",ROUND(J5+J6+J7+J8-J9,2))</f>
-        <v/>
-      </c>
-      <c r="K14" s="29">
-        <f>IF(K9="","",ROUND(K5+K6+K7+K8-K9,2))</f>
-        <v/>
-      </c>
-      <c r="L14" s="29">
-        <f>IF(L9="","",ROUND(L5+L6+L7+L8-L9,2))</f>
-        <v/>
-      </c>
-      <c r="M14" s="29">
-        <f>IF(M9="","",ROUND(M5+M6+M7+M8-M9,2))</f>
-        <v/>
-      </c>
-      <c r="N14" s="29">
-        <f>IF(N9="","",ROUND(N5+N6+N7+N8-N9,2))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="23" t="inlineStr">
-        <is>
-          <t>Meses de despesa cobertos: caixa disponível ÷ média do pago nos últimos 3 meses.</t>
+      <c r="C15" s="29">
+        <f>IF(C10="","",ROUND(C5+C6+C7+C8+C9-C10,2))</f>
+        <v/>
+      </c>
+      <c r="D15" s="29">
+        <f>IF(D10="","",ROUND(D5+D6+D7+D8+D9-D10,2))</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>IF(E10="","",ROUND(E5+E6+E7+E8+E9-E10,2))</f>
+        <v/>
+      </c>
+      <c r="F15" s="29">
+        <f>IF(F10="","",ROUND(F5+F6+F7+F8+F9-F10,2))</f>
+        <v/>
+      </c>
+      <c r="G15" s="29">
+        <f>IF(G10="","",ROUND(G5+G6+G7+G8+G9-G10,2))</f>
+        <v/>
+      </c>
+      <c r="H15" s="29">
+        <f>IF(H10="","",ROUND(H5+H6+H7+H8+H9-H10,2))</f>
+        <v/>
+      </c>
+      <c r="I15" s="29">
+        <f>IF(I10="","",ROUND(I5+I6+I7+I8+I9-I10,2))</f>
+        <v/>
+      </c>
+      <c r="J15" s="29">
+        <f>IF(J10="","",ROUND(J5+J6+J7+J8+J9-J10,2))</f>
+        <v/>
+      </c>
+      <c r="K15" s="29">
+        <f>IF(K10="","",ROUND(K5+K6+K7+K8+K9-K10,2))</f>
+        <v/>
+      </c>
+      <c r="L15" s="29">
+        <f>IF(L10="","",ROUND(L5+L6+L7+L8+L9-L10,2))</f>
+        <v/>
+      </c>
+      <c r="M15" s="29">
+        <f>IF(M10="","",ROUND(M5+M6+M7+M8+M9-M10,2))</f>
+        <v/>
+      </c>
+      <c r="N15" s="29">
+        <f>IF(N10="","",ROUND(N5+N6+N7+N8+N9-N10,2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Meses de despesa cobertos: caixa disponível ÷ média do pago nos últimos 3 meses. Rendimentos: CDB, reserva remunerada e CDI informados no fechamento.</t>
         </is>
       </c>
     </row>
@@ -10137,7 +10234,7 @@
       <formula>COLUMN(C4)-2=Dados!$AI$6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:N14">
+  <conditionalFormatting sqref="C5:N15">
     <cfRule type="expression" priority="2" dxfId="3">
       <formula>COLUMN(C5)-2=Dados!$AI$6</formula>
     </cfRule>

</xml_diff>